<commit_message>
Add Innotrust Gold schema data validation test cases and consolidated audit
</commit_message>
<xml_diff>
--- a/Gold_Data_Validation_Test_Cases.xlsx
+++ b/Gold_Data_Validation_Test_Cases.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Coverage Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="All Gold Tests (Master)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Black Diamond Gold" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Schwab Gold" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Salentica Gold" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Tamarac Gold" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Consolidated SK Audit" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Gold Tests (Master)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Black Diamond Gold" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schwab Gold" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salentica Gold" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tamarac Gold" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Innotrust Gold" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidated SK Audit" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -585,7 +586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -640,19 +641,19 @@
     </row>
     <row r="5" ht="28" customHeight="1">
       <c r="A5" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C5" s="4" t="n">
+        <v>57</v>
+      </c>
+      <c r="E5" s="4" t="n">
         <v>43</v>
       </c>
-      <c r="E5" s="4" t="n">
-        <v>32</v>
-      </c>
       <c r="F5" s="4" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" ht="26" customHeight="1">
@@ -816,32 +817,63 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="26" customHeight="1">
-      <c r="A12" s="14" t="inlineStr">
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Innotrust</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>innotrust</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>11</v>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>TC_COMB_SK_INNO_05</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>All 5 dimensions: dim_account_master, category_codes, type_codes, sec_index, characteristics</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="26" customHeight="1">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B12" s="14" t="inlineStr">
-        <is>
-          <t>All 4 Gold Schemas</t>
-        </is>
-      </c>
-      <c r="C12" s="15" t="n">
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>All 5 Gold Schemas</t>
+        </is>
+      </c>
+      <c r="C13" s="15" t="n">
+        <v>57</v>
+      </c>
+      <c r="D13" s="15" t="n">
         <v>43</v>
       </c>
-      <c r="D12" s="15" t="n">
-        <v>32</v>
-      </c>
-      <c r="E12" s="15" t="n">
-        <v>11</v>
-      </c>
-      <c r="F12" s="15" t="inlineStr">
-        <is>
-          <t>4 Combined Audits</t>
-        </is>
-      </c>
-      <c r="G12" s="14" t="inlineStr">
+      <c r="E13" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="F13" s="15" t="inlineStr">
+        <is>
+          <t>5 Combined Audits</t>
+        </is>
+      </c>
+      <c r="G13" s="14" t="inlineStr">
         <is>
           <t>100% Core Verification</t>
         </is>
@@ -866,7 +898,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I45"/>
+  <dimension ref="A1:I59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2971,45 +3003,715 @@
     <row r="42" ht="54" customHeight="1">
       <c r="A42" s="8" t="inlineStr">
         <is>
+          <t>Innotrust</t>
+        </is>
+      </c>
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>TC_INNO_GOLD_01</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>SCD2 Deduplication</t>
+        </is>
+      </c>
+      <c r="D42" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_master</t>
+        </is>
+      </c>
+      <c r="F42" s="7" t="inlineStr">
+        <is>
+          <t>Verify Active Deduplication on Business Key ['customer_account_number'] (is_current = 1)</t>
+        </is>
+      </c>
+      <c r="G42" s="7" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_master populated</t>
+        </is>
+      </c>
+      <c r="H42" s="7" t="inlineStr">
+        <is>
+          <t>Zero duplicate active accounts. Exactly one is_current = 1 record per customer_account_number.</t>
+        </is>
+      </c>
+      <c r="I42" s="18" t="inlineStr">
+        <is>
+          <t>SELECT customer_account_number, COUNT(*) AS ActiveDuplicateCount
+FROM Gold_Warehouse.innotrust.dim_account_master
+WHERE is_current = 1
+GROUP BY customer_account_number
+HAVING COUNT(*) &gt; 1;</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="54" customHeight="1">
+      <c r="A43" s="12" t="inlineStr">
+        <is>
+          <t>Innotrust</t>
+        </is>
+      </c>
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>TC_INNO_GOLD_02</t>
+        </is>
+      </c>
+      <c r="C43" s="13" t="inlineStr">
+        <is>
+          <t>SK Uniqueness</t>
+        </is>
+      </c>
+      <c r="D43" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E43" s="10" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_master</t>
+        </is>
+      </c>
+      <c r="F43" s="11" t="inlineStr">
+        <is>
+          <t>Verify Primary Surrogate Key (dim_account_master_sk) uniqueness and non-null constraint</t>
+        </is>
+      </c>
+      <c r="G43" s="11" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_master populated</t>
+        </is>
+      </c>
+      <c r="H43" s="11" t="inlineStr">
+        <is>
+          <t>dim_account_master_sk is strictly unique across all versions with zero NULL values.</t>
+        </is>
+      </c>
+      <c r="I43" s="17" t="inlineStr">
+        <is>
+          <t>SELECT dim_account_master_sk, COUNT(*) AS DuplicateCount
+FROM Gold_Warehouse.innotrust.dim_account_master
+GROUP BY dim_account_master_sk
+HAVING COUNT(*) &gt; 1
+UNION ALL
+SELECT NULL, COUNT(*)
+FROM Gold_Warehouse.innotrust.dim_account_master
+WHERE dim_account_master_sk IS NULL
+HAVING COUNT(*) &gt; 0;</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="54" customHeight="1">
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>Innotrust</t>
+        </is>
+      </c>
+      <c r="B44" s="8" t="inlineStr">
+        <is>
+          <t>TC_INNO_GOLD_03</t>
+        </is>
+      </c>
+      <c r="C44" s="9" t="inlineStr">
+        <is>
+          <t>SCD2 Deduplication</t>
+        </is>
+      </c>
+      <c r="D44" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E44" s="6" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_category_codes</t>
+        </is>
+      </c>
+      <c r="F44" s="7" t="inlineStr">
+        <is>
+          <t>Verify Active Deduplication on Business Key ['account_category_code'] (is_current = 1)</t>
+        </is>
+      </c>
+      <c r="G44" s="7" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_category_codes populated</t>
+        </is>
+      </c>
+      <c r="H44" s="7" t="inlineStr">
+        <is>
+          <t>Zero duplicate active category codes per account_category_code.</t>
+        </is>
+      </c>
+      <c r="I44" s="18" t="inlineStr">
+        <is>
+          <t>SELECT account_category_code, COUNT(*) AS ActiveDuplicateCount
+FROM Gold_Warehouse.innotrust.dim_account_category_codes
+WHERE is_current = 1
+GROUP BY account_category_code
+HAVING COUNT(*) &gt; 1;</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="54" customHeight="1">
+      <c r="A45" s="12" t="inlineStr">
+        <is>
+          <t>Innotrust</t>
+        </is>
+      </c>
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>TC_INNO_GOLD_04</t>
+        </is>
+      </c>
+      <c r="C45" s="13" t="inlineStr">
+        <is>
+          <t>SK Uniqueness</t>
+        </is>
+      </c>
+      <c r="D45" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E45" s="10" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_category_codes</t>
+        </is>
+      </c>
+      <c r="F45" s="11" t="inlineStr">
+        <is>
+          <t>Verify Primary Surrogate Key (dim_account_master_sk) uniqueness on dim_account_category_codes</t>
+        </is>
+      </c>
+      <c r="G45" s="11" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_category_codes populated</t>
+        </is>
+      </c>
+      <c r="H45" s="11" t="inlineStr">
+        <is>
+          <t>Surrogate key dim_account_master_sk is unique across all rows with zero NULLs.</t>
+        </is>
+      </c>
+      <c r="I45" s="17" t="inlineStr">
+        <is>
+          <t>SELECT dim_account_master_sk, COUNT(*) AS DuplicateCount
+FROM Gold_Warehouse.innotrust.dim_account_category_codes
+GROUP BY dim_account_master_sk
+HAVING COUNT(*) &gt; 1;</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="54" customHeight="1">
+      <c r="A46" s="8" t="inlineStr">
+        <is>
+          <t>Innotrust</t>
+        </is>
+      </c>
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>TC_INNO_GOLD_05</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="inlineStr">
+        <is>
+          <t>SCD2 Deduplication</t>
+        </is>
+      </c>
+      <c r="D46" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_type_codes</t>
+        </is>
+      </c>
+      <c r="F46" s="7" t="inlineStr">
+        <is>
+          <t>Verify Active Deduplication on Business Key ['account_type_code'] (is_current = 1)</t>
+        </is>
+      </c>
+      <c r="G46" s="7" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_type_codes populated</t>
+        </is>
+      </c>
+      <c r="H46" s="7" t="inlineStr">
+        <is>
+          <t>Zero duplicate active account types per account_type_code.</t>
+        </is>
+      </c>
+      <c r="I46" s="18" t="inlineStr">
+        <is>
+          <t>SELECT account_type_code, COUNT(*) AS ActiveDuplicateCount
+FROM Gold_Warehouse.innotrust.dim_account_type_codes
+WHERE is_current = 1
+GROUP BY account_type_code
+HAVING COUNT(*) &gt; 1;</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="54" customHeight="1">
+      <c r="A47" s="12" t="inlineStr">
+        <is>
+          <t>Innotrust</t>
+        </is>
+      </c>
+      <c r="B47" s="12" t="inlineStr">
+        <is>
+          <t>TC_INNO_GOLD_06</t>
+        </is>
+      </c>
+      <c r="C47" s="13" t="inlineStr">
+        <is>
+          <t>SK Uniqueness</t>
+        </is>
+      </c>
+      <c r="D47" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E47" s="10" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_type_codes</t>
+        </is>
+      </c>
+      <c r="F47" s="11" t="inlineStr">
+        <is>
+          <t>Verify Primary Surrogate Key (dim_account_type_codes_sk) uniqueness and non-null constraint</t>
+        </is>
+      </c>
+      <c r="G47" s="11" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_type_codes populated</t>
+        </is>
+      </c>
+      <c r="H47" s="11" t="inlineStr">
+        <is>
+          <t>dim_account_type_codes_sk is strictly unique across all versions with zero NULLs.</t>
+        </is>
+      </c>
+      <c r="I47" s="17" t="inlineStr">
+        <is>
+          <t>SELECT dim_account_type_codes_sk, COUNT(*) AS DuplicateCount
+FROM Gold_Warehouse.innotrust.dim_account_type_codes
+GROUP BY dim_account_type_codes_sk
+HAVING COUNT(*) &gt; 1;</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="54" customHeight="1">
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>Innotrust</t>
+        </is>
+      </c>
+      <c r="B48" s="8" t="inlineStr">
+        <is>
+          <t>TC_INNO_GOLD_07</t>
+        </is>
+      </c>
+      <c r="C48" s="9" t="inlineStr">
+        <is>
+          <t>SCD2 Deduplication</t>
+        </is>
+      </c>
+      <c r="D48" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="inlineStr">
+        <is>
+          <t>innotrust.dim_master_sec_index</t>
+        </is>
+      </c>
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t>Verify Active Deduplication on Security Primary Key ['isin'] (is_current = 1)</t>
+        </is>
+      </c>
+      <c r="G48" s="7" t="inlineStr">
+        <is>
+          <t>innotrust.dim_master_sec_index populated</t>
+        </is>
+      </c>
+      <c r="H48" s="7" t="inlineStr">
+        <is>
+          <t>Zero duplicate active securities. Exactly one is_current = 1 record per isin.</t>
+        </is>
+      </c>
+      <c r="I48" s="18" t="inlineStr">
+        <is>
+          <t>SELECT isin, COUNT(*) AS ActiveDuplicateCount
+FROM Gold_Warehouse.innotrust.dim_master_sec_index
+WHERE is_current = 1
+GROUP BY isin
+HAVING COUNT(*) &gt; 1;</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="54" customHeight="1">
+      <c r="A49" s="12" t="inlineStr">
+        <is>
+          <t>Innotrust</t>
+        </is>
+      </c>
+      <c r="B49" s="12" t="inlineStr">
+        <is>
+          <t>TC_INNO_GOLD_08</t>
+        </is>
+      </c>
+      <c r="C49" s="13" t="inlineStr">
+        <is>
+          <t>SK Uniqueness</t>
+        </is>
+      </c>
+      <c r="D49" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E49" s="10" t="inlineStr">
+        <is>
+          <t>innotrust.dim_master_sec_index</t>
+        </is>
+      </c>
+      <c r="F49" s="11" t="inlineStr">
+        <is>
+          <t>Verify Primary Surrogate Key (dim_master_sec_index_sk) uniqueness across all records</t>
+        </is>
+      </c>
+      <c r="G49" s="11" t="inlineStr">
+        <is>
+          <t>innotrust.dim_master_sec_index populated</t>
+        </is>
+      </c>
+      <c r="H49" s="11" t="inlineStr">
+        <is>
+          <t>dim_master_sec_index_sk is strictly unique across all versions with zero NULLs.</t>
+        </is>
+      </c>
+      <c r="I49" s="17" t="inlineStr">
+        <is>
+          <t>SELECT dim_master_sec_index_sk, COUNT(*) AS DuplicateCount
+FROM Gold_Warehouse.innotrust.dim_master_sec_index
+GROUP BY dim_master_sec_index_sk
+HAVING COUNT(*) &gt; 1;</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="54" customHeight="1">
+      <c r="A50" s="8" t="inlineStr">
+        <is>
+          <t>Innotrust</t>
+        </is>
+      </c>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>TC_INNO_GOLD_09</t>
+        </is>
+      </c>
+      <c r="C50" s="9" t="inlineStr">
+        <is>
+          <t>SCD2 Deduplication</t>
+        </is>
+      </c>
+      <c r="D50" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="inlineStr">
+        <is>
+          <t>innotrust.dim_security_characteristics_codes</t>
+        </is>
+      </c>
+      <c r="F50" s="7" t="inlineStr">
+        <is>
+          <t>Verify Active Deduplication on Business Key ['security_type_code'] (is_current = 1)</t>
+        </is>
+      </c>
+      <c r="G50" s="7" t="inlineStr">
+        <is>
+          <t>innotrust.dim_security_characteristics_codes populated</t>
+        </is>
+      </c>
+      <c r="H50" s="7" t="inlineStr">
+        <is>
+          <t>Zero duplicate active security type codes per security_type_code.</t>
+        </is>
+      </c>
+      <c r="I50" s="18" t="inlineStr">
+        <is>
+          <t>SELECT security_type_code, COUNT(*) AS ActiveDuplicateCount
+FROM Gold_Warehouse.innotrust.dim_security_characteristics_codes
+WHERE is_current = 1
+GROUP BY security_type_code
+HAVING COUNT(*) &gt; 1;</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="54" customHeight="1">
+      <c r="A51" s="12" t="inlineStr">
+        <is>
+          <t>Innotrust</t>
+        </is>
+      </c>
+      <c r="B51" s="12" t="inlineStr">
+        <is>
+          <t>TC_INNO_GOLD_10</t>
+        </is>
+      </c>
+      <c r="C51" s="13" t="inlineStr">
+        <is>
+          <t>SK Uniqueness</t>
+        </is>
+      </c>
+      <c r="D51" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E51" s="10" t="inlineStr">
+        <is>
+          <t>innotrust.dim_security_characteristics_codes</t>
+        </is>
+      </c>
+      <c r="F51" s="11" t="inlineStr">
+        <is>
+          <t>Verify Primary Surrogate Key (dim_securitycharacteristicscodes) uniqueness and non-null constraint</t>
+        </is>
+      </c>
+      <c r="G51" s="11" t="inlineStr">
+        <is>
+          <t>innotrust.dim_security_characteristics_codes populated</t>
+        </is>
+      </c>
+      <c r="H51" s="11" t="inlineStr">
+        <is>
+          <t>dim_securitycharacteristicscodes is strictly unique across all versions with zero NULLs.</t>
+        </is>
+      </c>
+      <c r="I51" s="17" t="inlineStr">
+        <is>
+          <t>SELECT dim_securitycharacteristicscodes, COUNT(*) AS DuplicateCount
+FROM Gold_Warehouse.innotrust.dim_security_characteristics_codes
+GROUP BY dim_securitycharacteristicscodes
+HAVING COUNT(*) &gt; 1;</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="54" customHeight="1">
+      <c r="A52" s="8" t="inlineStr">
+        <is>
+          <t>Innotrust</t>
+        </is>
+      </c>
+      <c r="B52" s="8" t="inlineStr">
+        <is>
+          <t>TC_INNO_GOLD_11</t>
+        </is>
+      </c>
+      <c r="C52" s="9" t="inlineStr">
+        <is>
+          <t>Audit &amp; Date Logic</t>
+        </is>
+      </c>
+      <c r="D52" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E52" s="6" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_master</t>
+        </is>
+      </c>
+      <c r="F52" s="7" t="inlineStr">
+        <is>
+          <t>Verify business_date, updated_at, effective_start_date &amp; effective_end_date integrity on active records</t>
+        </is>
+      </c>
+      <c r="G52" s="7" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_master populated</t>
+        </is>
+      </c>
+      <c r="H52" s="7" t="inlineStr">
+        <is>
+          <t>Zero NULLs in business_date or updated_at; effective_end_date &gt;= effective_start_date.</t>
+        </is>
+      </c>
+      <c r="I52" s="18" t="inlineStr">
+        <is>
+          <t>SELECT 
+    COUNT(*) AS TotalActiveRows,
+    SUM(CASE WHEN business_date IS NULL THEN 1 ELSE 0 END) AS Null_BusinessDate,
+    SUM(CASE WHEN updated_at IS NULL THEN 1 ELSE 0 END) AS Null_UpdatedAt,
+    SUM(CASE WHEN effective_start_date IS NULL THEN 1 ELSE 0 END) AS Null_EffectiveStartDate,
+    SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) AS InvertedEffectiveDates
+FROM Gold_Warehouse.innotrust.dim_account_master
+WHERE is_current = 1;</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="54" customHeight="1">
+      <c r="A53" s="12" t="inlineStr">
+        <is>
+          <t>Innotrust</t>
+        </is>
+      </c>
+      <c r="B53" s="12" t="inlineStr">
+        <is>
+          <t>TC_INNO_GOLD_12</t>
+        </is>
+      </c>
+      <c r="C53" s="13" t="inlineStr">
+        <is>
+          <t>Cross-Table Linkage</t>
+        </is>
+      </c>
+      <c r="D53" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E53" s="10" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_master</t>
+        </is>
+      </c>
+      <c r="F53" s="11" t="inlineStr">
+        <is>
+          <t>Verify Referential Integrity: account_category_code and account_type_code resolve to active codes</t>
+        </is>
+      </c>
+      <c r="G53" s="11" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_master populated</t>
+        </is>
+      </c>
+      <c r="H53" s="11" t="inlineStr">
+        <is>
+          <t>All non-null account_category_code and account_type_code exist in corresponding dimension code tables.</t>
+        </is>
+      </c>
+      <c r="I53" s="17" t="inlineStr">
+        <is>
+          <t>SELECT 
+    SUM(CASE WHEN m.account_category_code IS NOT NULL AND cat.account_category_code IS NULL THEN 1 ELSE 0 END) AS Orphan_CategoryCodes,
+    SUM(CASE WHEN m.account_type_code IS NOT NULL AND typ.account_type_code IS NULL THEN 1 ELSE 0 END) AS Orphan_TypeCodes
+FROM Gold_Warehouse.innotrust.dim_account_master m
+LEFT JOIN Gold_Warehouse.innotrust.dim_account_category_codes cat 
+    ON m.account_category_code = cat.account_category_code AND cat.is_current = 1
+LEFT JOIN Gold_Warehouse.innotrust.dim_account_type_codes typ 
+    ON m.account_type_code = typ.account_type_code AND typ.is_current = 1
+WHERE m.is_current = 1;</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="54" customHeight="1">
+      <c r="A54" s="8" t="inlineStr">
+        <is>
+          <t>Innotrust</t>
+        </is>
+      </c>
+      <c r="B54" s="8" t="inlineStr">
+        <is>
+          <t>TC_INNO_GOLD_13</t>
+        </is>
+      </c>
+      <c r="C54" s="9" t="inlineStr">
+        <is>
+          <t>Cross-Table Linkage</t>
+        </is>
+      </c>
+      <c r="D54" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="inlineStr">
+        <is>
+          <t>innotrust.dim_master_sec_index</t>
+        </is>
+      </c>
+      <c r="F54" s="7" t="inlineStr">
+        <is>
+          <t>Verify Security Referential Integrity: security_type_code resolves to active security characteristics</t>
+        </is>
+      </c>
+      <c r="G54" s="7" t="inlineStr">
+        <is>
+          <t>innotrust.dim_master_sec_index populated</t>
+        </is>
+      </c>
+      <c r="H54" s="7" t="inlineStr">
+        <is>
+          <t>All non-null security_type_code values exist in dim_security_characteristics_codes.</t>
+        </is>
+      </c>
+      <c r="I54" s="18" t="inlineStr">
+        <is>
+          <t>SELECT COUNT(*) AS Orphan_SecurityTypeCodes
+FROM Gold_Warehouse.innotrust.dim_master_sec_index s
+LEFT JOIN Gold_Warehouse.innotrust.dim_security_characteristics_codes sc 
+    ON s.security_type_code = sc.security_type_code AND sc.is_current = 1
+WHERE s.is_current = 1 AND s.security_type_code IS NOT NULL AND sc.security_type_code IS NULL;</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="54" customHeight="1">
+      <c r="A55" s="12" t="inlineStr">
+        <is>
           <t>Black Diamond (Consolidated)</t>
         </is>
       </c>
-      <c r="B42" s="8" t="inlineStr">
+      <c r="B55" s="12" t="inlineStr">
         <is>
           <t>TC_COMB_SK_BD_01</t>
         </is>
       </c>
-      <c r="C42" s="9" t="inlineStr">
+      <c r="C55" s="13" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D42" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E42" s="6" t="inlineStr">
+      <c r="D55" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E55" s="10" t="inlineStr">
         <is>
           <t>All 9 Child &amp; Fact Tables (holdings, transactions, taxlots, class/segment, details, tags, team, targets)</t>
         </is>
       </c>
-      <c r="F42" s="7" t="inlineStr">
+      <c r="F55" s="11" t="inlineStr">
         <is>
           <t>Black Diamond: Cross-Object account_sk vs dim_accounts Natural Key (accountid == da.id) Verification - Executes a single consolidated UNION ALL query across all 9 child/fact tables to verify that the attached account_sk strictly points to the exact same account natural key (child.accountid == da.id). Guarantees zero wrong account links.</t>
         </is>
       </c>
-      <c r="G42" s="7" t="inlineStr">
+      <c r="G55" s="11" t="inlineStr">
         <is>
           <t>All Gold tables populated for Black Diamond</t>
         </is>
       </c>
-      <c r="H42" s="7" t="inlineStr">
+      <c r="H55" s="11" t="inlineStr">
         <is>
           <t>Duplicate_BusinessKey_Count = 0, MismatchedAccountIdCount = 0, Null_AccountSK_Count = 0, Orphan_AccountSK_Count = 0 across all 9 objects.</t>
         </is>
       </c>
-      <c r="I42" s="18" t="inlineStr">
+      <c r="I55" s="17" t="inlineStr">
         <is>
           <t>SELECT 
     'dim_accounts_classallocation' AS TableName, 
@@ -3118,48 +3820,48 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="54" customHeight="1">
-      <c r="A43" s="12" t="inlineStr">
+    <row r="56" ht="54" customHeight="1">
+      <c r="A56" s="8" t="inlineStr">
         <is>
           <t>Schwab (Consolidated)</t>
         </is>
       </c>
-      <c r="B43" s="12" t="inlineStr">
+      <c r="B56" s="8" t="inlineStr">
         <is>
           <t>TC_COMB_SK_SC_02</t>
         </is>
       </c>
-      <c r="C43" s="13" t="inlineStr">
+      <c r="C56" s="9" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D43" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E43" s="10" t="inlineStr">
+      <c r="D56" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E56" s="6" t="inlineStr">
         <is>
           <t>All 8 Objects (dim_accounts &amp; 7 Fact Tables: recon_d1/d2, daily_closing, security, transactions, ult/uln lots)</t>
         </is>
       </c>
-      <c r="F43" s="11" t="inlineStr">
+      <c r="F56" s="7" t="inlineStr">
         <is>
           <t>Schwab: Consolidated Multi-Object SK Mapping, PK Deduplication &amp; Audit Date Health Check - Single unified query executing across all 8 Schwab Gold tables. Validates that every fact record's account_sk correctly matches dim_accounts on composite natural keys (account_id, custodian_id), confirms primary SK uniqueness, and ensures 100% audit dates populated.</t>
         </is>
       </c>
-      <c r="G43" s="11" t="inlineStr">
+      <c r="G56" s="7" t="inlineStr">
         <is>
           <t>All Gold tables populated for Schwab</t>
         </is>
       </c>
-      <c r="H43" s="11" t="inlineStr">
+      <c r="H56" s="7" t="inlineStr">
         <is>
           <t>Mismatched_AccountId_Count = 0 and Orphan_AccountSK_Count = 0 across all fact tables. All mapped account_sk strictly match the natural account_id.</t>
         </is>
       </c>
-      <c r="I43" s="17" t="inlineStr">
+      <c r="I56" s="18" t="inlineStr">
         <is>
           <t>SELECT 
     'fact_recon_position_d1' AS TableName,
@@ -3218,48 +3920,48 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="54" customHeight="1">
-      <c r="A44" s="8" t="inlineStr">
+    <row r="57" ht="54" customHeight="1">
+      <c r="A57" s="12" t="inlineStr">
         <is>
           <t>Salentica CRM (Consolidated)</t>
         </is>
       </c>
-      <c r="B44" s="8" t="inlineStr">
+      <c r="B57" s="12" t="inlineStr">
         <is>
           <t>TC_COMB_SK_SAL_03</t>
         </is>
       </c>
-      <c r="C44" s="9" t="inlineStr">
+      <c r="C57" s="13" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D44" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E44" s="6" t="inlineStr">
+      <c r="D57" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E57" s="10" t="inlineStr">
         <is>
           <t>All 6 Core CRM Entities (dim_account, dim_contact_core, dim_family, fact_lead, fact_opportunity, fact_investmentaccount)</t>
         </is>
       </c>
-      <c r="F44" s="7" t="inlineStr">
+      <c r="F57" s="11" t="inlineStr">
         <is>
           <t>Salentica: Consolidated Point-in-Time Referential SK Mapping (Active &amp; Historical Mapping Validation) - Single unified query executing across all 6 core Salentica CRM tables. Validates that every attached foreign SK resolves to the same Natural Key in parent dimensions (allowing active OR expired parent versions to preserve point-in-time audit history) and checks for broken orphans.</t>
         </is>
       </c>
-      <c r="G44" s="7" t="inlineStr">
+      <c r="G57" s="11" t="inlineStr">
         <is>
           <t>All Gold tables populated for Salentica CRM</t>
         </is>
       </c>
-      <c r="H44" s="7" t="inlineStr">
+      <c r="H57" s="11" t="inlineStr">
         <is>
           <t>Mismatched_PrimaryContact_NK = 0, Mismatched_BusinessUnit_NK = 0, Broken_Orphan_Count = 0 across all 6 CRM tables.</t>
         </is>
       </c>
-      <c r="I44" s="18" t="inlineStr">
+      <c r="I57" s="17" t="inlineStr">
         <is>
           <t>SELECT 'dim_account' AS TableName, COUNT(*) AS TotalActiveRows,
     SUM(CASE WHEN a.primarycontactid IS NOT NULL AND a.primarycontactid_sk &lt;&gt; -1 AND a.primarycontactid &lt;&gt; c.contactid THEN 1 ELSE 0 END) AS Mismatched_PrimaryContact_NK,
@@ -3323,48 +4025,48 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="54" customHeight="1">
-      <c r="A45" s="12" t="inlineStr">
+    <row r="58" ht="54" customHeight="1">
+      <c r="A58" s="8" t="inlineStr">
         <is>
           <t>Tamarac (Consolidated)</t>
         </is>
       </c>
-      <c r="B45" s="12" t="inlineStr">
+      <c r="B58" s="8" t="inlineStr">
         <is>
           <t>TC_COMB_SK_TAM_04</t>
         </is>
       </c>
-      <c r="C45" s="13" t="inlineStr">
+      <c r="C58" s="9" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D45" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E45" s="10" t="inlineStr">
+      <c r="D58" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="inlineStr">
         <is>
           <t>Both Tables (dim_account_information, dim_account_model_allocation)</t>
         </is>
       </c>
-      <c r="F45" s="11" t="inlineStr">
+      <c r="F58" s="7" t="inlineStr">
         <is>
           <t>Tamarac: Consolidated Multi-Object PK Deduplication, Primary SK &amp; Cross-Table Linkage - Single unified query validating SCD2 active uniqueness on exact PK columns (['account_number'] and ['account_number', 'model_name']), surrogate key uniqueness, and cross-table referential integrity between model allocations and accounts.</t>
         </is>
       </c>
-      <c r="G45" s="11" t="inlineStr">
+      <c r="G58" s="7" t="inlineStr">
         <is>
           <t>All Gold tables populated for Tamarac</t>
         </is>
       </c>
-      <c r="H45" s="11" t="inlineStr">
+      <c r="H58" s="7" t="inlineStr">
         <is>
           <t>PK_Active_Duplicates = 0, Duplicate_Primary_SK = 0, Orphan_Accounts = 0, Missing_BusinessDate = 0 across both tables.</t>
         </is>
       </c>
-      <c r="I45" s="17" t="inlineStr">
+      <c r="I58" s="18" t="inlineStr">
         <is>
           <t>SELECT 'dim_account_information' AS TableName, COUNT(*) AS TotalActiveRows,
     (SELECT COUNT(*) FROM (SELECT account_number FROM Gold_Warehouse.tamarac.dim_account_information WHERE is_current = 'True' GROUP BY account_number HAVING COUNT(*) &gt; 1) d) AS PK_Active_Duplicates,
@@ -3384,6 +4086,97 @@
 LEFT JOIN Gold_Warehouse.tamarac.dim_account_information info 
     ON ma.account_number = info.account_number AND info.is_current = 'True'
 WHERE ma.is_current = 'True';</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="54" customHeight="1">
+      <c r="A59" s="12" t="inlineStr">
+        <is>
+          <t>Innotrust (Consolidated)</t>
+        </is>
+      </c>
+      <c r="B59" s="12" t="inlineStr">
+        <is>
+          <t>TC_COMB_SK_INNO_05</t>
+        </is>
+      </c>
+      <c r="C59" s="13" t="inlineStr">
+        <is>
+          <t>Consolidated Multi-Object SK Audit</t>
+        </is>
+      </c>
+      <c r="D59" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E59" s="10" t="inlineStr">
+        <is>
+          <t>All 5 Innotrust Dimensions (dim_account_master, category_codes, type_codes, sec_index, characteristics)</t>
+        </is>
+      </c>
+      <c r="F59" s="11" t="inlineStr">
+        <is>
+          <t>Innotrust: Consolidated Multi-Object PK Deduplication, Primary SK &amp; Cross-Dimension Linkage - Single unified query validating SCD2 active uniqueness on exact natural keys, primary surrogate key uniqueness, and cross-dimension referential integrity between master entities and classification codes.</t>
+        </is>
+      </c>
+      <c r="G59" s="11" t="inlineStr">
+        <is>
+          <t>All Gold tables populated for Innotrust</t>
+        </is>
+      </c>
+      <c r="H59" s="11" t="inlineStr">
+        <is>
+          <t>PK_Active_Duplicates = 0, Duplicate_Primary_SK = 0, Orphan_Foreign_References = 0, Missing_BusinessDate = 0 across all 5 Innotrust tables.</t>
+        </is>
+      </c>
+      <c r="I59" s="17" t="inlineStr">
+        <is>
+          <t>SELECT 'dim_account_master' AS TableName, COUNT(*) AS TotalActiveRows,
+    (SELECT COUNT(*) FROM (SELECT customer_account_number FROM Gold_Warehouse.innotrust.dim_account_master WHERE is_current = 1 GROUP BY customer_account_number HAVING COUNT(*) &gt; 1) d) AS PK_Active_Duplicates,
+    (COUNT(*) - COUNT(DISTINCT dim_account_master_sk)) AS Duplicate_Primary_SK,
+    SUM(CASE WHEN (m.account_category_code IS NOT NULL AND cat.account_category_code IS NULL)
+               OR (m.account_type_code IS NOT NULL AND typ.account_type_code IS NULL) THEN 1 ELSE 0 END) AS Orphan_Foreign_References,
+    SUM(CASE WHEN m.business_date IS NULL THEN 1 ELSE 0 END) AS Missing_BusinessDate,
+    SUM(CASE WHEN m.updated_at IS NULL THEN 1 ELSE 0 END) AS Missing_UpdatedAt
+FROM Gold_Warehouse.innotrust.dim_account_master m
+LEFT JOIN Gold_Warehouse.innotrust.dim_account_category_codes cat ON m.account_category_code = cat.account_category_code AND cat.is_current = 1
+LEFT JOIN Gold_Warehouse.innotrust.dim_account_type_codes typ ON m.account_type_code = typ.account_type_code AND typ.is_current = 1
+WHERE m.is_current = 1
+UNION ALL
+SELECT 'dim_account_category_codes', COUNT(*),
+    (SELECT COUNT(*) FROM (SELECT account_category_code FROM Gold_Warehouse.innotrust.dim_account_category_codes WHERE is_current = 1 GROUP BY account_category_code HAVING COUNT(*) &gt; 1) d),
+    (COUNT(*) - COUNT(DISTINCT dim_account_master_sk)),
+    0,
+    SUM(CASE WHEN business_date IS NULL THEN 1 ELSE 0 END),
+    SUM(CASE WHEN updated_at IS NULL THEN 1 ELSE 0 END)
+FROM Gold_Warehouse.innotrust.dim_account_category_codes WHERE is_current = 1
+UNION ALL
+SELECT 'dim_account_type_codes', COUNT(*),
+    (SELECT COUNT(*) FROM (SELECT account_type_code FROM Gold_Warehouse.innotrust.dim_account_type_codes WHERE is_current = 1 GROUP BY account_type_code HAVING COUNT(*) &gt; 1) d),
+    (COUNT(*) - COUNT(DISTINCT dim_account_type_codes_sk)),
+    0,
+    SUM(CASE WHEN business_date IS NULL THEN 1 ELSE 0 END),
+    SUM(CASE WHEN updated_at IS NULL THEN 1 ELSE 0 END)
+FROM Gold_Warehouse.innotrust.dim_account_type_codes WHERE is_current = 1
+UNION ALL
+SELECT 'dim_master_sec_index', COUNT(*),
+    (SELECT COUNT(*) FROM (SELECT isin FROM Gold_Warehouse.innotrust.dim_master_sec_index WHERE is_current = 1 GROUP BY isin HAVING COUNT(*) &gt; 1) d),
+    (COUNT(*) - COUNT(DISTINCT dim_master_sec_index_sk)),
+    SUM(CASE WHEN s.security_type_code IS NOT NULL AND sc.security_type_code IS NULL THEN 1 ELSE 0 END),
+    SUM(CASE WHEN s.business_date IS NULL THEN 1 ELSE 0 END),
+    SUM(CASE WHEN s.updated_at IS NULL THEN 1 ELSE 0 END)
+FROM Gold_Warehouse.innotrust.dim_master_sec_index s
+LEFT JOIN Gold_Warehouse.innotrust.dim_security_characteristics_codes sc ON s.security_type_code = sc.security_type_code AND sc.is_current = 1
+WHERE s.is_current = 1
+UNION ALL
+SELECT 'dim_security_characteristics_codes', COUNT(*),
+    (SELECT COUNT(*) FROM (SELECT security_type_code FROM Gold_Warehouse.innotrust.dim_security_characteristics_codes WHERE is_current = 1 GROUP BY security_type_code HAVING COUNT(*) &gt; 1) d),
+    (COUNT(*) - COUNT(DISTINCT dim_securitycharacteristicscodes)),
+    0,
+    SUM(CASE WHEN business_date IS NULL THEN 1 ELSE 0 END),
+    SUM(CASE WHEN updated_at IS NULL THEN 1 ELSE 0 END)
+FROM Gold_Warehouse.innotrust.dim_security_characteristics_codes WHERE is_current = 1;</t>
         </is>
       </c>
     </row>
@@ -5544,7 +6337,688 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="70" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>INNOTRUST GOLD LAYER VALIDATION SUITE</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="26" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Test Category</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Target Table</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Test Scenario Description</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>SQL Validation Query</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="54" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>TC_INNO_GOLD_01</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>SCD2 Deduplication</t>
+        </is>
+      </c>
+      <c r="C3" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_master</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>Verify Active Deduplication on Business Key ['customer_account_number'] (is_current = 1)</t>
+        </is>
+      </c>
+      <c r="F3" s="11" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_master populated</t>
+        </is>
+      </c>
+      <c r="G3" s="11" t="inlineStr">
+        <is>
+          <t>Zero duplicate active accounts. Exactly one is_current = 1 record per customer_account_number.</t>
+        </is>
+      </c>
+      <c r="H3" s="17" t="inlineStr">
+        <is>
+          <t>SELECT customer_account_number, COUNT(*) AS ActiveDuplicateCount
+FROM Gold_Warehouse.innotrust.dim_account_master
+WHERE is_current = 1
+GROUP BY customer_account_number
+HAVING COUNT(*) &gt; 1;</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="54" customHeight="1">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>TC_INNO_GOLD_02</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>SK Uniqueness</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_master</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Verify Primary Surrogate Key (dim_account_master_sk) uniqueness and non-null constraint</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_master populated</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>dim_account_master_sk is strictly unique across all versions with zero NULL values.</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>SELECT dim_account_master_sk, COUNT(*) AS DuplicateCount
+FROM Gold_Warehouse.innotrust.dim_account_master
+GROUP BY dim_account_master_sk
+HAVING COUNT(*) &gt; 1
+UNION ALL
+SELECT NULL, COUNT(*)
+FROM Gold_Warehouse.innotrust.dim_account_master
+WHERE dim_account_master_sk IS NULL
+HAVING COUNT(*) &gt; 0;</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="54" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>TC_INNO_GOLD_03</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>SCD2 Deduplication</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_category_codes</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>Verify Active Deduplication on Business Key ['account_category_code'] (is_current = 1)</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_category_codes populated</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>Zero duplicate active category codes per account_category_code.</t>
+        </is>
+      </c>
+      <c r="H5" s="17" t="inlineStr">
+        <is>
+          <t>SELECT account_category_code, COUNT(*) AS ActiveDuplicateCount
+FROM Gold_Warehouse.innotrust.dim_account_category_codes
+WHERE is_current = 1
+GROUP BY account_category_code
+HAVING COUNT(*) &gt; 1;</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="54" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>TC_INNO_GOLD_04</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>SK Uniqueness</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_category_codes</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Verify Primary Surrogate Key (dim_account_master_sk) uniqueness on dim_account_category_codes</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_category_codes populated</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>Surrogate key dim_account_master_sk is unique across all rows with zero NULLs.</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>SELECT dim_account_master_sk, COUNT(*) AS DuplicateCount
+FROM Gold_Warehouse.innotrust.dim_account_category_codes
+GROUP BY dim_account_master_sk
+HAVING COUNT(*) &gt; 1;</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="54" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>TC_INNO_GOLD_05</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>SCD2 Deduplication</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_type_codes</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>Verify Active Deduplication on Business Key ['account_type_code'] (is_current = 1)</t>
+        </is>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_type_codes populated</t>
+        </is>
+      </c>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>Zero duplicate active account types per account_type_code.</t>
+        </is>
+      </c>
+      <c r="H7" s="17" t="inlineStr">
+        <is>
+          <t>SELECT account_type_code, COUNT(*) AS ActiveDuplicateCount
+FROM Gold_Warehouse.innotrust.dim_account_type_codes
+WHERE is_current = 1
+GROUP BY account_type_code
+HAVING COUNT(*) &gt; 1;</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="54" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>TC_INNO_GOLD_06</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>SK Uniqueness</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_type_codes</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Verify Primary Surrogate Key (dim_account_type_codes_sk) uniqueness and non-null constraint</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_type_codes populated</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>dim_account_type_codes_sk is strictly unique across all versions with zero NULLs.</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>SELECT dim_account_type_codes_sk, COUNT(*) AS DuplicateCount
+FROM Gold_Warehouse.innotrust.dim_account_type_codes
+GROUP BY dim_account_type_codes_sk
+HAVING COUNT(*) &gt; 1;</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="54" customHeight="1">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>TC_INNO_GOLD_07</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>SCD2 Deduplication</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>innotrust.dim_master_sec_index</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>Verify Active Deduplication on Security Primary Key ['isin'] (is_current = 1)</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>innotrust.dim_master_sec_index populated</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>Zero duplicate active securities. Exactly one is_current = 1 record per isin.</t>
+        </is>
+      </c>
+      <c r="H9" s="17" t="inlineStr">
+        <is>
+          <t>SELECT isin, COUNT(*) AS ActiveDuplicateCount
+FROM Gold_Warehouse.innotrust.dim_master_sec_index
+WHERE is_current = 1
+GROUP BY isin
+HAVING COUNT(*) &gt; 1;</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="54" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>TC_INNO_GOLD_08</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>SK Uniqueness</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>innotrust.dim_master_sec_index</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Verify Primary Surrogate Key (dim_master_sec_index_sk) uniqueness across all records</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>innotrust.dim_master_sec_index populated</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>dim_master_sec_index_sk is strictly unique across all versions with zero NULLs.</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>SELECT dim_master_sec_index_sk, COUNT(*) AS DuplicateCount
+FROM Gold_Warehouse.innotrust.dim_master_sec_index
+GROUP BY dim_master_sec_index_sk
+HAVING COUNT(*) &gt; 1;</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="54" customHeight="1">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>TC_INNO_GOLD_09</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>SCD2 Deduplication</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>innotrust.dim_security_characteristics_codes</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>Verify Active Deduplication on Business Key ['security_type_code'] (is_current = 1)</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>innotrust.dim_security_characteristics_codes populated</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>Zero duplicate active security type codes per security_type_code.</t>
+        </is>
+      </c>
+      <c r="H11" s="17" t="inlineStr">
+        <is>
+          <t>SELECT security_type_code, COUNT(*) AS ActiveDuplicateCount
+FROM Gold_Warehouse.innotrust.dim_security_characteristics_codes
+WHERE is_current = 1
+GROUP BY security_type_code
+HAVING COUNT(*) &gt; 1;</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="54" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>TC_INNO_GOLD_10</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>SK Uniqueness</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>innotrust.dim_security_characteristics_codes</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Verify Primary Surrogate Key (dim_securitycharacteristicscodes) uniqueness and non-null constraint</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>innotrust.dim_security_characteristics_codes populated</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>dim_securitycharacteristicscodes is strictly unique across all versions with zero NULLs.</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>SELECT dim_securitycharacteristicscodes, COUNT(*) AS DuplicateCount
+FROM Gold_Warehouse.innotrust.dim_security_characteristics_codes
+GROUP BY dim_securitycharacteristicscodes
+HAVING COUNT(*) &gt; 1;</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="54" customHeight="1">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>TC_INNO_GOLD_11</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Audit &amp; Date Logic</t>
+        </is>
+      </c>
+      <c r="C13" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_master</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>Verify business_date, updated_at, effective_start_date &amp; effective_end_date integrity on active records</t>
+        </is>
+      </c>
+      <c r="F13" s="11" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_master populated</t>
+        </is>
+      </c>
+      <c r="G13" s="11" t="inlineStr">
+        <is>
+          <t>Zero NULLs in business_date or updated_at; effective_end_date &gt;= effective_start_date.</t>
+        </is>
+      </c>
+      <c r="H13" s="17" t="inlineStr">
+        <is>
+          <t>SELECT 
+    COUNT(*) AS TotalActiveRows,
+    SUM(CASE WHEN business_date IS NULL THEN 1 ELSE 0 END) AS Null_BusinessDate,
+    SUM(CASE WHEN updated_at IS NULL THEN 1 ELSE 0 END) AS Null_UpdatedAt,
+    SUM(CASE WHEN effective_start_date IS NULL THEN 1 ELSE 0 END) AS Null_EffectiveStartDate,
+    SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) AS InvertedEffectiveDates
+FROM Gold_Warehouse.innotrust.dim_account_master
+WHERE is_current = 1;</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="54" customHeight="1">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>TC_INNO_GOLD_12</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Cross-Table Linkage</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_master</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Verify Referential Integrity: account_category_code and account_type_code resolve to active codes</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_master populated</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>All non-null account_category_code and account_type_code exist in corresponding dimension code tables.</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>SELECT 
+    SUM(CASE WHEN m.account_category_code IS NOT NULL AND cat.account_category_code IS NULL THEN 1 ELSE 0 END) AS Orphan_CategoryCodes,
+    SUM(CASE WHEN m.account_type_code IS NOT NULL AND typ.account_type_code IS NULL THEN 1 ELSE 0 END) AS Orphan_TypeCodes
+FROM Gold_Warehouse.innotrust.dim_account_master m
+LEFT JOIN Gold_Warehouse.innotrust.dim_account_category_codes cat 
+    ON m.account_category_code = cat.account_category_code AND cat.is_current = 1
+LEFT JOIN Gold_Warehouse.innotrust.dim_account_type_codes typ 
+    ON m.account_type_code = typ.account_type_code AND typ.is_current = 1
+WHERE m.is_current = 1;</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="54" customHeight="1">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>TC_INNO_GOLD_13</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>Cross-Table Linkage</t>
+        </is>
+      </c>
+      <c r="C15" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>innotrust.dim_master_sec_index</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>Verify Security Referential Integrity: security_type_code resolves to active security characteristics</t>
+        </is>
+      </c>
+      <c r="F15" s="11" t="inlineStr">
+        <is>
+          <t>innotrust.dim_master_sec_index populated</t>
+        </is>
+      </c>
+      <c r="G15" s="11" t="inlineStr">
+        <is>
+          <t>All non-null security_type_code values exist in dim_security_characteristics_codes.</t>
+        </is>
+      </c>
+      <c r="H15" s="17" t="inlineStr">
+        <is>
+          <t>SELECT COUNT(*) AS Orphan_SecurityTypeCodes
+FROM Gold_Warehouse.innotrust.dim_master_sec_index s
+LEFT JOIN Gold_Warehouse.innotrust.dim_security_characteristics_codes sc 
+    ON s.security_type_code = sc.security_type_code AND sc.is_current = 1
+WHERE s.is_current = 1 AND s.security_type_code IS NOT NULL AND sc.security_type_code IS NULL;</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6009,6 +7483,93 @@
         </is>
       </c>
     </row>
+    <row r="7" ht="110" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>TC_COMB_SK_INNO_05</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>Innotrust</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>All 5 Innotrust Dimensions (dim_account_master, category_codes, type_codes, sec_index, characteristics)</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>Innotrust: Consolidated Multi-Object PK Deduplication, Primary SK &amp; Cross-Dimension Linkage
+Single unified query validating SCD2 active uniqueness on exact natural keys, primary surrogate key uniqueness, and cross-dimension referential integrity between master entities and classification codes.</t>
+        </is>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>All Gold tables loaded for Innotrust</t>
+        </is>
+      </c>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>PK_Active_Duplicates = 0, Duplicate_Primary_SK = 0, Orphan_Foreign_References = 0, Missing_BusinessDate = 0 across all 5 Innotrust tables.</t>
+        </is>
+      </c>
+      <c r="H7" s="17" t="inlineStr">
+        <is>
+          <t>SELECT 'dim_account_master' AS TableName, COUNT(*) AS TotalActiveRows,
+    (SELECT COUNT(*) FROM (SELECT customer_account_number FROM Gold_Warehouse.innotrust.dim_account_master WHERE is_current = 1 GROUP BY customer_account_number HAVING COUNT(*) &gt; 1) d) AS PK_Active_Duplicates,
+    (COUNT(*) - COUNT(DISTINCT dim_account_master_sk)) AS Duplicate_Primary_SK,
+    SUM(CASE WHEN (m.account_category_code IS NOT NULL AND cat.account_category_code IS NULL)
+               OR (m.account_type_code IS NOT NULL AND typ.account_type_code IS NULL) THEN 1 ELSE 0 END) AS Orphan_Foreign_References,
+    SUM(CASE WHEN m.business_date IS NULL THEN 1 ELSE 0 END) AS Missing_BusinessDate,
+    SUM(CASE WHEN m.updated_at IS NULL THEN 1 ELSE 0 END) AS Missing_UpdatedAt
+FROM Gold_Warehouse.innotrust.dim_account_master m
+LEFT JOIN Gold_Warehouse.innotrust.dim_account_category_codes cat ON m.account_category_code = cat.account_category_code AND cat.is_current = 1
+LEFT JOIN Gold_Warehouse.innotrust.dim_account_type_codes typ ON m.account_type_code = typ.account_type_code AND typ.is_current = 1
+WHERE m.is_current = 1
+UNION ALL
+SELECT 'dim_account_category_codes', COUNT(*),
+    (SELECT COUNT(*) FROM (SELECT account_category_code FROM Gold_Warehouse.innotrust.dim_account_category_codes WHERE is_current = 1 GROUP BY account_category_code HAVING COUNT(*) &gt; 1) d),
+    (COUNT(*) - COUNT(DISTINCT dim_account_master_sk)),
+    0,
+    SUM(CASE WHEN business_date IS NULL THEN 1 ELSE 0 END),
+    SUM(CASE WHEN updated_at IS NULL THEN 1 ELSE 0 END)
+FROM Gold_Warehouse.innotrust.dim_account_category_codes WHERE is_current = 1
+UNION ALL
+SELECT 'dim_account_type_codes', COUNT(*),
+    (SELECT COUNT(*) FROM (SELECT account_type_code FROM Gold_Warehouse.innotrust.dim_account_type_codes WHERE is_current = 1 GROUP BY account_type_code HAVING COUNT(*) &gt; 1) d),
+    (COUNT(*) - COUNT(DISTINCT dim_account_type_codes_sk)),
+    0,
+    SUM(CASE WHEN business_date IS NULL THEN 1 ELSE 0 END),
+    SUM(CASE WHEN updated_at IS NULL THEN 1 ELSE 0 END)
+FROM Gold_Warehouse.innotrust.dim_account_type_codes WHERE is_current = 1
+UNION ALL
+SELECT 'dim_master_sec_index', COUNT(*),
+    (SELECT COUNT(*) FROM (SELECT isin FROM Gold_Warehouse.innotrust.dim_master_sec_index WHERE is_current = 1 GROUP BY isin HAVING COUNT(*) &gt; 1) d),
+    (COUNT(*) - COUNT(DISTINCT dim_master_sec_index_sk)),
+    SUM(CASE WHEN s.security_type_code IS NOT NULL AND sc.security_type_code IS NULL THEN 1 ELSE 0 END),
+    SUM(CASE WHEN s.business_date IS NULL THEN 1 ELSE 0 END),
+    SUM(CASE WHEN s.updated_at IS NULL THEN 1 ELSE 0 END)
+FROM Gold_Warehouse.innotrust.dim_master_sec_index s
+LEFT JOIN Gold_Warehouse.innotrust.dim_security_characteristics_codes sc ON s.security_type_code = sc.security_type_code AND sc.is_current = 1
+WHERE s.is_current = 1
+UNION ALL
+SELECT 'dim_security_characteristics_codes', COUNT(*),
+    (SELECT COUNT(*) FROM (SELECT security_type_code FROM Gold_Warehouse.innotrust.dim_security_characteristics_codes WHERE is_current = 1 GROUP BY security_type_code HAVING COUNT(*) &gt; 1) d),
+    (COUNT(*) - COUNT(DISTINCT dim_securitycharacteristicscodes)),
+    0,
+    SUM(CASE WHEN business_date IS NULL THEN 1 ELSE 0 END),
+    SUM(CASE WHEN updated_at IS NULL THEN 1 ELSE 0 END)
+FROM Gold_Warehouse.innotrust.dim_security_characteristics_codes WHERE is_current = 1;</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>

</xml_diff>

<commit_message>
Add Innotrust SCD2 effective date validation test cases and consolidated audit
</commit_message>
<xml_diff>
--- a/Gold_Data_Validation_Test_Cases.xlsx
+++ b/Gold_Data_Validation_Test_Cases.xlsx
@@ -644,16 +644,16 @@
         <v>5</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F5" s="4" t="n">
         <v>14</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" ht="26" customHeight="1">
@@ -829,22 +829,22 @@
         </is>
       </c>
       <c r="C12" s="8" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E12" s="9" t="n">
         <v>3</v>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>TC_COMB_SK_INNO_05</t>
+          <t>TC_COMB_SK_INNO_05 / 06</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>All 5 dimensions: dim_account_master, category_codes, type_codes, sec_index, characteristics</t>
+          <t>All 5 dimensions: PK dedup, SK uniqueness, cross-table linkage &amp; SCD2 date rules (End Date &lt;= Today - 1)</t>
         </is>
       </c>
     </row>
@@ -860,10 +860,10 @@
         </is>
       </c>
       <c r="C13" s="15" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D13" s="15" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E13" s="15" t="n">
         <v>14</v>
@@ -898,7 +898,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I59"/>
+  <dimension ref="A1:I61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3673,45 +3673,105 @@
     <row r="55" ht="54" customHeight="1">
       <c r="A55" s="12" t="inlineStr">
         <is>
+          <t>Innotrust</t>
+        </is>
+      </c>
+      <c r="B55" s="12" t="inlineStr">
+        <is>
+          <t>TC_INNO_GOLD_14</t>
+        </is>
+      </c>
+      <c r="C55" s="13" t="inlineStr">
+        <is>
+          <t>SCD2 Date Validation</t>
+        </is>
+      </c>
+      <c r="D55" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E55" s="10" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_master</t>
+        </is>
+      </c>
+      <c r="F55" s="11" t="inlineStr">
+        <is>
+          <t>Verify SCD2 Effective Date Rules: Inactive records effective_end_date &lt;= (Current Day - 1), non-null end date, and valid active start date</t>
+        </is>
+      </c>
+      <c r="G55" s="11" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_master populated with SCD2 tracking columns</t>
+        </is>
+      </c>
+      <c r="H55" s="11" t="inlineStr">
+        <is>
+          <t>Inactive_End_Date_Breach_Count = 0, Inactive_Missing_End_Date = 0, Active_Future_Start_Date = 0, Inverted_Date_Range_Count = 0. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="I55" s="17" t="inlineStr">
+        <is>
+          <t>SELECT 
+    'dim_account_master' AS TableName,
+    COUNT(*) AS TotalRecords,
+    SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END) AS Inactive_End_Date_Breach_Count,
+    SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END) AS Inactive_Missing_End_Date,
+    SUM(CASE WHEN is_current = 1 AND effective_start_date &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END) AS Active_Future_Start_Date,
+    SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) AS Inverted_Date_Range_Count,
+    CASE 
+        WHEN SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END AS TestStatus
+FROM Gold_Warehouse.innotrust.dim_account_master;</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="54" customHeight="1">
+      <c r="A56" s="8" t="inlineStr">
+        <is>
           <t>Black Diamond (Consolidated)</t>
         </is>
       </c>
-      <c r="B55" s="12" t="inlineStr">
+      <c r="B56" s="8" t="inlineStr">
         <is>
           <t>TC_COMB_SK_BD_01</t>
         </is>
       </c>
-      <c r="C55" s="13" t="inlineStr">
+      <c r="C56" s="9" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D55" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E55" s="10" t="inlineStr">
+      <c r="D56" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E56" s="6" t="inlineStr">
         <is>
           <t>All 9 Child &amp; Fact Tables (holdings, transactions, taxlots, class/segment, details, tags, team, targets)</t>
         </is>
       </c>
-      <c r="F55" s="11" t="inlineStr">
+      <c r="F56" s="7" t="inlineStr">
         <is>
           <t>Black Diamond: Cross-Object account_sk vs dim_accounts Natural Key (accountid == da.id) Verification - Executes a single consolidated UNION ALL query across all 9 child/fact tables to verify that the attached account_sk strictly points to the exact same account natural key (child.accountid == da.id). Guarantees zero wrong account links.</t>
         </is>
       </c>
-      <c r="G55" s="11" t="inlineStr">
+      <c r="G56" s="7" t="inlineStr">
         <is>
           <t>All Gold tables populated for Black Diamond</t>
         </is>
       </c>
-      <c r="H55" s="11" t="inlineStr">
+      <c r="H56" s="7" t="inlineStr">
         <is>
           <t>Duplicate_BusinessKey_Count = 0, MismatchedAccountIdCount = 0, Null_AccountSK_Count = 0, Orphan_AccountSK_Count = 0 across all 9 objects.</t>
         </is>
       </c>
-      <c r="I55" s="17" t="inlineStr">
+      <c r="I56" s="18" t="inlineStr">
         <is>
           <t>SELECT 
     'dim_accounts_classallocation' AS TableName, 
@@ -3820,48 +3880,48 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="54" customHeight="1">
-      <c r="A56" s="8" t="inlineStr">
+    <row r="57" ht="54" customHeight="1">
+      <c r="A57" s="12" t="inlineStr">
         <is>
           <t>Schwab (Consolidated)</t>
         </is>
       </c>
-      <c r="B56" s="8" t="inlineStr">
+      <c r="B57" s="12" t="inlineStr">
         <is>
           <t>TC_COMB_SK_SC_02</t>
         </is>
       </c>
-      <c r="C56" s="9" t="inlineStr">
+      <c r="C57" s="13" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D56" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E56" s="6" t="inlineStr">
+      <c r="D57" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E57" s="10" t="inlineStr">
         <is>
           <t>All 8 Objects (dim_accounts &amp; 7 Fact Tables: recon_d1/d2, daily_closing, security, transactions, ult/uln lots)</t>
         </is>
       </c>
-      <c r="F56" s="7" t="inlineStr">
+      <c r="F57" s="11" t="inlineStr">
         <is>
           <t>Schwab: Consolidated Multi-Object SK Mapping, PK Deduplication &amp; Audit Date Health Check - Single unified query executing across all 8 Schwab Gold tables. Validates that every fact record's account_sk correctly matches dim_accounts on composite natural keys (account_id, custodian_id), confirms primary SK uniqueness, and ensures 100% audit dates populated.</t>
         </is>
       </c>
-      <c r="G56" s="7" t="inlineStr">
+      <c r="G57" s="11" t="inlineStr">
         <is>
           <t>All Gold tables populated for Schwab</t>
         </is>
       </c>
-      <c r="H56" s="7" t="inlineStr">
+      <c r="H57" s="11" t="inlineStr">
         <is>
           <t>Mismatched_AccountId_Count = 0 and Orphan_AccountSK_Count = 0 across all fact tables. All mapped account_sk strictly match the natural account_id.</t>
         </is>
       </c>
-      <c r="I56" s="18" t="inlineStr">
+      <c r="I57" s="17" t="inlineStr">
         <is>
           <t>SELECT 
     'fact_recon_position_d1' AS TableName,
@@ -3920,48 +3980,48 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="54" customHeight="1">
-      <c r="A57" s="12" t="inlineStr">
+    <row r="58" ht="54" customHeight="1">
+      <c r="A58" s="8" t="inlineStr">
         <is>
           <t>Salentica CRM (Consolidated)</t>
         </is>
       </c>
-      <c r="B57" s="12" t="inlineStr">
+      <c r="B58" s="8" t="inlineStr">
         <is>
           <t>TC_COMB_SK_SAL_03</t>
         </is>
       </c>
-      <c r="C57" s="13" t="inlineStr">
+      <c r="C58" s="9" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D57" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E57" s="10" t="inlineStr">
+      <c r="D58" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="inlineStr">
         <is>
           <t>All 6 Core CRM Entities (dim_account, dim_contact_core, dim_family, fact_lead, fact_opportunity, fact_investmentaccount)</t>
         </is>
       </c>
-      <c r="F57" s="11" t="inlineStr">
+      <c r="F58" s="7" t="inlineStr">
         <is>
           <t>Salentica: Consolidated Point-in-Time Referential SK Mapping (Active &amp; Historical Mapping Validation) - Single unified query executing across all 6 core Salentica CRM tables. Validates that every attached foreign SK resolves to the same Natural Key in parent dimensions (allowing active OR expired parent versions to preserve point-in-time audit history) and checks for broken orphans.</t>
         </is>
       </c>
-      <c r="G57" s="11" t="inlineStr">
+      <c r="G58" s="7" t="inlineStr">
         <is>
           <t>All Gold tables populated for Salentica CRM</t>
         </is>
       </c>
-      <c r="H57" s="11" t="inlineStr">
+      <c r="H58" s="7" t="inlineStr">
         <is>
           <t>Mismatched_PrimaryContact_NK = 0, Mismatched_BusinessUnit_NK = 0, Broken_Orphan_Count = 0 across all 6 CRM tables.</t>
         </is>
       </c>
-      <c r="I57" s="17" t="inlineStr">
+      <c r="I58" s="18" t="inlineStr">
         <is>
           <t>SELECT 'dim_account' AS TableName, COUNT(*) AS TotalActiveRows,
     SUM(CASE WHEN a.primarycontactid IS NOT NULL AND a.primarycontactid_sk &lt;&gt; -1 AND a.primarycontactid &lt;&gt; c.contactid THEN 1 ELSE 0 END) AS Mismatched_PrimaryContact_NK,
@@ -4025,48 +4085,48 @@
         </is>
       </c>
     </row>
-    <row r="58" ht="54" customHeight="1">
-      <c r="A58" s="8" t="inlineStr">
+    <row r="59" ht="54" customHeight="1">
+      <c r="A59" s="12" t="inlineStr">
         <is>
           <t>Tamarac (Consolidated)</t>
         </is>
       </c>
-      <c r="B58" s="8" t="inlineStr">
+      <c r="B59" s="12" t="inlineStr">
         <is>
           <t>TC_COMB_SK_TAM_04</t>
         </is>
       </c>
-      <c r="C58" s="9" t="inlineStr">
+      <c r="C59" s="13" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D58" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E58" s="6" t="inlineStr">
+      <c r="D59" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E59" s="10" t="inlineStr">
         <is>
           <t>Both Tables (dim_account_information, dim_account_model_allocation)</t>
         </is>
       </c>
-      <c r="F58" s="7" t="inlineStr">
+      <c r="F59" s="11" t="inlineStr">
         <is>
           <t>Tamarac: Consolidated Multi-Object PK Deduplication, Primary SK &amp; Cross-Table Linkage - Single unified query validating SCD2 active uniqueness on exact PK columns (['account_number'] and ['account_number', 'model_name']), surrogate key uniqueness, and cross-table referential integrity between model allocations and accounts.</t>
         </is>
       </c>
-      <c r="G58" s="7" t="inlineStr">
+      <c r="G59" s="11" t="inlineStr">
         <is>
           <t>All Gold tables populated for Tamarac</t>
         </is>
       </c>
-      <c r="H58" s="7" t="inlineStr">
+      <c r="H59" s="11" t="inlineStr">
         <is>
           <t>PK_Active_Duplicates = 0, Duplicate_Primary_SK = 0, Orphan_Accounts = 0, Missing_BusinessDate = 0 across both tables.</t>
         </is>
       </c>
-      <c r="I58" s="18" t="inlineStr">
+      <c r="I59" s="17" t="inlineStr">
         <is>
           <t>SELECT 'dim_account_information' AS TableName, COUNT(*) AS TotalActiveRows,
     (SELECT COUNT(*) FROM (SELECT account_number FROM Gold_Warehouse.tamarac.dim_account_information WHERE is_current = 'True' GROUP BY account_number HAVING COUNT(*) &gt; 1) d) AS PK_Active_Duplicates,
@@ -4089,48 +4149,48 @@
         </is>
       </c>
     </row>
-    <row r="59" ht="54" customHeight="1">
-      <c r="A59" s="12" t="inlineStr">
+    <row r="60" ht="54" customHeight="1">
+      <c r="A60" s="8" t="inlineStr">
         <is>
           <t>Innotrust (Consolidated)</t>
         </is>
       </c>
-      <c r="B59" s="12" t="inlineStr">
+      <c r="B60" s="8" t="inlineStr">
         <is>
           <t>TC_COMB_SK_INNO_05</t>
         </is>
       </c>
-      <c r="C59" s="13" t="inlineStr">
+      <c r="C60" s="9" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D59" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E59" s="10" t="inlineStr">
+      <c r="D60" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E60" s="6" t="inlineStr">
         <is>
           <t>All 5 Innotrust Dimensions (dim_account_master, category_codes, type_codes, sec_index, characteristics)</t>
         </is>
       </c>
-      <c r="F59" s="11" t="inlineStr">
+      <c r="F60" s="7" t="inlineStr">
         <is>
           <t>Innotrust: Consolidated Multi-Object PK Deduplication, Primary SK &amp; Cross-Dimension Linkage - Single unified query validating SCD2 active uniqueness on exact natural keys, primary surrogate key uniqueness, and cross-dimension referential integrity between master entities and classification codes.</t>
         </is>
       </c>
-      <c r="G59" s="11" t="inlineStr">
+      <c r="G60" s="7" t="inlineStr">
         <is>
           <t>All Gold tables populated for Innotrust</t>
         </is>
       </c>
-      <c r="H59" s="11" t="inlineStr">
+      <c r="H60" s="7" t="inlineStr">
         <is>
           <t>PK_Active_Duplicates = 0, Duplicate_Primary_SK = 0, Orphan_Foreign_References = 0, Missing_BusinessDate = 0 across all 5 Innotrust tables.</t>
         </is>
       </c>
-      <c r="I59" s="17" t="inlineStr">
+      <c r="I60" s="18" t="inlineStr">
         <is>
           <t>SELECT 'dim_account_master' AS TableName, COUNT(*) AS TotalActiveRows,
     (SELECT COUNT(*) FROM (SELECT customer_account_number FROM Gold_Warehouse.innotrust.dim_account_master WHERE is_current = 1 GROUP BY customer_account_number HAVING COUNT(*) &gt; 1) d) AS PK_Active_Duplicates,
@@ -4180,6 +4240,126 @@
         </is>
       </c>
     </row>
+    <row r="61" ht="54" customHeight="1">
+      <c r="A61" s="12" t="inlineStr">
+        <is>
+          <t>Innotrust (Consolidated)</t>
+        </is>
+      </c>
+      <c r="B61" s="12" t="inlineStr">
+        <is>
+          <t>TC_COMB_SK_INNO_06</t>
+        </is>
+      </c>
+      <c r="C61" s="13" t="inlineStr">
+        <is>
+          <t>Consolidated Multi-Object SK Audit</t>
+        </is>
+      </c>
+      <c r="D61" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E61" s="10" t="inlineStr">
+        <is>
+          <t>All 5 Innotrust Dimensions (dim_account_master, category_codes, type_codes, sec_index, characteristics)</t>
+        </is>
+      </c>
+      <c r="F61" s="11" t="inlineStr">
+        <is>
+          <t>Innotrust: Consolidated Multi-Object SCD2 Effective Start &amp; End Date Audit (End Date &lt;= Today - 1) - Validates across all 5 Innotrust dimensions that inactive records (is_current = 0) have effective_end_date &lt;= (current day - 1), non-null end dates, active records have non-future start dates, and zero inverted date ranges.</t>
+        </is>
+      </c>
+      <c r="G61" s="11" t="inlineStr">
+        <is>
+          <t>All Gold tables populated for Innotrust</t>
+        </is>
+      </c>
+      <c r="H61" s="11" t="inlineStr">
+        <is>
+          <t>Inactive_End_Date_Breach_Count = 0, Inactive_Missing_End_Date = 0, Active_Future_Start_Date = 0, Inverted_Date_Range_Count = 0 across all 5 tables.</t>
+        </is>
+      </c>
+      <c r="I61" s="17" t="inlineStr">
+        <is>
+          <t>SELECT 
+    'dim_account_master' AS TableName,
+    COUNT(*) AS TotalRecords,
+    SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END) AS Inactive_End_Date_Breach_Count,
+    SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END) AS Inactive_Missing_End_Date,
+    SUM(CASE WHEN is_current = 1 AND effective_start_date &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END) AS Active_Future_Start_Date,
+    SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) AS Inverted_Date_Range_Count,
+    CASE 
+        WHEN SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END AS TestStatus
+FROM Gold_Warehouse.innotrust.dim_account_master
+UNION ALL
+SELECT 
+    'dim_master_sec_index' AS TableName,
+    COUNT(*),
+    SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END),
+    SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END),
+    SUM(CASE WHEN is_current = 1 AND effective_start_date &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END),
+    SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END),
+    CASE 
+        WHEN SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END
+FROM Gold_Warehouse.innotrust.dim_master_sec_index
+UNION ALL
+SELECT 
+    'dim_account_category_codes',
+    COUNT(*),
+    SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END),
+    SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END),
+    SUM(CASE WHEN is_current = 1 AND effective_start_date &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END),
+    SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END),
+    CASE 
+        WHEN SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END
+FROM Gold_Warehouse.innotrust.dim_account_category_codes
+UNION ALL
+SELECT 
+    'dim_account_type_codes',
+    COUNT(*),
+    SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END),
+    SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END),
+    SUM(CASE WHEN is_current = 1 AND effective_start_date &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END),
+    SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END),
+    CASE 
+        WHEN SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END
+FROM Gold_Warehouse.innotrust.dim_account_type_codes
+UNION ALL
+SELECT 
+    'dim_security_characteristics_codes',
+    COUNT(*),
+    SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END),
+    SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END),
+    SUM(CASE WHEN is_current = 1 AND effective_start_date &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END),
+    SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END),
+    CASE 
+        WHEN SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END
+FROM Gold_Warehouse.innotrust.dim_security_characteristics_codes;</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>
@@ -6337,7 +6517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7004,6 +7184,61 @@
         </is>
       </c>
     </row>
+    <row r="16" ht="54" customHeight="1">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>TC_INNO_GOLD_14</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>SCD2 Date Validation</t>
+        </is>
+      </c>
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_master</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>Verify SCD2 Effective Date Rules: Inactive records effective_end_date &lt;= (Current Day - 1), non-null end date, and valid active start date</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>innotrust.dim_account_master populated with SCD2 tracking columns</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>Inactive_End_Date_Breach_Count = 0, Inactive_Missing_End_Date = 0, Active_Future_Start_Date = 0, Inverted_Date_Range_Count = 0. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>SELECT 
+    'dim_account_master' AS TableName,
+    COUNT(*) AS TotalRecords,
+    SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END) AS Inactive_End_Date_Breach_Count,
+    SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END) AS Inactive_Missing_End_Date,
+    SUM(CASE WHEN is_current = 1 AND effective_start_date &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END) AS Active_Future_Start_Date,
+    SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) AS Inverted_Date_Range_Count,
+    CASE 
+        WHEN SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END AS TestStatus
+FROM Gold_Warehouse.innotrust.dim_account_master;</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
@@ -7018,7 +7253,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7570,6 +7805,122 @@
         </is>
       </c>
     </row>
+    <row r="8" ht="110" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>TC_COMB_SK_INNO_06</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Innotrust</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>All 5 Innotrust Dimensions (dim_account_master, category_codes, type_codes, sec_index, characteristics)</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Innotrust: Consolidated Multi-Object SCD2 Effective Start &amp; End Date Audit (End Date &lt;= Today - 1)
+Validates across all 5 Innotrust dimensions that inactive records (is_current = 0) have effective_end_date &lt;= (current day - 1), non-null end dates, active records have non-future start dates, and zero inverted date ranges.</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>All Gold tables loaded for Innotrust</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>Inactive_End_Date_Breach_Count = 0, Inactive_Missing_End_Date = 0, Active_Future_Start_Date = 0, Inverted_Date_Range_Count = 0 across all 5 tables.</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>SELECT 
+    'dim_account_master' AS TableName,
+    COUNT(*) AS TotalRecords,
+    SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END) AS Inactive_End_Date_Breach_Count,
+    SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END) AS Inactive_Missing_End_Date,
+    SUM(CASE WHEN is_current = 1 AND effective_start_date &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END) AS Active_Future_Start_Date,
+    SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) AS Inverted_Date_Range_Count,
+    CASE 
+        WHEN SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END AS TestStatus
+FROM Gold_Warehouse.innotrust.dim_account_master
+UNION ALL
+SELECT 
+    'dim_master_sec_index' AS TableName,
+    COUNT(*),
+    SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END),
+    SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END),
+    SUM(CASE WHEN is_current = 1 AND effective_start_date &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END),
+    SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END),
+    CASE 
+        WHEN SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END
+FROM Gold_Warehouse.innotrust.dim_master_sec_index
+UNION ALL
+SELECT 
+    'dim_account_category_codes',
+    COUNT(*),
+    SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END),
+    SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END),
+    SUM(CASE WHEN is_current = 1 AND effective_start_date &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END),
+    SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END),
+    CASE 
+        WHEN SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END
+FROM Gold_Warehouse.innotrust.dim_account_category_codes
+UNION ALL
+SELECT 
+    'dim_account_type_codes',
+    COUNT(*),
+    SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END),
+    SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END),
+    SUM(CASE WHEN is_current = 1 AND effective_start_date &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END),
+    SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END),
+    CASE 
+        WHEN SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END
+FROM Gold_Warehouse.innotrust.dim_account_type_codes
+UNION ALL
+SELECT 
+    'dim_security_characteristics_codes',
+    COUNT(*),
+    SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END),
+    SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END),
+    SUM(CASE WHEN is_current = 1 AND effective_start_date &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END),
+    SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END),
+    CASE 
+        WHEN SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END
+FROM Gold_Warehouse.innotrust.dim_security_characteristics_codes;</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>

</xml_diff>

<commit_message>
Add full suite of Tamarac SCD2 effective dates, timeline continuity, and SK monotonicity tests
</commit_message>
<xml_diff>
--- a/Gold_Data_Validation_Test_Cases.xlsx
+++ b/Gold_Data_Validation_Test_Cases.xlsx
@@ -644,13 +644,13 @@
         <v>5</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G5" s="4" t="n">
         <v>6</v>
@@ -798,13 +798,13 @@
         </is>
       </c>
       <c r="C11" s="12" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="D11" s="13" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="E11" s="13" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
@@ -860,13 +860,13 @@
         </is>
       </c>
       <c r="C13" s="15" t="n">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="D13" s="15" t="n">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="E13" s="15" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F13" s="15" t="inlineStr">
         <is>
@@ -898,7 +898,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I61"/>
+  <dimension ref="A1:I69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3003,45 +3003,536 @@
     <row r="42" ht="54" customHeight="1">
       <c r="A42" s="8" t="inlineStr">
         <is>
+          <t>Tamarac</t>
+        </is>
+      </c>
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>TC_TAM_GOLD_07</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>SCD2 Date Validation</t>
+        </is>
+      </c>
+      <c r="D42" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
+        <is>
+          <t>tamarac.dim_account_information</t>
+        </is>
+      </c>
+      <c r="F42" s="7" t="inlineStr">
+        <is>
+          <t>Verify Inactive End Date Rule: effective_end_date &lt;= (MAX(file_business_date) - 1 day) and non-null</t>
+        </is>
+      </c>
+      <c r="G42" s="7" t="inlineStr">
+        <is>
+          <t>dim_account_information populated with inactive records</t>
+        </is>
+      </c>
+      <c r="H42" s="7" t="inlineStr">
+        <is>
+          <t>Exceeded_Cutoff_Count = 0, Null_End_Date_Count = 0. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="I42" s="18" t="inlineStr">
+        <is>
+          <t>SELECT 
+    'dim_account_information' AS TableName,
+    COUNT(*) AS TotalInactiveRows,
+    CAST(m.CutoffDate AS VARCHAR(10)) AS Max_Cutoff_Allowed,
+    SUM(CASE WHEN a.effective_end_date &gt; m.CutoffDate THEN 1 ELSE 0 END) AS Exceeded_Cutoff_Count,
+    SUM(CASE WHEN a.effective_end_date IS NULL THEN 1 ELSE 0 END) AS Null_End_Date_Count,
+    CASE 
+        WHEN SUM(CASE WHEN a.effective_end_date &gt; m.CutoffDate THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN a.effective_end_date IS NULL THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END AS TestStatus
+FROM Gold_Warehouse.tamarac.dim_account_information a
+CROSS JOIN (SELECT DATEADD(day, -1, MAX(file_business_date)) AS CutoffDate FROM Gold_Warehouse.tamarac.dim_account_information) m
+WHERE a.is_current = 'False'
+GROUP BY m.CutoffDate;</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="54" customHeight="1">
+      <c r="A43" s="12" t="inlineStr">
+        <is>
+          <t>Tamarac</t>
+        </is>
+      </c>
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>TC_TAM_GOLD_08</t>
+        </is>
+      </c>
+      <c r="C43" s="13" t="inlineStr">
+        <is>
+          <t>SCD2 Date Validation</t>
+        </is>
+      </c>
+      <c r="D43" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E43" s="10" t="inlineStr">
+        <is>
+          <t>tamarac.dim_account_model_allocation</t>
+        </is>
+      </c>
+      <c r="F43" s="11" t="inlineStr">
+        <is>
+          <t>Verify Inactive End Date Rule: effective_end_date &lt;= (MAX(file_business_date) - 1 day) and non-null</t>
+        </is>
+      </c>
+      <c r="G43" s="11" t="inlineStr">
+        <is>
+          <t>dim_account_model_allocation populated with inactive records</t>
+        </is>
+      </c>
+      <c r="H43" s="11" t="inlineStr">
+        <is>
+          <t>Exceeded_Cutoff_Count = 0, Null_End_Date_Count = 0. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="I43" s="17" t="inlineStr">
+        <is>
+          <t>SELECT 
+    'dim_account_model_allocation' AS TableName,
+    COUNT(*) AS TotalInactiveRows,
+    CAST(m.CutoffDate AS VARCHAR(10)) AS Max_Cutoff_Allowed,
+    SUM(CASE WHEN a.effective_end_date &gt; m.CutoffDate THEN 1 ELSE 0 END) AS Exceeded_Cutoff_Count,
+    SUM(CASE WHEN a.effective_end_date IS NULL THEN 1 ELSE 0 END) AS Null_End_Date_Count,
+    CASE 
+        WHEN SUM(CASE WHEN a.effective_end_date &gt; m.CutoffDate THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN a.effective_end_date IS NULL THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END AS TestStatus
+FROM Gold_Warehouse.tamarac.dim_account_model_allocation a
+CROSS JOIN (SELECT DATEADD(day, -1, MAX(file_business_date)) AS CutoffDate FROM Gold_Warehouse.tamarac.dim_account_model_allocation) m
+WHERE a.is_current = 'False'
+GROUP BY m.CutoffDate;</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="54" customHeight="1">
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>Tamarac</t>
+        </is>
+      </c>
+      <c r="B44" s="8" t="inlineStr">
+        <is>
+          <t>TC_TAM_GOLD_09</t>
+        </is>
+      </c>
+      <c r="C44" s="9" t="inlineStr">
+        <is>
+          <t>SCD2 Timeline &amp; SK Monotonicity</t>
+        </is>
+      </c>
+      <c r="D44" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E44" s="6" t="inlineStr">
+        <is>
+          <t>tamarac.dim_account_information</t>
+        </is>
+      </c>
+      <c r="F44" s="7" t="inlineStr">
+        <is>
+          <t>Verify SCD2 Timeline Continuity (Zero Gaps, Zero Overlaps) &amp; SK Monotonic Increment</t>
+        </is>
+      </c>
+      <c r="G44" s="7" t="inlineStr">
+        <is>
+          <t>dim_account_information with multiple versions per account_number</t>
+        </is>
+      </c>
+      <c r="H44" s="7" t="inlineStr">
+        <is>
+          <t>Timeline_Gap_Or_Overlap_Count = 0, SK_Non_Incrementing_Violation_Count = 0. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="I44" s="18" t="inlineStr">
+        <is>
+          <t>;WITH InfoTimeline AS (
+    SELECT 
+        account_number,
+        account_information_SK,
+        effective_start_date,
+        effective_end_date,
+        is_current,
+        LEAD(effective_start_date) OVER (PARTITION BY account_number ORDER BY effective_start_date, account_information_SK) AS next_start_date,
+        LEAD(account_information_SK) OVER (PARTITION BY account_number ORDER BY effective_start_date, account_information_SK) AS next_sk
+    FROM Gold_Warehouse.tamarac.dim_account_information
+)
+SELECT 
+    'dim_account_information' AS TableName,
+    COUNT(*) AS MultiVersionRecordsChecked,
+    SUM(CASE WHEN next_start_date IS NOT NULL AND effective_end_date &lt;&gt; DATEADD(day, -1, next_start_date) THEN 1 ELSE 0 END) AS Timeline_Gap_Or_Overlap_Count,
+    SUM(CASE WHEN next_sk IS NOT NULL AND next_sk &lt;= account_information_SK THEN 1 ELSE 0 END) AS SK_Non_Incrementing_Violation_Count,
+    CASE 
+        WHEN SUM(CASE WHEN next_start_date IS NOT NULL AND effective_end_date &lt;&gt; DATEADD(day, -1, next_start_date) THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN next_sk IS NOT NULL AND next_sk &lt;= account_information_SK THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END AS TestStatus
+FROM InfoTimeline
+WHERE next_start_date IS NOT NULL;</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="54" customHeight="1">
+      <c r="A45" s="12" t="inlineStr">
+        <is>
+          <t>Tamarac</t>
+        </is>
+      </c>
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>TC_TAM_GOLD_10</t>
+        </is>
+      </c>
+      <c r="C45" s="13" t="inlineStr">
+        <is>
+          <t>SCD2 Timeline &amp; SK Monotonicity</t>
+        </is>
+      </c>
+      <c r="D45" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E45" s="10" t="inlineStr">
+        <is>
+          <t>tamarac.dim_account_model_allocation</t>
+        </is>
+      </c>
+      <c r="F45" s="11" t="inlineStr">
+        <is>
+          <t>Verify SCD2 Timeline Continuity (Zero Gaps, Zero Overlaps) &amp; SK Monotonic Increment</t>
+        </is>
+      </c>
+      <c r="G45" s="11" t="inlineStr">
+        <is>
+          <t>dim_account_model_allocation with multiple versions per composite key</t>
+        </is>
+      </c>
+      <c r="H45" s="11" t="inlineStr">
+        <is>
+          <t>Timeline_Gap_Or_Overlap_Count = 0, SK_Non_Incrementing_Violation_Count = 0. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="I45" s="17" t="inlineStr">
+        <is>
+          <t>;WITH ModelTimeline AS (
+    SELECT 
+        account_number,
+        model_name,
+        account_model_SK,
+        effective_start_date,
+        effective_end_date,
+        is_current,
+        LEAD(effective_start_date) OVER (PARTITION BY account_number, model_name ORDER BY effective_start_date, account_model_SK) AS next_start_date,
+        LEAD(account_model_SK) OVER (PARTITION BY account_number, model_name ORDER BY effective_start_date, account_model_SK) AS next_sk
+    FROM Gold_Warehouse.tamarac.dim_account_model_allocation
+)
+SELECT 
+    'dim_account_model_allocation' AS TableName,
+    COUNT(*) AS MultiVersionRecordsChecked,
+    SUM(CASE WHEN next_start_date IS NOT NULL AND effective_end_date &lt;&gt; DATEADD(day, -1, next_start_date) THEN 1 ELSE 0 END) AS Timeline_Gap_Or_Overlap_Count,
+    SUM(CASE WHEN next_sk IS NOT NULL AND next_sk &lt;= account_model_SK THEN 1 ELSE 0 END) AS SK_Non_Incrementing_Violation_Count,
+    CASE 
+        WHEN SUM(CASE WHEN next_start_date IS NOT NULL AND effective_end_date &lt;&gt; DATEADD(day, -1, next_start_date) THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN next_sk IS NOT NULL AND next_sk &lt;= account_model_SK THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END AS TestStatus
+FROM ModelTimeline
+WHERE next_start_date IS NOT NULL;</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="54" customHeight="1">
+      <c r="A46" s="8" t="inlineStr">
+        <is>
+          <t>Tamarac</t>
+        </is>
+      </c>
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>TC_TAM_GOLD_11</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="inlineStr">
+        <is>
+          <t>Date Sanity &amp; Inversions</t>
+        </is>
+      </c>
+      <c r="D46" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t>tamarac.dim_account_information</t>
+        </is>
+      </c>
+      <c r="F46" s="7" t="inlineStr">
+        <is>
+          <t>Verify Date Sanity: Zero inverted dates (start &gt; end) and active records have non-future start dates</t>
+        </is>
+      </c>
+      <c r="G46" s="7" t="inlineStr">
+        <is>
+          <t>dim_account_information populated</t>
+        </is>
+      </c>
+      <c r="H46" s="7" t="inlineStr">
+        <is>
+          <t>Inverted_Date_Count = 0, Future_Active_Start_Date = 0, Null_Start_Date_Count = 0. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="I46" s="18" t="inlineStr">
+        <is>
+          <t>SELECT 
+    'dim_account_information' AS TableName,
+    COUNT(*) AS TotalRecords,
+    SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) AS Inverted_Date_Count,
+    SUM(CASE WHEN is_current = 'True' AND effective_start_date &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END) AS Future_Active_Start_Date,
+    SUM(CASE WHEN effective_start_date IS NULL THEN 1 ELSE 0 END) AS Null_Start_Date_Count,
+    CASE 
+        WHEN SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN is_current = 'True' AND effective_start_date &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN effective_start_date IS NULL THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END AS TestStatus
+FROM Gold_Warehouse.tamarac.dim_account_information;</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="54" customHeight="1">
+      <c r="A47" s="12" t="inlineStr">
+        <is>
+          <t>Tamarac</t>
+        </is>
+      </c>
+      <c r="B47" s="12" t="inlineStr">
+        <is>
+          <t>TC_TAM_GOLD_12</t>
+        </is>
+      </c>
+      <c r="C47" s="13" t="inlineStr">
+        <is>
+          <t>Date Sanity &amp; Inversions</t>
+        </is>
+      </c>
+      <c r="D47" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E47" s="10" t="inlineStr">
+        <is>
+          <t>tamarac.dim_account_model_allocation</t>
+        </is>
+      </c>
+      <c r="F47" s="11" t="inlineStr">
+        <is>
+          <t>Verify Date Sanity: Zero inverted dates (start &gt; end) and active records have non-future start dates</t>
+        </is>
+      </c>
+      <c r="G47" s="11" t="inlineStr">
+        <is>
+          <t>dim_account_model_allocation populated</t>
+        </is>
+      </c>
+      <c r="H47" s="11" t="inlineStr">
+        <is>
+          <t>Inverted_Date_Count = 0, Future_Active_Start_Date = 0, Null_Start_Date_Count = 0. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="I47" s="17" t="inlineStr">
+        <is>
+          <t>SELECT 
+    'dim_account_model_allocation' AS TableName,
+    COUNT(*) AS TotalRecords,
+    SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) AS Inverted_Date_Count,
+    SUM(CASE WHEN is_current = 'True' AND effective_start_date &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END) AS Future_Active_Start_Date,
+    SUM(CASE WHEN effective_start_date IS NULL THEN 1 ELSE 0 END) AS Null_Start_Date_Count,
+    CASE 
+        WHEN SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN is_current = 'True' AND effective_start_date &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN effective_start_date IS NULL THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END AS TestStatus
+FROM Gold_Warehouse.tamarac.dim_account_model_allocation;</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="54" customHeight="1">
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>Tamarac</t>
+        </is>
+      </c>
+      <c r="B48" s="8" t="inlineStr">
+        <is>
+          <t>TC_TAM_GOLD_13</t>
+        </is>
+      </c>
+      <c r="C48" s="9" t="inlineStr">
+        <is>
+          <t>Open-Ended Active Records</t>
+        </is>
+      </c>
+      <c r="D48" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="inlineStr">
+        <is>
+          <t>tamarac.dim_account_information</t>
+        </is>
+      </c>
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t>Verify Active Records are Open-Ended (effective_end_date is NULL or '9999-12-31')</t>
+        </is>
+      </c>
+      <c r="G48" s="7" t="inlineStr">
+        <is>
+          <t>dim_account_information where is_current = 'True'</t>
+        </is>
+      </c>
+      <c r="H48" s="7" t="inlineStr">
+        <is>
+          <t>Prematurely_Ended_Active_Records = 0. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="I48" s="18" t="inlineStr">
+        <is>
+          <t>SELECT 
+    'dim_account_information' AS TableName,
+    COUNT(*) AS TotalActiveRecords,
+    SUM(CASE WHEN effective_end_date IS NOT NULL AND effective_end_date NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END) AS Prematurely_Ended_Active_Records,
+    CASE 
+        WHEN SUM(CASE WHEN effective_end_date IS NOT NULL AND effective_end_date NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END) = 0 
+        THEN 'PASSED' ELSE 'FAILED'
+    END AS TestStatus
+FROM Gold_Warehouse.tamarac.dim_account_information
+WHERE is_current = 'True';</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="54" customHeight="1">
+      <c r="A49" s="12" t="inlineStr">
+        <is>
+          <t>Tamarac</t>
+        </is>
+      </c>
+      <c r="B49" s="12" t="inlineStr">
+        <is>
+          <t>TC_TAM_GOLD_14</t>
+        </is>
+      </c>
+      <c r="C49" s="13" t="inlineStr">
+        <is>
+          <t>Open-Ended Active Records</t>
+        </is>
+      </c>
+      <c r="D49" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E49" s="10" t="inlineStr">
+        <is>
+          <t>tamarac.dim_account_model_allocation</t>
+        </is>
+      </c>
+      <c r="F49" s="11" t="inlineStr">
+        <is>
+          <t>Verify Active Records are Open-Ended (effective_end_date is NULL or '9999-12-31')</t>
+        </is>
+      </c>
+      <c r="G49" s="11" t="inlineStr">
+        <is>
+          <t>dim_account_model_allocation where is_current = 'True'</t>
+        </is>
+      </c>
+      <c r="H49" s="11" t="inlineStr">
+        <is>
+          <t>Prematurely_Ended_Active_Records = 0. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="I49" s="17" t="inlineStr">
+        <is>
+          <t>SELECT 
+    'dim_account_model_allocation' AS TableName,
+    COUNT(*) AS TotalActiveRecords,
+    SUM(CASE WHEN effective_end_date IS NOT NULL AND effective_end_date NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END) AS Prematurely_Ended_Active_Records,
+    CASE 
+        WHEN SUM(CASE WHEN effective_end_date IS NOT NULL AND effective_end_date NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END) = 0 
+        THEN 'PASSED' ELSE 'FAILED'
+    END AS TestStatus
+FROM Gold_Warehouse.tamarac.dim_account_model_allocation
+WHERE is_current = 'True';</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="54" customHeight="1">
+      <c r="A50" s="8" t="inlineStr">
+        <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B42" s="8" t="inlineStr">
+      <c r="B50" s="8" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_01</t>
         </is>
       </c>
-      <c r="C42" s="9" t="inlineStr">
+      <c r="C50" s="9" t="inlineStr">
         <is>
           <t>SCD2 Deduplication</t>
         </is>
       </c>
-      <c r="D42" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E42" s="6" t="inlineStr">
+      <c r="D50" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master</t>
         </is>
       </c>
-      <c r="F42" s="7" t="inlineStr">
+      <c r="F50" s="7" t="inlineStr">
         <is>
           <t>Verify Active Deduplication on Business Key ['customer_account_number'] (is_current = 1)</t>
         </is>
       </c>
-      <c r="G42" s="7" t="inlineStr">
+      <c r="G50" s="7" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master populated</t>
         </is>
       </c>
-      <c r="H42" s="7" t="inlineStr">
+      <c r="H50" s="7" t="inlineStr">
         <is>
           <t>Zero duplicate active accounts. Exactly one is_current = 1 record per customer_account_number.</t>
         </is>
       </c>
-      <c r="I42" s="18" t="inlineStr">
+      <c r="I50" s="18" t="inlineStr">
         <is>
           <t>SELECT customer_account_number, COUNT(*) AS ActiveDuplicateCount
 FROM Gold_Warehouse.innotrust.dim_account_master
@@ -3051,48 +3542,48 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="54" customHeight="1">
-      <c r="A43" s="12" t="inlineStr">
+    <row r="51" ht="54" customHeight="1">
+      <c r="A51" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B43" s="12" t="inlineStr">
+      <c r="B51" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_02</t>
         </is>
       </c>
-      <c r="C43" s="13" t="inlineStr">
+      <c r="C51" s="13" t="inlineStr">
         <is>
           <t>SK Uniqueness</t>
         </is>
       </c>
-      <c r="D43" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E43" s="10" t="inlineStr">
+      <c r="D51" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E51" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master</t>
         </is>
       </c>
-      <c r="F43" s="11" t="inlineStr">
+      <c r="F51" s="11" t="inlineStr">
         <is>
           <t>Verify Primary Surrogate Key (dim_account_master_sk) uniqueness and non-null constraint</t>
         </is>
       </c>
-      <c r="G43" s="11" t="inlineStr">
+      <c r="G51" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master populated</t>
         </is>
       </c>
-      <c r="H43" s="11" t="inlineStr">
+      <c r="H51" s="11" t="inlineStr">
         <is>
           <t>dim_account_master_sk is strictly unique across all versions with zero NULL values.</t>
         </is>
       </c>
-      <c r="I43" s="17" t="inlineStr">
+      <c r="I51" s="17" t="inlineStr">
         <is>
           <t>SELECT dim_account_master_sk, COUNT(*) AS DuplicateCount
 FROM Gold_Warehouse.innotrust.dim_account_master
@@ -3106,48 +3597,48 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="54" customHeight="1">
-      <c r="A44" s="8" t="inlineStr">
+    <row r="52" ht="54" customHeight="1">
+      <c r="A52" s="8" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B44" s="8" t="inlineStr">
+      <c r="B52" s="8" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_03</t>
         </is>
       </c>
-      <c r="C44" s="9" t="inlineStr">
+      <c r="C52" s="9" t="inlineStr">
         <is>
           <t>SCD2 Deduplication</t>
         </is>
       </c>
-      <c r="D44" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E44" s="6" t="inlineStr">
+      <c r="D52" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E52" s="6" t="inlineStr">
         <is>
           <t>innotrust.dim_account_category_codes</t>
         </is>
       </c>
-      <c r="F44" s="7" t="inlineStr">
+      <c r="F52" s="7" t="inlineStr">
         <is>
           <t>Verify Active Deduplication on Business Key ['account_category_code'] (is_current = 1)</t>
         </is>
       </c>
-      <c r="G44" s="7" t="inlineStr">
+      <c r="G52" s="7" t="inlineStr">
         <is>
           <t>innotrust.dim_account_category_codes populated</t>
         </is>
       </c>
-      <c r="H44" s="7" t="inlineStr">
+      <c r="H52" s="7" t="inlineStr">
         <is>
           <t>Zero duplicate active category codes per account_category_code.</t>
         </is>
       </c>
-      <c r="I44" s="18" t="inlineStr">
+      <c r="I52" s="18" t="inlineStr">
         <is>
           <t>SELECT account_category_code, COUNT(*) AS ActiveDuplicateCount
 FROM Gold_Warehouse.innotrust.dim_account_category_codes
@@ -3157,48 +3648,48 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="54" customHeight="1">
-      <c r="A45" s="12" t="inlineStr">
+    <row r="53" ht="54" customHeight="1">
+      <c r="A53" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B45" s="12" t="inlineStr">
+      <c r="B53" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_04</t>
         </is>
       </c>
-      <c r="C45" s="13" t="inlineStr">
+      <c r="C53" s="13" t="inlineStr">
         <is>
           <t>SK Uniqueness</t>
         </is>
       </c>
-      <c r="D45" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E45" s="10" t="inlineStr">
+      <c r="D53" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E53" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_account_category_codes</t>
         </is>
       </c>
-      <c r="F45" s="11" t="inlineStr">
+      <c r="F53" s="11" t="inlineStr">
         <is>
           <t>Verify Primary Surrogate Key (dim_account_master_sk) uniqueness on dim_account_category_codes</t>
         </is>
       </c>
-      <c r="G45" s="11" t="inlineStr">
+      <c r="G53" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_account_category_codes populated</t>
         </is>
       </c>
-      <c r="H45" s="11" t="inlineStr">
+      <c r="H53" s="11" t="inlineStr">
         <is>
           <t>Surrogate key dim_account_master_sk is unique across all rows with zero NULLs.</t>
         </is>
       </c>
-      <c r="I45" s="17" t="inlineStr">
+      <c r="I53" s="17" t="inlineStr">
         <is>
           <t>SELECT dim_account_master_sk, COUNT(*) AS DuplicateCount
 FROM Gold_Warehouse.innotrust.dim_account_category_codes
@@ -3207,48 +3698,48 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="54" customHeight="1">
-      <c r="A46" s="8" t="inlineStr">
+    <row r="54" ht="54" customHeight="1">
+      <c r="A54" s="8" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B46" s="8" t="inlineStr">
+      <c r="B54" s="8" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_05</t>
         </is>
       </c>
-      <c r="C46" s="9" t="inlineStr">
+      <c r="C54" s="9" t="inlineStr">
         <is>
           <t>SCD2 Deduplication</t>
         </is>
       </c>
-      <c r="D46" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E46" s="6" t="inlineStr">
+      <c r="D54" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="inlineStr">
         <is>
           <t>innotrust.dim_account_type_codes</t>
         </is>
       </c>
-      <c r="F46" s="7" t="inlineStr">
+      <c r="F54" s="7" t="inlineStr">
         <is>
           <t>Verify Active Deduplication on Business Key ['account_type_code'] (is_current = 1)</t>
         </is>
       </c>
-      <c r="G46" s="7" t="inlineStr">
+      <c r="G54" s="7" t="inlineStr">
         <is>
           <t>innotrust.dim_account_type_codes populated</t>
         </is>
       </c>
-      <c r="H46" s="7" t="inlineStr">
+      <c r="H54" s="7" t="inlineStr">
         <is>
           <t>Zero duplicate active account types per account_type_code.</t>
         </is>
       </c>
-      <c r="I46" s="18" t="inlineStr">
+      <c r="I54" s="18" t="inlineStr">
         <is>
           <t>SELECT account_type_code, COUNT(*) AS ActiveDuplicateCount
 FROM Gold_Warehouse.innotrust.dim_account_type_codes
@@ -3258,48 +3749,48 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="54" customHeight="1">
-      <c r="A47" s="12" t="inlineStr">
+    <row r="55" ht="54" customHeight="1">
+      <c r="A55" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B47" s="12" t="inlineStr">
+      <c r="B55" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_06</t>
         </is>
       </c>
-      <c r="C47" s="13" t="inlineStr">
+      <c r="C55" s="13" t="inlineStr">
         <is>
           <t>SK Uniqueness</t>
         </is>
       </c>
-      <c r="D47" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E47" s="10" t="inlineStr">
+      <c r="D55" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E55" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_account_type_codes</t>
         </is>
       </c>
-      <c r="F47" s="11" t="inlineStr">
+      <c r="F55" s="11" t="inlineStr">
         <is>
           <t>Verify Primary Surrogate Key (dim_account_type_codes_sk) uniqueness and non-null constraint</t>
         </is>
       </c>
-      <c r="G47" s="11" t="inlineStr">
+      <c r="G55" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_account_type_codes populated</t>
         </is>
       </c>
-      <c r="H47" s="11" t="inlineStr">
+      <c r="H55" s="11" t="inlineStr">
         <is>
           <t>dim_account_type_codes_sk is strictly unique across all versions with zero NULLs.</t>
         </is>
       </c>
-      <c r="I47" s="17" t="inlineStr">
+      <c r="I55" s="17" t="inlineStr">
         <is>
           <t>SELECT dim_account_type_codes_sk, COUNT(*) AS DuplicateCount
 FROM Gold_Warehouse.innotrust.dim_account_type_codes
@@ -3308,48 +3799,48 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="54" customHeight="1">
-      <c r="A48" s="8" t="inlineStr">
+    <row r="56" ht="54" customHeight="1">
+      <c r="A56" s="8" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B48" s="8" t="inlineStr">
+      <c r="B56" s="8" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_07</t>
         </is>
       </c>
-      <c r="C48" s="9" t="inlineStr">
+      <c r="C56" s="9" t="inlineStr">
         <is>
           <t>SCD2 Deduplication</t>
         </is>
       </c>
-      <c r="D48" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E48" s="6" t="inlineStr">
+      <c r="D56" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E56" s="6" t="inlineStr">
         <is>
           <t>innotrust.dim_master_sec_index</t>
         </is>
       </c>
-      <c r="F48" s="7" t="inlineStr">
+      <c r="F56" s="7" t="inlineStr">
         <is>
           <t>Verify Active Deduplication on Security Primary Key ['isin'] (is_current = 1)</t>
         </is>
       </c>
-      <c r="G48" s="7" t="inlineStr">
+      <c r="G56" s="7" t="inlineStr">
         <is>
           <t>innotrust.dim_master_sec_index populated</t>
         </is>
       </c>
-      <c r="H48" s="7" t="inlineStr">
+      <c r="H56" s="7" t="inlineStr">
         <is>
           <t>Zero duplicate active securities. Exactly one is_current = 1 record per isin.</t>
         </is>
       </c>
-      <c r="I48" s="18" t="inlineStr">
+      <c r="I56" s="18" t="inlineStr">
         <is>
           <t>SELECT isin, COUNT(*) AS ActiveDuplicateCount
 FROM Gold_Warehouse.innotrust.dim_master_sec_index
@@ -3359,48 +3850,48 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="54" customHeight="1">
-      <c r="A49" s="12" t="inlineStr">
+    <row r="57" ht="54" customHeight="1">
+      <c r="A57" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B49" s="12" t="inlineStr">
+      <c r="B57" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_08</t>
         </is>
       </c>
-      <c r="C49" s="13" t="inlineStr">
+      <c r="C57" s="13" t="inlineStr">
         <is>
           <t>SK Uniqueness</t>
         </is>
       </c>
-      <c r="D49" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E49" s="10" t="inlineStr">
+      <c r="D57" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E57" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_master_sec_index</t>
         </is>
       </c>
-      <c r="F49" s="11" t="inlineStr">
+      <c r="F57" s="11" t="inlineStr">
         <is>
           <t>Verify Primary Surrogate Key (dim_master_sec_index_sk) uniqueness across all records</t>
         </is>
       </c>
-      <c r="G49" s="11" t="inlineStr">
+      <c r="G57" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_master_sec_index populated</t>
         </is>
       </c>
-      <c r="H49" s="11" t="inlineStr">
+      <c r="H57" s="11" t="inlineStr">
         <is>
           <t>dim_master_sec_index_sk is strictly unique across all versions with zero NULLs.</t>
         </is>
       </c>
-      <c r="I49" s="17" t="inlineStr">
+      <c r="I57" s="17" t="inlineStr">
         <is>
           <t>SELECT dim_master_sec_index_sk, COUNT(*) AS DuplicateCount
 FROM Gold_Warehouse.innotrust.dim_master_sec_index
@@ -3409,48 +3900,48 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="54" customHeight="1">
-      <c r="A50" s="8" t="inlineStr">
+    <row r="58" ht="54" customHeight="1">
+      <c r="A58" s="8" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B50" s="8" t="inlineStr">
+      <c r="B58" s="8" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_09</t>
         </is>
       </c>
-      <c r="C50" s="9" t="inlineStr">
+      <c r="C58" s="9" t="inlineStr">
         <is>
           <t>SCD2 Deduplication</t>
         </is>
       </c>
-      <c r="D50" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E50" s="6" t="inlineStr">
+      <c r="D58" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="inlineStr">
         <is>
           <t>innotrust.dim_security_characteristics_codes</t>
         </is>
       </c>
-      <c r="F50" s="7" t="inlineStr">
+      <c r="F58" s="7" t="inlineStr">
         <is>
           <t>Verify Active Deduplication on Business Key ['security_type_code'] (is_current = 1)</t>
         </is>
       </c>
-      <c r="G50" s="7" t="inlineStr">
+      <c r="G58" s="7" t="inlineStr">
         <is>
           <t>innotrust.dim_security_characteristics_codes populated</t>
         </is>
       </c>
-      <c r="H50" s="7" t="inlineStr">
+      <c r="H58" s="7" t="inlineStr">
         <is>
           <t>Zero duplicate active security type codes per security_type_code.</t>
         </is>
       </c>
-      <c r="I50" s="18" t="inlineStr">
+      <c r="I58" s="18" t="inlineStr">
         <is>
           <t>SELECT security_type_code, COUNT(*) AS ActiveDuplicateCount
 FROM Gold_Warehouse.innotrust.dim_security_characteristics_codes
@@ -3460,48 +3951,48 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="54" customHeight="1">
-      <c r="A51" s="12" t="inlineStr">
+    <row r="59" ht="54" customHeight="1">
+      <c r="A59" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B51" s="12" t="inlineStr">
+      <c r="B59" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_10</t>
         </is>
       </c>
-      <c r="C51" s="13" t="inlineStr">
+      <c r="C59" s="13" t="inlineStr">
         <is>
           <t>SK Uniqueness</t>
         </is>
       </c>
-      <c r="D51" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E51" s="10" t="inlineStr">
+      <c r="D59" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E59" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_security_characteristics_codes</t>
         </is>
       </c>
-      <c r="F51" s="11" t="inlineStr">
+      <c r="F59" s="11" t="inlineStr">
         <is>
           <t>Verify Primary Surrogate Key (dim_securitycharacteristicscodes) uniqueness and non-null constraint</t>
         </is>
       </c>
-      <c r="G51" s="11" t="inlineStr">
+      <c r="G59" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_security_characteristics_codes populated</t>
         </is>
       </c>
-      <c r="H51" s="11" t="inlineStr">
+      <c r="H59" s="11" t="inlineStr">
         <is>
           <t>dim_securitycharacteristicscodes is strictly unique across all versions with zero NULLs.</t>
         </is>
       </c>
-      <c r="I51" s="17" t="inlineStr">
+      <c r="I59" s="17" t="inlineStr">
         <is>
           <t>SELECT dim_securitycharacteristicscodes, COUNT(*) AS DuplicateCount
 FROM Gold_Warehouse.innotrust.dim_security_characteristics_codes
@@ -3510,48 +4001,48 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="54" customHeight="1">
-      <c r="A52" s="8" t="inlineStr">
+    <row r="60" ht="54" customHeight="1">
+      <c r="A60" s="8" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B52" s="8" t="inlineStr">
+      <c r="B60" s="8" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_11</t>
         </is>
       </c>
-      <c r="C52" s="9" t="inlineStr">
+      <c r="C60" s="9" t="inlineStr">
         <is>
           <t>Audit &amp; Date Logic</t>
         </is>
       </c>
-      <c r="D52" s="19" t="inlineStr">
+      <c r="D60" s="19" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E52" s="6" t="inlineStr">
+      <c r="E60" s="6" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master</t>
         </is>
       </c>
-      <c r="F52" s="7" t="inlineStr">
+      <c r="F60" s="7" t="inlineStr">
         <is>
           <t>Verify business_date, updated_at, effective_start_date &amp; effective_end_date integrity on active records</t>
         </is>
       </c>
-      <c r="G52" s="7" t="inlineStr">
+      <c r="G60" s="7" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master populated</t>
         </is>
       </c>
-      <c r="H52" s="7" t="inlineStr">
+      <c r="H60" s="7" t="inlineStr">
         <is>
           <t>Zero NULLs in business_date or updated_at; effective_end_date &gt;= effective_start_date.</t>
         </is>
       </c>
-      <c r="I52" s="18" t="inlineStr">
+      <c r="I60" s="18" t="inlineStr">
         <is>
           <t>SELECT 
     COUNT(*) AS TotalActiveRows,
@@ -3564,48 +4055,48 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="54" customHeight="1">
-      <c r="A53" s="12" t="inlineStr">
+    <row r="61" ht="54" customHeight="1">
+      <c r="A61" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B53" s="12" t="inlineStr">
+      <c r="B61" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_12</t>
         </is>
       </c>
-      <c r="C53" s="13" t="inlineStr">
+      <c r="C61" s="13" t="inlineStr">
         <is>
           <t>Cross-Table Linkage</t>
         </is>
       </c>
-      <c r="D53" s="19" t="inlineStr">
+      <c r="D61" s="19" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E53" s="10" t="inlineStr">
+      <c r="E61" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master</t>
         </is>
       </c>
-      <c r="F53" s="11" t="inlineStr">
+      <c r="F61" s="11" t="inlineStr">
         <is>
           <t>Verify Referential Integrity: account_category_code and account_type_code resolve to active codes</t>
         </is>
       </c>
-      <c r="G53" s="11" t="inlineStr">
+      <c r="G61" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master populated</t>
         </is>
       </c>
-      <c r="H53" s="11" t="inlineStr">
+      <c r="H61" s="11" t="inlineStr">
         <is>
           <t>All non-null account_category_code and account_type_code exist in corresponding dimension code tables.</t>
         </is>
       </c>
-      <c r="I53" s="17" t="inlineStr">
+      <c r="I61" s="17" t="inlineStr">
         <is>
           <t>SELECT 
     SUM(CASE WHEN m.account_category_code IS NOT NULL AND cat.account_category_code IS NULL THEN 1 ELSE 0 END) AS Orphan_CategoryCodes,
@@ -3619,48 +4110,48 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="54" customHeight="1">
-      <c r="A54" s="8" t="inlineStr">
+    <row r="62" ht="54" customHeight="1">
+      <c r="A62" s="8" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B54" s="8" t="inlineStr">
+      <c r="B62" s="8" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_13</t>
         </is>
       </c>
-      <c r="C54" s="9" t="inlineStr">
+      <c r="C62" s="9" t="inlineStr">
         <is>
           <t>Cross-Table Linkage</t>
         </is>
       </c>
-      <c r="D54" s="19" t="inlineStr">
+      <c r="D62" s="19" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E54" s="6" t="inlineStr">
+      <c r="E62" s="6" t="inlineStr">
         <is>
           <t>innotrust.dim_master_sec_index</t>
         </is>
       </c>
-      <c r="F54" s="7" t="inlineStr">
+      <c r="F62" s="7" t="inlineStr">
         <is>
           <t>Verify Security Referential Integrity: security_type_code resolves to active security characteristics</t>
         </is>
       </c>
-      <c r="G54" s="7" t="inlineStr">
+      <c r="G62" s="7" t="inlineStr">
         <is>
           <t>innotrust.dim_master_sec_index populated</t>
         </is>
       </c>
-      <c r="H54" s="7" t="inlineStr">
+      <c r="H62" s="7" t="inlineStr">
         <is>
           <t>All non-null security_type_code values exist in dim_security_characteristics_codes.</t>
         </is>
       </c>
-      <c r="I54" s="18" t="inlineStr">
+      <c r="I62" s="18" t="inlineStr">
         <is>
           <t>SELECT COUNT(*) AS Orphan_SecurityTypeCodes
 FROM Gold_Warehouse.innotrust.dim_master_sec_index s
@@ -3670,48 +4161,48 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="54" customHeight="1">
-      <c r="A55" s="12" t="inlineStr">
+    <row r="63" ht="54" customHeight="1">
+      <c r="A63" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B55" s="12" t="inlineStr">
+      <c r="B63" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_14</t>
         </is>
       </c>
-      <c r="C55" s="13" t="inlineStr">
+      <c r="C63" s="13" t="inlineStr">
         <is>
           <t>SCD2 Date Validation</t>
         </is>
       </c>
-      <c r="D55" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E55" s="10" t="inlineStr">
+      <c r="D63" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E63" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master</t>
         </is>
       </c>
-      <c r="F55" s="11" t="inlineStr">
+      <c r="F63" s="11" t="inlineStr">
         <is>
           <t>Verify SCD2 Effective Date Rules: Inactive records effective_end_date &lt;= (Current Day - 1), non-null end date, and valid active start date</t>
         </is>
       </c>
-      <c r="G55" s="11" t="inlineStr">
+      <c r="G63" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master populated with SCD2 tracking columns</t>
         </is>
       </c>
-      <c r="H55" s="11" t="inlineStr">
+      <c r="H63" s="11" t="inlineStr">
         <is>
           <t>Inactive_End_Date_Breach_Count = 0, Inactive_Missing_End_Date = 0, Active_Future_Start_Date = 0, Inverted_Date_Range_Count = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I55" s="17" t="inlineStr">
+      <c r="I63" s="17" t="inlineStr">
         <is>
           <t>SELECT 
     'dim_account_master' AS TableName,
@@ -3730,48 +4221,48 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="54" customHeight="1">
-      <c r="A56" s="8" t="inlineStr">
+    <row r="64" ht="54" customHeight="1">
+      <c r="A64" s="8" t="inlineStr">
         <is>
           <t>Black Diamond (Consolidated)</t>
         </is>
       </c>
-      <c r="B56" s="8" t="inlineStr">
+      <c r="B64" s="8" t="inlineStr">
         <is>
           <t>TC_COMB_SK_BD_01</t>
         </is>
       </c>
-      <c r="C56" s="9" t="inlineStr">
+      <c r="C64" s="9" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D56" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E56" s="6" t="inlineStr">
+      <c r="D64" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E64" s="6" t="inlineStr">
         <is>
           <t>All 9 Child &amp; Fact Tables (holdings, transactions, taxlots, class/segment, details, tags, team, targets)</t>
         </is>
       </c>
-      <c r="F56" s="7" t="inlineStr">
+      <c r="F64" s="7" t="inlineStr">
         <is>
           <t>Black Diamond: Cross-Object account_sk vs dim_accounts Natural Key (accountid == da.id) Verification - Executes a single consolidated UNION ALL query across all 9 child/fact tables to verify that the attached account_sk strictly points to the exact same account natural key (child.accountid == da.id). Guarantees zero wrong account links.</t>
         </is>
       </c>
-      <c r="G56" s="7" t="inlineStr">
+      <c r="G64" s="7" t="inlineStr">
         <is>
           <t>All Gold tables populated for Black Diamond</t>
         </is>
       </c>
-      <c r="H56" s="7" t="inlineStr">
+      <c r="H64" s="7" t="inlineStr">
         <is>
           <t>Duplicate_BusinessKey_Count = 0, MismatchedAccountIdCount = 0, Null_AccountSK_Count = 0, Orphan_AccountSK_Count = 0 across all 9 objects.</t>
         </is>
       </c>
-      <c r="I56" s="18" t="inlineStr">
+      <c r="I64" s="18" t="inlineStr">
         <is>
           <t>SELECT 
     'dim_accounts_classallocation' AS TableName, 
@@ -3880,48 +4371,48 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="54" customHeight="1">
-      <c r="A57" s="12" t="inlineStr">
+    <row r="65" ht="54" customHeight="1">
+      <c r="A65" s="12" t="inlineStr">
         <is>
           <t>Schwab (Consolidated)</t>
         </is>
       </c>
-      <c r="B57" s="12" t="inlineStr">
+      <c r="B65" s="12" t="inlineStr">
         <is>
           <t>TC_COMB_SK_SC_02</t>
         </is>
       </c>
-      <c r="C57" s="13" t="inlineStr">
+      <c r="C65" s="13" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D57" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E57" s="10" t="inlineStr">
+      <c r="D65" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E65" s="10" t="inlineStr">
         <is>
           <t>All 8 Objects (dim_accounts &amp; 7 Fact Tables: recon_d1/d2, daily_closing, security, transactions, ult/uln lots)</t>
         </is>
       </c>
-      <c r="F57" s="11" t="inlineStr">
+      <c r="F65" s="11" t="inlineStr">
         <is>
           <t>Schwab: Consolidated Multi-Object SK Mapping, PK Deduplication &amp; Audit Date Health Check - Single unified query executing across all 8 Schwab Gold tables. Validates that every fact record's account_sk correctly matches dim_accounts on composite natural keys (account_id, custodian_id), confirms primary SK uniqueness, and ensures 100% audit dates populated.</t>
         </is>
       </c>
-      <c r="G57" s="11" t="inlineStr">
+      <c r="G65" s="11" t="inlineStr">
         <is>
           <t>All Gold tables populated for Schwab</t>
         </is>
       </c>
-      <c r="H57" s="11" t="inlineStr">
+      <c r="H65" s="11" t="inlineStr">
         <is>
           <t>Mismatched_AccountId_Count = 0 and Orphan_AccountSK_Count = 0 across all fact tables. All mapped account_sk strictly match the natural account_id.</t>
         </is>
       </c>
-      <c r="I57" s="17" t="inlineStr">
+      <c r="I65" s="17" t="inlineStr">
         <is>
           <t>SELECT 
     'fact_recon_position_d1' AS TableName,
@@ -3980,48 +4471,48 @@
         </is>
       </c>
     </row>
-    <row r="58" ht="54" customHeight="1">
-      <c r="A58" s="8" t="inlineStr">
+    <row r="66" ht="54" customHeight="1">
+      <c r="A66" s="8" t="inlineStr">
         <is>
           <t>Salentica CRM (Consolidated)</t>
         </is>
       </c>
-      <c r="B58" s="8" t="inlineStr">
+      <c r="B66" s="8" t="inlineStr">
         <is>
           <t>TC_COMB_SK_SAL_03</t>
         </is>
       </c>
-      <c r="C58" s="9" t="inlineStr">
+      <c r="C66" s="9" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D58" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E58" s="6" t="inlineStr">
+      <c r="D66" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E66" s="6" t="inlineStr">
         <is>
           <t>All 6 Core CRM Entities (dim_account, dim_contact_core, dim_family, fact_lead, fact_opportunity, fact_investmentaccount)</t>
         </is>
       </c>
-      <c r="F58" s="7" t="inlineStr">
+      <c r="F66" s="7" t="inlineStr">
         <is>
           <t>Salentica: Consolidated Point-in-Time Referential SK Mapping (Active &amp; Historical Mapping Validation) - Single unified query executing across all 6 core Salentica CRM tables. Validates that every attached foreign SK resolves to the same Natural Key in parent dimensions (allowing active OR expired parent versions to preserve point-in-time audit history) and checks for broken orphans.</t>
         </is>
       </c>
-      <c r="G58" s="7" t="inlineStr">
+      <c r="G66" s="7" t="inlineStr">
         <is>
           <t>All Gold tables populated for Salentica CRM</t>
         </is>
       </c>
-      <c r="H58" s="7" t="inlineStr">
+      <c r="H66" s="7" t="inlineStr">
         <is>
           <t>Mismatched_PrimaryContact_NK = 0, Mismatched_BusinessUnit_NK = 0, Broken_Orphan_Count = 0 across all 6 CRM tables.</t>
         </is>
       </c>
-      <c r="I58" s="18" t="inlineStr">
+      <c r="I66" s="18" t="inlineStr">
         <is>
           <t>SELECT 'dim_account' AS TableName, COUNT(*) AS TotalActiveRows,
     SUM(CASE WHEN a.primarycontactid IS NOT NULL AND a.primarycontactid_sk &lt;&gt; -1 AND a.primarycontactid &lt;&gt; c.contactid THEN 1 ELSE 0 END) AS Mismatched_PrimaryContact_NK,
@@ -4085,48 +4576,48 @@
         </is>
       </c>
     </row>
-    <row r="59" ht="54" customHeight="1">
-      <c r="A59" s="12" t="inlineStr">
+    <row r="67" ht="54" customHeight="1">
+      <c r="A67" s="12" t="inlineStr">
         <is>
           <t>Tamarac (Consolidated)</t>
         </is>
       </c>
-      <c r="B59" s="12" t="inlineStr">
+      <c r="B67" s="12" t="inlineStr">
         <is>
           <t>TC_COMB_SK_TAM_04</t>
         </is>
       </c>
-      <c r="C59" s="13" t="inlineStr">
+      <c r="C67" s="13" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D59" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E59" s="10" t="inlineStr">
+      <c r="D67" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E67" s="10" t="inlineStr">
         <is>
           <t>Both Tables (dim_account_information, dim_account_model_allocation)</t>
         </is>
       </c>
-      <c r="F59" s="11" t="inlineStr">
+      <c r="F67" s="11" t="inlineStr">
         <is>
           <t>Tamarac: Consolidated Multi-Object PK Deduplication, Primary SK &amp; Cross-Table Linkage - Single unified query validating SCD2 active uniqueness on exact PK columns (['account_number'] and ['account_number', 'model_name']), surrogate key uniqueness, and cross-table referential integrity between model allocations and accounts.</t>
         </is>
       </c>
-      <c r="G59" s="11" t="inlineStr">
+      <c r="G67" s="11" t="inlineStr">
         <is>
           <t>All Gold tables populated for Tamarac</t>
         </is>
       </c>
-      <c r="H59" s="11" t="inlineStr">
+      <c r="H67" s="11" t="inlineStr">
         <is>
           <t>PK_Active_Duplicates = 0, Duplicate_Primary_SK = 0, Orphan_Accounts = 0, Missing_BusinessDate = 0 across both tables.</t>
         </is>
       </c>
-      <c r="I59" s="17" t="inlineStr">
+      <c r="I67" s="17" t="inlineStr">
         <is>
           <t>SELECT 'dim_account_information' AS TableName, COUNT(*) AS TotalActiveRows,
     (SELECT COUNT(*) FROM (SELECT account_number FROM Gold_Warehouse.tamarac.dim_account_information WHERE is_current = 'True' GROUP BY account_number HAVING COUNT(*) &gt; 1) d) AS PK_Active_Duplicates,
@@ -4149,48 +4640,48 @@
         </is>
       </c>
     </row>
-    <row r="60" ht="54" customHeight="1">
-      <c r="A60" s="8" t="inlineStr">
+    <row r="68" ht="54" customHeight="1">
+      <c r="A68" s="8" t="inlineStr">
         <is>
           <t>Innotrust (Consolidated)</t>
         </is>
       </c>
-      <c r="B60" s="8" t="inlineStr">
+      <c r="B68" s="8" t="inlineStr">
         <is>
           <t>TC_COMB_SK_INNO_05</t>
         </is>
       </c>
-      <c r="C60" s="9" t="inlineStr">
+      <c r="C68" s="9" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D60" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E60" s="6" t="inlineStr">
+      <c r="D68" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E68" s="6" t="inlineStr">
         <is>
           <t>All 5 Innotrust Dimensions (dim_account_master, category_codes, type_codes, sec_index, characteristics)</t>
         </is>
       </c>
-      <c r="F60" s="7" t="inlineStr">
+      <c r="F68" s="7" t="inlineStr">
         <is>
           <t>Innotrust: Consolidated Multi-Object PK Deduplication, Primary SK &amp; Cross-Dimension Linkage - Single unified query validating SCD2 active uniqueness on exact natural keys, primary surrogate key uniqueness, and cross-dimension referential integrity between master entities and classification codes.</t>
         </is>
       </c>
-      <c r="G60" s="7" t="inlineStr">
+      <c r="G68" s="7" t="inlineStr">
         <is>
           <t>All Gold tables populated for Innotrust</t>
         </is>
       </c>
-      <c r="H60" s="7" t="inlineStr">
+      <c r="H68" s="7" t="inlineStr">
         <is>
           <t>PK_Active_Duplicates = 0, Duplicate_Primary_SK = 0, Orphan_Foreign_References = 0, Missing_BusinessDate = 0 across all 5 Innotrust tables.</t>
         </is>
       </c>
-      <c r="I60" s="18" t="inlineStr">
+      <c r="I68" s="18" t="inlineStr">
         <is>
           <t>SELECT 'dim_account_master' AS TableName, COUNT(*) AS TotalActiveRows,
     (SELECT COUNT(*) FROM (SELECT customer_account_number FROM Gold_Warehouse.innotrust.dim_account_master WHERE is_current = 1 GROUP BY customer_account_number HAVING COUNT(*) &gt; 1) d) AS PK_Active_Duplicates,
@@ -4240,48 +4731,48 @@
         </is>
       </c>
     </row>
-    <row r="61" ht="54" customHeight="1">
-      <c r="A61" s="12" t="inlineStr">
+    <row r="69" ht="54" customHeight="1">
+      <c r="A69" s="12" t="inlineStr">
         <is>
           <t>Innotrust (Consolidated)</t>
         </is>
       </c>
-      <c r="B61" s="12" t="inlineStr">
+      <c r="B69" s="12" t="inlineStr">
         <is>
           <t>TC_COMB_SK_INNO_06</t>
         </is>
       </c>
-      <c r="C61" s="13" t="inlineStr">
+      <c r="C69" s="13" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D61" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E61" s="10" t="inlineStr">
+      <c r="D69" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E69" s="10" t="inlineStr">
         <is>
           <t>All 5 Innotrust Dimensions (dim_account_master, category_codes, type_codes, sec_index, characteristics)</t>
         </is>
       </c>
-      <c r="F61" s="11" t="inlineStr">
+      <c r="F69" s="11" t="inlineStr">
         <is>
           <t>Innotrust: Consolidated Multi-Object SCD2 Effective Start &amp; End Date Audit (End Date &lt;= Today - 1) - Validates across all 5 Innotrust dimensions that inactive records (is_current = 0) have effective_end_date &lt;= (current day - 1), non-null end dates, active records have non-future start dates, and zero inverted date ranges.</t>
         </is>
       </c>
-      <c r="G61" s="11" t="inlineStr">
+      <c r="G69" s="11" t="inlineStr">
         <is>
           <t>All Gold tables populated for Innotrust</t>
         </is>
       </c>
-      <c r="H61" s="11" t="inlineStr">
+      <c r="H69" s="11" t="inlineStr">
         <is>
           <t>Inactive_End_Date_Breach_Count = 0, Inactive_Missing_End_Date = 0, Active_Future_Start_Date = 0, Inverted_Date_Range_Count = 0 across all 5 tables.</t>
         </is>
       </c>
-      <c r="I61" s="17" t="inlineStr">
+      <c r="I69" s="17" t="inlineStr">
         <is>
           <t>SELECT 
     'dim_account_master' AS TableName,
@@ -6165,7 +6656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6500,6 +6991,457 @@
     ON ma.account_number = info.account_number AND info.is_current = 'True'
 WHERE ma.is_current = 'True' 
   AND info.account_information_SK IS NULL;</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="54" customHeight="1">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>TC_TAM_GOLD_07</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>SCD2 Date Validation</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>tamarac.dim_account_information</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>Verify Inactive End Date Rule: effective_end_date &lt;= (MAX(file_business_date) - 1 day) and non-null</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>dim_account_information populated with inactive records</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>Exceeded_Cutoff_Count = 0, Null_End_Date_Count = 0. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="H9" s="17" t="inlineStr">
+        <is>
+          <t>SELECT 
+    'dim_account_information' AS TableName,
+    COUNT(*) AS TotalInactiveRows,
+    CAST(m.CutoffDate AS VARCHAR(10)) AS Max_Cutoff_Allowed,
+    SUM(CASE WHEN a.effective_end_date &gt; m.CutoffDate THEN 1 ELSE 0 END) AS Exceeded_Cutoff_Count,
+    SUM(CASE WHEN a.effective_end_date IS NULL THEN 1 ELSE 0 END) AS Null_End_Date_Count,
+    CASE 
+        WHEN SUM(CASE WHEN a.effective_end_date &gt; m.CutoffDate THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN a.effective_end_date IS NULL THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END AS TestStatus
+FROM Gold_Warehouse.tamarac.dim_account_information a
+CROSS JOIN (SELECT DATEADD(day, -1, MAX(file_business_date)) AS CutoffDate FROM Gold_Warehouse.tamarac.dim_account_information) m
+WHERE a.is_current = 'False'
+GROUP BY m.CutoffDate;</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="54" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>TC_TAM_GOLD_08</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>SCD2 Date Validation</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>tamarac.dim_account_model_allocation</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Verify Inactive End Date Rule: effective_end_date &lt;= (MAX(file_business_date) - 1 day) and non-null</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>dim_account_model_allocation populated with inactive records</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>Exceeded_Cutoff_Count = 0, Null_End_Date_Count = 0. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>SELECT 
+    'dim_account_model_allocation' AS TableName,
+    COUNT(*) AS TotalInactiveRows,
+    CAST(m.CutoffDate AS VARCHAR(10)) AS Max_Cutoff_Allowed,
+    SUM(CASE WHEN a.effective_end_date &gt; m.CutoffDate THEN 1 ELSE 0 END) AS Exceeded_Cutoff_Count,
+    SUM(CASE WHEN a.effective_end_date IS NULL THEN 1 ELSE 0 END) AS Null_End_Date_Count,
+    CASE 
+        WHEN SUM(CASE WHEN a.effective_end_date &gt; m.CutoffDate THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN a.effective_end_date IS NULL THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END AS TestStatus
+FROM Gold_Warehouse.tamarac.dim_account_model_allocation a
+CROSS JOIN (SELECT DATEADD(day, -1, MAX(file_business_date)) AS CutoffDate FROM Gold_Warehouse.tamarac.dim_account_model_allocation) m
+WHERE a.is_current = 'False'
+GROUP BY m.CutoffDate;</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="54" customHeight="1">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>TC_TAM_GOLD_09</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>SCD2 Timeline &amp; SK Monotonicity</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>tamarac.dim_account_information</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>Verify SCD2 Timeline Continuity (Zero Gaps, Zero Overlaps) &amp; SK Monotonic Increment</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>dim_account_information with multiple versions per account_number</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>Timeline_Gap_Or_Overlap_Count = 0, SK_Non_Incrementing_Violation_Count = 0. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="H11" s="17" t="inlineStr">
+        <is>
+          <t>;WITH InfoTimeline AS (
+    SELECT 
+        account_number,
+        account_information_SK,
+        effective_start_date,
+        effective_end_date,
+        is_current,
+        LEAD(effective_start_date) OVER (PARTITION BY account_number ORDER BY effective_start_date, account_information_SK) AS next_start_date,
+        LEAD(account_information_SK) OVER (PARTITION BY account_number ORDER BY effective_start_date, account_information_SK) AS next_sk
+    FROM Gold_Warehouse.tamarac.dim_account_information
+)
+SELECT 
+    'dim_account_information' AS TableName,
+    COUNT(*) AS MultiVersionRecordsChecked,
+    SUM(CASE WHEN next_start_date IS NOT NULL AND effective_end_date &lt;&gt; DATEADD(day, -1, next_start_date) THEN 1 ELSE 0 END) AS Timeline_Gap_Or_Overlap_Count,
+    SUM(CASE WHEN next_sk IS NOT NULL AND next_sk &lt;= account_information_SK THEN 1 ELSE 0 END) AS SK_Non_Incrementing_Violation_Count,
+    CASE 
+        WHEN SUM(CASE WHEN next_start_date IS NOT NULL AND effective_end_date &lt;&gt; DATEADD(day, -1, next_start_date) THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN next_sk IS NOT NULL AND next_sk &lt;= account_information_SK THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END AS TestStatus
+FROM InfoTimeline
+WHERE next_start_date IS NOT NULL;</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="54" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>TC_TAM_GOLD_10</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>SCD2 Timeline &amp; SK Monotonicity</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>tamarac.dim_account_model_allocation</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Verify SCD2 Timeline Continuity (Zero Gaps, Zero Overlaps) &amp; SK Monotonic Increment</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>dim_account_model_allocation with multiple versions per composite key</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>Timeline_Gap_Or_Overlap_Count = 0, SK_Non_Incrementing_Violation_Count = 0. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>;WITH ModelTimeline AS (
+    SELECT 
+        account_number,
+        model_name,
+        account_model_SK,
+        effective_start_date,
+        effective_end_date,
+        is_current,
+        LEAD(effective_start_date) OVER (PARTITION BY account_number, model_name ORDER BY effective_start_date, account_model_SK) AS next_start_date,
+        LEAD(account_model_SK) OVER (PARTITION BY account_number, model_name ORDER BY effective_start_date, account_model_SK) AS next_sk
+    FROM Gold_Warehouse.tamarac.dim_account_model_allocation
+)
+SELECT 
+    'dim_account_model_allocation' AS TableName,
+    COUNT(*) AS MultiVersionRecordsChecked,
+    SUM(CASE WHEN next_start_date IS NOT NULL AND effective_end_date &lt;&gt; DATEADD(day, -1, next_start_date) THEN 1 ELSE 0 END) AS Timeline_Gap_Or_Overlap_Count,
+    SUM(CASE WHEN next_sk IS NOT NULL AND next_sk &lt;= account_model_SK THEN 1 ELSE 0 END) AS SK_Non_Incrementing_Violation_Count,
+    CASE 
+        WHEN SUM(CASE WHEN next_start_date IS NOT NULL AND effective_end_date &lt;&gt; DATEADD(day, -1, next_start_date) THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN next_sk IS NOT NULL AND next_sk &lt;= account_model_SK THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END AS TestStatus
+FROM ModelTimeline
+WHERE next_start_date IS NOT NULL;</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="54" customHeight="1">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>TC_TAM_GOLD_11</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Date Sanity &amp; Inversions</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>tamarac.dim_account_information</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>Verify Date Sanity: Zero inverted dates (start &gt; end) and active records have non-future start dates</t>
+        </is>
+      </c>
+      <c r="F13" s="11" t="inlineStr">
+        <is>
+          <t>dim_account_information populated</t>
+        </is>
+      </c>
+      <c r="G13" s="11" t="inlineStr">
+        <is>
+          <t>Inverted_Date_Count = 0, Future_Active_Start_Date = 0, Null_Start_Date_Count = 0. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="H13" s="17" t="inlineStr">
+        <is>
+          <t>SELECT 
+    'dim_account_information' AS TableName,
+    COUNT(*) AS TotalRecords,
+    SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) AS Inverted_Date_Count,
+    SUM(CASE WHEN is_current = 'True' AND effective_start_date &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END) AS Future_Active_Start_Date,
+    SUM(CASE WHEN effective_start_date IS NULL THEN 1 ELSE 0 END) AS Null_Start_Date_Count,
+    CASE 
+        WHEN SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN is_current = 'True' AND effective_start_date &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN effective_start_date IS NULL THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END AS TestStatus
+FROM Gold_Warehouse.tamarac.dim_account_information;</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="54" customHeight="1">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>TC_TAM_GOLD_12</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Date Sanity &amp; Inversions</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>tamarac.dim_account_model_allocation</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Verify Date Sanity: Zero inverted dates (start &gt; end) and active records have non-future start dates</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>dim_account_model_allocation populated</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>Inverted_Date_Count = 0, Future_Active_Start_Date = 0, Null_Start_Date_Count = 0. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>SELECT 
+    'dim_account_model_allocation' AS TableName,
+    COUNT(*) AS TotalRecords,
+    SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) AS Inverted_Date_Count,
+    SUM(CASE WHEN is_current = 'True' AND effective_start_date &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END) AS Future_Active_Start_Date,
+    SUM(CASE WHEN effective_start_date IS NULL THEN 1 ELSE 0 END) AS Null_Start_Date_Count,
+    CASE 
+        WHEN SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN is_current = 'True' AND effective_start_date &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN effective_start_date IS NULL THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END AS TestStatus
+FROM Gold_Warehouse.tamarac.dim_account_model_allocation;</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="54" customHeight="1">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>TC_TAM_GOLD_13</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>Open-Ended Active Records</t>
+        </is>
+      </c>
+      <c r="C15" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>tamarac.dim_account_information</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>Verify Active Records are Open-Ended (effective_end_date is NULL or '9999-12-31')</t>
+        </is>
+      </c>
+      <c r="F15" s="11" t="inlineStr">
+        <is>
+          <t>dim_account_information where is_current = 'True'</t>
+        </is>
+      </c>
+      <c r="G15" s="11" t="inlineStr">
+        <is>
+          <t>Prematurely_Ended_Active_Records = 0. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="H15" s="17" t="inlineStr">
+        <is>
+          <t>SELECT 
+    'dim_account_information' AS TableName,
+    COUNT(*) AS TotalActiveRecords,
+    SUM(CASE WHEN effective_end_date IS NOT NULL AND effective_end_date NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END) AS Prematurely_Ended_Active_Records,
+    CASE 
+        WHEN SUM(CASE WHEN effective_end_date IS NOT NULL AND effective_end_date NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END) = 0 
+        THEN 'PASSED' ELSE 'FAILED'
+    END AS TestStatus
+FROM Gold_Warehouse.tamarac.dim_account_information
+WHERE is_current = 'True';</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="54" customHeight="1">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>TC_TAM_GOLD_14</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Open-Ended Active Records</t>
+        </is>
+      </c>
+      <c r="C16" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>tamarac.dim_account_model_allocation</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>Verify Active Records are Open-Ended (effective_end_date is NULL or '9999-12-31')</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>dim_account_model_allocation where is_current = 'True'</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>Prematurely_Ended_Active_Records = 0. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>SELECT 
+    'dim_account_model_allocation' AS TableName,
+    COUNT(*) AS TotalActiveRecords,
+    SUM(CASE WHEN effective_end_date IS NOT NULL AND effective_end_date NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END) AS Prematurely_Ended_Active_Records,
+    CASE 
+        WHEN SUM(CASE WHEN effective_end_date IS NOT NULL AND effective_end_date NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END) = 0 
+        THEN 'PASSED' ELSE 'FAILED'
+    END AS TestStatus
+FROM Gold_Warehouse.tamarac.dim_account_model_allocation
+WHERE is_current = 'True';</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add TC_TAM_GOLD_15 and TC_TAM_GOLD_16: Version evolution, incremental SK and advancing effective start date audits
</commit_message>
<xml_diff>
--- a/Gold_Data_Validation_Test_Cases.xlsx
+++ b/Gold_Data_Validation_Test_Cases.xlsx
@@ -644,10 +644,10 @@
         <v>5</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F5" s="4" t="n">
         <v>16</v>
@@ -798,10 +798,10 @@
         </is>
       </c>
       <c r="C11" s="12" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D11" s="13" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E11" s="13" t="n">
         <v>4</v>
@@ -860,10 +860,10 @@
         </is>
       </c>
       <c r="C13" s="15" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D13" s="15" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E13" s="15" t="n">
         <v>16</v>
@@ -898,7 +898,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I69"/>
+  <dimension ref="A1:I71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3494,45 +3494,196 @@
     <row r="50" ht="54" customHeight="1">
       <c r="A50" s="8" t="inlineStr">
         <is>
+          <t>Tamarac</t>
+        </is>
+      </c>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>TC_TAM_GOLD_15</t>
+        </is>
+      </c>
+      <c r="C50" s="9" t="inlineStr">
+        <is>
+          <t>Version Evolution Audit</t>
+        </is>
+      </c>
+      <c r="D50" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="inlineStr">
+        <is>
+          <t>tamarac.dim_account_information</t>
+        </is>
+      </c>
+      <c r="F50" s="7" t="inlineStr">
+        <is>
+          <t>Verify Run Evolution: Every new run produces New Incremented SK, Advancing Start Date, and Latest Version is Active</t>
+        </is>
+      </c>
+      <c r="G50" s="7" t="inlineStr">
+        <is>
+          <t>dim_account_information with historical batch progression</t>
+        </is>
+      </c>
+      <c r="H50" s="7" t="inlineStr">
+        <is>
+          <t>Reused_Or_NonIncrementing_SK_Count = 0, NonAdvancing_EffectiveStartDate_Count = 0, Timeline_Gap_Or_Overlap_Count = 0, LatestVersion_Not_Active_Count = 0. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="I50" s="18" t="inlineStr">
+        <is>
+          <t>;WITH VersionChains AS (
+    SELECT 
+        account_number,
+        account_information_SK,
+        effective_start_date,
+        effective_end_date,
+        is_current,
+        file_business_date,
+        updated_at,
+        LEAD(account_information_SK) OVER (PARTITION BY account_number ORDER BY effective_start_date, account_information_SK) AS next_sk,
+        LEAD(effective_start_date) OVER (PARTITION BY account_number ORDER BY effective_start_date, account_information_SK) AS next_start_date,
+        ROW_NUMBER() OVER (PARTITION BY account_number ORDER BY effective_start_date DESC, account_information_SK DESC) AS rn_latest
+    FROM Gold_Warehouse.tamarac.dim_account_information
+)
+SELECT 
+    'dim_account_information' AS TableName,
+    COUNT(*) AS TotalVersionsAudited,
+    SUM(CASE WHEN next_sk IS NOT NULL AND next_sk &lt;= account_information_SK THEN 1 ELSE 0 END) AS Reused_Or_NonIncrementing_SK_Count,
+    SUM(CASE WHEN next_start_date IS NOT NULL AND next_start_date &lt;= effective_start_date THEN 1 ELSE 0 END) AS NonAdvancing_EffectiveStartDate_Count,
+    SUM(CASE WHEN next_start_date IS NOT NULL AND effective_end_date &lt;&gt; DATEADD(day, -1, next_start_date) THEN 1 ELSE 0 END) AS Timeline_Gap_Or_Overlap_Count,
+    SUM(CASE WHEN rn_latest = 1 AND is_current &lt;&gt; 'True' THEN 1 ELSE 0 END) AS LatestVersion_Not_Active_Count,
+    CASE 
+        WHEN SUM(CASE WHEN next_sk IS NOT NULL AND next_sk &lt;= account_information_SK THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN next_start_date IS NOT NULL AND next_start_date &lt;= effective_start_date THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN next_start_date IS NOT NULL AND effective_end_date &lt;&gt; DATEADD(day, -1, next_start_date) THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN rn_latest = 1 AND is_current &lt;&gt; 'True' THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END AS TestStatus
+FROM VersionChains;</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="54" customHeight="1">
+      <c r="A51" s="12" t="inlineStr">
+        <is>
+          <t>Tamarac</t>
+        </is>
+      </c>
+      <c r="B51" s="12" t="inlineStr">
+        <is>
+          <t>TC_TAM_GOLD_16</t>
+        </is>
+      </c>
+      <c r="C51" s="13" t="inlineStr">
+        <is>
+          <t>Version Evolution Audit</t>
+        </is>
+      </c>
+      <c r="D51" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E51" s="10" t="inlineStr">
+        <is>
+          <t>tamarac.dim_account_model_allocation</t>
+        </is>
+      </c>
+      <c r="F51" s="11" t="inlineStr">
+        <is>
+          <t>Verify Run Evolution: Every new run produces New Incremented SK, Advancing Start Date, and Latest Version is Active</t>
+        </is>
+      </c>
+      <c r="G51" s="11" t="inlineStr">
+        <is>
+          <t>dim_account_model_allocation with historical batch progression</t>
+        </is>
+      </c>
+      <c r="H51" s="11" t="inlineStr">
+        <is>
+          <t>Reused_Or_NonIncrementing_SK_Count = 0, NonAdvancing_EffectiveStartDate_Count = 0, Timeline_Gap_Or_Overlap_Count = 0, LatestVersion_Not_Active_Count = 0. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="I51" s="17" t="inlineStr">
+        <is>
+          <t>;WITH ModelChains AS (
+    SELECT 
+        account_number,
+        model_name,
+        account_model_SK,
+        effective_start_date,
+        effective_end_date,
+        is_current,
+        file_business_date,
+        updated_at,
+        LEAD(account_model_SK) OVER (PARTITION BY account_number, model_name ORDER BY effective_start_date, account_model_SK) AS next_sk,
+        LEAD(effective_start_date) OVER (PARTITION BY account_number, model_name ORDER BY effective_start_date, account_model_SK) AS next_start_date,
+        ROW_NUMBER() OVER (PARTITION BY account_number, model_name ORDER BY effective_start_date DESC, account_model_SK DESC) AS rn_latest
+    FROM Gold_Warehouse.tamarac.dim_account_model_allocation
+)
+SELECT 
+    'dim_account_model_allocation' AS TableName,
+    COUNT(*) AS TotalVersionsAudited,
+    SUM(CASE WHEN next_sk IS NOT NULL AND next_sk &lt;= account_model_SK THEN 1 ELSE 0 END) AS Reused_Or_NonIncrementing_SK_Count,
+    SUM(CASE WHEN next_start_date IS NOT NULL AND next_start_date &lt;= effective_start_date THEN 1 ELSE 0 END) AS NonAdvancing_EffectiveStartDate_Count,
+    SUM(CASE WHEN next_start_date IS NOT NULL AND effective_end_date &lt;&gt; DATEADD(day, -1, next_start_date) THEN 1 ELSE 0 END) AS Timeline_Gap_Or_Overlap_Count,
+    SUM(CASE WHEN rn_latest = 1 AND is_current &lt;&gt; 'True' THEN 1 ELSE 0 END) AS LatestVersion_Not_Active_Count,
+    CASE 
+        WHEN SUM(CASE WHEN next_sk IS NOT NULL AND next_sk &lt;= account_model_SK THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN next_start_date IS NOT NULL AND next_start_date &lt;= effective_start_date THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN next_start_date IS NOT NULL AND effective_end_date &lt;&gt; DATEADD(day, -1, next_start_date) THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN rn_latest = 1 AND is_current &lt;&gt; 'True' THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END AS TestStatus
+FROM ModelChains;</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="54" customHeight="1">
+      <c r="A52" s="8" t="inlineStr">
+        <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B50" s="8" t="inlineStr">
+      <c r="B52" s="8" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_01</t>
         </is>
       </c>
-      <c r="C50" s="9" t="inlineStr">
+      <c r="C52" s="9" t="inlineStr">
         <is>
           <t>SCD2 Deduplication</t>
         </is>
       </c>
-      <c r="D50" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E50" s="6" t="inlineStr">
+      <c r="D52" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E52" s="6" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master</t>
         </is>
       </c>
-      <c r="F50" s="7" t="inlineStr">
+      <c r="F52" s="7" t="inlineStr">
         <is>
           <t>Verify Active Deduplication on Business Key ['customer_account_number'] (is_current = 1)</t>
         </is>
       </c>
-      <c r="G50" s="7" t="inlineStr">
+      <c r="G52" s="7" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master populated</t>
         </is>
       </c>
-      <c r="H50" s="7" t="inlineStr">
+      <c r="H52" s="7" t="inlineStr">
         <is>
           <t>Zero duplicate active accounts. Exactly one is_current = 1 record per customer_account_number.</t>
         </is>
       </c>
-      <c r="I50" s="18" t="inlineStr">
+      <c r="I52" s="18" t="inlineStr">
         <is>
           <t>SELECT customer_account_number, COUNT(*) AS ActiveDuplicateCount
 FROM Gold_Warehouse.innotrust.dim_account_master
@@ -3542,48 +3693,48 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="54" customHeight="1">
-      <c r="A51" s="12" t="inlineStr">
+    <row r="53" ht="54" customHeight="1">
+      <c r="A53" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B51" s="12" t="inlineStr">
+      <c r="B53" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_02</t>
         </is>
       </c>
-      <c r="C51" s="13" t="inlineStr">
+      <c r="C53" s="13" t="inlineStr">
         <is>
           <t>SK Uniqueness</t>
         </is>
       </c>
-      <c r="D51" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E51" s="10" t="inlineStr">
+      <c r="D53" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E53" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master</t>
         </is>
       </c>
-      <c r="F51" s="11" t="inlineStr">
+      <c r="F53" s="11" t="inlineStr">
         <is>
           <t>Verify Primary Surrogate Key (dim_account_master_sk) uniqueness and non-null constraint</t>
         </is>
       </c>
-      <c r="G51" s="11" t="inlineStr">
+      <c r="G53" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master populated</t>
         </is>
       </c>
-      <c r="H51" s="11" t="inlineStr">
+      <c r="H53" s="11" t="inlineStr">
         <is>
           <t>dim_account_master_sk is strictly unique across all versions with zero NULL values.</t>
         </is>
       </c>
-      <c r="I51" s="17" t="inlineStr">
+      <c r="I53" s="17" t="inlineStr">
         <is>
           <t>SELECT dim_account_master_sk, COUNT(*) AS DuplicateCount
 FROM Gold_Warehouse.innotrust.dim_account_master
@@ -3597,48 +3748,48 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="54" customHeight="1">
-      <c r="A52" s="8" t="inlineStr">
+    <row r="54" ht="54" customHeight="1">
+      <c r="A54" s="8" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B52" s="8" t="inlineStr">
+      <c r="B54" s="8" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_03</t>
         </is>
       </c>
-      <c r="C52" s="9" t="inlineStr">
+      <c r="C54" s="9" t="inlineStr">
         <is>
           <t>SCD2 Deduplication</t>
         </is>
       </c>
-      <c r="D52" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E52" s="6" t="inlineStr">
+      <c r="D54" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="inlineStr">
         <is>
           <t>innotrust.dim_account_category_codes</t>
         </is>
       </c>
-      <c r="F52" s="7" t="inlineStr">
+      <c r="F54" s="7" t="inlineStr">
         <is>
           <t>Verify Active Deduplication on Business Key ['account_category_code'] (is_current = 1)</t>
         </is>
       </c>
-      <c r="G52" s="7" t="inlineStr">
+      <c r="G54" s="7" t="inlineStr">
         <is>
           <t>innotrust.dim_account_category_codes populated</t>
         </is>
       </c>
-      <c r="H52" s="7" t="inlineStr">
+      <c r="H54" s="7" t="inlineStr">
         <is>
           <t>Zero duplicate active category codes per account_category_code.</t>
         </is>
       </c>
-      <c r="I52" s="18" t="inlineStr">
+      <c r="I54" s="18" t="inlineStr">
         <is>
           <t>SELECT account_category_code, COUNT(*) AS ActiveDuplicateCount
 FROM Gold_Warehouse.innotrust.dim_account_category_codes
@@ -3648,48 +3799,48 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="54" customHeight="1">
-      <c r="A53" s="12" t="inlineStr">
+    <row r="55" ht="54" customHeight="1">
+      <c r="A55" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B53" s="12" t="inlineStr">
+      <c r="B55" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_04</t>
         </is>
       </c>
-      <c r="C53" s="13" t="inlineStr">
+      <c r="C55" s="13" t="inlineStr">
         <is>
           <t>SK Uniqueness</t>
         </is>
       </c>
-      <c r="D53" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E53" s="10" t="inlineStr">
+      <c r="D55" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E55" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_account_category_codes</t>
         </is>
       </c>
-      <c r="F53" s="11" t="inlineStr">
+      <c r="F55" s="11" t="inlineStr">
         <is>
           <t>Verify Primary Surrogate Key (dim_account_master_sk) uniqueness on dim_account_category_codes</t>
         </is>
       </c>
-      <c r="G53" s="11" t="inlineStr">
+      <c r="G55" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_account_category_codes populated</t>
         </is>
       </c>
-      <c r="H53" s="11" t="inlineStr">
+      <c r="H55" s="11" t="inlineStr">
         <is>
           <t>Surrogate key dim_account_master_sk is unique across all rows with zero NULLs.</t>
         </is>
       </c>
-      <c r="I53" s="17" t="inlineStr">
+      <c r="I55" s="17" t="inlineStr">
         <is>
           <t>SELECT dim_account_master_sk, COUNT(*) AS DuplicateCount
 FROM Gold_Warehouse.innotrust.dim_account_category_codes
@@ -3698,48 +3849,48 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="54" customHeight="1">
-      <c r="A54" s="8" t="inlineStr">
+    <row r="56" ht="54" customHeight="1">
+      <c r="A56" s="8" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B54" s="8" t="inlineStr">
+      <c r="B56" s="8" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_05</t>
         </is>
       </c>
-      <c r="C54" s="9" t="inlineStr">
+      <c r="C56" s="9" t="inlineStr">
         <is>
           <t>SCD2 Deduplication</t>
         </is>
       </c>
-      <c r="D54" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E54" s="6" t="inlineStr">
+      <c r="D56" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E56" s="6" t="inlineStr">
         <is>
           <t>innotrust.dim_account_type_codes</t>
         </is>
       </c>
-      <c r="F54" s="7" t="inlineStr">
+      <c r="F56" s="7" t="inlineStr">
         <is>
           <t>Verify Active Deduplication on Business Key ['account_type_code'] (is_current = 1)</t>
         </is>
       </c>
-      <c r="G54" s="7" t="inlineStr">
+      <c r="G56" s="7" t="inlineStr">
         <is>
           <t>innotrust.dim_account_type_codes populated</t>
         </is>
       </c>
-      <c r="H54" s="7" t="inlineStr">
+      <c r="H56" s="7" t="inlineStr">
         <is>
           <t>Zero duplicate active account types per account_type_code.</t>
         </is>
       </c>
-      <c r="I54" s="18" t="inlineStr">
+      <c r="I56" s="18" t="inlineStr">
         <is>
           <t>SELECT account_type_code, COUNT(*) AS ActiveDuplicateCount
 FROM Gold_Warehouse.innotrust.dim_account_type_codes
@@ -3749,48 +3900,48 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="54" customHeight="1">
-      <c r="A55" s="12" t="inlineStr">
+    <row r="57" ht="54" customHeight="1">
+      <c r="A57" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B55" s="12" t="inlineStr">
+      <c r="B57" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_06</t>
         </is>
       </c>
-      <c r="C55" s="13" t="inlineStr">
+      <c r="C57" s="13" t="inlineStr">
         <is>
           <t>SK Uniqueness</t>
         </is>
       </c>
-      <c r="D55" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E55" s="10" t="inlineStr">
+      <c r="D57" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E57" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_account_type_codes</t>
         </is>
       </c>
-      <c r="F55" s="11" t="inlineStr">
+      <c r="F57" s="11" t="inlineStr">
         <is>
           <t>Verify Primary Surrogate Key (dim_account_type_codes_sk) uniqueness and non-null constraint</t>
         </is>
       </c>
-      <c r="G55" s="11" t="inlineStr">
+      <c r="G57" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_account_type_codes populated</t>
         </is>
       </c>
-      <c r="H55" s="11" t="inlineStr">
+      <c r="H57" s="11" t="inlineStr">
         <is>
           <t>dim_account_type_codes_sk is strictly unique across all versions with zero NULLs.</t>
         </is>
       </c>
-      <c r="I55" s="17" t="inlineStr">
+      <c r="I57" s="17" t="inlineStr">
         <is>
           <t>SELECT dim_account_type_codes_sk, COUNT(*) AS DuplicateCount
 FROM Gold_Warehouse.innotrust.dim_account_type_codes
@@ -3799,48 +3950,48 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="54" customHeight="1">
-      <c r="A56" s="8" t="inlineStr">
+    <row r="58" ht="54" customHeight="1">
+      <c r="A58" s="8" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B56" s="8" t="inlineStr">
+      <c r="B58" s="8" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_07</t>
         </is>
       </c>
-      <c r="C56" s="9" t="inlineStr">
+      <c r="C58" s="9" t="inlineStr">
         <is>
           <t>SCD2 Deduplication</t>
         </is>
       </c>
-      <c r="D56" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E56" s="6" t="inlineStr">
+      <c r="D58" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="inlineStr">
         <is>
           <t>innotrust.dim_master_sec_index</t>
         </is>
       </c>
-      <c r="F56" s="7" t="inlineStr">
+      <c r="F58" s="7" t="inlineStr">
         <is>
           <t>Verify Active Deduplication on Security Primary Key ['isin'] (is_current = 1)</t>
         </is>
       </c>
-      <c r="G56" s="7" t="inlineStr">
+      <c r="G58" s="7" t="inlineStr">
         <is>
           <t>innotrust.dim_master_sec_index populated</t>
         </is>
       </c>
-      <c r="H56" s="7" t="inlineStr">
+      <c r="H58" s="7" t="inlineStr">
         <is>
           <t>Zero duplicate active securities. Exactly one is_current = 1 record per isin.</t>
         </is>
       </c>
-      <c r="I56" s="18" t="inlineStr">
+      <c r="I58" s="18" t="inlineStr">
         <is>
           <t>SELECT isin, COUNT(*) AS ActiveDuplicateCount
 FROM Gold_Warehouse.innotrust.dim_master_sec_index
@@ -3850,48 +4001,48 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="54" customHeight="1">
-      <c r="A57" s="12" t="inlineStr">
+    <row r="59" ht="54" customHeight="1">
+      <c r="A59" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B57" s="12" t="inlineStr">
+      <c r="B59" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_08</t>
         </is>
       </c>
-      <c r="C57" s="13" t="inlineStr">
+      <c r="C59" s="13" t="inlineStr">
         <is>
           <t>SK Uniqueness</t>
         </is>
       </c>
-      <c r="D57" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E57" s="10" t="inlineStr">
+      <c r="D59" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E59" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_master_sec_index</t>
         </is>
       </c>
-      <c r="F57" s="11" t="inlineStr">
+      <c r="F59" s="11" t="inlineStr">
         <is>
           <t>Verify Primary Surrogate Key (dim_master_sec_index_sk) uniqueness across all records</t>
         </is>
       </c>
-      <c r="G57" s="11" t="inlineStr">
+      <c r="G59" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_master_sec_index populated</t>
         </is>
       </c>
-      <c r="H57" s="11" t="inlineStr">
+      <c r="H59" s="11" t="inlineStr">
         <is>
           <t>dim_master_sec_index_sk is strictly unique across all versions with zero NULLs.</t>
         </is>
       </c>
-      <c r="I57" s="17" t="inlineStr">
+      <c r="I59" s="17" t="inlineStr">
         <is>
           <t>SELECT dim_master_sec_index_sk, COUNT(*) AS DuplicateCount
 FROM Gold_Warehouse.innotrust.dim_master_sec_index
@@ -3900,48 +4051,48 @@
         </is>
       </c>
     </row>
-    <row r="58" ht="54" customHeight="1">
-      <c r="A58" s="8" t="inlineStr">
+    <row r="60" ht="54" customHeight="1">
+      <c r="A60" s="8" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B58" s="8" t="inlineStr">
+      <c r="B60" s="8" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_09</t>
         </is>
       </c>
-      <c r="C58" s="9" t="inlineStr">
+      <c r="C60" s="9" t="inlineStr">
         <is>
           <t>SCD2 Deduplication</t>
         </is>
       </c>
-      <c r="D58" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E58" s="6" t="inlineStr">
+      <c r="D60" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E60" s="6" t="inlineStr">
         <is>
           <t>innotrust.dim_security_characteristics_codes</t>
         </is>
       </c>
-      <c r="F58" s="7" t="inlineStr">
+      <c r="F60" s="7" t="inlineStr">
         <is>
           <t>Verify Active Deduplication on Business Key ['security_type_code'] (is_current = 1)</t>
         </is>
       </c>
-      <c r="G58" s="7" t="inlineStr">
+      <c r="G60" s="7" t="inlineStr">
         <is>
           <t>innotrust.dim_security_characteristics_codes populated</t>
         </is>
       </c>
-      <c r="H58" s="7" t="inlineStr">
+      <c r="H60" s="7" t="inlineStr">
         <is>
           <t>Zero duplicate active security type codes per security_type_code.</t>
         </is>
       </c>
-      <c r="I58" s="18" t="inlineStr">
+      <c r="I60" s="18" t="inlineStr">
         <is>
           <t>SELECT security_type_code, COUNT(*) AS ActiveDuplicateCount
 FROM Gold_Warehouse.innotrust.dim_security_characteristics_codes
@@ -3951,48 +4102,48 @@
         </is>
       </c>
     </row>
-    <row r="59" ht="54" customHeight="1">
-      <c r="A59" s="12" t="inlineStr">
+    <row r="61" ht="54" customHeight="1">
+      <c r="A61" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B59" s="12" t="inlineStr">
+      <c r="B61" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_10</t>
         </is>
       </c>
-      <c r="C59" s="13" t="inlineStr">
+      <c r="C61" s="13" t="inlineStr">
         <is>
           <t>SK Uniqueness</t>
         </is>
       </c>
-      <c r="D59" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E59" s="10" t="inlineStr">
+      <c r="D61" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E61" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_security_characteristics_codes</t>
         </is>
       </c>
-      <c r="F59" s="11" t="inlineStr">
+      <c r="F61" s="11" t="inlineStr">
         <is>
           <t>Verify Primary Surrogate Key (dim_securitycharacteristicscodes) uniqueness and non-null constraint</t>
         </is>
       </c>
-      <c r="G59" s="11" t="inlineStr">
+      <c r="G61" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_security_characteristics_codes populated</t>
         </is>
       </c>
-      <c r="H59" s="11" t="inlineStr">
+      <c r="H61" s="11" t="inlineStr">
         <is>
           <t>dim_securitycharacteristicscodes is strictly unique across all versions with zero NULLs.</t>
         </is>
       </c>
-      <c r="I59" s="17" t="inlineStr">
+      <c r="I61" s="17" t="inlineStr">
         <is>
           <t>SELECT dim_securitycharacteristicscodes, COUNT(*) AS DuplicateCount
 FROM Gold_Warehouse.innotrust.dim_security_characteristics_codes
@@ -4001,48 +4152,48 @@
         </is>
       </c>
     </row>
-    <row r="60" ht="54" customHeight="1">
-      <c r="A60" s="8" t="inlineStr">
+    <row r="62" ht="54" customHeight="1">
+      <c r="A62" s="8" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B60" s="8" t="inlineStr">
+      <c r="B62" s="8" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_11</t>
         </is>
       </c>
-      <c r="C60" s="9" t="inlineStr">
+      <c r="C62" s="9" t="inlineStr">
         <is>
           <t>Audit &amp; Date Logic</t>
         </is>
       </c>
-      <c r="D60" s="19" t="inlineStr">
+      <c r="D62" s="19" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E60" s="6" t="inlineStr">
+      <c r="E62" s="6" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master</t>
         </is>
       </c>
-      <c r="F60" s="7" t="inlineStr">
+      <c r="F62" s="7" t="inlineStr">
         <is>
           <t>Verify business_date, updated_at, effective_start_date &amp; effective_end_date integrity on active records</t>
         </is>
       </c>
-      <c r="G60" s="7" t="inlineStr">
+      <c r="G62" s="7" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master populated</t>
         </is>
       </c>
-      <c r="H60" s="7" t="inlineStr">
+      <c r="H62" s="7" t="inlineStr">
         <is>
           <t>Zero NULLs in business_date or updated_at; effective_end_date &gt;= effective_start_date.</t>
         </is>
       </c>
-      <c r="I60" s="18" t="inlineStr">
+      <c r="I62" s="18" t="inlineStr">
         <is>
           <t>SELECT 
     COUNT(*) AS TotalActiveRows,
@@ -4055,48 +4206,48 @@
         </is>
       </c>
     </row>
-    <row r="61" ht="54" customHeight="1">
-      <c r="A61" s="12" t="inlineStr">
+    <row r="63" ht="54" customHeight="1">
+      <c r="A63" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B61" s="12" t="inlineStr">
+      <c r="B63" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_12</t>
         </is>
       </c>
-      <c r="C61" s="13" t="inlineStr">
+      <c r="C63" s="13" t="inlineStr">
         <is>
           <t>Cross-Table Linkage</t>
         </is>
       </c>
-      <c r="D61" s="19" t="inlineStr">
+      <c r="D63" s="19" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E61" s="10" t="inlineStr">
+      <c r="E63" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master</t>
         </is>
       </c>
-      <c r="F61" s="11" t="inlineStr">
+      <c r="F63" s="11" t="inlineStr">
         <is>
           <t>Verify Referential Integrity: account_category_code and account_type_code resolve to active codes</t>
         </is>
       </c>
-      <c r="G61" s="11" t="inlineStr">
+      <c r="G63" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master populated</t>
         </is>
       </c>
-      <c r="H61" s="11" t="inlineStr">
+      <c r="H63" s="11" t="inlineStr">
         <is>
           <t>All non-null account_category_code and account_type_code exist in corresponding dimension code tables.</t>
         </is>
       </c>
-      <c r="I61" s="17" t="inlineStr">
+      <c r="I63" s="17" t="inlineStr">
         <is>
           <t>SELECT 
     SUM(CASE WHEN m.account_category_code IS NOT NULL AND cat.account_category_code IS NULL THEN 1 ELSE 0 END) AS Orphan_CategoryCodes,
@@ -4110,48 +4261,48 @@
         </is>
       </c>
     </row>
-    <row r="62" ht="54" customHeight="1">
-      <c r="A62" s="8" t="inlineStr">
+    <row r="64" ht="54" customHeight="1">
+      <c r="A64" s="8" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B62" s="8" t="inlineStr">
+      <c r="B64" s="8" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_13</t>
         </is>
       </c>
-      <c r="C62" s="9" t="inlineStr">
+      <c r="C64" s="9" t="inlineStr">
         <is>
           <t>Cross-Table Linkage</t>
         </is>
       </c>
-      <c r="D62" s="19" t="inlineStr">
+      <c r="D64" s="19" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E62" s="6" t="inlineStr">
+      <c r="E64" s="6" t="inlineStr">
         <is>
           <t>innotrust.dim_master_sec_index</t>
         </is>
       </c>
-      <c r="F62" s="7" t="inlineStr">
+      <c r="F64" s="7" t="inlineStr">
         <is>
           <t>Verify Security Referential Integrity: security_type_code resolves to active security characteristics</t>
         </is>
       </c>
-      <c r="G62" s="7" t="inlineStr">
+      <c r="G64" s="7" t="inlineStr">
         <is>
           <t>innotrust.dim_master_sec_index populated</t>
         </is>
       </c>
-      <c r="H62" s="7" t="inlineStr">
+      <c r="H64" s="7" t="inlineStr">
         <is>
           <t>All non-null security_type_code values exist in dim_security_characteristics_codes.</t>
         </is>
       </c>
-      <c r="I62" s="18" t="inlineStr">
+      <c r="I64" s="18" t="inlineStr">
         <is>
           <t>SELECT COUNT(*) AS Orphan_SecurityTypeCodes
 FROM Gold_Warehouse.innotrust.dim_master_sec_index s
@@ -4161,48 +4312,48 @@
         </is>
       </c>
     </row>
-    <row r="63" ht="54" customHeight="1">
-      <c r="A63" s="12" t="inlineStr">
+    <row r="65" ht="54" customHeight="1">
+      <c r="A65" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B63" s="12" t="inlineStr">
+      <c r="B65" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_14</t>
         </is>
       </c>
-      <c r="C63" s="13" t="inlineStr">
+      <c r="C65" s="13" t="inlineStr">
         <is>
           <t>SCD2 Date Validation</t>
         </is>
       </c>
-      <c r="D63" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E63" s="10" t="inlineStr">
+      <c r="D65" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E65" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master</t>
         </is>
       </c>
-      <c r="F63" s="11" t="inlineStr">
+      <c r="F65" s="11" t="inlineStr">
         <is>
           <t>Verify SCD2 Effective Date Rules: Inactive records effective_end_date &lt;= (Current Day - 1), non-null end date, and valid active start date</t>
         </is>
       </c>
-      <c r="G63" s="11" t="inlineStr">
+      <c r="G65" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master populated with SCD2 tracking columns</t>
         </is>
       </c>
-      <c r="H63" s="11" t="inlineStr">
+      <c r="H65" s="11" t="inlineStr">
         <is>
           <t>Inactive_End_Date_Breach_Count = 0, Inactive_Missing_End_Date = 0, Active_Future_Start_Date = 0, Inverted_Date_Range_Count = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I63" s="17" t="inlineStr">
+      <c r="I65" s="17" t="inlineStr">
         <is>
           <t>SELECT 
     'dim_account_master' AS TableName,
@@ -4221,48 +4372,48 @@
         </is>
       </c>
     </row>
-    <row r="64" ht="54" customHeight="1">
-      <c r="A64" s="8" t="inlineStr">
+    <row r="66" ht="54" customHeight="1">
+      <c r="A66" s="8" t="inlineStr">
         <is>
           <t>Black Diamond (Consolidated)</t>
         </is>
       </c>
-      <c r="B64" s="8" t="inlineStr">
+      <c r="B66" s="8" t="inlineStr">
         <is>
           <t>TC_COMB_SK_BD_01</t>
         </is>
       </c>
-      <c r="C64" s="9" t="inlineStr">
+      <c r="C66" s="9" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D64" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E64" s="6" t="inlineStr">
+      <c r="D66" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E66" s="6" t="inlineStr">
         <is>
           <t>All 9 Child &amp; Fact Tables (holdings, transactions, taxlots, class/segment, details, tags, team, targets)</t>
         </is>
       </c>
-      <c r="F64" s="7" t="inlineStr">
+      <c r="F66" s="7" t="inlineStr">
         <is>
           <t>Black Diamond: Cross-Object account_sk vs dim_accounts Natural Key (accountid == da.id) Verification - Executes a single consolidated UNION ALL query across all 9 child/fact tables to verify that the attached account_sk strictly points to the exact same account natural key (child.accountid == da.id). Guarantees zero wrong account links.</t>
         </is>
       </c>
-      <c r="G64" s="7" t="inlineStr">
+      <c r="G66" s="7" t="inlineStr">
         <is>
           <t>All Gold tables populated for Black Diamond</t>
         </is>
       </c>
-      <c r="H64" s="7" t="inlineStr">
+      <c r="H66" s="7" t="inlineStr">
         <is>
           <t>Duplicate_BusinessKey_Count = 0, MismatchedAccountIdCount = 0, Null_AccountSK_Count = 0, Orphan_AccountSK_Count = 0 across all 9 objects.</t>
         </is>
       </c>
-      <c r="I64" s="18" t="inlineStr">
+      <c r="I66" s="18" t="inlineStr">
         <is>
           <t>SELECT 
     'dim_accounts_classallocation' AS TableName, 
@@ -4371,48 +4522,48 @@
         </is>
       </c>
     </row>
-    <row r="65" ht="54" customHeight="1">
-      <c r="A65" s="12" t="inlineStr">
+    <row r="67" ht="54" customHeight="1">
+      <c r="A67" s="12" t="inlineStr">
         <is>
           <t>Schwab (Consolidated)</t>
         </is>
       </c>
-      <c r="B65" s="12" t="inlineStr">
+      <c r="B67" s="12" t="inlineStr">
         <is>
           <t>TC_COMB_SK_SC_02</t>
         </is>
       </c>
-      <c r="C65" s="13" t="inlineStr">
+      <c r="C67" s="13" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D65" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E65" s="10" t="inlineStr">
+      <c r="D67" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E67" s="10" t="inlineStr">
         <is>
           <t>All 8 Objects (dim_accounts &amp; 7 Fact Tables: recon_d1/d2, daily_closing, security, transactions, ult/uln lots)</t>
         </is>
       </c>
-      <c r="F65" s="11" t="inlineStr">
+      <c r="F67" s="11" t="inlineStr">
         <is>
           <t>Schwab: Consolidated Multi-Object SK Mapping, PK Deduplication &amp; Audit Date Health Check - Single unified query executing across all 8 Schwab Gold tables. Validates that every fact record's account_sk correctly matches dim_accounts on composite natural keys (account_id, custodian_id), confirms primary SK uniqueness, and ensures 100% audit dates populated.</t>
         </is>
       </c>
-      <c r="G65" s="11" t="inlineStr">
+      <c r="G67" s="11" t="inlineStr">
         <is>
           <t>All Gold tables populated for Schwab</t>
         </is>
       </c>
-      <c r="H65" s="11" t="inlineStr">
+      <c r="H67" s="11" t="inlineStr">
         <is>
           <t>Mismatched_AccountId_Count = 0 and Orphan_AccountSK_Count = 0 across all fact tables. All mapped account_sk strictly match the natural account_id.</t>
         </is>
       </c>
-      <c r="I65" s="17" t="inlineStr">
+      <c r="I67" s="17" t="inlineStr">
         <is>
           <t>SELECT 
     'fact_recon_position_d1' AS TableName,
@@ -4471,48 +4622,48 @@
         </is>
       </c>
     </row>
-    <row r="66" ht="54" customHeight="1">
-      <c r="A66" s="8" t="inlineStr">
+    <row r="68" ht="54" customHeight="1">
+      <c r="A68" s="8" t="inlineStr">
         <is>
           <t>Salentica CRM (Consolidated)</t>
         </is>
       </c>
-      <c r="B66" s="8" t="inlineStr">
+      <c r="B68" s="8" t="inlineStr">
         <is>
           <t>TC_COMB_SK_SAL_03</t>
         </is>
       </c>
-      <c r="C66" s="9" t="inlineStr">
+      <c r="C68" s="9" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D66" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E66" s="6" t="inlineStr">
+      <c r="D68" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E68" s="6" t="inlineStr">
         <is>
           <t>All 6 Core CRM Entities (dim_account, dim_contact_core, dim_family, fact_lead, fact_opportunity, fact_investmentaccount)</t>
         </is>
       </c>
-      <c r="F66" s="7" t="inlineStr">
+      <c r="F68" s="7" t="inlineStr">
         <is>
           <t>Salentica: Consolidated Point-in-Time Referential SK Mapping (Active &amp; Historical Mapping Validation) - Single unified query executing across all 6 core Salentica CRM tables. Validates that every attached foreign SK resolves to the same Natural Key in parent dimensions (allowing active OR expired parent versions to preserve point-in-time audit history) and checks for broken orphans.</t>
         </is>
       </c>
-      <c r="G66" s="7" t="inlineStr">
+      <c r="G68" s="7" t="inlineStr">
         <is>
           <t>All Gold tables populated for Salentica CRM</t>
         </is>
       </c>
-      <c r="H66" s="7" t="inlineStr">
+      <c r="H68" s="7" t="inlineStr">
         <is>
           <t>Mismatched_PrimaryContact_NK = 0, Mismatched_BusinessUnit_NK = 0, Broken_Orphan_Count = 0 across all 6 CRM tables.</t>
         </is>
       </c>
-      <c r="I66" s="18" t="inlineStr">
+      <c r="I68" s="18" t="inlineStr">
         <is>
           <t>SELECT 'dim_account' AS TableName, COUNT(*) AS TotalActiveRows,
     SUM(CASE WHEN a.primarycontactid IS NOT NULL AND a.primarycontactid_sk &lt;&gt; -1 AND a.primarycontactid &lt;&gt; c.contactid THEN 1 ELSE 0 END) AS Mismatched_PrimaryContact_NK,
@@ -4576,48 +4727,48 @@
         </is>
       </c>
     </row>
-    <row r="67" ht="54" customHeight="1">
-      <c r="A67" s="12" t="inlineStr">
+    <row r="69" ht="54" customHeight="1">
+      <c r="A69" s="12" t="inlineStr">
         <is>
           <t>Tamarac (Consolidated)</t>
         </is>
       </c>
-      <c r="B67" s="12" t="inlineStr">
+      <c r="B69" s="12" t="inlineStr">
         <is>
           <t>TC_COMB_SK_TAM_04</t>
         </is>
       </c>
-      <c r="C67" s="13" t="inlineStr">
+      <c r="C69" s="13" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D67" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E67" s="10" t="inlineStr">
+      <c r="D69" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E69" s="10" t="inlineStr">
         <is>
           <t>Both Tables (dim_account_information, dim_account_model_allocation)</t>
         </is>
       </c>
-      <c r="F67" s="11" t="inlineStr">
+      <c r="F69" s="11" t="inlineStr">
         <is>
           <t>Tamarac: Consolidated Multi-Object PK Deduplication, Primary SK &amp; Cross-Table Linkage - Single unified query validating SCD2 active uniqueness on exact PK columns (['account_number'] and ['account_number', 'model_name']), surrogate key uniqueness, and cross-table referential integrity between model allocations and accounts.</t>
         </is>
       </c>
-      <c r="G67" s="11" t="inlineStr">
+      <c r="G69" s="11" t="inlineStr">
         <is>
           <t>All Gold tables populated for Tamarac</t>
         </is>
       </c>
-      <c r="H67" s="11" t="inlineStr">
+      <c r="H69" s="11" t="inlineStr">
         <is>
           <t>PK_Active_Duplicates = 0, Duplicate_Primary_SK = 0, Orphan_Accounts = 0, Missing_BusinessDate = 0 across both tables.</t>
         </is>
       </c>
-      <c r="I67" s="17" t="inlineStr">
+      <c r="I69" s="17" t="inlineStr">
         <is>
           <t>SELECT 'dim_account_information' AS TableName, COUNT(*) AS TotalActiveRows,
     (SELECT COUNT(*) FROM (SELECT account_number FROM Gold_Warehouse.tamarac.dim_account_information WHERE is_current = 'True' GROUP BY account_number HAVING COUNT(*) &gt; 1) d) AS PK_Active_Duplicates,
@@ -4640,48 +4791,48 @@
         </is>
       </c>
     </row>
-    <row r="68" ht="54" customHeight="1">
-      <c r="A68" s="8" t="inlineStr">
+    <row r="70" ht="54" customHeight="1">
+      <c r="A70" s="8" t="inlineStr">
         <is>
           <t>Innotrust (Consolidated)</t>
         </is>
       </c>
-      <c r="B68" s="8" t="inlineStr">
+      <c r="B70" s="8" t="inlineStr">
         <is>
           <t>TC_COMB_SK_INNO_05</t>
         </is>
       </c>
-      <c r="C68" s="9" t="inlineStr">
+      <c r="C70" s="9" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D68" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E68" s="6" t="inlineStr">
+      <c r="D70" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E70" s="6" t="inlineStr">
         <is>
           <t>All 5 Innotrust Dimensions (dim_account_master, category_codes, type_codes, sec_index, characteristics)</t>
         </is>
       </c>
-      <c r="F68" s="7" t="inlineStr">
+      <c r="F70" s="7" t="inlineStr">
         <is>
           <t>Innotrust: Consolidated Multi-Object PK Deduplication, Primary SK &amp; Cross-Dimension Linkage - Single unified query validating SCD2 active uniqueness on exact natural keys, primary surrogate key uniqueness, and cross-dimension referential integrity between master entities and classification codes.</t>
         </is>
       </c>
-      <c r="G68" s="7" t="inlineStr">
+      <c r="G70" s="7" t="inlineStr">
         <is>
           <t>All Gold tables populated for Innotrust</t>
         </is>
       </c>
-      <c r="H68" s="7" t="inlineStr">
+      <c r="H70" s="7" t="inlineStr">
         <is>
           <t>PK_Active_Duplicates = 0, Duplicate_Primary_SK = 0, Orphan_Foreign_References = 0, Missing_BusinessDate = 0 across all 5 Innotrust tables.</t>
         </is>
       </c>
-      <c r="I68" s="18" t="inlineStr">
+      <c r="I70" s="18" t="inlineStr">
         <is>
           <t>SELECT 'dim_account_master' AS TableName, COUNT(*) AS TotalActiveRows,
     (SELECT COUNT(*) FROM (SELECT customer_account_number FROM Gold_Warehouse.innotrust.dim_account_master WHERE is_current = 1 GROUP BY customer_account_number HAVING COUNT(*) &gt; 1) d) AS PK_Active_Duplicates,
@@ -4731,48 +4882,48 @@
         </is>
       </c>
     </row>
-    <row r="69" ht="54" customHeight="1">
-      <c r="A69" s="12" t="inlineStr">
+    <row r="71" ht="54" customHeight="1">
+      <c r="A71" s="12" t="inlineStr">
         <is>
           <t>Innotrust (Consolidated)</t>
         </is>
       </c>
-      <c r="B69" s="12" t="inlineStr">
+      <c r="B71" s="12" t="inlineStr">
         <is>
           <t>TC_COMB_SK_INNO_06</t>
         </is>
       </c>
-      <c r="C69" s="13" t="inlineStr">
+      <c r="C71" s="13" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D69" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E69" s="10" t="inlineStr">
+      <c r="D71" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E71" s="10" t="inlineStr">
         <is>
           <t>All 5 Innotrust Dimensions (dim_account_master, category_codes, type_codes, sec_index, characteristics)</t>
         </is>
       </c>
-      <c r="F69" s="11" t="inlineStr">
+      <c r="F71" s="11" t="inlineStr">
         <is>
           <t>Innotrust: Consolidated Multi-Object SCD2 Effective Start &amp; End Date Audit (End Date &lt;= Today - 1) - Validates across all 5 Innotrust dimensions that inactive records (is_current = 0) have effective_end_date &lt;= (current day - 1), non-null end dates, active records have non-future start dates, and zero inverted date ranges.</t>
         </is>
       </c>
-      <c r="G69" s="11" t="inlineStr">
+      <c r="G71" s="11" t="inlineStr">
         <is>
           <t>All Gold tables populated for Innotrust</t>
         </is>
       </c>
-      <c r="H69" s="11" t="inlineStr">
+      <c r="H71" s="11" t="inlineStr">
         <is>
           <t>Inactive_End_Date_Breach_Count = 0, Inactive_Missing_End_Date = 0, Active_Future_Start_Date = 0, Inverted_Date_Range_Count = 0 across all 5 tables.</t>
         </is>
       </c>
-      <c r="I69" s="17" t="inlineStr">
+      <c r="I71" s="17" t="inlineStr">
         <is>
           <t>SELECT 
     'dim_account_master' AS TableName,
@@ -6656,7 +6807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7442,6 +7593,147 @@
     END AS TestStatus
 FROM Gold_Warehouse.tamarac.dim_account_model_allocation
 WHERE is_current = 'True';</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="54" customHeight="1">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>TC_TAM_GOLD_15</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>Version Evolution Audit</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>tamarac.dim_account_information</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="inlineStr">
+        <is>
+          <t>Verify Run Evolution: Every new run produces New Incremented SK, Advancing Start Date, and Latest Version is Active</t>
+        </is>
+      </c>
+      <c r="F17" s="11" t="inlineStr">
+        <is>
+          <t>dim_account_information with historical batch progression</t>
+        </is>
+      </c>
+      <c r="G17" s="11" t="inlineStr">
+        <is>
+          <t>Reused_Or_NonIncrementing_SK_Count = 0, NonAdvancing_EffectiveStartDate_Count = 0, Timeline_Gap_Or_Overlap_Count = 0, LatestVersion_Not_Active_Count = 0. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="H17" s="17" t="inlineStr">
+        <is>
+          <t>;WITH VersionChains AS (
+    SELECT 
+        account_number,
+        account_information_SK,
+        effective_start_date,
+        effective_end_date,
+        is_current,
+        file_business_date,
+        updated_at,
+        LEAD(account_information_SK) OVER (PARTITION BY account_number ORDER BY effective_start_date, account_information_SK) AS next_sk,
+        LEAD(effective_start_date) OVER (PARTITION BY account_number ORDER BY effective_start_date, account_information_SK) AS next_start_date,
+        ROW_NUMBER() OVER (PARTITION BY account_number ORDER BY effective_start_date DESC, account_information_SK DESC) AS rn_latest
+    FROM Gold_Warehouse.tamarac.dim_account_information
+)
+SELECT 
+    'dim_account_information' AS TableName,
+    COUNT(*) AS TotalVersionsAudited,
+    SUM(CASE WHEN next_sk IS NOT NULL AND next_sk &lt;= account_information_SK THEN 1 ELSE 0 END) AS Reused_Or_NonIncrementing_SK_Count,
+    SUM(CASE WHEN next_start_date IS NOT NULL AND next_start_date &lt;= effective_start_date THEN 1 ELSE 0 END) AS NonAdvancing_EffectiveStartDate_Count,
+    SUM(CASE WHEN next_start_date IS NOT NULL AND effective_end_date &lt;&gt; DATEADD(day, -1, next_start_date) THEN 1 ELSE 0 END) AS Timeline_Gap_Or_Overlap_Count,
+    SUM(CASE WHEN rn_latest = 1 AND is_current &lt;&gt; 'True' THEN 1 ELSE 0 END) AS LatestVersion_Not_Active_Count,
+    CASE 
+        WHEN SUM(CASE WHEN next_sk IS NOT NULL AND next_sk &lt;= account_information_SK THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN next_start_date IS NOT NULL AND next_start_date &lt;= effective_start_date THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN next_start_date IS NOT NULL AND effective_end_date &lt;&gt; DATEADD(day, -1, next_start_date) THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN rn_latest = 1 AND is_current &lt;&gt; 'True' THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END AS TestStatus
+FROM VersionChains;</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="54" customHeight="1">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>TC_TAM_GOLD_16</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Version Evolution Audit</t>
+        </is>
+      </c>
+      <c r="C18" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>tamarac.dim_account_model_allocation</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>Verify Run Evolution: Every new run produces New Incremented SK, Advancing Start Date, and Latest Version is Active</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>dim_account_model_allocation with historical batch progression</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>Reused_Or_NonIncrementing_SK_Count = 0, NonAdvancing_EffectiveStartDate_Count = 0, Timeline_Gap_Or_Overlap_Count = 0, LatestVersion_Not_Active_Count = 0. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>;WITH ModelChains AS (
+    SELECT 
+        account_number,
+        model_name,
+        account_model_SK,
+        effective_start_date,
+        effective_end_date,
+        is_current,
+        file_business_date,
+        updated_at,
+        LEAD(account_model_SK) OVER (PARTITION BY account_number, model_name ORDER BY effective_start_date, account_model_SK) AS next_sk,
+        LEAD(effective_start_date) OVER (PARTITION BY account_number, model_name ORDER BY effective_start_date, account_model_SK) AS next_start_date,
+        ROW_NUMBER() OVER (PARTITION BY account_number, model_name ORDER BY effective_start_date DESC, account_model_SK DESC) AS rn_latest
+    FROM Gold_Warehouse.tamarac.dim_account_model_allocation
+)
+SELECT 
+    'dim_account_model_allocation' AS TableName,
+    COUNT(*) AS TotalVersionsAudited,
+    SUM(CASE WHEN next_sk IS NOT NULL AND next_sk &lt;= account_model_SK THEN 1 ELSE 0 END) AS Reused_Or_NonIncrementing_SK_Count,
+    SUM(CASE WHEN next_start_date IS NOT NULL AND next_start_date &lt;= effective_start_date THEN 1 ELSE 0 END) AS NonAdvancing_EffectiveStartDate_Count,
+    SUM(CASE WHEN next_start_date IS NOT NULL AND effective_end_date &lt;&gt; DATEADD(day, -1, next_start_date) THEN 1 ELSE 0 END) AS Timeline_Gap_Or_Overlap_Count,
+    SUM(CASE WHEN rn_latest = 1 AND is_current &lt;&gt; 'True' THEN 1 ELSE 0 END) AS LatestVersion_Not_Active_Count,
+    CASE 
+        WHEN SUM(CASE WHEN next_sk IS NOT NULL AND next_sk &lt;= account_model_SK THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN next_start_date IS NOT NULL AND next_start_date &lt;= effective_start_date THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN next_start_date IS NOT NULL AND effective_end_date &lt;&gt; DATEADD(day, -1, next_start_date) THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN rn_latest = 1 AND is_current &lt;&gt; 'True' THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END AS TestStatus
+FROM ModelChains;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(schwab): add SCD2 dimension sanity & client-ready fact health validation tests TC_SC_GOLD_09-13
</commit_message>
<xml_diff>
--- a/Gold_Data_Validation_Test_Cases.xlsx
+++ b/Gold_Data_Validation_Test_Cases.xlsx
@@ -644,13 +644,13 @@
         <v>5</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G5" s="4" t="n">
         <v>6</v>
@@ -736,13 +736,13 @@
         </is>
       </c>
       <c r="C9" s="12" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="D9" s="13" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
@@ -860,13 +860,13 @@
         </is>
       </c>
       <c r="C13" s="15" t="n">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="D13" s="15" t="n">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E13" s="15" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F13" s="15" t="inlineStr">
         <is>
@@ -898,7 +898,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I71"/>
+  <dimension ref="A1:I76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2326,45 +2326,459 @@
     <row r="29" ht="54" customHeight="1">
       <c r="A29" s="12" t="inlineStr">
         <is>
+          <t>Schwab</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>TC_SC_GOLD_09</t>
+        </is>
+      </c>
+      <c r="C29" s="13" t="inlineStr">
+        <is>
+          <t>SCD2 Inactive Date Rules</t>
+        </is>
+      </c>
+      <c r="D29" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E29" s="10" t="inlineStr">
+        <is>
+          <t>schwab.dim_accounts</t>
+        </is>
+      </c>
+      <c r="F29" s="11" t="inlineStr">
+        <is>
+          <t>Verify SCD2 Inactive Date Rule: Inactive records (IsCurrent = 0) must have EffectiveTo &lt;= file_business_date - 1 (or next EffectiveFrom - 1)</t>
+        </is>
+      </c>
+      <c r="G29" s="11" t="inlineStr">
+        <is>
+          <t>dim_accounts populated with SCD2 tracking columns</t>
+        </is>
+      </c>
+      <c r="H29" s="11" t="inlineStr">
+        <is>
+          <t>Zero active records marked expired prematurely, zero inactive records with open/invalid EffectiveTo. DefectCount = 0.</t>
+        </is>
+      </c>
+      <c r="I29" s="17" t="inlineStr">
+        <is>
+          <t>SELECT 
+    account_id,
+    account_sk,
+    file_business_date,
+    EffectiveFrom,
+    EffectiveTo,
+    IsCurrent,
+    Audit_Update_Date
+FROM Gold_Warehouse.schwab.dim_accounts
+WHERE IsCurrent = 0 
+  AND (EffectiveTo IS NULL OR EffectiveTo &gt; file_business_date)
+ORDER BY account_id, EffectiveFrom;</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="54" customHeight="1">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>Schwab</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>TC_SC_GOLD_10</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>Date Sanity &amp; Inversions</t>
+        </is>
+      </c>
+      <c r="D30" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>schwab.dim_accounts</t>
+        </is>
+      </c>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>Verify Date Sanity: Zero inverted dates (EffectiveTo &lt; EffectiveFrom) and active records have non-future start dates</t>
+        </is>
+      </c>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>dim_accounts populated</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>Inverted_Date_Count = 0, Future_Active_Start_Date = 0, Null_Start_Date_Count = 0. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="I30" s="18" t="inlineStr">
+        <is>
+          <t>SELECT 
+    'schwab.dim_accounts' AS TableName,
+    COUNT(*) AS TotalRecords,
+    SUM(CASE WHEN EffectiveTo &lt; EffectiveFrom THEN 1 ELSE 0 END) AS Inverted_Date_Count,
+    SUM(CASE WHEN IsCurrent = 1 AND EffectiveFrom &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END) AS Future_Active_Start_Date,
+    SUM(CASE WHEN EffectiveFrom IS NULL THEN 1 ELSE 0 END) AS Null_Start_Date_Count,
+    CASE 
+        WHEN SUM(CASE WHEN EffectiveTo &lt; EffectiveFrom THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN IsCurrent = 1 AND EffectiveFrom &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN EffectiveFrom IS NULL THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END AS TestStatus
+FROM Gold_Warehouse.schwab.dim_accounts;</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="54" customHeight="1">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>Schwab</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>TC_SC_GOLD_11</t>
+        </is>
+      </c>
+      <c r="C31" s="13" t="inlineStr">
+        <is>
+          <t>Open-Ended Active Records</t>
+        </is>
+      </c>
+      <c r="D31" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E31" s="10" t="inlineStr">
+        <is>
+          <t>schwab.dim_accounts</t>
+        </is>
+      </c>
+      <c r="F31" s="11" t="inlineStr">
+        <is>
+          <t>Verify Active Records are Open-Ended (EffectiveTo is NULL or '9999-12-31')</t>
+        </is>
+      </c>
+      <c r="G31" s="11" t="inlineStr">
+        <is>
+          <t>dim_accounts where IsCurrent = 1</t>
+        </is>
+      </c>
+      <c r="H31" s="11" t="inlineStr">
+        <is>
+          <t>Prematurely_Ended_Active_Records = 0. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="I31" s="17" t="inlineStr">
+        <is>
+          <t>SELECT 
+    'schwab.dim_accounts' AS TableName,
+    COUNT(*) AS TotalActiveRecords,
+    SUM(CASE WHEN EffectiveTo IS NOT NULL AND EffectiveTo NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END) AS Prematurely_Ended_Active_Records,
+    CASE 
+        WHEN SUM(CASE WHEN EffectiveTo IS NOT NULL AND EffectiveTo NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END) = 0 
+        THEN 'PASSED' ELSE 'FAILED'
+    END AS TestStatus
+FROM Gold_Warehouse.schwab.dim_accounts
+WHERE IsCurrent = 1;</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="54" customHeight="1">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>Schwab</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>TC_SC_GOLD_12</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>Version Evolution Audit</t>
+        </is>
+      </c>
+      <c r="D32" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>schwab.dim_accounts</t>
+        </is>
+      </c>
+      <c r="F32" s="7" t="inlineStr">
+        <is>
+          <t>Verify SCD2 Version Evolution: Monotonic SK increments, advancing EffectiveFrom, continuous timeline (EffectiveTo = next EffectiveFrom - 1), and latest version active</t>
+        </is>
+      </c>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>dim_accounts with multiple version rows per account_id</t>
+        </is>
+      </c>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
+          <t>Reused_Or_NonIncrementing_SK_Count = 0, NonAdvancing_EffectiveFrom_Count = 0, Timeline_Gap_Or_Overlap_Count = 0, LatestVersion_Not_Active_Count = 0. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="I32" s="18" t="inlineStr">
+        <is>
+          <t>WITH SchwabEvolution AS (
+    SELECT 
+        account_id,
+        account_sk,
+        EffectiveFrom,
+        EffectiveTo,
+        IsCurrent,
+        file_business_date,
+        Audit_Update_Date,
+        LEAD(account_sk) OVER (PARTITION BY account_id ORDER BY EffectiveFrom, account_sk) AS next_sk,
+        LEAD(EffectiveFrom) OVER (PARTITION BY account_id ORDER BY EffectiveFrom, account_sk) AS next_start_date,
+        ROW_NUMBER() OVER (PARTITION BY account_id ORDER BY EffectiveFrom DESC, account_sk DESC) AS rn_latest
+    FROM Gold_Warehouse.schwab.dim_accounts
+)
+SELECT 
+    'schwab.dim_accounts' AS TableName,
+    'Version Evolution &amp; Progression' AS TestName,
+    COUNT(*) AS TotalVersionsAudited,
+    SUM(CASE WHEN next_sk IS NOT NULL AND next_sk &lt;= account_sk THEN 1 ELSE 0 END) AS Reused_Or_NonIncrementing_SK_Count,
+    SUM(CASE WHEN next_start_date IS NOT NULL AND next_start_date &lt;= EffectiveFrom THEN 1 ELSE 0 END) AS NonAdvancing_EffectiveFrom_Count,
+    SUM(CASE WHEN next_start_date IS NOT NULL AND EffectiveTo &lt;&gt; DATEADD(day, -1, next_start_date) THEN 1 ELSE 0 END) AS Timeline_Gap_Or_Overlap_Count,
+    SUM(CASE WHEN rn_latest = 1 AND IsCurrent &lt;&gt; 1 THEN 1 ELSE 0 END) AS LatestVersion_Not_Active_Count,
+    CASE 
+        WHEN SUM(CASE WHEN next_sk IS NOT NULL AND next_sk &lt;= account_sk THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN next_start_date IS NOT NULL AND next_start_date &lt;= EffectiveFrom THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN next_start_date IS NOT NULL AND EffectiveTo &lt;&gt; DATEADD(day, -1, next_start_date) THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN rn_latest = 1 AND IsCurrent &lt;&gt; 1 THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END AS TestStatus
+FROM SchwabEvolution;</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="54" customHeight="1">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t>Schwab</t>
+        </is>
+      </c>
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>TC_SC_GOLD_13</t>
+        </is>
+      </c>
+      <c r="C33" s="13" t="inlineStr">
+        <is>
+          <t>Fact Health &amp; Historical Retention</t>
+        </is>
+      </c>
+      <c r="D33" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E33" s="10" t="inlineStr">
+        <is>
+          <t>schwab.fact_recon_position_d1, fact_recon_position_d2, fact_daily_closing_lots, fact_transactions, fact_ult_lot_daily_taxable, fact_uln_lot_daily_non_taxable</t>
+        </is>
+      </c>
+      <c r="F33" s="11" t="inlineStr">
+        <is>
+          <t>Verify Fact Tables Health: Active SK mapping for fresh runs, historical closed version preservation for unrepeated rows, exact natural account match, and orphan SK detection</t>
+        </is>
+      </c>
+      <c r="G33" s="11" t="inlineStr">
+        <is>
+          <t>All 6 Schwab Fact tables loaded into Gold Warehouse</t>
+        </is>
+      </c>
+      <c r="H33" s="11" t="inlineStr">
+        <is>
+          <t>Fresh records map to active SK (IsCurrent = 1), past records retain historical SK, Exact_Account_Match_Count covers all non-orphan rows, Defect_Orphan_Unmapped_SK = 0, Defect_Wrong_Account_Mismatch = 0. OverallStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="I33" s="17" t="inlineStr">
+        <is>
+          <t>WITH MaxRuns AS (
+    SELECT 'fact_recon_position_d1' AS TableName, MAX(updated_at) AS LatestRunTimestamp FROM Gold_Warehouse.schwab.fact_recon_position_d1 UNION ALL
+    SELECT 'fact_recon_position_d2', MAX(updated_at) FROM Gold_Warehouse.schwab.fact_recon_position_d2 UNION ALL
+    SELECT 'fact_daily_closing_lots', MAX(updated_at) FROM Gold_Warehouse.schwab.fact_daily_closing_lots UNION ALL
+    SELECT 'fact_transactions', MAX(updated_at) FROM Gold_Warehouse.schwab.fact_transactions UNION ALL
+    SELECT 'fact_ult_lot_daily_taxable', MAX(updated_at) FROM Gold_Warehouse.schwab.fact_ult_lot_daily_taxable UNION ALL
+    SELECT 'fact_uln_lot_daily_non_taxable', MAX(updated_at) FROM Gold_Warehouse.schwab.fact_uln_lot_daily_non_taxable
+),
+FactBreakdown AS (
+    SELECT 
+        'fact_recon_position_d1' AS TableName,
+        COUNT(*) AS TotalFactRows,
+        MAX(f.file_business_date) AS LatestBatchDate,
+        SUM(CASE WHEN f.updated_at = m.LatestRunTimestamp AND da.IsCurrent = 1 AND f.account_id = da.account_id THEN 1 ELSE 0 END) AS Fresh_Run_Active_Mapped,
+        SUM(CASE WHEN f.updated_at &lt; m.LatestRunTimestamp AND da.IsCurrent = 1 AND f.account_id = da.account_id THEN 1 ELSE 0 END) AS Past_Run_Active_Retained,
+        SUM(CASE WHEN f.updated_at &lt; m.LatestRunTimestamp AND da.IsCurrent = 0 AND f.account_id = da.account_id THEN 1 ELSE 0 END) AS Past_Run_Expired_Version_Retained,
+        SUM(CASE WHEN da.account_sk IS NOT NULL AND f.account_id = da.account_id THEN 1 ELSE 0 END) AS Exact_Account_Match_Count,
+        SUM(CASE WHEN f.account_sk = -1 OR da.account_sk IS NULL THEN 1 ELSE 0 END) AS Defect_Orphan_Unmapped_SK,
+        SUM(CASE WHEN da.account_sk IS NOT NULL AND f.account_id &lt;&gt; da.account_id THEN 1 ELSE 0 END) AS Defect_Wrong_Account_Mismatch
+    FROM Gold_Warehouse.schwab.fact_recon_position_d1 f
+    JOIN MaxRuns m ON m.TableName = 'fact_recon_position_d1'
+    LEFT JOIN Gold_Warehouse.schwab.dim_accounts da ON f.account_sk = da.account_sk
+    GROUP BY m.LatestRunTimestamp
+    UNION ALL
+    SELECT 
+        'fact_recon_position_d2',
+        COUNT(*),
+        MAX(f.file_business_date),
+        SUM(CASE WHEN f.updated_at = m.LatestRunTimestamp AND da.IsCurrent = 1 AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.updated_at &lt; m.LatestRunTimestamp AND da.IsCurrent = 1 AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.updated_at &lt; m.LatestRunTimestamp AND da.IsCurrent = 0 AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.account_sk IS NOT NULL AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.account_sk = -1 OR da.account_sk IS NULL THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.account_sk IS NOT NULL AND f.account_id &lt;&gt; da.account_id THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.schwab.fact_recon_position_d2 f
+    JOIN MaxRuns m ON m.TableName = 'fact_recon_position_d2'
+    LEFT JOIN Gold_Warehouse.schwab.dim_accounts da ON f.account_sk = da.account_sk
+    GROUP BY m.LatestRunTimestamp
+    UNION ALL
+    SELECT 
+        'fact_daily_closing_lots',
+        COUNT(*),
+        MAX(f.file_business_date),
+        SUM(CASE WHEN f.updated_at = m.LatestRunTimestamp AND da.IsCurrent = 1 AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.updated_at &lt; m.LatestRunTimestamp AND da.IsCurrent = 1 AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.updated_at &lt; m.LatestRunTimestamp AND da.IsCurrent = 0 AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.account_sk IS NOT NULL AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.account_sk = -1 OR da.account_sk IS NULL THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.account_sk IS NOT NULL AND f.account_id &lt;&gt; da.account_id THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.schwab.fact_daily_closing_lots f
+    JOIN MaxRuns m ON m.TableName = 'fact_daily_closing_lots'
+    LEFT JOIN Gold_Warehouse.schwab.dim_accounts da ON f.account_sk = da.account_sk
+    GROUP BY m.LatestRunTimestamp
+    UNION ALL
+    SELECT 
+        'fact_transactions',
+        COUNT(*),
+        MAX(f.file_business_date),
+        SUM(CASE WHEN f.updated_at = m.LatestRunTimestamp AND da.IsCurrent = 1 AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.updated_at &lt; m.LatestRunTimestamp AND da.IsCurrent = 1 AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.updated_at &lt; m.LatestRunTimestamp AND da.IsCurrent = 0 AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.account_sk IS NOT NULL AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.account_sk = -1 OR da.account_sk IS NULL THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.account_sk IS NOT NULL AND f.account_id &lt;&gt; da.account_id THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.schwab.fact_transactions f
+    JOIN MaxRuns m ON m.TableName = 'fact_transactions'
+    LEFT JOIN Gold_Warehouse.schwab.dim_accounts da ON f.account_sk = da.account_sk
+    GROUP BY m.LatestRunTimestamp
+    UNION ALL
+    SELECT 
+        'fact_ult_lot_daily_taxable',
+        COUNT(*),
+        MAX(f.file_business_date),
+        SUM(CASE WHEN f.updated_at = m.LatestRunTimestamp AND da.IsCurrent = 1 AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.updated_at &lt; m.LatestRunTimestamp AND da.IsCurrent = 1 AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.updated_at &lt; m.LatestRunTimestamp AND da.IsCurrent = 0 AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.account_sk IS NOT NULL AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.account_sk = -1 OR da.account_sk IS NULL THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.account_sk IS NOT NULL AND f.account_id &lt;&gt; da.account_id THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.schwab.fact_ult_lot_daily_taxable f
+    JOIN MaxRuns m ON m.TableName = 'fact_ult_lot_daily_taxable'
+    LEFT JOIN Gold_Warehouse.schwab.dim_accounts da ON f.account_sk = da.account_sk
+    GROUP BY m.LatestRunTimestamp
+    UNION ALL
+    SELECT 
+        'fact_uln_lot_daily_non_taxable',
+        COUNT(*),
+        MAX(f.file_business_date),
+        SUM(CASE WHEN f.updated_at = m.LatestRunTimestamp AND da.IsCurrent = 1 AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.updated_at &lt; m.LatestRunTimestamp AND da.IsCurrent = 1 AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.updated_at &lt; m.LatestRunTimestamp AND da.IsCurrent = 0 AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.account_sk IS NOT NULL AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.account_sk = -1 OR da.account_sk IS NULL THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.account_sk IS NOT NULL AND f.account_id &lt;&gt; da.account_id THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.schwab.fact_uln_lot_daily_non_taxable f
+    JOIN MaxRuns m ON m.TableName = 'fact_uln_lot_daily_non_taxable'
+    LEFT JOIN Gold_Warehouse.schwab.dim_accounts da ON f.account_sk = da.account_sk
+    GROUP BY m.LatestRunTimestamp
+)
+SELECT 
+    TableName,
+    TotalFactRows,
+    LatestBatchDate,
+    Fresh_Run_Active_Mapped,
+    Past_Run_Active_Retained,
+    Past_Run_Expired_Version_Retained AS Historical_Closed_Version_Retained,
+    Exact_Account_Match_Count,
+    Defect_Orphan_Unmapped_SK,
+    Defect_Wrong_Account_Mismatch,
+    CASE 
+        WHEN Defect_Orphan_Unmapped_SK = 0 AND Defect_Wrong_Account_Mismatch = 0 THEN 'PASSED'
+        ELSE 'FAILED'
+    END AS OverallStatus,
+    CASE 
+        WHEN Defect_Orphan_Unmapped_SK &gt; 0 THEN CONCAT(Defect_Orphan_Unmapped_SK, ' Orphan Record(s) (SK = -1)')
+        WHEN Defect_Wrong_Account_Mismatch &gt; 0 THEN 'Account Mismatch Defect'
+        ELSE 'All Active &amp; Historical Records Correctly Preserved'
+    END AS Remarks
+FROM FactBreakdown;</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="54" customHeight="1">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
           <t>Salentica</t>
         </is>
       </c>
-      <c r="B29" s="12" t="inlineStr">
+      <c r="B34" s="8" t="inlineStr">
         <is>
           <t>TC_SAL_GOLD_01</t>
         </is>
       </c>
-      <c r="C29" s="13" t="inlineStr">
+      <c r="C34" s="9" t="inlineStr">
         <is>
           <t>SK Mapping &amp; Joins</t>
         </is>
       </c>
-      <c r="D29" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E29" s="10" t="inlineStr">
+      <c r="D34" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
         <is>
           <t>salentica.dim_account</t>
         </is>
       </c>
-      <c r="F29" s="11" t="inlineStr">
+      <c r="F34" s="7" t="inlineStr">
         <is>
           <t>Verify Foreign SK Resolution in dim_account (primarycontactid_sk, owningbusinessunit_sk)</t>
         </is>
       </c>
-      <c r="G29" s="11" t="inlineStr">
+      <c r="G34" s="7" t="inlineStr">
         <is>
           <t>dim_account populated with Point-in-Time referential keys</t>
         </is>
       </c>
-      <c r="H29" s="11" t="inlineStr">
+      <c r="H34" s="7" t="inlineStr">
         <is>
           <t>Foreign SKs resolve to matching natural keys in parent dimensions (Active or Expired). Unmapped default to -1.</t>
         </is>
       </c>
-      <c r="I29" s="17" t="inlineStr">
+      <c r="I34" s="18" t="inlineStr">
         <is>
           <t>SELECT COUNT(*) AS MismatchedNaturalKeyCount
 FROM Gold_Warehouse.salentica.dim_account a
@@ -2376,48 +2790,48 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="54" customHeight="1">
-      <c r="A30" s="8" t="inlineStr">
+    <row r="35" ht="54" customHeight="1">
+      <c r="A35" s="12" t="inlineStr">
         <is>
           <t>Salentica</t>
         </is>
       </c>
-      <c r="B30" s="8" t="inlineStr">
+      <c r="B35" s="12" t="inlineStr">
         <is>
           <t>TC_SAL_GOLD_02</t>
         </is>
       </c>
-      <c r="C30" s="9" t="inlineStr">
+      <c r="C35" s="13" t="inlineStr">
         <is>
           <t>SK Mapping &amp; Joins</t>
         </is>
       </c>
-      <c r="D30" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E30" s="6" t="inlineStr">
+      <c r="D35" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E35" s="10" t="inlineStr">
         <is>
           <t>salentica.dim_contact_core</t>
         </is>
       </c>
-      <c r="F30" s="7" t="inlineStr">
+      <c r="F35" s="11" t="inlineStr">
         <is>
           <t>Verify Foreign SK Resolution in dim_contact_core (accountid_sk, owningbusinessunit_sk)</t>
         </is>
       </c>
-      <c r="G30" s="7" t="inlineStr">
+      <c r="G35" s="11" t="inlineStr">
         <is>
           <t>dim_contact_core populated</t>
         </is>
       </c>
-      <c r="H30" s="7" t="inlineStr">
+      <c r="H35" s="11" t="inlineStr">
         <is>
           <t>Foreign SKs resolve to matching natural keys in dim_account &amp; dim_businessunit. Zero referential mismatches.</t>
         </is>
       </c>
-      <c r="I30" s="18" t="inlineStr">
+      <c r="I35" s="17" t="inlineStr">
         <is>
           <t>SELECT COUNT(*) AS MismatchedNaturalKeyCount
 FROM Gold_Warehouse.salentica.dim_contact_core c
@@ -2429,48 +2843,48 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="54" customHeight="1">
-      <c r="A31" s="12" t="inlineStr">
+    <row r="36" ht="54" customHeight="1">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t>Salentica</t>
         </is>
       </c>
-      <c r="B31" s="12" t="inlineStr">
+      <c r="B36" s="8" t="inlineStr">
         <is>
           <t>TC_SAL_GOLD_03</t>
         </is>
       </c>
-      <c r="C31" s="13" t="inlineStr">
+      <c r="C36" s="9" t="inlineStr">
         <is>
           <t>SK Mapping &amp; Joins</t>
         </is>
       </c>
-      <c r="D31" s="19" t="inlineStr">
+      <c r="D36" s="19" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E31" s="10" t="inlineStr">
+      <c r="E36" s="6" t="inlineStr">
         <is>
           <t>salentica.dim_family</t>
         </is>
       </c>
-      <c r="F31" s="11" t="inlineStr">
+      <c r="F36" s="7" t="inlineStr">
         <is>
           <t>Verify Foreign SK Resolution in dim_family (si_primarycontact_sk, owningbusinessunit_sk)</t>
         </is>
       </c>
-      <c r="G31" s="11" t="inlineStr">
+      <c r="G36" s="7" t="inlineStr">
         <is>
           <t>dim_family populated</t>
         </is>
       </c>
-      <c r="H31" s="11" t="inlineStr">
+      <c r="H36" s="7" t="inlineStr">
         <is>
           <t>Foreign SKs accurately resolve to contactid &amp; businessunitid. Zero mismatches.</t>
         </is>
       </c>
-      <c r="I31" s="17" t="inlineStr">
+      <c r="I36" s="18" t="inlineStr">
         <is>
           <t>SELECT COUNT(*) AS MismatchedFamilyLinks
 FROM Gold_Warehouse.salentica.dim_family f
@@ -2482,48 +2896,48 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="54" customHeight="1">
-      <c r="A32" s="8" t="inlineStr">
+    <row r="37" ht="54" customHeight="1">
+      <c r="A37" s="12" t="inlineStr">
         <is>
           <t>Salentica</t>
         </is>
       </c>
-      <c r="B32" s="8" t="inlineStr">
+      <c r="B37" s="12" t="inlineStr">
         <is>
           <t>TC_SAL_GOLD_04</t>
         </is>
       </c>
-      <c r="C32" s="9" t="inlineStr">
+      <c r="C37" s="13" t="inlineStr">
         <is>
           <t>SK Mapping &amp; Joins</t>
         </is>
       </c>
-      <c r="D32" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E32" s="6" t="inlineStr">
+      <c r="D37" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E37" s="10" t="inlineStr">
         <is>
           <t>salentica.fact_lead</t>
         </is>
       </c>
-      <c r="F32" s="7" t="inlineStr">
+      <c r="F37" s="11" t="inlineStr">
         <is>
           <t>Verify Foreign SK Resolution in fact_lead (accountid_sk, contactid_sk)</t>
         </is>
       </c>
-      <c r="G32" s="7" t="inlineStr">
+      <c r="G37" s="11" t="inlineStr">
         <is>
           <t>fact_lead populated</t>
         </is>
       </c>
-      <c r="H32" s="7" t="inlineStr">
+      <c r="H37" s="11" t="inlineStr">
         <is>
           <t>Foreign SKs resolve to matching accountid and contactid (Active or Expired versions). Zero mismatches.</t>
         </is>
       </c>
-      <c r="I32" s="18" t="inlineStr">
+      <c r="I37" s="17" t="inlineStr">
         <is>
           <t>SELECT COUNT(*) AS MismatchedLeadLinks
 FROM Gold_Warehouse.salentica.fact_lead l
@@ -2535,48 +2949,48 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="54" customHeight="1">
-      <c r="A33" s="12" t="inlineStr">
+    <row r="38" ht="54" customHeight="1">
+      <c r="A38" s="8" t="inlineStr">
         <is>
           <t>Salentica</t>
         </is>
       </c>
-      <c r="B33" s="12" t="inlineStr">
+      <c r="B38" s="8" t="inlineStr">
         <is>
           <t>TC_SAL_GOLD_05</t>
         </is>
       </c>
-      <c r="C33" s="13" t="inlineStr">
+      <c r="C38" s="9" t="inlineStr">
         <is>
           <t>SK Mapping &amp; Joins</t>
         </is>
       </c>
-      <c r="D33" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E33" s="10" t="inlineStr">
+      <c r="D38" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="inlineStr">
         <is>
           <t>salentica.fact_opportunity</t>
         </is>
       </c>
-      <c r="F33" s="11" t="inlineStr">
+      <c r="F38" s="7" t="inlineStr">
         <is>
           <t>Verify Point-in-Time SK Resolution in fact_opportunity (accountid_sk, contactid_sk)</t>
         </is>
       </c>
-      <c r="G33" s="11" t="inlineStr">
+      <c r="G38" s="7" t="inlineStr">
         <is>
           <t>fact_opportunity populated</t>
         </is>
       </c>
-      <c r="H33" s="11" t="inlineStr">
+      <c r="H38" s="7" t="inlineStr">
         <is>
           <t>opp.accountid_sk &amp; contactid_sk resolve to matching natural keys in Dim (Active or Expired). Zero mismatches.</t>
         </is>
       </c>
-      <c r="I33" s="17" t="inlineStr">
+      <c r="I38" s="18" t="inlineStr">
         <is>
           <t>SELECT COUNT(*) AS MismatchedOpportunityLinks
 FROM Gold_Warehouse.salentica.fact_opportunity opp
@@ -2588,48 +3002,48 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="54" customHeight="1">
-      <c r="A34" s="8" t="inlineStr">
+    <row r="39" ht="54" customHeight="1">
+      <c r="A39" s="12" t="inlineStr">
         <is>
           <t>Salentica</t>
         </is>
       </c>
-      <c r="B34" s="8" t="inlineStr">
+      <c r="B39" s="12" t="inlineStr">
         <is>
           <t>TC_SAL_GOLD_06</t>
         </is>
       </c>
-      <c r="C34" s="9" t="inlineStr">
+      <c r="C39" s="13" t="inlineStr">
         <is>
           <t>SK Mapping &amp; Joins</t>
         </is>
       </c>
-      <c r="D34" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E34" s="6" t="inlineStr">
+      <c r="D39" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E39" s="10" t="inlineStr">
         <is>
           <t>salentica.fact_investmentaccount</t>
         </is>
       </c>
-      <c r="F34" s="7" t="inlineStr">
+      <c r="F39" s="11" t="inlineStr">
         <is>
           <t>Verify Foreign SK Resolution in fact_investmentaccount (si_family_sk, si_portfolio_sk)</t>
         </is>
       </c>
-      <c r="G34" s="7" t="inlineStr">
+      <c r="G39" s="11" t="inlineStr">
         <is>
           <t>fact_investmentaccount populated</t>
         </is>
       </c>
-      <c r="H34" s="7" t="inlineStr">
+      <c r="H39" s="11" t="inlineStr">
         <is>
           <t>Attached SKs resolve to matching si_familyid &amp; si_portfolioid. Zero mismatches.</t>
         </is>
       </c>
-      <c r="I34" s="18" t="inlineStr">
+      <c r="I39" s="17" t="inlineStr">
         <is>
           <t>SELECT COUNT(*) AS MismatchedInvestmentLinks
 FROM Gold_Warehouse.salentica.fact_investmentaccount ia
@@ -2641,48 +3055,48 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="54" customHeight="1">
-      <c r="A35" s="12" t="inlineStr">
+    <row r="40" ht="54" customHeight="1">
+      <c r="A40" s="8" t="inlineStr">
         <is>
           <t>Salentica</t>
         </is>
       </c>
-      <c r="B35" s="12" t="inlineStr">
+      <c r="B40" s="8" t="inlineStr">
         <is>
           <t>TC_SAL_GOLD_07</t>
         </is>
       </c>
-      <c r="C35" s="13" t="inlineStr">
+      <c r="C40" s="9" t="inlineStr">
         <is>
           <t>Orphan &amp; -1 Fallback</t>
         </is>
       </c>
-      <c r="D35" s="19" t="inlineStr">
+      <c r="D40" s="19" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E35" s="10" t="inlineStr">
+      <c r="E40" s="6" t="inlineStr">
         <is>
           <t>salentica.fact_opportunity</t>
         </is>
       </c>
-      <c r="F35" s="11" t="inlineStr">
+      <c r="F40" s="7" t="inlineStr">
         <is>
           <t>Verify SG_SAL_22 Fallback: Unmapped Foreign References Default to -1 (Zero Orphan NULLs)</t>
         </is>
       </c>
-      <c r="G35" s="11" t="inlineStr">
+      <c r="G40" s="7" t="inlineStr">
         <is>
           <t>fact_opportunity populated</t>
         </is>
       </c>
-      <c r="H35" s="11" t="inlineStr">
+      <c r="H40" s="7" t="inlineStr">
         <is>
           <t>When natural ID is NULL, the corresponding SK defaults to -1. Zero unmapped NULLs in SK columns.</t>
         </is>
       </c>
-      <c r="I35" s="17" t="inlineStr">
+      <c r="I40" s="18" t="inlineStr">
         <is>
           <t>SELECT 
     SUM(CASE WHEN accountid IS NULL AND accountid_sk = -1 THEN 1 ELSE 0 END) AS ProperlyDefaulted_AccountSK,
@@ -2694,48 +3108,48 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="54" customHeight="1">
-      <c r="A36" s="8" t="inlineStr">
+    <row r="41" ht="54" customHeight="1">
+      <c r="A41" s="12" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B36" s="8" t="inlineStr">
+      <c r="B41" s="12" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_01</t>
         </is>
       </c>
-      <c r="C36" s="9" t="inlineStr">
+      <c r="C41" s="13" t="inlineStr">
         <is>
           <t>SCD2 Deduplication</t>
         </is>
       </c>
-      <c r="D36" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E36" s="6" t="inlineStr">
+      <c r="D41" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E41" s="10" t="inlineStr">
         <is>
           <t>tamarac.dim_account_information</t>
         </is>
       </c>
-      <c r="F36" s="7" t="inlineStr">
+      <c r="F41" s="11" t="inlineStr">
         <is>
           <t>Verify Active Deduplication on PK ['account_number'] (is_current = 'True')</t>
         </is>
       </c>
-      <c r="G36" s="7" t="inlineStr">
+      <c r="G41" s="11" t="inlineStr">
         <is>
           <t>dim_account_information populated</t>
         </is>
       </c>
-      <c r="H36" s="7" t="inlineStr">
+      <c r="H41" s="11" t="inlineStr">
         <is>
           <t>Zero duplicate active accounts. Exactly one is_current = 'True' row per account_number.</t>
         </is>
       </c>
-      <c r="I36" s="18" t="inlineStr">
+      <c r="I41" s="17" t="inlineStr">
         <is>
           <t>SELECT account_number, COUNT(*) AS ActiveDuplicateCount
 FROM Gold_Warehouse.tamarac.dim_account_information
@@ -2745,48 +3159,48 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="54" customHeight="1">
-      <c r="A37" s="12" t="inlineStr">
+    <row r="42" ht="54" customHeight="1">
+      <c r="A42" s="8" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B37" s="12" t="inlineStr">
+      <c r="B42" s="8" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_02</t>
         </is>
       </c>
-      <c r="C37" s="13" t="inlineStr">
+      <c r="C42" s="9" t="inlineStr">
         <is>
           <t>SK Uniqueness</t>
         </is>
       </c>
-      <c r="D37" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E37" s="10" t="inlineStr">
+      <c r="D42" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
         <is>
           <t>tamarac.dim_account_information</t>
         </is>
       </c>
-      <c r="F37" s="11" t="inlineStr">
+      <c r="F42" s="7" t="inlineStr">
         <is>
           <t>Verify Primary Surrogate Key (account_information_SK) uniqueness across all records</t>
         </is>
       </c>
-      <c r="G37" s="11" t="inlineStr">
+      <c r="G42" s="7" t="inlineStr">
         <is>
           <t>dim_account_information populated</t>
         </is>
       </c>
-      <c r="H37" s="11" t="inlineStr">
+      <c r="H42" s="7" t="inlineStr">
         <is>
           <t>Surrogate key account_information_SK is strictly unique across all rows. Zero duplicates.</t>
         </is>
       </c>
-      <c r="I37" s="17" t="inlineStr">
+      <c r="I42" s="18" t="inlineStr">
         <is>
           <t>SELECT account_information_SK, COUNT(*) AS DuplicateCount
 FROM Gold_Warehouse.tamarac.dim_account_information
@@ -2795,48 +3209,48 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="54" customHeight="1">
-      <c r="A38" s="8" t="inlineStr">
+    <row r="43" ht="54" customHeight="1">
+      <c r="A43" s="12" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B38" s="8" t="inlineStr">
+      <c r="B43" s="12" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_03</t>
         </is>
       </c>
-      <c r="C38" s="9" t="inlineStr">
+      <c r="C43" s="13" t="inlineStr">
         <is>
           <t>Audit Columns</t>
         </is>
       </c>
-      <c r="D38" s="19" t="inlineStr">
+      <c r="D43" s="19" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E38" s="6" t="inlineStr">
+      <c r="E43" s="10" t="inlineStr">
         <is>
           <t>tamarac.dim_account_information</t>
         </is>
       </c>
-      <c r="F38" s="7" t="inlineStr">
+      <c r="F43" s="11" t="inlineStr">
         <is>
           <t>Verify file_business_date and updated_at populated on active Tamarac accounts</t>
         </is>
       </c>
-      <c r="G38" s="7" t="inlineStr">
+      <c r="G43" s="11" t="inlineStr">
         <is>
           <t>dim_account_information populated</t>
         </is>
       </c>
-      <c r="H38" s="7" t="inlineStr">
+      <c r="H43" s="11" t="inlineStr">
         <is>
           <t>file_business_date and updated_at are non-null and &lt;= current calendar date.</t>
         </is>
       </c>
-      <c r="I38" s="18" t="inlineStr">
+      <c r="I43" s="17" t="inlineStr">
         <is>
           <t>SELECT 
     COUNT(*) AS TotalRows,
@@ -2847,48 +3261,48 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="54" customHeight="1">
-      <c r="A39" s="12" t="inlineStr">
+    <row r="44" ht="54" customHeight="1">
+      <c r="A44" s="8" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B39" s="12" t="inlineStr">
+      <c r="B44" s="8" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_04</t>
         </is>
       </c>
-      <c r="C39" s="13" t="inlineStr">
+      <c r="C44" s="9" t="inlineStr">
         <is>
           <t>SCD2 Deduplication</t>
         </is>
       </c>
-      <c r="D39" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E39" s="10" t="inlineStr">
+      <c r="D44" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E44" s="6" t="inlineStr">
         <is>
           <t>tamarac.dim_account_model_allocation</t>
         </is>
       </c>
-      <c r="F39" s="11" t="inlineStr">
+      <c r="F44" s="7" t="inlineStr">
         <is>
           <t>Verify Active Deduplication on Composite PK ['account_number', 'model_name']</t>
         </is>
       </c>
-      <c r="G39" s="11" t="inlineStr">
+      <c r="G44" s="7" t="inlineStr">
         <is>
           <t>dim_account_model_allocation populated</t>
         </is>
       </c>
-      <c r="H39" s="11" t="inlineStr">
+      <c r="H44" s="7" t="inlineStr">
         <is>
           <t>Zero duplicate active model allocations per (account_number, model_name).</t>
         </is>
       </c>
-      <c r="I39" s="17" t="inlineStr">
+      <c r="I44" s="18" t="inlineStr">
         <is>
           <t>SELECT account_number, model_name, COUNT(*) AS ActiveDuplicateAllocations
 FROM Gold_Warehouse.tamarac.dim_account_model_allocation
@@ -2898,48 +3312,48 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="54" customHeight="1">
-      <c r="A40" s="8" t="inlineStr">
+    <row r="45" ht="54" customHeight="1">
+      <c r="A45" s="12" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B40" s="8" t="inlineStr">
+      <c r="B45" s="12" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_05</t>
         </is>
       </c>
-      <c r="C40" s="9" t="inlineStr">
+      <c r="C45" s="13" t="inlineStr">
         <is>
           <t>SK Uniqueness</t>
         </is>
       </c>
-      <c r="D40" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E40" s="6" t="inlineStr">
+      <c r="D45" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E45" s="10" t="inlineStr">
         <is>
           <t>tamarac.dim_account_model_allocation</t>
         </is>
       </c>
-      <c r="F40" s="7" t="inlineStr">
+      <c r="F45" s="11" t="inlineStr">
         <is>
           <t>Verify Primary Surrogate Key (account_model_SK) uniqueness</t>
         </is>
       </c>
-      <c r="G40" s="7" t="inlineStr">
+      <c r="G45" s="11" t="inlineStr">
         <is>
           <t>dim_account_model_allocation populated</t>
         </is>
       </c>
-      <c r="H40" s="7" t="inlineStr">
+      <c r="H45" s="11" t="inlineStr">
         <is>
           <t>account_model_SK is unique with zero NULL values.</t>
         </is>
       </c>
-      <c r="I40" s="18" t="inlineStr">
+      <c r="I45" s="17" t="inlineStr">
         <is>
           <t>SELECT account_model_SK, COUNT(*) AS DuplicateModelSK
 FROM Gold_Warehouse.tamarac.dim_account_model_allocation
@@ -2948,48 +3362,48 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="54" customHeight="1">
-      <c r="A41" s="12" t="inlineStr">
+    <row r="46" ht="54" customHeight="1">
+      <c r="A46" s="8" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B41" s="12" t="inlineStr">
+      <c r="B46" s="8" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_06</t>
         </is>
       </c>
-      <c r="C41" s="13" t="inlineStr">
+      <c r="C46" s="9" t="inlineStr">
         <is>
           <t>Cross-Table Linkage</t>
         </is>
       </c>
-      <c r="D41" s="19" t="inlineStr">
+      <c r="D46" s="19" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E41" s="10" t="inlineStr">
+      <c r="E46" s="6" t="inlineStr">
         <is>
           <t>tamarac.dim_account_model_allocation</t>
         </is>
       </c>
-      <c r="F41" s="11" t="inlineStr">
+      <c r="F46" s="7" t="inlineStr">
         <is>
           <t>Verify Cross-Table Linkage: Every account_number exists in dim_account_information</t>
         </is>
       </c>
-      <c r="G41" s="11" t="inlineStr">
+      <c r="G46" s="7" t="inlineStr">
         <is>
           <t>dim_account_model_allocation populated</t>
         </is>
       </c>
-      <c r="H41" s="11" t="inlineStr">
+      <c r="H46" s="7" t="inlineStr">
         <is>
           <t>Zero orphan model allocation accounts. All account_number values exist in parent dimension.</t>
         </is>
       </c>
-      <c r="I41" s="17" t="inlineStr">
+      <c r="I46" s="18" t="inlineStr">
         <is>
           <t>SELECT COUNT(*) AS OrphanModelAllocations
 FROM Gold_Warehouse.tamarac.dim_account_model_allocation ma
@@ -3000,48 +3414,48 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="54" customHeight="1">
-      <c r="A42" s="8" t="inlineStr">
+    <row r="47" ht="54" customHeight="1">
+      <c r="A47" s="12" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B42" s="8" t="inlineStr">
+      <c r="B47" s="12" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_07</t>
         </is>
       </c>
-      <c r="C42" s="9" t="inlineStr">
+      <c r="C47" s="13" t="inlineStr">
         <is>
           <t>SCD2 Date Validation</t>
         </is>
       </c>
-      <c r="D42" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E42" s="6" t="inlineStr">
+      <c r="D47" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E47" s="10" t="inlineStr">
         <is>
           <t>tamarac.dim_account_information</t>
         </is>
       </c>
-      <c r="F42" s="7" t="inlineStr">
+      <c r="F47" s="11" t="inlineStr">
         <is>
           <t>Verify Inactive End Date Rule: effective_end_date &lt;= (MAX(file_business_date) - 1 day) and non-null</t>
         </is>
       </c>
-      <c r="G42" s="7" t="inlineStr">
+      <c r="G47" s="11" t="inlineStr">
         <is>
           <t>dim_account_information populated with inactive records</t>
         </is>
       </c>
-      <c r="H42" s="7" t="inlineStr">
+      <c r="H47" s="11" t="inlineStr">
         <is>
           <t>Exceeded_Cutoff_Count = 0, Null_End_Date_Count = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I42" s="18" t="inlineStr">
+      <c r="I47" s="17" t="inlineStr">
         <is>
           <t>SELECT 
     'dim_account_information' AS TableName,
@@ -3061,48 +3475,48 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="54" customHeight="1">
-      <c r="A43" s="12" t="inlineStr">
+    <row r="48" ht="54" customHeight="1">
+      <c r="A48" s="8" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B43" s="12" t="inlineStr">
+      <c r="B48" s="8" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_08</t>
         </is>
       </c>
-      <c r="C43" s="13" t="inlineStr">
+      <c r="C48" s="9" t="inlineStr">
         <is>
           <t>SCD2 Date Validation</t>
         </is>
       </c>
-      <c r="D43" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E43" s="10" t="inlineStr">
+      <c r="D48" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="inlineStr">
         <is>
           <t>tamarac.dim_account_model_allocation</t>
         </is>
       </c>
-      <c r="F43" s="11" t="inlineStr">
+      <c r="F48" s="7" t="inlineStr">
         <is>
           <t>Verify Inactive End Date Rule: effective_end_date &lt;= (MAX(file_business_date) - 1 day) and non-null</t>
         </is>
       </c>
-      <c r="G43" s="11" t="inlineStr">
+      <c r="G48" s="7" t="inlineStr">
         <is>
           <t>dim_account_model_allocation populated with inactive records</t>
         </is>
       </c>
-      <c r="H43" s="11" t="inlineStr">
+      <c r="H48" s="7" t="inlineStr">
         <is>
           <t>Exceeded_Cutoff_Count = 0, Null_End_Date_Count = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I43" s="17" t="inlineStr">
+      <c r="I48" s="18" t="inlineStr">
         <is>
           <t>SELECT 
     'dim_account_model_allocation' AS TableName,
@@ -3122,48 +3536,48 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="54" customHeight="1">
-      <c r="A44" s="8" t="inlineStr">
+    <row r="49" ht="54" customHeight="1">
+      <c r="A49" s="12" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B44" s="8" t="inlineStr">
+      <c r="B49" s="12" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_09</t>
         </is>
       </c>
-      <c r="C44" s="9" t="inlineStr">
+      <c r="C49" s="13" t="inlineStr">
         <is>
           <t>SCD2 Timeline &amp; SK Monotonicity</t>
         </is>
       </c>
-      <c r="D44" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E44" s="6" t="inlineStr">
+      <c r="D49" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E49" s="10" t="inlineStr">
         <is>
           <t>tamarac.dim_account_information</t>
         </is>
       </c>
-      <c r="F44" s="7" t="inlineStr">
+      <c r="F49" s="11" t="inlineStr">
         <is>
           <t>Verify SCD2 Timeline Continuity (Zero Gaps, Zero Overlaps) &amp; SK Monotonic Increment</t>
         </is>
       </c>
-      <c r="G44" s="7" t="inlineStr">
+      <c r="G49" s="11" t="inlineStr">
         <is>
           <t>dim_account_information with multiple versions per account_number</t>
         </is>
       </c>
-      <c r="H44" s="7" t="inlineStr">
+      <c r="H49" s="11" t="inlineStr">
         <is>
           <t>Timeline_Gap_Or_Overlap_Count = 0, SK_Non_Incrementing_Violation_Count = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I44" s="18" t="inlineStr">
+      <c r="I49" s="17" t="inlineStr">
         <is>
           <t>;WITH InfoTimeline AS (
     SELECT 
@@ -3191,48 +3605,48 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="54" customHeight="1">
-      <c r="A45" s="12" t="inlineStr">
+    <row r="50" ht="54" customHeight="1">
+      <c r="A50" s="8" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B45" s="12" t="inlineStr">
+      <c r="B50" s="8" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_10</t>
         </is>
       </c>
-      <c r="C45" s="13" t="inlineStr">
+      <c r="C50" s="9" t="inlineStr">
         <is>
           <t>SCD2 Timeline &amp; SK Monotonicity</t>
         </is>
       </c>
-      <c r="D45" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E45" s="10" t="inlineStr">
+      <c r="D50" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="inlineStr">
         <is>
           <t>tamarac.dim_account_model_allocation</t>
         </is>
       </c>
-      <c r="F45" s="11" t="inlineStr">
+      <c r="F50" s="7" t="inlineStr">
         <is>
           <t>Verify SCD2 Timeline Continuity (Zero Gaps, Zero Overlaps) &amp; SK Monotonic Increment</t>
         </is>
       </c>
-      <c r="G45" s="11" t="inlineStr">
+      <c r="G50" s="7" t="inlineStr">
         <is>
           <t>dim_account_model_allocation with multiple versions per composite key</t>
         </is>
       </c>
-      <c r="H45" s="11" t="inlineStr">
+      <c r="H50" s="7" t="inlineStr">
         <is>
           <t>Timeline_Gap_Or_Overlap_Count = 0, SK_Non_Incrementing_Violation_Count = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I45" s="17" t="inlineStr">
+      <c r="I50" s="18" t="inlineStr">
         <is>
           <t>;WITH ModelTimeline AS (
     SELECT 
@@ -3261,48 +3675,48 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="54" customHeight="1">
-      <c r="A46" s="8" t="inlineStr">
+    <row r="51" ht="54" customHeight="1">
+      <c r="A51" s="12" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B46" s="8" t="inlineStr">
+      <c r="B51" s="12" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_11</t>
         </is>
       </c>
-      <c r="C46" s="9" t="inlineStr">
+      <c r="C51" s="13" t="inlineStr">
         <is>
           <t>Date Sanity &amp; Inversions</t>
         </is>
       </c>
-      <c r="D46" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E46" s="6" t="inlineStr">
+      <c r="D51" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E51" s="10" t="inlineStr">
         <is>
           <t>tamarac.dim_account_information</t>
         </is>
       </c>
-      <c r="F46" s="7" t="inlineStr">
+      <c r="F51" s="11" t="inlineStr">
         <is>
           <t>Verify Date Sanity: Zero inverted dates (start &gt; end) and active records have non-future start dates</t>
         </is>
       </c>
-      <c r="G46" s="7" t="inlineStr">
+      <c r="G51" s="11" t="inlineStr">
         <is>
           <t>dim_account_information populated</t>
         </is>
       </c>
-      <c r="H46" s="7" t="inlineStr">
+      <c r="H51" s="11" t="inlineStr">
         <is>
           <t>Inverted_Date_Count = 0, Future_Active_Start_Date = 0, Null_Start_Date_Count = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I46" s="18" t="inlineStr">
+      <c r="I51" s="17" t="inlineStr">
         <is>
           <t>SELECT 
     'dim_account_information' AS TableName,
@@ -3320,48 +3734,48 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="54" customHeight="1">
-      <c r="A47" s="12" t="inlineStr">
+    <row r="52" ht="54" customHeight="1">
+      <c r="A52" s="8" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B47" s="12" t="inlineStr">
+      <c r="B52" s="8" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_12</t>
         </is>
       </c>
-      <c r="C47" s="13" t="inlineStr">
+      <c r="C52" s="9" t="inlineStr">
         <is>
           <t>Date Sanity &amp; Inversions</t>
         </is>
       </c>
-      <c r="D47" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E47" s="10" t="inlineStr">
+      <c r="D52" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E52" s="6" t="inlineStr">
         <is>
           <t>tamarac.dim_account_model_allocation</t>
         </is>
       </c>
-      <c r="F47" s="11" t="inlineStr">
+      <c r="F52" s="7" t="inlineStr">
         <is>
           <t>Verify Date Sanity: Zero inverted dates (start &gt; end) and active records have non-future start dates</t>
         </is>
       </c>
-      <c r="G47" s="11" t="inlineStr">
+      <c r="G52" s="7" t="inlineStr">
         <is>
           <t>dim_account_model_allocation populated</t>
         </is>
       </c>
-      <c r="H47" s="11" t="inlineStr">
+      <c r="H52" s="7" t="inlineStr">
         <is>
           <t>Inverted_Date_Count = 0, Future_Active_Start_Date = 0, Null_Start_Date_Count = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I47" s="17" t="inlineStr">
+      <c r="I52" s="18" t="inlineStr">
         <is>
           <t>SELECT 
     'dim_account_model_allocation' AS TableName,
@@ -3379,48 +3793,48 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="54" customHeight="1">
-      <c r="A48" s="8" t="inlineStr">
+    <row r="53" ht="54" customHeight="1">
+      <c r="A53" s="12" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B48" s="8" t="inlineStr">
+      <c r="B53" s="12" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_13</t>
         </is>
       </c>
-      <c r="C48" s="9" t="inlineStr">
+      <c r="C53" s="13" t="inlineStr">
         <is>
           <t>Open-Ended Active Records</t>
         </is>
       </c>
-      <c r="D48" s="19" t="inlineStr">
+      <c r="D53" s="19" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E48" s="6" t="inlineStr">
+      <c r="E53" s="10" t="inlineStr">
         <is>
           <t>tamarac.dim_account_information</t>
         </is>
       </c>
-      <c r="F48" s="7" t="inlineStr">
+      <c r="F53" s="11" t="inlineStr">
         <is>
           <t>Verify Active Records are Open-Ended (effective_end_date is NULL or '9999-12-31')</t>
         </is>
       </c>
-      <c r="G48" s="7" t="inlineStr">
+      <c r="G53" s="11" t="inlineStr">
         <is>
           <t>dim_account_information where is_current = 'True'</t>
         </is>
       </c>
-      <c r="H48" s="7" t="inlineStr">
+      <c r="H53" s="11" t="inlineStr">
         <is>
           <t>Prematurely_Ended_Active_Records = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I48" s="18" t="inlineStr">
+      <c r="I53" s="17" t="inlineStr">
         <is>
           <t>SELECT 
     'dim_account_information' AS TableName,
@@ -3435,48 +3849,48 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="54" customHeight="1">
-      <c r="A49" s="12" t="inlineStr">
+    <row r="54" ht="54" customHeight="1">
+      <c r="A54" s="8" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B49" s="12" t="inlineStr">
+      <c r="B54" s="8" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_14</t>
         </is>
       </c>
-      <c r="C49" s="13" t="inlineStr">
+      <c r="C54" s="9" t="inlineStr">
         <is>
           <t>Open-Ended Active Records</t>
         </is>
       </c>
-      <c r="D49" s="19" t="inlineStr">
+      <c r="D54" s="19" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E49" s="10" t="inlineStr">
+      <c r="E54" s="6" t="inlineStr">
         <is>
           <t>tamarac.dim_account_model_allocation</t>
         </is>
       </c>
-      <c r="F49" s="11" t="inlineStr">
+      <c r="F54" s="7" t="inlineStr">
         <is>
           <t>Verify Active Records are Open-Ended (effective_end_date is NULL or '9999-12-31')</t>
         </is>
       </c>
-      <c r="G49" s="11" t="inlineStr">
+      <c r="G54" s="7" t="inlineStr">
         <is>
           <t>dim_account_model_allocation where is_current = 'True'</t>
         </is>
       </c>
-      <c r="H49" s="11" t="inlineStr">
+      <c r="H54" s="7" t="inlineStr">
         <is>
           <t>Prematurely_Ended_Active_Records = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I49" s="17" t="inlineStr">
+      <c r="I54" s="18" t="inlineStr">
         <is>
           <t>SELECT 
     'dim_account_model_allocation' AS TableName,
@@ -3491,48 +3905,48 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="54" customHeight="1">
-      <c r="A50" s="8" t="inlineStr">
+    <row r="55" ht="54" customHeight="1">
+      <c r="A55" s="12" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B50" s="8" t="inlineStr">
+      <c r="B55" s="12" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_15</t>
         </is>
       </c>
-      <c r="C50" s="9" t="inlineStr">
+      <c r="C55" s="13" t="inlineStr">
         <is>
           <t>Version Evolution Audit</t>
         </is>
       </c>
-      <c r="D50" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E50" s="6" t="inlineStr">
+      <c r="D55" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E55" s="10" t="inlineStr">
         <is>
           <t>tamarac.dim_account_information</t>
         </is>
       </c>
-      <c r="F50" s="7" t="inlineStr">
+      <c r="F55" s="11" t="inlineStr">
         <is>
           <t>Verify Run Evolution: Every new run produces New Incremented SK, Advancing Start Date, and Latest Version is Active</t>
         </is>
       </c>
-      <c r="G50" s="7" t="inlineStr">
+      <c r="G55" s="11" t="inlineStr">
         <is>
           <t>dim_account_information with historical batch progression</t>
         </is>
       </c>
-      <c r="H50" s="7" t="inlineStr">
+      <c r="H55" s="11" t="inlineStr">
         <is>
           <t>Reused_Or_NonIncrementing_SK_Count = 0, NonAdvancing_EffectiveStartDate_Count = 0, Timeline_Gap_Or_Overlap_Count = 0, LatestVersion_Not_Active_Count = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I50" s="18" t="inlineStr">
+      <c r="I55" s="17" t="inlineStr">
         <is>
           <t>;WITH VersionChains AS (
     SELECT 
@@ -3566,48 +3980,48 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="54" customHeight="1">
-      <c r="A51" s="12" t="inlineStr">
+    <row r="56" ht="54" customHeight="1">
+      <c r="A56" s="8" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B51" s="12" t="inlineStr">
+      <c r="B56" s="8" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_16</t>
         </is>
       </c>
-      <c r="C51" s="13" t="inlineStr">
+      <c r="C56" s="9" t="inlineStr">
         <is>
           <t>Version Evolution Audit</t>
         </is>
       </c>
-      <c r="D51" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E51" s="10" t="inlineStr">
+      <c r="D56" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E56" s="6" t="inlineStr">
         <is>
           <t>tamarac.dim_account_model_allocation</t>
         </is>
       </c>
-      <c r="F51" s="11" t="inlineStr">
+      <c r="F56" s="7" t="inlineStr">
         <is>
           <t>Verify Run Evolution: Every new run produces New Incremented SK, Advancing Start Date, and Latest Version is Active</t>
         </is>
       </c>
-      <c r="G51" s="11" t="inlineStr">
+      <c r="G56" s="7" t="inlineStr">
         <is>
           <t>dim_account_model_allocation with historical batch progression</t>
         </is>
       </c>
-      <c r="H51" s="11" t="inlineStr">
+      <c r="H56" s="7" t="inlineStr">
         <is>
           <t>Reused_Or_NonIncrementing_SK_Count = 0, NonAdvancing_EffectiveStartDate_Count = 0, Timeline_Gap_Or_Overlap_Count = 0, LatestVersion_Not_Active_Count = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I51" s="17" t="inlineStr">
+      <c r="I56" s="18" t="inlineStr">
         <is>
           <t>;WITH ModelChains AS (
     SELECT 
@@ -3642,48 +4056,48 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="54" customHeight="1">
-      <c r="A52" s="8" t="inlineStr">
+    <row r="57" ht="54" customHeight="1">
+      <c r="A57" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B52" s="8" t="inlineStr">
+      <c r="B57" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_01</t>
         </is>
       </c>
-      <c r="C52" s="9" t="inlineStr">
+      <c r="C57" s="13" t="inlineStr">
         <is>
           <t>SCD2 Deduplication</t>
         </is>
       </c>
-      <c r="D52" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E52" s="6" t="inlineStr">
+      <c r="D57" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E57" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master</t>
         </is>
       </c>
-      <c r="F52" s="7" t="inlineStr">
+      <c r="F57" s="11" t="inlineStr">
         <is>
           <t>Verify Active Deduplication on Business Key ['customer_account_number'] (is_current = 1)</t>
         </is>
       </c>
-      <c r="G52" s="7" t="inlineStr">
+      <c r="G57" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master populated</t>
         </is>
       </c>
-      <c r="H52" s="7" t="inlineStr">
+      <c r="H57" s="11" t="inlineStr">
         <is>
           <t>Zero duplicate active accounts. Exactly one is_current = 1 record per customer_account_number.</t>
         </is>
       </c>
-      <c r="I52" s="18" t="inlineStr">
+      <c r="I57" s="17" t="inlineStr">
         <is>
           <t>SELECT customer_account_number, COUNT(*) AS ActiveDuplicateCount
 FROM Gold_Warehouse.innotrust.dim_account_master
@@ -3693,48 +4107,48 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="54" customHeight="1">
-      <c r="A53" s="12" t="inlineStr">
+    <row r="58" ht="54" customHeight="1">
+      <c r="A58" s="8" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B53" s="12" t="inlineStr">
+      <c r="B58" s="8" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_02</t>
         </is>
       </c>
-      <c r="C53" s="13" t="inlineStr">
+      <c r="C58" s="9" t="inlineStr">
         <is>
           <t>SK Uniqueness</t>
         </is>
       </c>
-      <c r="D53" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E53" s="10" t="inlineStr">
+      <c r="D58" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master</t>
         </is>
       </c>
-      <c r="F53" s="11" t="inlineStr">
+      <c r="F58" s="7" t="inlineStr">
         <is>
           <t>Verify Primary Surrogate Key (dim_account_master_sk) uniqueness and non-null constraint</t>
         </is>
       </c>
-      <c r="G53" s="11" t="inlineStr">
+      <c r="G58" s="7" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master populated</t>
         </is>
       </c>
-      <c r="H53" s="11" t="inlineStr">
+      <c r="H58" s="7" t="inlineStr">
         <is>
           <t>dim_account_master_sk is strictly unique across all versions with zero NULL values.</t>
         </is>
       </c>
-      <c r="I53" s="17" t="inlineStr">
+      <c r="I58" s="18" t="inlineStr">
         <is>
           <t>SELECT dim_account_master_sk, COUNT(*) AS DuplicateCount
 FROM Gold_Warehouse.innotrust.dim_account_master
@@ -3748,48 +4162,48 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="54" customHeight="1">
-      <c r="A54" s="8" t="inlineStr">
+    <row r="59" ht="54" customHeight="1">
+      <c r="A59" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B54" s="8" t="inlineStr">
+      <c r="B59" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_03</t>
         </is>
       </c>
-      <c r="C54" s="9" t="inlineStr">
+      <c r="C59" s="13" t="inlineStr">
         <is>
           <t>SCD2 Deduplication</t>
         </is>
       </c>
-      <c r="D54" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E54" s="6" t="inlineStr">
+      <c r="D59" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E59" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_account_category_codes</t>
         </is>
       </c>
-      <c r="F54" s="7" t="inlineStr">
+      <c r="F59" s="11" t="inlineStr">
         <is>
           <t>Verify Active Deduplication on Business Key ['account_category_code'] (is_current = 1)</t>
         </is>
       </c>
-      <c r="G54" s="7" t="inlineStr">
+      <c r="G59" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_account_category_codes populated</t>
         </is>
       </c>
-      <c r="H54" s="7" t="inlineStr">
+      <c r="H59" s="11" t="inlineStr">
         <is>
           <t>Zero duplicate active category codes per account_category_code.</t>
         </is>
       </c>
-      <c r="I54" s="18" t="inlineStr">
+      <c r="I59" s="17" t="inlineStr">
         <is>
           <t>SELECT account_category_code, COUNT(*) AS ActiveDuplicateCount
 FROM Gold_Warehouse.innotrust.dim_account_category_codes
@@ -3799,48 +4213,48 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="54" customHeight="1">
-      <c r="A55" s="12" t="inlineStr">
+    <row r="60" ht="54" customHeight="1">
+      <c r="A60" s="8" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B55" s="12" t="inlineStr">
+      <c r="B60" s="8" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_04</t>
         </is>
       </c>
-      <c r="C55" s="13" t="inlineStr">
+      <c r="C60" s="9" t="inlineStr">
         <is>
           <t>SK Uniqueness</t>
         </is>
       </c>
-      <c r="D55" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E55" s="10" t="inlineStr">
+      <c r="D60" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E60" s="6" t="inlineStr">
         <is>
           <t>innotrust.dim_account_category_codes</t>
         </is>
       </c>
-      <c r="F55" s="11" t="inlineStr">
+      <c r="F60" s="7" t="inlineStr">
         <is>
           <t>Verify Primary Surrogate Key (dim_account_master_sk) uniqueness on dim_account_category_codes</t>
         </is>
       </c>
-      <c r="G55" s="11" t="inlineStr">
+      <c r="G60" s="7" t="inlineStr">
         <is>
           <t>innotrust.dim_account_category_codes populated</t>
         </is>
       </c>
-      <c r="H55" s="11" t="inlineStr">
+      <c r="H60" s="7" t="inlineStr">
         <is>
           <t>Surrogate key dim_account_master_sk is unique across all rows with zero NULLs.</t>
         </is>
       </c>
-      <c r="I55" s="17" t="inlineStr">
+      <c r="I60" s="18" t="inlineStr">
         <is>
           <t>SELECT dim_account_master_sk, COUNT(*) AS DuplicateCount
 FROM Gold_Warehouse.innotrust.dim_account_category_codes
@@ -3849,48 +4263,48 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="54" customHeight="1">
-      <c r="A56" s="8" t="inlineStr">
+    <row r="61" ht="54" customHeight="1">
+      <c r="A61" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B56" s="8" t="inlineStr">
+      <c r="B61" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_05</t>
         </is>
       </c>
-      <c r="C56" s="9" t="inlineStr">
+      <c r="C61" s="13" t="inlineStr">
         <is>
           <t>SCD2 Deduplication</t>
         </is>
       </c>
-      <c r="D56" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E56" s="6" t="inlineStr">
+      <c r="D61" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E61" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_account_type_codes</t>
         </is>
       </c>
-      <c r="F56" s="7" t="inlineStr">
+      <c r="F61" s="11" t="inlineStr">
         <is>
           <t>Verify Active Deduplication on Business Key ['account_type_code'] (is_current = 1)</t>
         </is>
       </c>
-      <c r="G56" s="7" t="inlineStr">
+      <c r="G61" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_account_type_codes populated</t>
         </is>
       </c>
-      <c r="H56" s="7" t="inlineStr">
+      <c r="H61" s="11" t="inlineStr">
         <is>
           <t>Zero duplicate active account types per account_type_code.</t>
         </is>
       </c>
-      <c r="I56" s="18" t="inlineStr">
+      <c r="I61" s="17" t="inlineStr">
         <is>
           <t>SELECT account_type_code, COUNT(*) AS ActiveDuplicateCount
 FROM Gold_Warehouse.innotrust.dim_account_type_codes
@@ -3900,48 +4314,48 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="54" customHeight="1">
-      <c r="A57" s="12" t="inlineStr">
+    <row r="62" ht="54" customHeight="1">
+      <c r="A62" s="8" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B57" s="12" t="inlineStr">
+      <c r="B62" s="8" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_06</t>
         </is>
       </c>
-      <c r="C57" s="13" t="inlineStr">
+      <c r="C62" s="9" t="inlineStr">
         <is>
           <t>SK Uniqueness</t>
         </is>
       </c>
-      <c r="D57" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E57" s="10" t="inlineStr">
+      <c r="D62" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E62" s="6" t="inlineStr">
         <is>
           <t>innotrust.dim_account_type_codes</t>
         </is>
       </c>
-      <c r="F57" s="11" t="inlineStr">
+      <c r="F62" s="7" t="inlineStr">
         <is>
           <t>Verify Primary Surrogate Key (dim_account_type_codes_sk) uniqueness and non-null constraint</t>
         </is>
       </c>
-      <c r="G57" s="11" t="inlineStr">
+      <c r="G62" s="7" t="inlineStr">
         <is>
           <t>innotrust.dim_account_type_codes populated</t>
         </is>
       </c>
-      <c r="H57" s="11" t="inlineStr">
+      <c r="H62" s="7" t="inlineStr">
         <is>
           <t>dim_account_type_codes_sk is strictly unique across all versions with zero NULLs.</t>
         </is>
       </c>
-      <c r="I57" s="17" t="inlineStr">
+      <c r="I62" s="18" t="inlineStr">
         <is>
           <t>SELECT dim_account_type_codes_sk, COUNT(*) AS DuplicateCount
 FROM Gold_Warehouse.innotrust.dim_account_type_codes
@@ -3950,48 +4364,48 @@
         </is>
       </c>
     </row>
-    <row r="58" ht="54" customHeight="1">
-      <c r="A58" s="8" t="inlineStr">
+    <row r="63" ht="54" customHeight="1">
+      <c r="A63" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B58" s="8" t="inlineStr">
+      <c r="B63" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_07</t>
         </is>
       </c>
-      <c r="C58" s="9" t="inlineStr">
+      <c r="C63" s="13" t="inlineStr">
         <is>
           <t>SCD2 Deduplication</t>
         </is>
       </c>
-      <c r="D58" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E58" s="6" t="inlineStr">
+      <c r="D63" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E63" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_master_sec_index</t>
         </is>
       </c>
-      <c r="F58" s="7" t="inlineStr">
+      <c r="F63" s="11" t="inlineStr">
         <is>
           <t>Verify Active Deduplication on Security Primary Key ['isin'] (is_current = 1)</t>
         </is>
       </c>
-      <c r="G58" s="7" t="inlineStr">
+      <c r="G63" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_master_sec_index populated</t>
         </is>
       </c>
-      <c r="H58" s="7" t="inlineStr">
+      <c r="H63" s="11" t="inlineStr">
         <is>
           <t>Zero duplicate active securities. Exactly one is_current = 1 record per isin.</t>
         </is>
       </c>
-      <c r="I58" s="18" t="inlineStr">
+      <c r="I63" s="17" t="inlineStr">
         <is>
           <t>SELECT isin, COUNT(*) AS ActiveDuplicateCount
 FROM Gold_Warehouse.innotrust.dim_master_sec_index
@@ -4001,48 +4415,48 @@
         </is>
       </c>
     </row>
-    <row r="59" ht="54" customHeight="1">
-      <c r="A59" s="12" t="inlineStr">
+    <row r="64" ht="54" customHeight="1">
+      <c r="A64" s="8" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B59" s="12" t="inlineStr">
+      <c r="B64" s="8" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_08</t>
         </is>
       </c>
-      <c r="C59" s="13" t="inlineStr">
+      <c r="C64" s="9" t="inlineStr">
         <is>
           <t>SK Uniqueness</t>
         </is>
       </c>
-      <c r="D59" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E59" s="10" t="inlineStr">
+      <c r="D64" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E64" s="6" t="inlineStr">
         <is>
           <t>innotrust.dim_master_sec_index</t>
         </is>
       </c>
-      <c r="F59" s="11" t="inlineStr">
+      <c r="F64" s="7" t="inlineStr">
         <is>
           <t>Verify Primary Surrogate Key (dim_master_sec_index_sk) uniqueness across all records</t>
         </is>
       </c>
-      <c r="G59" s="11" t="inlineStr">
+      <c r="G64" s="7" t="inlineStr">
         <is>
           <t>innotrust.dim_master_sec_index populated</t>
         </is>
       </c>
-      <c r="H59" s="11" t="inlineStr">
+      <c r="H64" s="7" t="inlineStr">
         <is>
           <t>dim_master_sec_index_sk is strictly unique across all versions with zero NULLs.</t>
         </is>
       </c>
-      <c r="I59" s="17" t="inlineStr">
+      <c r="I64" s="18" t="inlineStr">
         <is>
           <t>SELECT dim_master_sec_index_sk, COUNT(*) AS DuplicateCount
 FROM Gold_Warehouse.innotrust.dim_master_sec_index
@@ -4051,48 +4465,48 @@
         </is>
       </c>
     </row>
-    <row r="60" ht="54" customHeight="1">
-      <c r="A60" s="8" t="inlineStr">
+    <row r="65" ht="54" customHeight="1">
+      <c r="A65" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B60" s="8" t="inlineStr">
+      <c r="B65" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_09</t>
         </is>
       </c>
-      <c r="C60" s="9" t="inlineStr">
+      <c r="C65" s="13" t="inlineStr">
         <is>
           <t>SCD2 Deduplication</t>
         </is>
       </c>
-      <c r="D60" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E60" s="6" t="inlineStr">
+      <c r="D65" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E65" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_security_characteristics_codes</t>
         </is>
       </c>
-      <c r="F60" s="7" t="inlineStr">
+      <c r="F65" s="11" t="inlineStr">
         <is>
           <t>Verify Active Deduplication on Business Key ['security_type_code'] (is_current = 1)</t>
         </is>
       </c>
-      <c r="G60" s="7" t="inlineStr">
+      <c r="G65" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_security_characteristics_codes populated</t>
         </is>
       </c>
-      <c r="H60" s="7" t="inlineStr">
+      <c r="H65" s="11" t="inlineStr">
         <is>
           <t>Zero duplicate active security type codes per security_type_code.</t>
         </is>
       </c>
-      <c r="I60" s="18" t="inlineStr">
+      <c r="I65" s="17" t="inlineStr">
         <is>
           <t>SELECT security_type_code, COUNT(*) AS ActiveDuplicateCount
 FROM Gold_Warehouse.innotrust.dim_security_characteristics_codes
@@ -4102,48 +4516,48 @@
         </is>
       </c>
     </row>
-    <row r="61" ht="54" customHeight="1">
-      <c r="A61" s="12" t="inlineStr">
+    <row r="66" ht="54" customHeight="1">
+      <c r="A66" s="8" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B61" s="12" t="inlineStr">
+      <c r="B66" s="8" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_10</t>
         </is>
       </c>
-      <c r="C61" s="13" t="inlineStr">
+      <c r="C66" s="9" t="inlineStr">
         <is>
           <t>SK Uniqueness</t>
         </is>
       </c>
-      <c r="D61" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E61" s="10" t="inlineStr">
+      <c r="D66" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E66" s="6" t="inlineStr">
         <is>
           <t>innotrust.dim_security_characteristics_codes</t>
         </is>
       </c>
-      <c r="F61" s="11" t="inlineStr">
+      <c r="F66" s="7" t="inlineStr">
         <is>
           <t>Verify Primary Surrogate Key (dim_securitycharacteristicscodes) uniqueness and non-null constraint</t>
         </is>
       </c>
-      <c r="G61" s="11" t="inlineStr">
+      <c r="G66" s="7" t="inlineStr">
         <is>
           <t>innotrust.dim_security_characteristics_codes populated</t>
         </is>
       </c>
-      <c r="H61" s="11" t="inlineStr">
+      <c r="H66" s="7" t="inlineStr">
         <is>
           <t>dim_securitycharacteristicscodes is strictly unique across all versions with zero NULLs.</t>
         </is>
       </c>
-      <c r="I61" s="17" t="inlineStr">
+      <c r="I66" s="18" t="inlineStr">
         <is>
           <t>SELECT dim_securitycharacteristicscodes, COUNT(*) AS DuplicateCount
 FROM Gold_Warehouse.innotrust.dim_security_characteristics_codes
@@ -4152,48 +4566,48 @@
         </is>
       </c>
     </row>
-    <row r="62" ht="54" customHeight="1">
-      <c r="A62" s="8" t="inlineStr">
+    <row r="67" ht="54" customHeight="1">
+      <c r="A67" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B62" s="8" t="inlineStr">
+      <c r="B67" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_11</t>
         </is>
       </c>
-      <c r="C62" s="9" t="inlineStr">
+      <c r="C67" s="13" t="inlineStr">
         <is>
           <t>Audit &amp; Date Logic</t>
         </is>
       </c>
-      <c r="D62" s="19" t="inlineStr">
+      <c r="D67" s="19" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E62" s="6" t="inlineStr">
+      <c r="E67" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master</t>
         </is>
       </c>
-      <c r="F62" s="7" t="inlineStr">
+      <c r="F67" s="11" t="inlineStr">
         <is>
           <t>Verify business_date, updated_at, effective_start_date &amp; effective_end_date integrity on active records</t>
         </is>
       </c>
-      <c r="G62" s="7" t="inlineStr">
+      <c r="G67" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master populated</t>
         </is>
       </c>
-      <c r="H62" s="7" t="inlineStr">
+      <c r="H67" s="11" t="inlineStr">
         <is>
           <t>Zero NULLs in business_date or updated_at; effective_end_date &gt;= effective_start_date.</t>
         </is>
       </c>
-      <c r="I62" s="18" t="inlineStr">
+      <c r="I67" s="17" t="inlineStr">
         <is>
           <t>SELECT 
     COUNT(*) AS TotalActiveRows,
@@ -4206,48 +4620,48 @@
         </is>
       </c>
     </row>
-    <row r="63" ht="54" customHeight="1">
-      <c r="A63" s="12" t="inlineStr">
+    <row r="68" ht="54" customHeight="1">
+      <c r="A68" s="8" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B63" s="12" t="inlineStr">
+      <c r="B68" s="8" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_12</t>
         </is>
       </c>
-      <c r="C63" s="13" t="inlineStr">
+      <c r="C68" s="9" t="inlineStr">
         <is>
           <t>Cross-Table Linkage</t>
         </is>
       </c>
-      <c r="D63" s="19" t="inlineStr">
+      <c r="D68" s="19" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E63" s="10" t="inlineStr">
+      <c r="E68" s="6" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master</t>
         </is>
       </c>
-      <c r="F63" s="11" t="inlineStr">
+      <c r="F68" s="7" t="inlineStr">
         <is>
           <t>Verify Referential Integrity: account_category_code and account_type_code resolve to active codes</t>
         </is>
       </c>
-      <c r="G63" s="11" t="inlineStr">
+      <c r="G68" s="7" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master populated</t>
         </is>
       </c>
-      <c r="H63" s="11" t="inlineStr">
+      <c r="H68" s="7" t="inlineStr">
         <is>
           <t>All non-null account_category_code and account_type_code exist in corresponding dimension code tables.</t>
         </is>
       </c>
-      <c r="I63" s="17" t="inlineStr">
+      <c r="I68" s="18" t="inlineStr">
         <is>
           <t>SELECT 
     SUM(CASE WHEN m.account_category_code IS NOT NULL AND cat.account_category_code IS NULL THEN 1 ELSE 0 END) AS Orphan_CategoryCodes,
@@ -4261,48 +4675,48 @@
         </is>
       </c>
     </row>
-    <row r="64" ht="54" customHeight="1">
-      <c r="A64" s="8" t="inlineStr">
+    <row r="69" ht="54" customHeight="1">
+      <c r="A69" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B64" s="8" t="inlineStr">
+      <c r="B69" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_13</t>
         </is>
       </c>
-      <c r="C64" s="9" t="inlineStr">
+      <c r="C69" s="13" t="inlineStr">
         <is>
           <t>Cross-Table Linkage</t>
         </is>
       </c>
-      <c r="D64" s="19" t="inlineStr">
+      <c r="D69" s="19" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E64" s="6" t="inlineStr">
+      <c r="E69" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_master_sec_index</t>
         </is>
       </c>
-      <c r="F64" s="7" t="inlineStr">
+      <c r="F69" s="11" t="inlineStr">
         <is>
           <t>Verify Security Referential Integrity: security_type_code resolves to active security characteristics</t>
         </is>
       </c>
-      <c r="G64" s="7" t="inlineStr">
+      <c r="G69" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_master_sec_index populated</t>
         </is>
       </c>
-      <c r="H64" s="7" t="inlineStr">
+      <c r="H69" s="11" t="inlineStr">
         <is>
           <t>All non-null security_type_code values exist in dim_security_characteristics_codes.</t>
         </is>
       </c>
-      <c r="I64" s="18" t="inlineStr">
+      <c r="I69" s="17" t="inlineStr">
         <is>
           <t>SELECT COUNT(*) AS Orphan_SecurityTypeCodes
 FROM Gold_Warehouse.innotrust.dim_master_sec_index s
@@ -4312,48 +4726,48 @@
         </is>
       </c>
     </row>
-    <row r="65" ht="54" customHeight="1">
-      <c r="A65" s="12" t="inlineStr">
+    <row r="70" ht="54" customHeight="1">
+      <c r="A70" s="8" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B65" s="12" t="inlineStr">
+      <c r="B70" s="8" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_14</t>
         </is>
       </c>
-      <c r="C65" s="13" t="inlineStr">
+      <c r="C70" s="9" t="inlineStr">
         <is>
           <t>SCD2 Date Validation</t>
         </is>
       </c>
-      <c r="D65" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E65" s="10" t="inlineStr">
+      <c r="D70" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E70" s="6" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master</t>
         </is>
       </c>
-      <c r="F65" s="11" t="inlineStr">
+      <c r="F70" s="7" t="inlineStr">
         <is>
           <t>Verify SCD2 Effective Date Rules: Inactive records effective_end_date &lt;= (Current Day - 1), non-null end date, and valid active start date</t>
         </is>
       </c>
-      <c r="G65" s="11" t="inlineStr">
+      <c r="G70" s="7" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master populated with SCD2 tracking columns</t>
         </is>
       </c>
-      <c r="H65" s="11" t="inlineStr">
+      <c r="H70" s="7" t="inlineStr">
         <is>
           <t>Inactive_End_Date_Breach_Count = 0, Inactive_Missing_End_Date = 0, Active_Future_Start_Date = 0, Inverted_Date_Range_Count = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I65" s="17" t="inlineStr">
+      <c r="I70" s="18" t="inlineStr">
         <is>
           <t>SELECT 
     'dim_account_master' AS TableName,
@@ -4372,48 +4786,48 @@
         </is>
       </c>
     </row>
-    <row r="66" ht="54" customHeight="1">
-      <c r="A66" s="8" t="inlineStr">
+    <row r="71" ht="54" customHeight="1">
+      <c r="A71" s="12" t="inlineStr">
         <is>
           <t>Black Diamond (Consolidated)</t>
         </is>
       </c>
-      <c r="B66" s="8" t="inlineStr">
+      <c r="B71" s="12" t="inlineStr">
         <is>
           <t>TC_COMB_SK_BD_01</t>
         </is>
       </c>
-      <c r="C66" s="9" t="inlineStr">
+      <c r="C71" s="13" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D66" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E66" s="6" t="inlineStr">
+      <c r="D71" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E71" s="10" t="inlineStr">
         <is>
           <t>All 9 Child &amp; Fact Tables (holdings, transactions, taxlots, class/segment, details, tags, team, targets)</t>
         </is>
       </c>
-      <c r="F66" s="7" t="inlineStr">
+      <c r="F71" s="11" t="inlineStr">
         <is>
           <t>Black Diamond: Cross-Object account_sk vs dim_accounts Natural Key (accountid == da.id) Verification - Executes a single consolidated UNION ALL query across all 9 child/fact tables to verify that the attached account_sk strictly points to the exact same account natural key (child.accountid == da.id). Guarantees zero wrong account links.</t>
         </is>
       </c>
-      <c r="G66" s="7" t="inlineStr">
+      <c r="G71" s="11" t="inlineStr">
         <is>
           <t>All Gold tables populated for Black Diamond</t>
         </is>
       </c>
-      <c r="H66" s="7" t="inlineStr">
+      <c r="H71" s="11" t="inlineStr">
         <is>
           <t>Duplicate_BusinessKey_Count = 0, MismatchedAccountIdCount = 0, Null_AccountSK_Count = 0, Orphan_AccountSK_Count = 0 across all 9 objects.</t>
         </is>
       </c>
-      <c r="I66" s="18" t="inlineStr">
+      <c r="I71" s="17" t="inlineStr">
         <is>
           <t>SELECT 
     'dim_accounts_classallocation' AS TableName, 
@@ -4522,48 +4936,48 @@
         </is>
       </c>
     </row>
-    <row r="67" ht="54" customHeight="1">
-      <c r="A67" s="12" t="inlineStr">
+    <row r="72" ht="54" customHeight="1">
+      <c r="A72" s="8" t="inlineStr">
         <is>
           <t>Schwab (Consolidated)</t>
         </is>
       </c>
-      <c r="B67" s="12" t="inlineStr">
+      <c r="B72" s="8" t="inlineStr">
         <is>
           <t>TC_COMB_SK_SC_02</t>
         </is>
       </c>
-      <c r="C67" s="13" t="inlineStr">
+      <c r="C72" s="9" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D67" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E67" s="10" t="inlineStr">
+      <c r="D72" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E72" s="6" t="inlineStr">
         <is>
           <t>All 8 Objects (dim_accounts &amp; 7 Fact Tables: recon_d1/d2, daily_closing, security, transactions, ult/uln lots)</t>
         </is>
       </c>
-      <c r="F67" s="11" t="inlineStr">
+      <c r="F72" s="7" t="inlineStr">
         <is>
           <t>Schwab: Consolidated Multi-Object SK Mapping, PK Deduplication &amp; Audit Date Health Check - Single unified query executing across all 8 Schwab Gold tables. Validates that every fact record's account_sk correctly matches dim_accounts on composite natural keys (account_id, custodian_id), confirms primary SK uniqueness, and ensures 100% audit dates populated.</t>
         </is>
       </c>
-      <c r="G67" s="11" t="inlineStr">
+      <c r="G72" s="7" t="inlineStr">
         <is>
           <t>All Gold tables populated for Schwab</t>
         </is>
       </c>
-      <c r="H67" s="11" t="inlineStr">
+      <c r="H72" s="7" t="inlineStr">
         <is>
           <t>Mismatched_AccountId_Count = 0 and Orphan_AccountSK_Count = 0 across all fact tables. All mapped account_sk strictly match the natural account_id.</t>
         </is>
       </c>
-      <c r="I67" s="17" t="inlineStr">
+      <c r="I72" s="18" t="inlineStr">
         <is>
           <t>SELECT 
     'fact_recon_position_d1' AS TableName,
@@ -4622,48 +5036,48 @@
         </is>
       </c>
     </row>
-    <row r="68" ht="54" customHeight="1">
-      <c r="A68" s="8" t="inlineStr">
+    <row r="73" ht="54" customHeight="1">
+      <c r="A73" s="12" t="inlineStr">
         <is>
           <t>Salentica CRM (Consolidated)</t>
         </is>
       </c>
-      <c r="B68" s="8" t="inlineStr">
+      <c r="B73" s="12" t="inlineStr">
         <is>
           <t>TC_COMB_SK_SAL_03</t>
         </is>
       </c>
-      <c r="C68" s="9" t="inlineStr">
+      <c r="C73" s="13" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D68" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E68" s="6" t="inlineStr">
+      <c r="D73" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E73" s="10" t="inlineStr">
         <is>
           <t>All 6 Core CRM Entities (dim_account, dim_contact_core, dim_family, fact_lead, fact_opportunity, fact_investmentaccount)</t>
         </is>
       </c>
-      <c r="F68" s="7" t="inlineStr">
+      <c r="F73" s="11" t="inlineStr">
         <is>
           <t>Salentica: Consolidated Point-in-Time Referential SK Mapping (Active &amp; Historical Mapping Validation) - Single unified query executing across all 6 core Salentica CRM tables. Validates that every attached foreign SK resolves to the same Natural Key in parent dimensions (allowing active OR expired parent versions to preserve point-in-time audit history) and checks for broken orphans.</t>
         </is>
       </c>
-      <c r="G68" s="7" t="inlineStr">
+      <c r="G73" s="11" t="inlineStr">
         <is>
           <t>All Gold tables populated for Salentica CRM</t>
         </is>
       </c>
-      <c r="H68" s="7" t="inlineStr">
+      <c r="H73" s="11" t="inlineStr">
         <is>
           <t>Mismatched_PrimaryContact_NK = 0, Mismatched_BusinessUnit_NK = 0, Broken_Orphan_Count = 0 across all 6 CRM tables.</t>
         </is>
       </c>
-      <c r="I68" s="18" t="inlineStr">
+      <c r="I73" s="17" t="inlineStr">
         <is>
           <t>SELECT 'dim_account' AS TableName, COUNT(*) AS TotalActiveRows,
     SUM(CASE WHEN a.primarycontactid IS NOT NULL AND a.primarycontactid_sk &lt;&gt; -1 AND a.primarycontactid &lt;&gt; c.contactid THEN 1 ELSE 0 END) AS Mismatched_PrimaryContact_NK,
@@ -4727,48 +5141,48 @@
         </is>
       </c>
     </row>
-    <row r="69" ht="54" customHeight="1">
-      <c r="A69" s="12" t="inlineStr">
+    <row r="74" ht="54" customHeight="1">
+      <c r="A74" s="8" t="inlineStr">
         <is>
           <t>Tamarac (Consolidated)</t>
         </is>
       </c>
-      <c r="B69" s="12" t="inlineStr">
+      <c r="B74" s="8" t="inlineStr">
         <is>
           <t>TC_COMB_SK_TAM_04</t>
         </is>
       </c>
-      <c r="C69" s="13" t="inlineStr">
+      <c r="C74" s="9" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D69" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E69" s="10" t="inlineStr">
+      <c r="D74" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E74" s="6" t="inlineStr">
         <is>
           <t>Both Tables (dim_account_information, dim_account_model_allocation)</t>
         </is>
       </c>
-      <c r="F69" s="11" t="inlineStr">
+      <c r="F74" s="7" t="inlineStr">
         <is>
           <t>Tamarac: Consolidated Multi-Object PK Deduplication, Primary SK &amp; Cross-Table Linkage - Single unified query validating SCD2 active uniqueness on exact PK columns (['account_number'] and ['account_number', 'model_name']), surrogate key uniqueness, and cross-table referential integrity between model allocations and accounts.</t>
         </is>
       </c>
-      <c r="G69" s="11" t="inlineStr">
+      <c r="G74" s="7" t="inlineStr">
         <is>
           <t>All Gold tables populated for Tamarac</t>
         </is>
       </c>
-      <c r="H69" s="11" t="inlineStr">
+      <c r="H74" s="7" t="inlineStr">
         <is>
           <t>PK_Active_Duplicates = 0, Duplicate_Primary_SK = 0, Orphan_Accounts = 0, Missing_BusinessDate = 0 across both tables.</t>
         </is>
       </c>
-      <c r="I69" s="17" t="inlineStr">
+      <c r="I74" s="18" t="inlineStr">
         <is>
           <t>SELECT 'dim_account_information' AS TableName, COUNT(*) AS TotalActiveRows,
     (SELECT COUNT(*) FROM (SELECT account_number FROM Gold_Warehouse.tamarac.dim_account_information WHERE is_current = 'True' GROUP BY account_number HAVING COUNT(*) &gt; 1) d) AS PK_Active_Duplicates,
@@ -4791,48 +5205,48 @@
         </is>
       </c>
     </row>
-    <row r="70" ht="54" customHeight="1">
-      <c r="A70" s="8" t="inlineStr">
+    <row r="75" ht="54" customHeight="1">
+      <c r="A75" s="12" t="inlineStr">
         <is>
           <t>Innotrust (Consolidated)</t>
         </is>
       </c>
-      <c r="B70" s="8" t="inlineStr">
+      <c r="B75" s="12" t="inlineStr">
         <is>
           <t>TC_COMB_SK_INNO_05</t>
         </is>
       </c>
-      <c r="C70" s="9" t="inlineStr">
+      <c r="C75" s="13" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D70" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E70" s="6" t="inlineStr">
+      <c r="D75" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E75" s="10" t="inlineStr">
         <is>
           <t>All 5 Innotrust Dimensions (dim_account_master, category_codes, type_codes, sec_index, characteristics)</t>
         </is>
       </c>
-      <c r="F70" s="7" t="inlineStr">
+      <c r="F75" s="11" t="inlineStr">
         <is>
           <t>Innotrust: Consolidated Multi-Object PK Deduplication, Primary SK &amp; Cross-Dimension Linkage - Single unified query validating SCD2 active uniqueness on exact natural keys, primary surrogate key uniqueness, and cross-dimension referential integrity between master entities and classification codes.</t>
         </is>
       </c>
-      <c r="G70" s="7" t="inlineStr">
+      <c r="G75" s="11" t="inlineStr">
         <is>
           <t>All Gold tables populated for Innotrust</t>
         </is>
       </c>
-      <c r="H70" s="7" t="inlineStr">
+      <c r="H75" s="11" t="inlineStr">
         <is>
           <t>PK_Active_Duplicates = 0, Duplicate_Primary_SK = 0, Orphan_Foreign_References = 0, Missing_BusinessDate = 0 across all 5 Innotrust tables.</t>
         </is>
       </c>
-      <c r="I70" s="18" t="inlineStr">
+      <c r="I75" s="17" t="inlineStr">
         <is>
           <t>SELECT 'dim_account_master' AS TableName, COUNT(*) AS TotalActiveRows,
     (SELECT COUNT(*) FROM (SELECT customer_account_number FROM Gold_Warehouse.innotrust.dim_account_master WHERE is_current = 1 GROUP BY customer_account_number HAVING COUNT(*) &gt; 1) d) AS PK_Active_Duplicates,
@@ -4882,48 +5296,48 @@
         </is>
       </c>
     </row>
-    <row r="71" ht="54" customHeight="1">
-      <c r="A71" s="12" t="inlineStr">
+    <row r="76" ht="54" customHeight="1">
+      <c r="A76" s="8" t="inlineStr">
         <is>
           <t>Innotrust (Consolidated)</t>
         </is>
       </c>
-      <c r="B71" s="12" t="inlineStr">
+      <c r="B76" s="8" t="inlineStr">
         <is>
           <t>TC_COMB_SK_INNO_06</t>
         </is>
       </c>
-      <c r="C71" s="13" t="inlineStr">
+      <c r="C76" s="9" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D71" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E71" s="10" t="inlineStr">
+      <c r="D76" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E76" s="6" t="inlineStr">
         <is>
           <t>All 5 Innotrust Dimensions (dim_account_master, category_codes, type_codes, sec_index, characteristics)</t>
         </is>
       </c>
-      <c r="F71" s="11" t="inlineStr">
+      <c r="F76" s="7" t="inlineStr">
         <is>
           <t>Innotrust: Consolidated Multi-Object SCD2 Effective Start &amp; End Date Audit (End Date &lt;= Today - 1) - Validates across all 5 Innotrust dimensions that inactive records (is_current = 0) have effective_end_date &lt;= (current day - 1), non-null end dates, active records have non-future start dates, and zero inverted date ranges.</t>
         </is>
       </c>
-      <c r="G71" s="11" t="inlineStr">
+      <c r="G76" s="7" t="inlineStr">
         <is>
           <t>All Gold tables populated for Innotrust</t>
         </is>
       </c>
-      <c r="H71" s="11" t="inlineStr">
+      <c r="H76" s="7" t="inlineStr">
         <is>
           <t>Inactive_End_Date_Breach_Count = 0, Inactive_Missing_End_Date = 0, Active_Future_Start_Date = 0, Inverted_Date_Range_Count = 0 across all 5 tables.</t>
         </is>
       </c>
-      <c r="I71" s="17" t="inlineStr">
+      <c r="I76" s="18" t="inlineStr">
         <is>
           <t>SELECT 
     'dim_account_master' AS TableName,
@@ -5940,7 +6354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6378,6 +6792,395 @@
     SUM(CASE WHEN f.account_sk IS NOT NULL AND da.account_sk IS NULL THEN 1 ELSE 0 END) AS Orphan_AccountSK_Count
 FROM Gold_Warehouse.schwab.fact_uln_lot_daily_non_taxable f
 LEFT JOIN Gold_Warehouse.schwab.dim_accounts da ON f.account_sk = da.account_sk;</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="54" customHeight="1">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>TC_SC_GOLD_09</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>SCD2 Inactive Date Rules</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>schwab.dim_accounts</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>Verify SCD2 Inactive Date Rule: Inactive records (IsCurrent = 0) must have EffectiveTo &lt;= file_business_date - 1 (or next EffectiveFrom - 1)</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>dim_accounts populated with SCD2 tracking columns</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>Zero active records marked expired prematurely, zero inactive records with open/invalid EffectiveTo. DefectCount = 0.</t>
+        </is>
+      </c>
+      <c r="H11" s="17" t="inlineStr">
+        <is>
+          <t>SELECT 
+    account_id,
+    account_sk,
+    file_business_date,
+    EffectiveFrom,
+    EffectiveTo,
+    IsCurrent,
+    Audit_Update_Date
+FROM Gold_Warehouse.schwab.dim_accounts
+WHERE IsCurrent = 0 
+  AND (EffectiveTo IS NULL OR EffectiveTo &gt; file_business_date)
+ORDER BY account_id, EffectiveFrom;</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="54" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>TC_SC_GOLD_10</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Date Sanity &amp; Inversions</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>schwab.dim_accounts</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Verify Date Sanity: Zero inverted dates (EffectiveTo &lt; EffectiveFrom) and active records have non-future start dates</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>dim_accounts populated</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>Inverted_Date_Count = 0, Future_Active_Start_Date = 0, Null_Start_Date_Count = 0. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>SELECT 
+    'schwab.dim_accounts' AS TableName,
+    COUNT(*) AS TotalRecords,
+    SUM(CASE WHEN EffectiveTo &lt; EffectiveFrom THEN 1 ELSE 0 END) AS Inverted_Date_Count,
+    SUM(CASE WHEN IsCurrent = 1 AND EffectiveFrom &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END) AS Future_Active_Start_Date,
+    SUM(CASE WHEN EffectiveFrom IS NULL THEN 1 ELSE 0 END) AS Null_Start_Date_Count,
+    CASE 
+        WHEN SUM(CASE WHEN EffectiveTo &lt; EffectiveFrom THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN IsCurrent = 1 AND EffectiveFrom &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN EffectiveFrom IS NULL THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END AS TestStatus
+FROM Gold_Warehouse.schwab.dim_accounts;</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="54" customHeight="1">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>TC_SC_GOLD_11</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Open-Ended Active Records</t>
+        </is>
+      </c>
+      <c r="C13" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>schwab.dim_accounts</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>Verify Active Records are Open-Ended (EffectiveTo is NULL or '9999-12-31')</t>
+        </is>
+      </c>
+      <c r="F13" s="11" t="inlineStr">
+        <is>
+          <t>dim_accounts where IsCurrent = 1</t>
+        </is>
+      </c>
+      <c r="G13" s="11" t="inlineStr">
+        <is>
+          <t>Prematurely_Ended_Active_Records = 0. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="H13" s="17" t="inlineStr">
+        <is>
+          <t>SELECT 
+    'schwab.dim_accounts' AS TableName,
+    COUNT(*) AS TotalActiveRecords,
+    SUM(CASE WHEN EffectiveTo IS NOT NULL AND EffectiveTo NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END) AS Prematurely_Ended_Active_Records,
+    CASE 
+        WHEN SUM(CASE WHEN EffectiveTo IS NOT NULL AND EffectiveTo NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END) = 0 
+        THEN 'PASSED' ELSE 'FAILED'
+    END AS TestStatus
+FROM Gold_Warehouse.schwab.dim_accounts
+WHERE IsCurrent = 1;</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="54" customHeight="1">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>TC_SC_GOLD_12</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Version Evolution Audit</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>schwab.dim_accounts</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Verify SCD2 Version Evolution: Monotonic SK increments, advancing EffectiveFrom, continuous timeline (EffectiveTo = next EffectiveFrom - 1), and latest version active</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>dim_accounts with multiple version rows per account_id</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>Reused_Or_NonIncrementing_SK_Count = 0, NonAdvancing_EffectiveFrom_Count = 0, Timeline_Gap_Or_Overlap_Count = 0, LatestVersion_Not_Active_Count = 0. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>WITH SchwabEvolution AS (
+    SELECT 
+        account_id,
+        account_sk,
+        EffectiveFrom,
+        EffectiveTo,
+        IsCurrent,
+        file_business_date,
+        Audit_Update_Date,
+        LEAD(account_sk) OVER (PARTITION BY account_id ORDER BY EffectiveFrom, account_sk) AS next_sk,
+        LEAD(EffectiveFrom) OVER (PARTITION BY account_id ORDER BY EffectiveFrom, account_sk) AS next_start_date,
+        ROW_NUMBER() OVER (PARTITION BY account_id ORDER BY EffectiveFrom DESC, account_sk DESC) AS rn_latest
+    FROM Gold_Warehouse.schwab.dim_accounts
+)
+SELECT 
+    'schwab.dim_accounts' AS TableName,
+    'Version Evolution &amp; Progression' AS TestName,
+    COUNT(*) AS TotalVersionsAudited,
+    SUM(CASE WHEN next_sk IS NOT NULL AND next_sk &lt;= account_sk THEN 1 ELSE 0 END) AS Reused_Or_NonIncrementing_SK_Count,
+    SUM(CASE WHEN next_start_date IS NOT NULL AND next_start_date &lt;= EffectiveFrom THEN 1 ELSE 0 END) AS NonAdvancing_EffectiveFrom_Count,
+    SUM(CASE WHEN next_start_date IS NOT NULL AND EffectiveTo &lt;&gt; DATEADD(day, -1, next_start_date) THEN 1 ELSE 0 END) AS Timeline_Gap_Or_Overlap_Count,
+    SUM(CASE WHEN rn_latest = 1 AND IsCurrent &lt;&gt; 1 THEN 1 ELSE 0 END) AS LatestVersion_Not_Active_Count,
+    CASE 
+        WHEN SUM(CASE WHEN next_sk IS NOT NULL AND next_sk &lt;= account_sk THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN next_start_date IS NOT NULL AND next_start_date &lt;= EffectiveFrom THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN next_start_date IS NOT NULL AND EffectiveTo &lt;&gt; DATEADD(day, -1, next_start_date) THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN rn_latest = 1 AND IsCurrent &lt;&gt; 1 THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END AS TestStatus
+FROM SchwabEvolution;</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="54" customHeight="1">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>TC_SC_GOLD_13</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>Fact Health &amp; Historical Retention</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>schwab.fact_recon_position_d1, fact_recon_position_d2, fact_daily_closing_lots, fact_transactions, fact_ult_lot_daily_taxable, fact_uln_lot_daily_non_taxable</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>Verify Fact Tables Health: Active SK mapping for fresh runs, historical closed version preservation for unrepeated rows, exact natural account match, and orphan SK detection</t>
+        </is>
+      </c>
+      <c r="F15" s="11" t="inlineStr">
+        <is>
+          <t>All 6 Schwab Fact tables loaded into Gold Warehouse</t>
+        </is>
+      </c>
+      <c r="G15" s="11" t="inlineStr">
+        <is>
+          <t>Fresh records map to active SK (IsCurrent = 1), past records retain historical SK, Exact_Account_Match_Count covers all non-orphan rows, Defect_Orphan_Unmapped_SK = 0, Defect_Wrong_Account_Mismatch = 0. OverallStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="H15" s="17" t="inlineStr">
+        <is>
+          <t>WITH MaxRuns AS (
+    SELECT 'fact_recon_position_d1' AS TableName, MAX(updated_at) AS LatestRunTimestamp FROM Gold_Warehouse.schwab.fact_recon_position_d1 UNION ALL
+    SELECT 'fact_recon_position_d2', MAX(updated_at) FROM Gold_Warehouse.schwab.fact_recon_position_d2 UNION ALL
+    SELECT 'fact_daily_closing_lots', MAX(updated_at) FROM Gold_Warehouse.schwab.fact_daily_closing_lots UNION ALL
+    SELECT 'fact_transactions', MAX(updated_at) FROM Gold_Warehouse.schwab.fact_transactions UNION ALL
+    SELECT 'fact_ult_lot_daily_taxable', MAX(updated_at) FROM Gold_Warehouse.schwab.fact_ult_lot_daily_taxable UNION ALL
+    SELECT 'fact_uln_lot_daily_non_taxable', MAX(updated_at) FROM Gold_Warehouse.schwab.fact_uln_lot_daily_non_taxable
+),
+FactBreakdown AS (
+    SELECT 
+        'fact_recon_position_d1' AS TableName,
+        COUNT(*) AS TotalFactRows,
+        MAX(f.file_business_date) AS LatestBatchDate,
+        SUM(CASE WHEN f.updated_at = m.LatestRunTimestamp AND da.IsCurrent = 1 AND f.account_id = da.account_id THEN 1 ELSE 0 END) AS Fresh_Run_Active_Mapped,
+        SUM(CASE WHEN f.updated_at &lt; m.LatestRunTimestamp AND da.IsCurrent = 1 AND f.account_id = da.account_id THEN 1 ELSE 0 END) AS Past_Run_Active_Retained,
+        SUM(CASE WHEN f.updated_at &lt; m.LatestRunTimestamp AND da.IsCurrent = 0 AND f.account_id = da.account_id THEN 1 ELSE 0 END) AS Past_Run_Expired_Version_Retained,
+        SUM(CASE WHEN da.account_sk IS NOT NULL AND f.account_id = da.account_id THEN 1 ELSE 0 END) AS Exact_Account_Match_Count,
+        SUM(CASE WHEN f.account_sk = -1 OR da.account_sk IS NULL THEN 1 ELSE 0 END) AS Defect_Orphan_Unmapped_SK,
+        SUM(CASE WHEN da.account_sk IS NOT NULL AND f.account_id &lt;&gt; da.account_id THEN 1 ELSE 0 END) AS Defect_Wrong_Account_Mismatch
+    FROM Gold_Warehouse.schwab.fact_recon_position_d1 f
+    JOIN MaxRuns m ON m.TableName = 'fact_recon_position_d1'
+    LEFT JOIN Gold_Warehouse.schwab.dim_accounts da ON f.account_sk = da.account_sk
+    GROUP BY m.LatestRunTimestamp
+    UNION ALL
+    SELECT 
+        'fact_recon_position_d2',
+        COUNT(*),
+        MAX(f.file_business_date),
+        SUM(CASE WHEN f.updated_at = m.LatestRunTimestamp AND da.IsCurrent = 1 AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.updated_at &lt; m.LatestRunTimestamp AND da.IsCurrent = 1 AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.updated_at &lt; m.LatestRunTimestamp AND da.IsCurrent = 0 AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.account_sk IS NOT NULL AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.account_sk = -1 OR da.account_sk IS NULL THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.account_sk IS NOT NULL AND f.account_id &lt;&gt; da.account_id THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.schwab.fact_recon_position_d2 f
+    JOIN MaxRuns m ON m.TableName = 'fact_recon_position_d2'
+    LEFT JOIN Gold_Warehouse.schwab.dim_accounts da ON f.account_sk = da.account_sk
+    GROUP BY m.LatestRunTimestamp
+    UNION ALL
+    SELECT 
+        'fact_daily_closing_lots',
+        COUNT(*),
+        MAX(f.file_business_date),
+        SUM(CASE WHEN f.updated_at = m.LatestRunTimestamp AND da.IsCurrent = 1 AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.updated_at &lt; m.LatestRunTimestamp AND da.IsCurrent = 1 AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.updated_at &lt; m.LatestRunTimestamp AND da.IsCurrent = 0 AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.account_sk IS NOT NULL AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.account_sk = -1 OR da.account_sk IS NULL THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.account_sk IS NOT NULL AND f.account_id &lt;&gt; da.account_id THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.schwab.fact_daily_closing_lots f
+    JOIN MaxRuns m ON m.TableName = 'fact_daily_closing_lots'
+    LEFT JOIN Gold_Warehouse.schwab.dim_accounts da ON f.account_sk = da.account_sk
+    GROUP BY m.LatestRunTimestamp
+    UNION ALL
+    SELECT 
+        'fact_transactions',
+        COUNT(*),
+        MAX(f.file_business_date),
+        SUM(CASE WHEN f.updated_at = m.LatestRunTimestamp AND da.IsCurrent = 1 AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.updated_at &lt; m.LatestRunTimestamp AND da.IsCurrent = 1 AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.updated_at &lt; m.LatestRunTimestamp AND da.IsCurrent = 0 AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.account_sk IS NOT NULL AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.account_sk = -1 OR da.account_sk IS NULL THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.account_sk IS NOT NULL AND f.account_id &lt;&gt; da.account_id THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.schwab.fact_transactions f
+    JOIN MaxRuns m ON m.TableName = 'fact_transactions'
+    LEFT JOIN Gold_Warehouse.schwab.dim_accounts da ON f.account_sk = da.account_sk
+    GROUP BY m.LatestRunTimestamp
+    UNION ALL
+    SELECT 
+        'fact_ult_lot_daily_taxable',
+        COUNT(*),
+        MAX(f.file_business_date),
+        SUM(CASE WHEN f.updated_at = m.LatestRunTimestamp AND da.IsCurrent = 1 AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.updated_at &lt; m.LatestRunTimestamp AND da.IsCurrent = 1 AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.updated_at &lt; m.LatestRunTimestamp AND da.IsCurrent = 0 AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.account_sk IS NOT NULL AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.account_sk = -1 OR da.account_sk IS NULL THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.account_sk IS NOT NULL AND f.account_id &lt;&gt; da.account_id THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.schwab.fact_ult_lot_daily_taxable f
+    JOIN MaxRuns m ON m.TableName = 'fact_ult_lot_daily_taxable'
+    LEFT JOIN Gold_Warehouse.schwab.dim_accounts da ON f.account_sk = da.account_sk
+    GROUP BY m.LatestRunTimestamp
+    UNION ALL
+    SELECT 
+        'fact_uln_lot_daily_non_taxable',
+        COUNT(*),
+        MAX(f.file_business_date),
+        SUM(CASE WHEN f.updated_at = m.LatestRunTimestamp AND da.IsCurrent = 1 AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.updated_at &lt; m.LatestRunTimestamp AND da.IsCurrent = 1 AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.updated_at &lt; m.LatestRunTimestamp AND da.IsCurrent = 0 AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.account_sk IS NOT NULL AND f.account_id = da.account_id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.account_sk = -1 OR da.account_sk IS NULL THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.account_sk IS NOT NULL AND f.account_id &lt;&gt; da.account_id THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.schwab.fact_uln_lot_daily_non_taxable f
+    JOIN MaxRuns m ON m.TableName = 'fact_uln_lot_daily_non_taxable'
+    LEFT JOIN Gold_Warehouse.schwab.dim_accounts da ON f.account_sk = da.account_sk
+    GROUP BY m.LatestRunTimestamp
+)
+SELECT 
+    TableName,
+    TotalFactRows,
+    LatestBatchDate,
+    Fresh_Run_Active_Mapped,
+    Past_Run_Active_Retained,
+    Past_Run_Expired_Version_Retained AS Historical_Closed_Version_Retained,
+    Exact_Account_Match_Count,
+    Defect_Orphan_Unmapped_SK,
+    Defect_Wrong_Account_Mismatch,
+    CASE 
+        WHEN Defect_Orphan_Unmapped_SK = 0 AND Defect_Wrong_Account_Mismatch = 0 THEN 'PASSED'
+        ELSE 'FAILED'
+    END AS OverallStatus,
+    CASE 
+        WHEN Defect_Orphan_Unmapped_SK &gt; 0 THEN CONCAT(Defect_Orphan_Unmapped_SK, ' Orphan Record(s) (SK = -1)')
+        WHEN Defect_Wrong_Account_Mismatch &gt; 0 THEN 'Account Mismatch Defect'
+        ELSE 'All Active &amp; Historical Records Correctly Preserved'
+    END AS Remarks
+FROM FactBreakdown;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(schwab): enforce EffectiveTo <= Latest_Batch_Date - 1 and full SCD2 timeline rules in TC_SC_GOLD_09
</commit_message>
<xml_diff>
--- a/Gold_Data_Validation_Test_Cases.xlsx
+++ b/Gold_Data_Validation_Test_Cases.xlsx
@@ -2351,7 +2351,7 @@
       </c>
       <c r="F29" s="11" t="inlineStr">
         <is>
-          <t>Verify SCD2 Inactive Date Rule: Inactive records (IsCurrent = 0) must have EffectiveTo &lt;= file_business_date - 1 (or next EffectiveFrom - 1)</t>
+          <t>Verify SCD2 Timeline &amp; Date Rules: Inactive records (IsCurrent = 0) must have EffectiveTo &lt;= Latest_Batch_Date - 1, Active records must be open-ended, zero inverted dates</t>
         </is>
       </c>
       <c r="G29" s="11" t="inlineStr">
@@ -2361,23 +2361,38 @@
       </c>
       <c r="H29" s="11" t="inlineStr">
         <is>
-          <t>Zero active records marked expired prematurely, zero inactive records with open/invalid EffectiveTo. DefectCount = 0.</t>
+          <t>Defect_Inactive_EndDate_Not_Preceding_Batch = 0, Defect_Active_Prematurely_Closed = 0, Defect_Inverted_Dates = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
       <c r="I29" s="17" t="inlineStr">
         <is>
-          <t>SELECT 
-    account_id,
-    account_sk,
-    file_business_date,
-    EffectiveFrom,
-    EffectiveTo,
-    IsCurrent,
-    Audit_Update_Date
+          <t>;WITH LatestBatch AS (
+    SELECT MAX(file_business_date) AS LatestBatchDate FROM Gold_Warehouse.schwab.dim_accounts
+)
+SELECT 
+    'schwab.dim_accounts' AS TableName,
+    COUNT(*) AS TotalRecords,
+    b.LatestBatchDate,
+    SUM(CASE WHEN IsCurrent = 1 THEN 1 ELSE 0 END) AS Active_Records_Count,
+    SUM(CASE WHEN IsCurrent = 0 THEN 1 ELSE 0 END) AS Inactive_Records_Count,
+    -- Rule: Inactive records must have EffectiveTo &lt;= LatestBatchDate - 1
+    SUM(CASE WHEN IsCurrent = 0 AND (EffectiveTo IS NULL OR EffectiveTo &gt; DATEADD(day, -1, b.LatestBatchDate)) THEN 1 ELSE 0 END) AS Defect_Inactive_EndDate_Not_Preceding_Batch,
+    -- Rule: Active records must be open-ended (NULL or 9999-12-31)
+    SUM(CASE WHEN IsCurrent = 1 AND EffectiveTo IS NOT NULL AND EffectiveTo NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END) AS Defect_Active_Prematurely_Closed,
+    -- Rule: Start date cannot be after End date
+    SUM(CASE WHEN EffectiveTo &lt; EffectiveFrom THEN 1 ELSE 0 END) AS Defect_Inverted_Dates,
+    -- Rule: Active Start date cannot be in future
+    SUM(CASE WHEN IsCurrent = 1 AND EffectiveFrom &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END) AS Defect_Future_Active_Start_Date,
+    CASE 
+        WHEN SUM(CASE WHEN IsCurrent = 0 AND (EffectiveTo IS NULL OR EffectiveTo &gt; DATEADD(day, -1, b.LatestBatchDate)) THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN IsCurrent = 1 AND EffectiveTo IS NOT NULL AND EffectiveTo NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN EffectiveTo &lt; EffectiveFrom THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN IsCurrent = 1 AND EffectiveFrom &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END AS TestStatus
 FROM Gold_Warehouse.schwab.dim_accounts
-WHERE IsCurrent = 0 
-  AND (EffectiveTo IS NULL OR EffectiveTo &gt; file_business_date)
-ORDER BY account_id, EffectiveFrom;</t>
+CROSS JOIN LatestBatch b
+GROUP BY b.LatestBatchDate;</t>
         </is>
       </c>
     </row>
@@ -6818,7 +6833,7 @@
       </c>
       <c r="E11" s="11" t="inlineStr">
         <is>
-          <t>Verify SCD2 Inactive Date Rule: Inactive records (IsCurrent = 0) must have EffectiveTo &lt;= file_business_date - 1 (or next EffectiveFrom - 1)</t>
+          <t>Verify SCD2 Timeline &amp; Date Rules: Inactive records (IsCurrent = 0) must have EffectiveTo &lt;= Latest_Batch_Date - 1, Active records must be open-ended, zero inverted dates</t>
         </is>
       </c>
       <c r="F11" s="11" t="inlineStr">
@@ -6828,23 +6843,38 @@
       </c>
       <c r="G11" s="11" t="inlineStr">
         <is>
-          <t>Zero active records marked expired prematurely, zero inactive records with open/invalid EffectiveTo. DefectCount = 0.</t>
+          <t>Defect_Inactive_EndDate_Not_Preceding_Batch = 0, Defect_Active_Prematurely_Closed = 0, Defect_Inverted_Dates = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
       <c r="H11" s="17" t="inlineStr">
         <is>
-          <t>SELECT 
-    account_id,
-    account_sk,
-    file_business_date,
-    EffectiveFrom,
-    EffectiveTo,
-    IsCurrent,
-    Audit_Update_Date
+          <t>;WITH LatestBatch AS (
+    SELECT MAX(file_business_date) AS LatestBatchDate FROM Gold_Warehouse.schwab.dim_accounts
+)
+SELECT 
+    'schwab.dim_accounts' AS TableName,
+    COUNT(*) AS TotalRecords,
+    b.LatestBatchDate,
+    SUM(CASE WHEN IsCurrent = 1 THEN 1 ELSE 0 END) AS Active_Records_Count,
+    SUM(CASE WHEN IsCurrent = 0 THEN 1 ELSE 0 END) AS Inactive_Records_Count,
+    -- Rule: Inactive records must have EffectiveTo &lt;= LatestBatchDate - 1
+    SUM(CASE WHEN IsCurrent = 0 AND (EffectiveTo IS NULL OR EffectiveTo &gt; DATEADD(day, -1, b.LatestBatchDate)) THEN 1 ELSE 0 END) AS Defect_Inactive_EndDate_Not_Preceding_Batch,
+    -- Rule: Active records must be open-ended (NULL or 9999-12-31)
+    SUM(CASE WHEN IsCurrent = 1 AND EffectiveTo IS NOT NULL AND EffectiveTo NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END) AS Defect_Active_Prematurely_Closed,
+    -- Rule: Start date cannot be after End date
+    SUM(CASE WHEN EffectiveTo &lt; EffectiveFrom THEN 1 ELSE 0 END) AS Defect_Inverted_Dates,
+    -- Rule: Active Start date cannot be in future
+    SUM(CASE WHEN IsCurrent = 1 AND EffectiveFrom &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END) AS Defect_Future_Active_Start_Date,
+    CASE 
+        WHEN SUM(CASE WHEN IsCurrent = 0 AND (EffectiveTo IS NULL OR EffectiveTo &gt; DATEADD(day, -1, b.LatestBatchDate)) THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN IsCurrent = 1 AND EffectiveTo IS NOT NULL AND EffectiveTo NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN EffectiveTo &lt; EffectiveFrom THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN IsCurrent = 1 AND EffectiveFrom &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END AS TestStatus
 FROM Gold_Warehouse.schwab.dim_accounts
-WHERE IsCurrent = 0 
-  AND (EffectiveTo IS NULL OR EffectiveTo &gt; file_business_date)
-ORDER BY account_id, EffectiveFrom;</t>
+CROSS JOIN LatestBatch b
+GROUP BY b.LatestBatchDate;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(black_diamond): add consolidated SCD2 date rules (TC_BD_GOLD_19), evolution audit (TC_BD_GOLD_20), account_sk audit (TC_BD_GOLD_21) and fact retention (TC_BD_GOLD_22)
</commit_message>
<xml_diff>
--- a/Gold_Data_Validation_Test_Cases.xlsx
+++ b/Gold_Data_Validation_Test_Cases.xlsx
@@ -644,10 +644,10 @@
         <v>5</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F5" s="4" t="n">
         <v>17</v>
@@ -705,10 +705,10 @@
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="D8" s="9" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E8" s="9" t="n">
         <v>6</v>
@@ -860,10 +860,10 @@
         </is>
       </c>
       <c r="C13" s="15" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D13" s="15" t="n">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="E13" s="15" t="n">
         <v>17</v>
@@ -898,7 +898,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I76"/>
+  <dimension ref="A1:I80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1907,45 +1907,501 @@
     <row r="21" ht="54" customHeight="1">
       <c r="A21" s="12" t="inlineStr">
         <is>
+          <t>Black Diamond</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>TC_BD_GOLD_19</t>
+        </is>
+      </c>
+      <c r="C21" s="13" t="inlineStr">
+        <is>
+          <t>SCD2 Inactive Date Rules</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E21" s="10" t="inlineStr">
+        <is>
+          <t>black_diamond.dim_accounts (and ALL 13 Dim Tables)</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>Verify SCD2 Timeline &amp; Date Rules across ALL 13 Dim Tables: Inactive records (iscurrent = 'False') must have effectiveenddate &lt;= Latest_Batch_Date - 1, Active records must be open-ended, zero inverted dates</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="inlineStr">
+        <is>
+          <t>All 13 Black Diamond dimension tables loaded with SCD2 tracking columns</t>
+        </is>
+      </c>
+      <c r="H21" s="11" t="inlineStr">
+        <is>
+          <t>Defect_Inactive_EndDate_Not_DayMinus1 = 0, Defect_Active_Prematurely_Closed = 0, Defect_Inverted_Dates = 0, Defect_Future_Active_StartDate = 0 across all 13 tables. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="I21" s="17" t="inlineStr">
+        <is>
+          <t>;WITH DimSCD2Audit AS (
+    SELECT 'dim_accounts' AS TableName, COUNT(*) AS TotalRecords, MAX(file_business_date) AS LatestBatchDate,
+        SUM(CASE WHEN iscurrent = 'True' THEN 1 ELSE 0 END) AS Active_Count,
+        SUM(CASE WHEN iscurrent = 'False' THEN 1 ELSE 0 END) AS Inactive_Count,
+        SUM(CASE WHEN iscurrent = 'False' AND (effectiveenddate IS NULL OR effectiveenddate &gt; DATEADD(day, -1, b.MaxBatchDate)) THEN 1 ELSE 0 END) AS Defect_Inactive_EndDate_Not_DayMinus1,
+        SUM(CASE WHEN iscurrent = 'True' AND effectiveenddate IS NOT NULL AND effectiveenddate NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END) AS Defect_Active_Prematurely_Closed,
+        SUM(CASE WHEN effectiveenddate &lt; effectivestartdate THEN 1 ELSE 0 END) AS Defect_Inverted_Dates,
+        SUM(CASE WHEN iscurrent = 'True' AND effectivestartdate &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END) AS Defect_Future_Active_StartDate
+    FROM Gold_Warehouse.black_diamond.dim_accounts
+    CROSS JOIN (SELECT MAX(file_business_date) AS MaxBatchDate FROM Gold_Warehouse.black_diamond.dim_accounts) b
+    GROUP BY b.MaxBatchDate
+    UNION ALL
+    SELECT 'dim_asset', COUNT(*), MAX(file_business_date),
+        SUM(CASE WHEN iscurrent = 'True' THEN 1 ELSE 0 END), SUM(CASE WHEN iscurrent = 'False' THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'False' AND (effectiveenddate IS NULL OR effectiveenddate &gt; DATEADD(day, -1, b.MaxBatchDate)) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectiveenddate IS NOT NULL AND effectiveenddate NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END),
+        SUM(CASE WHEN effectiveenddate &lt; effectivestartdate THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectivestartdate &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.dim_asset
+    CROSS JOIN (SELECT MAX(file_business_date) AS MaxBatchDate FROM Gold_Warehouse.black_diamond.dim_asset) b GROUP BY b.MaxBatchDate
+    UNION ALL
+    SELECT 'dim_client', COUNT(*), MAX(file_business_date),
+        SUM(CASE WHEN iscurrent = 'True' THEN 1 ELSE 0 END), SUM(CASE WHEN iscurrent = 'False' THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'False' AND (effectiveenddate IS NULL OR effectiveenddate &gt; DATEADD(day, -1, b.MaxBatchDate)) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectiveenddate IS NOT NULL AND effectiveenddate NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END),
+        SUM(CASE WHEN effectiveenddate &lt; effectivestartdate THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectivestartdate &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.dim_client
+    CROSS JOIN (SELECT MAX(file_business_date) AS MaxBatchDate FROM Gold_Warehouse.black_diamond.dim_client) b GROUP BY b.MaxBatchDate
+    UNION ALL
+    SELECT 'dim_contact', COUNT(*), MAX(file_business_date),
+        SUM(CASE WHEN iscurrent = 'True' THEN 1 ELSE 0 END), SUM(CASE WHEN iscurrent = 'False' THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'False' AND (effectiveenddate IS NULL OR effectiveenddate &gt; DATEADD(day, -1, b.MaxBatchDate)) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectiveenddate IS NOT NULL AND effectiveenddate NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END),
+        SUM(CASE WHEN effectiveenddate &lt; effectivestartdate THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectivestartdate &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.dim_contact
+    CROSS JOIN (SELECT MAX(file_business_date) AS MaxBatchDate FROM Gold_Warehouse.black_diamond.dim_contact) b GROUP BY b.MaxBatchDate
+    UNION ALL
+    SELECT 'dim_portfoliogroup', COUNT(*), MAX(file_business_date),
+        SUM(CASE WHEN iscurrent = 'True' THEN 1 ELSE 0 END), SUM(CASE WHEN iscurrent = 'False' THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'False' AND (effectiveenddate IS NULL OR effectiveenddate &gt; DATEADD(day, -1, b.MaxBatchDate)) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectiveenddate IS NOT NULL AND effectiveenddate NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END),
+        SUM(CASE WHEN effectiveenddate &lt; effectivestartdate THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectivestartdate &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.dim_portfoliogroup
+    CROSS JOIN (SELECT MAX(file_business_date) AS MaxBatchDate FROM Gold_Warehouse.black_diamond.dim_portfoliogroup) b GROUP BY b.MaxBatchDate
+    UNION ALL
+    SELECT 'dim_relationshipv2', COUNT(*), MAX(file_business_date),
+        SUM(CASE WHEN iscurrent = 'True' THEN 1 ELSE 0 END), SUM(CASE WHEN iscurrent = 'False' THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'False' AND (effectiveenddate IS NULL OR effectiveenddate &gt; DATEADD(day, -1, b.MaxBatchDate)) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectiveenddate IS NOT NULL AND effectiveenddate NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END),
+        SUM(CASE WHEN effectiveenddate &lt; effectivestartdate THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectivestartdate &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.dim_relationshipv2
+    CROSS JOIN (SELECT MAX(file_business_date) AS MaxBatchDate FROM Gold_Warehouse.black_diamond.dim_relationshipv2) b GROUP BY b.MaxBatchDate
+    UNION ALL
+    SELECT 'dim_target', COUNT(*), MAX(file_business_date),
+        SUM(CASE WHEN iscurrent = 'True' THEN 1 ELSE 0 END), SUM(CASE WHEN iscurrent = 'False' THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'False' AND (effectiveenddate IS NULL OR effectiveenddate &gt; DATEADD(day, -1, b.MaxBatchDate)) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectiveenddate IS NOT NULL AND effectiveenddate NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END),
+        SUM(CASE WHEN effectiveenddate &lt; effectivestartdate THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectivestartdate &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.dim_target
+    CROSS JOIN (SELECT MAX(file_business_date) AS MaxBatchDate FROM Gold_Warehouse.black_diamond.dim_target) b GROUP BY b.MaxBatchDate
+    UNION ALL
+    SELECT 'dim_accounts_classallocation', COUNT(*), MAX(file_business_date),
+        SUM(CASE WHEN iscurrent = 'True' THEN 1 ELSE 0 END), SUM(CASE WHEN iscurrent = 'False' THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'False' AND (effectiveenddate IS NULL OR effectiveenddate &gt; DATEADD(day, -1, b.MaxBatchDate)) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectiveenddate IS NOT NULL AND effectiveenddate NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END),
+        SUM(CASE WHEN effectiveenddate &lt; effectivestartdate THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectivestartdate &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.dim_accounts_classallocation
+    CROSS JOIN (SELECT MAX(file_business_date) AS MaxBatchDate FROM Gold_Warehouse.black_diamond.dim_accounts_classallocation) b GROUP BY b.MaxBatchDate
+    UNION ALL
+    SELECT 'dim_accounts_details', COUNT(*), MAX(file_business_date),
+        SUM(CASE WHEN iscurrent = 'True' THEN 1 ELSE 0 END), SUM(CASE WHEN iscurrent = 'False' THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'False' AND (effectiveenddate IS NULL OR effectiveenddate &gt; DATEADD(day, -1, b.MaxBatchDate)) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectiveenddate IS NOT NULL AND effectiveenddate NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END),
+        SUM(CASE WHEN effectiveenddate &lt; effectivestartdate THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectivestartdate &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.dim_accounts_details
+    CROSS JOIN (SELECT MAX(file_business_date) AS MaxBatchDate FROM Gold_Warehouse.black_diamond.dim_accounts_details) b GROUP BY b.MaxBatchDate
+    UNION ALL
+    SELECT 'dim_accounts_segmentallocation', COUNT(*), MAX(file_business_date),
+        SUM(CASE WHEN iscurrent = 'True' THEN 1 ELSE 0 END), SUM(CASE WHEN iscurrent = 'False' THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'False' AND (effectiveenddate IS NULL OR effectiveenddate &gt; DATEADD(day, -1, b.MaxBatchDate)) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectiveenddate IS NOT NULL AND effectiveenddate NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END),
+        SUM(CASE WHEN effectiveenddate &lt; effectivestartdate THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectivestartdate &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.dim_accounts_segmentallocation
+    CROSS JOIN (SELECT MAX(file_business_date) AS MaxBatchDate FROM Gold_Warehouse.black_diamond.dim_accounts_segmentallocation) b GROUP BY b.MaxBatchDate
+    UNION ALL
+    SELECT 'dim_accounts_tags', COUNT(*), MAX(file_business_date),
+        SUM(CASE WHEN iscurrent = 'True' THEN 1 ELSE 0 END), SUM(CASE WHEN iscurrent = 'False' THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'False' AND (effectiveenddate IS NULL OR effectiveenddate &gt; DATEADD(day, -1, b.MaxBatchDate)) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectiveenddate IS NOT NULL AND effectiveenddate NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END),
+        SUM(CASE WHEN effectiveenddate &lt; effectivestartdate THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectivestartdate &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.dim_accounts_tags
+    CROSS JOIN (SELECT MAX(file_business_date) AS MaxBatchDate FROM Gold_Warehouse.black_diamond.dim_accounts_tags) b GROUP BY b.MaxBatchDate
+    UNION ALL
+    SELECT 'dim_accounts_targets', COUNT(*), MAX(file_business_date),
+        SUM(CASE WHEN iscurrent = 'True' THEN 1 ELSE 0 END), SUM(CASE WHEN iscurrent = 'False' THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'False' AND (effectiveenddate IS NULL OR effectiveenddate &gt; DATEADD(day, -1, b.MaxBatchDate)) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectiveenddate IS NOT NULL AND effectiveenddate NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END),
+        SUM(CASE WHEN effectiveenddate &lt; effectivestartdate THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectivestartdate &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.dim_accounts_targets
+    CROSS JOIN (SELECT MAX(file_business_date) AS MaxBatchDate FROM Gold_Warehouse.black_diamond.dim_accounts_targets) b GROUP BY b.MaxBatchDate
+    UNION ALL
+    SELECT 'dim_accounts_team', COUNT(*), MAX(file_business_date),
+        SUM(CASE WHEN iscurrent = 'True' THEN 1 ELSE 0 END), SUM(CASE WHEN iscurrent = 'False' THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'False' AND (effectiveenddate IS NULL OR effectiveenddate &gt; DATEADD(day, -1, b.MaxBatchDate)) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectiveenddate IS NOT NULL AND effectiveenddate NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END),
+        SUM(CASE WHEN effectiveenddate &lt; effectivestartdate THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectivestartdate &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.dim_accounts_team
+    CROSS JOIN (SELECT MAX(file_business_date) AS MaxBatchDate FROM Gold_Warehouse.black_diamond.dim_accounts_team) b GROUP BY b.MaxBatchDate
+)
+SELECT 
+    TableName, TotalRecords, LatestBatchDate, Active_Count, Inactive_Count,
+    Defect_Inactive_EndDate_Not_DayMinus1, Defect_Active_Prematurely_Closed, Defect_Inverted_Dates, Defect_Future_Active_StartDate,
+    CASE 
+        WHEN Defect_Inactive_EndDate_Not_DayMinus1 = 0 AND Defect_Active_Prematurely_Closed = 0 AND Defect_Inverted_Dates = 0 AND Defect_Future_Active_StartDate = 0 THEN 'PASSED'
+        ELSE 'FAILED'
+    END AS TestStatus
+FROM DimSCD2Audit;</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="54" customHeight="1">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Black Diamond</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>TC_BD_GOLD_20</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Version Evolution Audit</t>
+        </is>
+      </c>
+      <c r="D22" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>black_diamond.dim_accounts</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>Verify SCD2 Version Evolution: Monotonic accounts_SK increments, advancing effectivestartdate, continuous timeline (effectiveenddate = next effectivestartdate - 1), and latest version active</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>dim_accounts with multiple version rows per id</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>Reused_Or_NonIncrementing_SK_Count = 0, NonAdvancing_EffectiveStartDate_Count = 0, Timeline_Gap_Or_Overlap_Count = 0, LatestVersion_Not_Active_Count = 0. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="I22" s="18" t="inlineStr">
+        <is>
+          <t>;WITH VersionChains AS (
+    SELECT 
+        id, accounts_SK, effectivestartdate, effectiveenddate, iscurrent, file_business_date, updatedat,
+        LEAD(accounts_SK) OVER (PARTITION BY id ORDER BY effectivestartdate, accounts_SK) AS next_sk,
+        LEAD(effectivestartdate) OVER (PARTITION BY id ORDER BY effectivestartdate, accounts_SK) AS next_start_date,
+        ROW_NUMBER() OVER (PARTITION BY id ORDER BY effectivestartdate DESC, accounts_SK DESC) AS rn_latest
+    FROM Gold_Warehouse.black_diamond.dim_accounts
+)
+SELECT 
+    'black_diamond.dim_accounts' AS TableName,
+    'Version Evolution &amp; Progression' AS TestName,
+    COUNT(*) AS TotalVersionsAudited,
+    SUM(CASE WHEN next_sk IS NOT NULL AND next_sk &lt;= accounts_SK THEN 1 ELSE 0 END) AS Reused_Or_NonIncrementing_SK_Count,
+    SUM(CASE WHEN next_start_date IS NOT NULL AND next_start_date &lt;= effectivestartdate THEN 1 ELSE 0 END) AS NonAdvancing_EffectiveStartDate_Count,
+    SUM(CASE WHEN next_start_date IS NOT NULL AND effectiveenddate &lt;&gt; DATEADD(day, -1, next_start_date) THEN 1 ELSE 0 END) AS Timeline_Gap_Or_Overlap_Count,
+    SUM(CASE WHEN rn_latest = 1 AND iscurrent &lt;&gt; 'True' THEN 1 ELSE 0 END) AS LatestVersion_Not_Active_Count,
+    CASE 
+        WHEN SUM(CASE WHEN next_sk IS NOT NULL AND next_sk &lt;= accounts_SK THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN next_start_date IS NOT NULL AND next_start_date &lt;= effectivestartdate THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN next_start_date IS NOT NULL AND effectiveenddate &lt;&gt; DATEADD(day, -1, next_start_date) THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN rn_latest = 1 AND iscurrent &lt;&gt; 'True' THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END AS TestStatus
+FROM VersionChains;</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="54" customHeight="1">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>Black Diamond</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>TC_BD_GOLD_21</t>
+        </is>
+      </c>
+      <c r="C23" s="13" t="inlineStr">
+        <is>
+          <t>Foreign SK Referential Mapping</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E23" s="10" t="inlineStr">
+        <is>
+          <t>black_diamond (ALL 6 Child Dims + 3 Fact Tables)</t>
+        </is>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>Verify Consolidated account_sk Mapping: Audits that all 6 Child Dimensions and 3 Fact Tables have their attached account_sk strictly mapped to the exact matching id in dim_accounts</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="inlineStr">
+        <is>
+          <t>dim_accounts_classallocation, details, segmentallocation, tags, targets, team, holdings, transactions, taxlots populated</t>
+        </is>
+      </c>
+      <c r="H23" s="11" t="inlineStr">
+        <is>
+          <t>Defect_Orphan_Unmapped_SK = 0 and Defect_Wrong_Account_Mismatch = 0 across all 9 tables. Exact_Account_Match_Count covers 100% of rows. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="I23" s="17" t="inlineStr">
+        <is>
+          <t>;WITH AccountSKAudit AS (
+    SELECT 'dim_accounts_classallocation' AS TableName, 'Child Dimension' AS ObjectType, COUNT(*) AS TotalRecords,
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND c.accountid = da.id THEN 1 ELSE 0 END) AS Exact_Account_Match_Count,
+        SUM(CASE WHEN c.account_sk = -1 OR c.account_sk IS NULL OR da.accounts_SK IS NULL THEN 1 ELSE 0 END) AS Defect_Orphan_Unmapped_SK,
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND c.accountid &lt;&gt; da.id THEN 1 ELSE 0 END) AS Defect_Wrong_Account_Mismatch
+    FROM Gold_Warehouse.black_diamond.dim_accounts_classallocation c
+    LEFT JOIN Gold_Warehouse.black_diamond.dim_accounts da ON c.account_sk = da.accounts_SK
+    UNION ALL
+    SELECT 'dim_accounts_details', 'Child Dimension', COUNT(*),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND d.accountid = da.id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN d.account_sk = -1 OR d.account_sk IS NULL OR da.accounts_SK IS NULL THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND d.accountid &lt;&gt; da.id THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.dim_accounts_details d
+    LEFT JOIN Gold_Warehouse.black_diamond.dim_accounts da ON d.account_sk = da.accounts_SK
+    UNION ALL
+    SELECT 'dim_accounts_segmentallocation', 'Child Dimension', COUNT(*),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND s.accountid = da.id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN s.account_sk = -1 OR s.account_sk IS NULL OR da.accounts_SK IS NULL THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND s.accountid &lt;&gt; da.id THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.dim_accounts_segmentallocation s
+    LEFT JOIN Gold_Warehouse.black_diamond.dim_accounts da ON s.account_sk = da.accounts_SK
+    UNION ALL
+    SELECT 'dim_accounts_tags', 'Child Dimension', COUNT(*),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND t.accountid = da.id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN t.account_sk = -1 OR t.account_sk IS NULL OR da.accounts_SK IS NULL THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND t.accountid &lt;&gt; da.id THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.dim_accounts_tags t
+    LEFT JOIN Gold_Warehouse.black_diamond.dim_accounts da ON t.account_sk = da.accounts_SK
+    UNION ALL
+    SELECT 'dim_accounts_targets', 'Child Dimension', COUNT(*),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND tg.accountid = da.id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN tg.account_sk = -1 OR tg.account_sk IS NULL OR da.accounts_SK IS NULL THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND tg.accountid &lt;&gt; da.id THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.dim_accounts_targets tg
+    LEFT JOIN Gold_Warehouse.black_diamond.dim_accounts da ON tg.account_sk = da.accounts_SK
+    UNION ALL
+    SELECT 'dim_accounts_team', 'Child Dimension', COUNT(*),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND tm.accountid = da.id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN tm.account_sk = -1 OR tm.account_sk IS NULL OR da.accounts_SK IS NULL THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND tm.accountid &lt;&gt; da.id THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.dim_accounts_team tm
+    LEFT JOIN Gold_Warehouse.black_diamond.dim_accounts da ON tm.account_sk = da.accounts_SK
+    UNION ALL
+    SELECT 'fact_accounts_holdings', 'Fact Table', COUNT(*),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND h.accountid = da.id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN h.account_sk = -1 OR h.account_sk IS NULL OR da.accounts_SK IS NULL THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND h.accountid &lt;&gt; da.id THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.fact_accounts_holdings h
+    LEFT JOIN Gold_Warehouse.black_diamond.dim_accounts da ON h.account_sk = da.accounts_SK
+    UNION ALL
+    SELECT 'fact_accounts_transactions', 'Fact Table', COUNT(*),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND tx.accountid = da.id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN tx.account_sk = -1 OR tx.account_sk IS NULL OR da.accounts_SK IS NULL THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND tx.accountid &lt;&gt; da.id THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.fact_accounts_transactions tx
+    LEFT JOIN Gold_Warehouse.black_diamond.dim_accounts da ON tx.account_sk = da.accounts_SK
+    UNION ALL
+    SELECT 'fact_accounts_taxlots', 'Fact Table', COUNT(*),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND tl.accountid = da.id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN tl.account_sk = -1 OR tl.account_sk IS NULL OR da.accounts_SK IS NULL THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND tl.accountid &lt;&gt; da.id THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.fact_accounts_taxlots tl
+    LEFT JOIN Gold_Warehouse.black_diamond.dim_accounts da ON tl.account_sk = da.accounts_SK
+)
+SELECT TableName, ObjectType, TotalRecords, Exact_Account_Match_Count, Defect_Orphan_Unmapped_SK, Defect_Wrong_Account_Mismatch,
+    CASE WHEN Defect_Orphan_Unmapped_SK = 0 AND Defect_Wrong_Account_Mismatch = 0 THEN 'PASSED' ELSE 'FAILED' END AS TestStatus
+FROM AccountSKAudit;</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="54" customHeight="1">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Black Diamond</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>TC_BD_GOLD_22</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Fact Health &amp; Historical Retention</t>
+        </is>
+      </c>
+      <c r="D24" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>black_diamond.fact_accounts_holdings, fact_accounts_transactions, fact_accounts_taxlots</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>Verify Fact Tables Health: Active SK mapping for fresh runs, historical closed version preservation for unrepeated rows, exact natural account match, and orphan SK detection</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>All 3 Black Diamond Fact tables loaded into Gold Warehouse</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>Fresh records map to active SK (iscurrent = 'True'), past records retain historical SK, Exact_Account_Match_Count covers all non-orphan rows, Defect_Orphan_Unmapped_SK = 0, Defect_Wrong_Account_Mismatch = 0. OverallStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="I24" s="18" t="inlineStr">
+        <is>
+          <t>;WITH MaxRuns AS (
+    SELECT 'fact_accounts_holdings' AS TableName, MAX(updatedat) AS LatestRunTimestamp FROM Gold_Warehouse.black_diamond.fact_accounts_holdings UNION ALL
+    SELECT 'fact_accounts_transactions', MAX(updatedat) FROM Gold_Warehouse.black_diamond.fact_accounts_transactions UNION ALL
+    SELECT 'fact_accounts_taxlots', MAX(updatedat) FROM Gold_Warehouse.black_diamond.fact_accounts_taxlots
+),
+FactBreakdown AS (
+    SELECT 'fact_accounts_holdings' AS TableName, COUNT(*) AS TotalFactRows, MAX(f.file_business_date) AS LatestBatchDate,
+        SUM(CASE WHEN f.updatedat = m.LatestRunTimestamp AND da.iscurrent = 'True' AND f.accountid = da.id THEN 1 ELSE 0 END) AS Fresh_Run_Active_Mapped,
+        SUM(CASE WHEN f.updatedat &lt; m.LatestRunTimestamp AND da.iscurrent = 'True' AND f.accountid = da.id THEN 1 ELSE 0 END) AS Past_Run_Active_Retained,
+        SUM(CASE WHEN f.updatedat &lt; m.LatestRunTimestamp AND da.iscurrent = 'False' AND f.accountid = da.id THEN 1 ELSE 0 END) AS Past_Run_Expired_Version_Retained,
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND f.accountid = da.id THEN 1 ELSE 0 END) AS Exact_Account_Match_Count,
+        SUM(CASE WHEN f.account_sk = -1 OR da.accounts_SK IS NULL THEN 1 ELSE 0 END) AS Defect_Orphan_Unmapped_SK,
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND f.accountid &lt;&gt; da.id THEN 1 ELSE 0 END) AS Defect_Wrong_Account_Mismatch
+    FROM Gold_Warehouse.black_diamond.fact_accounts_holdings f
+    JOIN MaxRuns m ON m.TableName = 'fact_accounts_holdings'
+    LEFT JOIN Gold_Warehouse.black_diamond.dim_accounts da ON f.account_sk = da.accounts_SK
+    GROUP BY m.LatestRunTimestamp
+    UNION ALL
+    SELECT 'fact_accounts_transactions', COUNT(*), MAX(f.file_business_date),
+        SUM(CASE WHEN f.updatedat = m.LatestRunTimestamp AND da.iscurrent = 'True' AND f.accountid = da.id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.updatedat &lt; m.LatestRunTimestamp AND da.iscurrent = 'True' AND f.accountid = da.id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.updatedat &lt; m.LatestRunTimestamp AND da.iscurrent = 'False' AND f.accountid = da.id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND f.accountid = da.id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.account_sk = -1 OR da.accounts_SK IS NULL THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND f.accountid &lt;&gt; da.id THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.fact_accounts_transactions f
+    JOIN MaxRuns m ON m.TableName = 'fact_accounts_transactions'
+    LEFT JOIN Gold_Warehouse.black_diamond.dim_accounts da ON f.account_sk = da.accounts_SK
+    GROUP BY m.LatestRunTimestamp
+    UNION ALL
+    SELECT 'fact_accounts_taxlots', COUNT(*), MAX(f.file_business_date),
+        SUM(CASE WHEN f.updatedat = m.LatestRunTimestamp AND da.iscurrent = 'True' AND f.accountid = da.id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.updatedat &lt; m.LatestRunTimestamp AND da.iscurrent = 'True' AND f.accountid = da.id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.updatedat &lt; m.LatestRunTimestamp AND da.iscurrent = 'False' AND f.accountid = da.id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND f.accountid = da.id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.account_sk = -1 OR da.accounts_SK IS NULL THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND f.accountid &lt;&gt; da.id THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.fact_accounts_taxlots f
+    JOIN MaxRuns m ON m.TableName = 'fact_accounts_taxlots'
+    LEFT JOIN Gold_Warehouse.black_diamond.dim_accounts da ON f.account_sk = da.accounts_SK
+    GROUP BY m.LatestRunTimestamp
+)
+SELECT 
+    TableName, TotalFactRows, LatestBatchDate, Fresh_Run_Active_Mapped, Past_Run_Active_Retained,
+    Past_Run_Expired_Version_Retained AS Historical_Closed_Version_Retained, Exact_Account_Match_Count,
+    Defect_Orphan_Unmapped_SK, Defect_Wrong_Account_Mismatch,
+    CASE WHEN Defect_Orphan_Unmapped_SK = 0 AND Defect_Wrong_Account_Mismatch = 0 THEN 'PASSED' ELSE 'FAILED' END AS OverallStatus,
+    CASE 
+        WHEN Defect_Orphan_Unmapped_SK &gt; 0 THEN CONCAT(Defect_Orphan_Unmapped_SK, ' Orphan Record(s) (SK = -1)')
+        WHEN Defect_Wrong_Account_Mismatch &gt; 0 THEN 'Account Mismatch Defect'
+        ELSE 'All Active &amp; Historical Records Correctly Preserved'
+    END AS Remarks
+FROM FactBreakdown;</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="54" customHeight="1">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
           <t>Schwab</t>
         </is>
       </c>
-      <c r="B21" s="12" t="inlineStr">
+      <c r="B25" s="12" t="inlineStr">
         <is>
           <t>TC_SC_GOLD_01</t>
         </is>
       </c>
-      <c r="C21" s="13" t="inlineStr">
+      <c r="C25" s="13" t="inlineStr">
         <is>
           <t>SCD2 Deduplication</t>
         </is>
       </c>
-      <c r="D21" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E21" s="10" t="inlineStr">
+      <c r="D25" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E25" s="10" t="inlineStr">
         <is>
           <t>schwab.dim_accounts</t>
         </is>
       </c>
-      <c r="F21" s="11" t="inlineStr">
+      <c r="F25" s="11" t="inlineStr">
         <is>
           <t>Verify Active Deduplication on Composite Business Key ['account_id', 'custodian_id']</t>
         </is>
       </c>
-      <c r="G21" s="11" t="inlineStr">
+      <c r="G25" s="11" t="inlineStr">
         <is>
           <t>dim_accounts populated with IsCurrent flag</t>
         </is>
       </c>
-      <c r="H21" s="11" t="inlineStr">
+      <c r="H25" s="11" t="inlineStr">
         <is>
           <t>Zero duplicate active accounts; account_sk strictly unique across all rows.</t>
         </is>
       </c>
-      <c r="I21" s="17" t="inlineStr">
+      <c r="I25" s="17" t="inlineStr">
         <is>
           <t>SELECT account_id, custodian_id, COUNT(*) AS ActiveDuplicateCount
 FROM Gold_Warehouse.schwab.dim_accounts
@@ -1955,48 +2411,48 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="54" customHeight="1">
-      <c r="A22" s="8" t="inlineStr">
+    <row r="26" ht="54" customHeight="1">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>Schwab</t>
         </is>
       </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="B26" s="8" t="inlineStr">
         <is>
           <t>TC_SC_GOLD_02</t>
         </is>
       </c>
-      <c r="C22" s="9" t="inlineStr">
+      <c r="C26" s="9" t="inlineStr">
         <is>
           <t>Business Key &amp; SK Validation</t>
         </is>
       </c>
-      <c r="D22" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="inlineStr">
+      <c r="D26" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
         <is>
           <t>schwab.fact_recon_position_d1</t>
         </is>
       </c>
-      <c r="F22" s="7" t="inlineStr">
+      <c r="F26" s="7" t="inlineStr">
         <is>
           <t>Verify PK ['account_id', 'accounting_rule_code', 'item_issue_id', 'rule_set_suffix_id'] deduplication &amp; account_sk mapping</t>
         </is>
       </c>
-      <c r="G22" s="7" t="inlineStr">
+      <c r="G26" s="7" t="inlineStr">
         <is>
           <t>fact_recon_position_d1 populated</t>
         </is>
       </c>
-      <c r="H22" s="7" t="inlineStr">
+      <c r="H26" s="7" t="inlineStr">
         <is>
           <t>Zero duplicate rows on 4-column business key; attached account_sk strictly maps to the same account_id in dim_accounts.</t>
         </is>
       </c>
-      <c r="I22" s="18" t="inlineStr">
+      <c r="I26" s="18" t="inlineStr">
         <is>
           <t>SELECT 
     (SELECT COUNT(*) FROM (SELECT account_id, accounting_rule_code, item_issue_id, rule_set_suffix_id FROM Gold_Warehouse.schwab.fact_recon_position_d1 GROUP BY account_id, accounting_rule_code, item_issue_id, rule_set_suffix_id HAVING COUNT(*) &gt; 1) d) AS Duplicate_BusinessKey_Count,
@@ -2008,48 +2464,48 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="54" customHeight="1">
-      <c r="A23" s="12" t="inlineStr">
+    <row r="27" ht="54" customHeight="1">
+      <c r="A27" s="12" t="inlineStr">
         <is>
           <t>Schwab</t>
         </is>
       </c>
-      <c r="B23" s="12" t="inlineStr">
+      <c r="B27" s="12" t="inlineStr">
         <is>
           <t>TC_SC_GOLD_03</t>
         </is>
       </c>
-      <c r="C23" s="13" t="inlineStr">
+      <c r="C27" s="13" t="inlineStr">
         <is>
           <t>Business Key &amp; SK Validation</t>
         </is>
       </c>
-      <c r="D23" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E23" s="10" t="inlineStr">
+      <c r="D27" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E27" s="10" t="inlineStr">
         <is>
           <t>schwab.fact_recon_position_d2</t>
         </is>
       </c>
-      <c r="F23" s="11" t="inlineStr">
+      <c r="F27" s="11" t="inlineStr">
         <is>
           <t>Verify PK ['account_id'] deduplication &amp; account_sk referential mapping</t>
         </is>
       </c>
-      <c r="G23" s="11" t="inlineStr">
+      <c r="G27" s="11" t="inlineStr">
         <is>
           <t>fact_recon_position_d2 populated</t>
         </is>
       </c>
-      <c r="H23" s="11" t="inlineStr">
+      <c r="H27" s="11" t="inlineStr">
         <is>
           <t>Zero duplicate rows on account_id business key; attached account_sk strictly maps to dim_accounts.</t>
         </is>
       </c>
-      <c r="I23" s="17" t="inlineStr">
+      <c r="I27" s="17" t="inlineStr">
         <is>
           <t>SELECT 
     (SELECT COUNT(*) FROM (SELECT account_id FROM Gold_Warehouse.schwab.fact_recon_position_d2 GROUP BY account_id HAVING COUNT(*) &gt; 1) d) AS Duplicate_BusinessKey_Count,
@@ -2061,48 +2517,48 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="54" customHeight="1">
-      <c r="A24" s="8" t="inlineStr">
+    <row r="28" ht="54" customHeight="1">
+      <c r="A28" s="8" t="inlineStr">
         <is>
           <t>Schwab</t>
         </is>
       </c>
-      <c r="B24" s="8" t="inlineStr">
+      <c r="B28" s="8" t="inlineStr">
         <is>
           <t>TC_SC_GOLD_04</t>
         </is>
       </c>
-      <c r="C24" s="9" t="inlineStr">
+      <c r="C28" s="9" t="inlineStr">
         <is>
           <t>Business Key &amp; SK Validation</t>
         </is>
       </c>
-      <c r="D24" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E24" s="6" t="inlineStr">
+      <c r="D28" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
         <is>
           <t>schwab.fact_daily_closing_lots</t>
         </is>
       </c>
-      <c r="F24" s="7" t="inlineStr">
+      <c r="F28" s="7" t="inlineStr">
         <is>
           <t>Verify PK ['account_id', 'item_issue_id', 'close_event_id', 'close_open_event_id'] deduplication &amp; account_sk mapping</t>
         </is>
       </c>
-      <c r="G24" s="7" t="inlineStr">
+      <c r="G28" s="7" t="inlineStr">
         <is>
           <t>fact_daily_closing_lots populated</t>
         </is>
       </c>
-      <c r="H24" s="7" t="inlineStr">
+      <c r="H28" s="7" t="inlineStr">
         <is>
           <t>Zero duplicate rows on 4-column business key; account_sk strictly maps to dim_accounts (f.account_id == da.account_id).</t>
         </is>
       </c>
-      <c r="I24" s="18" t="inlineStr">
+      <c r="I28" s="18" t="inlineStr">
         <is>
           <t>SELECT 
     (SELECT COUNT(*) FROM (SELECT account_id, item_issue_id, close_event_id, close_open_event_id FROM Gold_Warehouse.schwab.fact_daily_closing_lots GROUP BY account_id, item_issue_id, close_event_id, close_open_event_id HAVING COUNT(*) &gt; 1) d) AS Duplicate_BusinessKey_Count,
@@ -2114,48 +2570,48 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="54" customHeight="1">
-      <c r="A25" s="12" t="inlineStr">
+    <row r="29" ht="54" customHeight="1">
+      <c r="A29" s="12" t="inlineStr">
         <is>
           <t>Schwab</t>
         </is>
       </c>
-      <c r="B25" s="12" t="inlineStr">
+      <c r="B29" s="12" t="inlineStr">
         <is>
           <t>TC_SC_GOLD_05</t>
         </is>
       </c>
-      <c r="C25" s="13" t="inlineStr">
+      <c r="C29" s="13" t="inlineStr">
         <is>
           <t>Business Key &amp; SK Uniqueness</t>
         </is>
       </c>
-      <c r="D25" s="19" t="inlineStr">
+      <c r="D29" s="19" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E25" s="10" t="inlineStr">
+      <c r="E29" s="10" t="inlineStr">
         <is>
           <t>schwab.fact_security</t>
         </is>
       </c>
-      <c r="F25" s="11" t="inlineStr">
+      <c r="F29" s="11" t="inlineStr">
         <is>
           <t>Verify PK ['schwab_security_number', 'item_issue_id'] deduplication, security_sk uniqueness and audit dates</t>
         </is>
       </c>
-      <c r="G25" s="11" t="inlineStr">
+      <c r="G29" s="11" t="inlineStr">
         <is>
           <t>fact_security populated</t>
         </is>
       </c>
-      <c r="H25" s="11" t="inlineStr">
+      <c r="H29" s="11" t="inlineStr">
         <is>
           <t>Zero duplicates on (schwab_security_number, item_issue_id); security_sk is strictly unique.</t>
         </is>
       </c>
-      <c r="I25" s="17" t="inlineStr">
+      <c r="I29" s="17" t="inlineStr">
         <is>
           <t>SELECT 
     (SELECT COUNT(*) FROM (SELECT schwab_security_number, item_issue_id FROM Gold_Warehouse.schwab.fact_security GROUP BY schwab_security_number, item_issue_id HAVING COUNT(*) &gt; 1) d) AS Duplicate_BusinessKey_Count,
@@ -2164,48 +2620,48 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="54" customHeight="1">
-      <c r="A26" s="8" t="inlineStr">
+    <row r="30" ht="54" customHeight="1">
+      <c r="A30" s="8" t="inlineStr">
         <is>
           <t>Schwab</t>
         </is>
       </c>
-      <c r="B26" s="8" t="inlineStr">
+      <c r="B30" s="8" t="inlineStr">
         <is>
           <t>TC_SC_GOLD_06</t>
         </is>
       </c>
-      <c r="C26" s="9" t="inlineStr">
+      <c r="C30" s="9" t="inlineStr">
         <is>
           <t>Business Key &amp; SK Validation</t>
         </is>
       </c>
-      <c r="D26" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E26" s="6" t="inlineStr">
+      <c r="D30" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
         <is>
           <t>schwab.fact_transactions</t>
         </is>
       </c>
-      <c r="F26" s="7" t="inlineStr">
+      <c r="F30" s="7" t="inlineStr">
         <is>
           <t>Verify PK ['account_id', 'transaction_process_date', 'transaction_cycle_identifier', 'transaction_random_number'] deduplication &amp; account_sk mapping</t>
         </is>
       </c>
-      <c r="G26" s="7" t="inlineStr">
+      <c r="G30" s="7" t="inlineStr">
         <is>
           <t>fact_transactions populated</t>
         </is>
       </c>
-      <c r="H26" s="7" t="inlineStr">
+      <c r="H30" s="7" t="inlineStr">
         <is>
           <t>Zero duplicate rows on 4-column business key; account_sk strictly matches dim_accounts.</t>
         </is>
       </c>
-      <c r="I26" s="18" t="inlineStr">
+      <c r="I30" s="18" t="inlineStr">
         <is>
           <t>SELECT 
     (SELECT COUNT(*) FROM (SELECT account_id, transaction_process_date, transaction_cycle_identifier, transaction_random_number FROM Gold_Warehouse.schwab.fact_transactions GROUP BY account_id, transaction_process_date, transaction_cycle_identifier, transaction_random_number HAVING COUNT(*) &gt; 1) d) AS Duplicate_BusinessKey_Count,
@@ -2217,48 +2673,48 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="54" customHeight="1">
-      <c r="A27" s="12" t="inlineStr">
+    <row r="31" ht="54" customHeight="1">
+      <c r="A31" s="12" t="inlineStr">
         <is>
           <t>Schwab</t>
         </is>
       </c>
-      <c r="B27" s="12" t="inlineStr">
+      <c r="B31" s="12" t="inlineStr">
         <is>
           <t>TC_SC_GOLD_07</t>
         </is>
       </c>
-      <c r="C27" s="13" t="inlineStr">
+      <c r="C31" s="13" t="inlineStr">
         <is>
           <t>Business Key &amp; SK Validation</t>
         </is>
       </c>
-      <c r="D27" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E27" s="10" t="inlineStr">
+      <c r="D31" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E31" s="10" t="inlineStr">
         <is>
           <t>schwab.fact_ult_lot_daily_taxable</t>
         </is>
       </c>
-      <c r="F27" s="11" t="inlineStr">
+      <c r="F31" s="11" t="inlineStr">
         <is>
           <t>Verify PK ['account_id', 'event_id', 'schwab_internal_id', 'item_issue_id', 'isin', 'sedol'] deduplication &amp; account_sk mapping</t>
         </is>
       </c>
-      <c r="G27" s="11" t="inlineStr">
+      <c r="G31" s="11" t="inlineStr">
         <is>
           <t>fact_ult_lot_daily_taxable populated</t>
         </is>
       </c>
-      <c r="H27" s="11" t="inlineStr">
+      <c r="H31" s="11" t="inlineStr">
         <is>
           <t>Zero duplicate rows on 6-column composite PK; account_sk strictly maps to dim_accounts.</t>
         </is>
       </c>
-      <c r="I27" s="17" t="inlineStr">
+      <c r="I31" s="17" t="inlineStr">
         <is>
           <t>SELECT 
     (SELECT COUNT(*) FROM (SELECT account_id, event_id, schwab_internal_id, item_issue_id, isin, sedol FROM Gold_Warehouse.schwab.fact_ult_lot_daily_taxable GROUP BY account_id, event_id, schwab_internal_id, item_issue_id, isin, sedol HAVING COUNT(*) &gt; 1) d) AS Duplicate_BusinessKey_Count,
@@ -2270,48 +2726,48 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="54" customHeight="1">
-      <c r="A28" s="8" t="inlineStr">
+    <row r="32" ht="54" customHeight="1">
+      <c r="A32" s="8" t="inlineStr">
         <is>
           <t>Schwab</t>
         </is>
       </c>
-      <c r="B28" s="8" t="inlineStr">
+      <c r="B32" s="8" t="inlineStr">
         <is>
           <t>TC_SC_GOLD_08</t>
         </is>
       </c>
-      <c r="C28" s="9" t="inlineStr">
+      <c r="C32" s="9" t="inlineStr">
         <is>
           <t>Business Key &amp; SK Validation</t>
         </is>
       </c>
-      <c r="D28" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E28" s="6" t="inlineStr">
+      <c r="D32" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
         <is>
           <t>schwab.fact_uln_lot_daily_non_taxable</t>
         </is>
       </c>
-      <c r="F28" s="7" t="inlineStr">
+      <c r="F32" s="7" t="inlineStr">
         <is>
           <t>Verify PK ['account_id', 'event_id'] deduplication &amp; account_sk referential mapping</t>
         </is>
       </c>
-      <c r="G28" s="7" t="inlineStr">
+      <c r="G32" s="7" t="inlineStr">
         <is>
           <t>fact_uln_lot_daily_non_taxable populated</t>
         </is>
       </c>
-      <c r="H28" s="7" t="inlineStr">
+      <c r="H32" s="7" t="inlineStr">
         <is>
           <t>Zero duplicate rows on (account_id, event_id); account_sk strictly maps to dim_accounts.</t>
         </is>
       </c>
-      <c r="I28" s="18" t="inlineStr">
+      <c r="I32" s="18" t="inlineStr">
         <is>
           <t>SELECT 
     (SELECT COUNT(*) FROM (SELECT account_id, event_id FROM Gold_Warehouse.schwab.fact_uln_lot_daily_non_taxable GROUP BY account_id, event_id HAVING COUNT(*) &gt; 1) d) AS Duplicate_BusinessKey_Count,
@@ -2323,48 +2779,48 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="54" customHeight="1">
-      <c r="A29" s="12" t="inlineStr">
+    <row r="33" ht="54" customHeight="1">
+      <c r="A33" s="12" t="inlineStr">
         <is>
           <t>Schwab</t>
         </is>
       </c>
-      <c r="B29" s="12" t="inlineStr">
+      <c r="B33" s="12" t="inlineStr">
         <is>
           <t>TC_SC_GOLD_09</t>
         </is>
       </c>
-      <c r="C29" s="13" t="inlineStr">
+      <c r="C33" s="13" t="inlineStr">
         <is>
           <t>SCD2 Inactive Date Rules</t>
         </is>
       </c>
-      <c r="D29" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E29" s="10" t="inlineStr">
+      <c r="D33" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E33" s="10" t="inlineStr">
         <is>
           <t>schwab.dim_accounts</t>
         </is>
       </c>
-      <c r="F29" s="11" t="inlineStr">
+      <c r="F33" s="11" t="inlineStr">
         <is>
           <t>Verify SCD2 Timeline &amp; Date Rules: Inactive records (IsCurrent = 0) must have EffectiveTo &lt;= Latest_Batch_Date - 1, Active records must be open-ended, zero inverted dates</t>
         </is>
       </c>
-      <c r="G29" s="11" t="inlineStr">
+      <c r="G33" s="11" t="inlineStr">
         <is>
           <t>dim_accounts populated with SCD2 tracking columns</t>
         </is>
       </c>
-      <c r="H29" s="11" t="inlineStr">
+      <c r="H33" s="11" t="inlineStr">
         <is>
           <t>Defect_Inactive_EndDate_Not_Preceding_Batch = 0, Defect_Active_Prematurely_Closed = 0, Defect_Inverted_Dates = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I29" s="17" t="inlineStr">
+      <c r="I33" s="17" t="inlineStr">
         <is>
           <t>;WITH LatestBatch AS (
     SELECT MAX(file_business_date) AS LatestBatchDate FROM Gold_Warehouse.schwab.dim_accounts
@@ -2396,48 +2852,48 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="54" customHeight="1">
-      <c r="A30" s="8" t="inlineStr">
+    <row r="34" ht="54" customHeight="1">
+      <c r="A34" s="8" t="inlineStr">
         <is>
           <t>Schwab</t>
         </is>
       </c>
-      <c r="B30" s="8" t="inlineStr">
+      <c r="B34" s="8" t="inlineStr">
         <is>
           <t>TC_SC_GOLD_10</t>
         </is>
       </c>
-      <c r="C30" s="9" t="inlineStr">
+      <c r="C34" s="9" t="inlineStr">
         <is>
           <t>Date Sanity &amp; Inversions</t>
         </is>
       </c>
-      <c r="D30" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E30" s="6" t="inlineStr">
+      <c r="D34" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
         <is>
           <t>schwab.dim_accounts</t>
         </is>
       </c>
-      <c r="F30" s="7" t="inlineStr">
+      <c r="F34" s="7" t="inlineStr">
         <is>
           <t>Verify Date Sanity: Zero inverted dates (EffectiveTo &lt; EffectiveFrom) and active records have non-future start dates</t>
         </is>
       </c>
-      <c r="G30" s="7" t="inlineStr">
+      <c r="G34" s="7" t="inlineStr">
         <is>
           <t>dim_accounts populated</t>
         </is>
       </c>
-      <c r="H30" s="7" t="inlineStr">
+      <c r="H34" s="7" t="inlineStr">
         <is>
           <t>Inverted_Date_Count = 0, Future_Active_Start_Date = 0, Null_Start_Date_Count = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I30" s="18" t="inlineStr">
+      <c r="I34" s="18" t="inlineStr">
         <is>
           <t>SELECT 
     'schwab.dim_accounts' AS TableName,
@@ -2455,48 +2911,48 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="54" customHeight="1">
-      <c r="A31" s="12" t="inlineStr">
+    <row r="35" ht="54" customHeight="1">
+      <c r="A35" s="12" t="inlineStr">
         <is>
           <t>Schwab</t>
         </is>
       </c>
-      <c r="B31" s="12" t="inlineStr">
+      <c r="B35" s="12" t="inlineStr">
         <is>
           <t>TC_SC_GOLD_11</t>
         </is>
       </c>
-      <c r="C31" s="13" t="inlineStr">
+      <c r="C35" s="13" t="inlineStr">
         <is>
           <t>Open-Ended Active Records</t>
         </is>
       </c>
-      <c r="D31" s="19" t="inlineStr">
+      <c r="D35" s="19" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E31" s="10" t="inlineStr">
+      <c r="E35" s="10" t="inlineStr">
         <is>
           <t>schwab.dim_accounts</t>
         </is>
       </c>
-      <c r="F31" s="11" t="inlineStr">
+      <c r="F35" s="11" t="inlineStr">
         <is>
           <t>Verify Active Records are Open-Ended (EffectiveTo is NULL or '9999-12-31')</t>
         </is>
       </c>
-      <c r="G31" s="11" t="inlineStr">
+      <c r="G35" s="11" t="inlineStr">
         <is>
           <t>dim_accounts where IsCurrent = 1</t>
         </is>
       </c>
-      <c r="H31" s="11" t="inlineStr">
+      <c r="H35" s="11" t="inlineStr">
         <is>
           <t>Prematurely_Ended_Active_Records = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I31" s="17" t="inlineStr">
+      <c r="I35" s="17" t="inlineStr">
         <is>
           <t>SELECT 
     'schwab.dim_accounts' AS TableName,
@@ -2511,48 +2967,48 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="54" customHeight="1">
-      <c r="A32" s="8" t="inlineStr">
+    <row r="36" ht="54" customHeight="1">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t>Schwab</t>
         </is>
       </c>
-      <c r="B32" s="8" t="inlineStr">
+      <c r="B36" s="8" t="inlineStr">
         <is>
           <t>TC_SC_GOLD_12</t>
         </is>
       </c>
-      <c r="C32" s="9" t="inlineStr">
+      <c r="C36" s="9" t="inlineStr">
         <is>
           <t>Version Evolution Audit</t>
         </is>
       </c>
-      <c r="D32" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E32" s="6" t="inlineStr">
+      <c r="D36" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
         <is>
           <t>schwab.dim_accounts</t>
         </is>
       </c>
-      <c r="F32" s="7" t="inlineStr">
+      <c r="F36" s="7" t="inlineStr">
         <is>
           <t>Verify SCD2 Version Evolution: Monotonic SK increments, advancing EffectiveFrom, continuous timeline (EffectiveTo = next EffectiveFrom - 1), and latest version active</t>
         </is>
       </c>
-      <c r="G32" s="7" t="inlineStr">
+      <c r="G36" s="7" t="inlineStr">
         <is>
           <t>dim_accounts with multiple version rows per account_id</t>
         </is>
       </c>
-      <c r="H32" s="7" t="inlineStr">
+      <c r="H36" s="7" t="inlineStr">
         <is>
           <t>Reused_Or_NonIncrementing_SK_Count = 0, NonAdvancing_EffectiveFrom_Count = 0, Timeline_Gap_Or_Overlap_Count = 0, LatestVersion_Not_Active_Count = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I32" s="18" t="inlineStr">
+      <c r="I36" s="18" t="inlineStr">
         <is>
           <t>WITH SchwabEvolution AS (
     SELECT 
@@ -2587,48 +3043,48 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="54" customHeight="1">
-      <c r="A33" s="12" t="inlineStr">
+    <row r="37" ht="54" customHeight="1">
+      <c r="A37" s="12" t="inlineStr">
         <is>
           <t>Schwab</t>
         </is>
       </c>
-      <c r="B33" s="12" t="inlineStr">
+      <c r="B37" s="12" t="inlineStr">
         <is>
           <t>TC_SC_GOLD_13</t>
         </is>
       </c>
-      <c r="C33" s="13" t="inlineStr">
+      <c r="C37" s="13" t="inlineStr">
         <is>
           <t>Fact Health &amp; Historical Retention</t>
         </is>
       </c>
-      <c r="D33" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E33" s="10" t="inlineStr">
+      <c r="D37" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E37" s="10" t="inlineStr">
         <is>
           <t>schwab.fact_recon_position_d1, fact_recon_position_d2, fact_daily_closing_lots, fact_transactions, fact_ult_lot_daily_taxable, fact_uln_lot_daily_non_taxable</t>
         </is>
       </c>
-      <c r="F33" s="11" t="inlineStr">
+      <c r="F37" s="11" t="inlineStr">
         <is>
           <t>Verify Fact Tables Health: Active SK mapping for fresh runs, historical closed version preservation for unrepeated rows, exact natural account match, and orphan SK detection</t>
         </is>
       </c>
-      <c r="G33" s="11" t="inlineStr">
+      <c r="G37" s="11" t="inlineStr">
         <is>
           <t>All 6 Schwab Fact tables loaded into Gold Warehouse</t>
         </is>
       </c>
-      <c r="H33" s="11" t="inlineStr">
+      <c r="H37" s="11" t="inlineStr">
         <is>
           <t>Fresh records map to active SK (IsCurrent = 1), past records retain historical SK, Exact_Account_Match_Count covers all non-orphan rows, Defect_Orphan_Unmapped_SK = 0, Defect_Wrong_Account_Mismatch = 0. OverallStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I33" s="17" t="inlineStr">
+      <c r="I37" s="17" t="inlineStr">
         <is>
           <t>WITH MaxRuns AS (
     SELECT 'fact_recon_position_d1' AS TableName, MAX(updated_at) AS LatestRunTimestamp FROM Gold_Warehouse.schwab.fact_recon_position_d1 UNION ALL
@@ -2752,48 +3208,48 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="54" customHeight="1">
-      <c r="A34" s="8" t="inlineStr">
+    <row r="38" ht="54" customHeight="1">
+      <c r="A38" s="8" t="inlineStr">
         <is>
           <t>Salentica</t>
         </is>
       </c>
-      <c r="B34" s="8" t="inlineStr">
+      <c r="B38" s="8" t="inlineStr">
         <is>
           <t>TC_SAL_GOLD_01</t>
         </is>
       </c>
-      <c r="C34" s="9" t="inlineStr">
+      <c r="C38" s="9" t="inlineStr">
         <is>
           <t>SK Mapping &amp; Joins</t>
         </is>
       </c>
-      <c r="D34" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E34" s="6" t="inlineStr">
+      <c r="D38" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="inlineStr">
         <is>
           <t>salentica.dim_account</t>
         </is>
       </c>
-      <c r="F34" s="7" t="inlineStr">
+      <c r="F38" s="7" t="inlineStr">
         <is>
           <t>Verify Foreign SK Resolution in dim_account (primarycontactid_sk, owningbusinessunit_sk)</t>
         </is>
       </c>
-      <c r="G34" s="7" t="inlineStr">
+      <c r="G38" s="7" t="inlineStr">
         <is>
           <t>dim_account populated with Point-in-Time referential keys</t>
         </is>
       </c>
-      <c r="H34" s="7" t="inlineStr">
+      <c r="H38" s="7" t="inlineStr">
         <is>
           <t>Foreign SKs resolve to matching natural keys in parent dimensions (Active or Expired). Unmapped default to -1.</t>
         </is>
       </c>
-      <c r="I34" s="18" t="inlineStr">
+      <c r="I38" s="18" t="inlineStr">
         <is>
           <t>SELECT COUNT(*) AS MismatchedNaturalKeyCount
 FROM Gold_Warehouse.salentica.dim_account a
@@ -2805,48 +3261,48 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="54" customHeight="1">
-      <c r="A35" s="12" t="inlineStr">
+    <row r="39" ht="54" customHeight="1">
+      <c r="A39" s="12" t="inlineStr">
         <is>
           <t>Salentica</t>
         </is>
       </c>
-      <c r="B35" s="12" t="inlineStr">
+      <c r="B39" s="12" t="inlineStr">
         <is>
           <t>TC_SAL_GOLD_02</t>
         </is>
       </c>
-      <c r="C35" s="13" t="inlineStr">
+      <c r="C39" s="13" t="inlineStr">
         <is>
           <t>SK Mapping &amp; Joins</t>
         </is>
       </c>
-      <c r="D35" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E35" s="10" t="inlineStr">
+      <c r="D39" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E39" s="10" t="inlineStr">
         <is>
           <t>salentica.dim_contact_core</t>
         </is>
       </c>
-      <c r="F35" s="11" t="inlineStr">
+      <c r="F39" s="11" t="inlineStr">
         <is>
           <t>Verify Foreign SK Resolution in dim_contact_core (accountid_sk, owningbusinessunit_sk)</t>
         </is>
       </c>
-      <c r="G35" s="11" t="inlineStr">
+      <c r="G39" s="11" t="inlineStr">
         <is>
           <t>dim_contact_core populated</t>
         </is>
       </c>
-      <c r="H35" s="11" t="inlineStr">
+      <c r="H39" s="11" t="inlineStr">
         <is>
           <t>Foreign SKs resolve to matching natural keys in dim_account &amp; dim_businessunit. Zero referential mismatches.</t>
         </is>
       </c>
-      <c r="I35" s="17" t="inlineStr">
+      <c r="I39" s="17" t="inlineStr">
         <is>
           <t>SELECT COUNT(*) AS MismatchedNaturalKeyCount
 FROM Gold_Warehouse.salentica.dim_contact_core c
@@ -2858,48 +3314,48 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="54" customHeight="1">
-      <c r="A36" s="8" t="inlineStr">
+    <row r="40" ht="54" customHeight="1">
+      <c r="A40" s="8" t="inlineStr">
         <is>
           <t>Salentica</t>
         </is>
       </c>
-      <c r="B36" s="8" t="inlineStr">
+      <c r="B40" s="8" t="inlineStr">
         <is>
           <t>TC_SAL_GOLD_03</t>
         </is>
       </c>
-      <c r="C36" s="9" t="inlineStr">
+      <c r="C40" s="9" t="inlineStr">
         <is>
           <t>SK Mapping &amp; Joins</t>
         </is>
       </c>
-      <c r="D36" s="19" t="inlineStr">
+      <c r="D40" s="19" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E36" s="6" t="inlineStr">
+      <c r="E40" s="6" t="inlineStr">
         <is>
           <t>salentica.dim_family</t>
         </is>
       </c>
-      <c r="F36" s="7" t="inlineStr">
+      <c r="F40" s="7" t="inlineStr">
         <is>
           <t>Verify Foreign SK Resolution in dim_family (si_primarycontact_sk, owningbusinessunit_sk)</t>
         </is>
       </c>
-      <c r="G36" s="7" t="inlineStr">
+      <c r="G40" s="7" t="inlineStr">
         <is>
           <t>dim_family populated</t>
         </is>
       </c>
-      <c r="H36" s="7" t="inlineStr">
+      <c r="H40" s="7" t="inlineStr">
         <is>
           <t>Foreign SKs accurately resolve to contactid &amp; businessunitid. Zero mismatches.</t>
         </is>
       </c>
-      <c r="I36" s="18" t="inlineStr">
+      <c r="I40" s="18" t="inlineStr">
         <is>
           <t>SELECT COUNT(*) AS MismatchedFamilyLinks
 FROM Gold_Warehouse.salentica.dim_family f
@@ -2911,48 +3367,48 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="54" customHeight="1">
-      <c r="A37" s="12" t="inlineStr">
+    <row r="41" ht="54" customHeight="1">
+      <c r="A41" s="12" t="inlineStr">
         <is>
           <t>Salentica</t>
         </is>
       </c>
-      <c r="B37" s="12" t="inlineStr">
+      <c r="B41" s="12" t="inlineStr">
         <is>
           <t>TC_SAL_GOLD_04</t>
         </is>
       </c>
-      <c r="C37" s="13" t="inlineStr">
+      <c r="C41" s="13" t="inlineStr">
         <is>
           <t>SK Mapping &amp; Joins</t>
         </is>
       </c>
-      <c r="D37" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E37" s="10" t="inlineStr">
+      <c r="D41" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E41" s="10" t="inlineStr">
         <is>
           <t>salentica.fact_lead</t>
         </is>
       </c>
-      <c r="F37" s="11" t="inlineStr">
+      <c r="F41" s="11" t="inlineStr">
         <is>
           <t>Verify Foreign SK Resolution in fact_lead (accountid_sk, contactid_sk)</t>
         </is>
       </c>
-      <c r="G37" s="11" t="inlineStr">
+      <c r="G41" s="11" t="inlineStr">
         <is>
           <t>fact_lead populated</t>
         </is>
       </c>
-      <c r="H37" s="11" t="inlineStr">
+      <c r="H41" s="11" t="inlineStr">
         <is>
           <t>Foreign SKs resolve to matching accountid and contactid (Active or Expired versions). Zero mismatches.</t>
         </is>
       </c>
-      <c r="I37" s="17" t="inlineStr">
+      <c r="I41" s="17" t="inlineStr">
         <is>
           <t>SELECT COUNT(*) AS MismatchedLeadLinks
 FROM Gold_Warehouse.salentica.fact_lead l
@@ -2964,48 +3420,48 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="54" customHeight="1">
-      <c r="A38" s="8" t="inlineStr">
+    <row r="42" ht="54" customHeight="1">
+      <c r="A42" s="8" t="inlineStr">
         <is>
           <t>Salentica</t>
         </is>
       </c>
-      <c r="B38" s="8" t="inlineStr">
+      <c r="B42" s="8" t="inlineStr">
         <is>
           <t>TC_SAL_GOLD_05</t>
         </is>
       </c>
-      <c r="C38" s="9" t="inlineStr">
+      <c r="C42" s="9" t="inlineStr">
         <is>
           <t>SK Mapping &amp; Joins</t>
         </is>
       </c>
-      <c r="D38" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E38" s="6" t="inlineStr">
+      <c r="D42" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
         <is>
           <t>salentica.fact_opportunity</t>
         </is>
       </c>
-      <c r="F38" s="7" t="inlineStr">
+      <c r="F42" s="7" t="inlineStr">
         <is>
           <t>Verify Point-in-Time SK Resolution in fact_opportunity (accountid_sk, contactid_sk)</t>
         </is>
       </c>
-      <c r="G38" s="7" t="inlineStr">
+      <c r="G42" s="7" t="inlineStr">
         <is>
           <t>fact_opportunity populated</t>
         </is>
       </c>
-      <c r="H38" s="7" t="inlineStr">
+      <c r="H42" s="7" t="inlineStr">
         <is>
           <t>opp.accountid_sk &amp; contactid_sk resolve to matching natural keys in Dim (Active or Expired). Zero mismatches.</t>
         </is>
       </c>
-      <c r="I38" s="18" t="inlineStr">
+      <c r="I42" s="18" t="inlineStr">
         <is>
           <t>SELECT COUNT(*) AS MismatchedOpportunityLinks
 FROM Gold_Warehouse.salentica.fact_opportunity opp
@@ -3017,48 +3473,48 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="54" customHeight="1">
-      <c r="A39" s="12" t="inlineStr">
+    <row r="43" ht="54" customHeight="1">
+      <c r="A43" s="12" t="inlineStr">
         <is>
           <t>Salentica</t>
         </is>
       </c>
-      <c r="B39" s="12" t="inlineStr">
+      <c r="B43" s="12" t="inlineStr">
         <is>
           <t>TC_SAL_GOLD_06</t>
         </is>
       </c>
-      <c r="C39" s="13" t="inlineStr">
+      <c r="C43" s="13" t="inlineStr">
         <is>
           <t>SK Mapping &amp; Joins</t>
         </is>
       </c>
-      <c r="D39" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E39" s="10" t="inlineStr">
+      <c r="D43" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E43" s="10" t="inlineStr">
         <is>
           <t>salentica.fact_investmentaccount</t>
         </is>
       </c>
-      <c r="F39" s="11" t="inlineStr">
+      <c r="F43" s="11" t="inlineStr">
         <is>
           <t>Verify Foreign SK Resolution in fact_investmentaccount (si_family_sk, si_portfolio_sk)</t>
         </is>
       </c>
-      <c r="G39" s="11" t="inlineStr">
+      <c r="G43" s="11" t="inlineStr">
         <is>
           <t>fact_investmentaccount populated</t>
         </is>
       </c>
-      <c r="H39" s="11" t="inlineStr">
+      <c r="H43" s="11" t="inlineStr">
         <is>
           <t>Attached SKs resolve to matching si_familyid &amp; si_portfolioid. Zero mismatches.</t>
         </is>
       </c>
-      <c r="I39" s="17" t="inlineStr">
+      <c r="I43" s="17" t="inlineStr">
         <is>
           <t>SELECT COUNT(*) AS MismatchedInvestmentLinks
 FROM Gold_Warehouse.salentica.fact_investmentaccount ia
@@ -3070,48 +3526,48 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="54" customHeight="1">
-      <c r="A40" s="8" t="inlineStr">
+    <row r="44" ht="54" customHeight="1">
+      <c r="A44" s="8" t="inlineStr">
         <is>
           <t>Salentica</t>
         </is>
       </c>
-      <c r="B40" s="8" t="inlineStr">
+      <c r="B44" s="8" t="inlineStr">
         <is>
           <t>TC_SAL_GOLD_07</t>
         </is>
       </c>
-      <c r="C40" s="9" t="inlineStr">
+      <c r="C44" s="9" t="inlineStr">
         <is>
           <t>Orphan &amp; -1 Fallback</t>
         </is>
       </c>
-      <c r="D40" s="19" t="inlineStr">
+      <c r="D44" s="19" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E40" s="6" t="inlineStr">
+      <c r="E44" s="6" t="inlineStr">
         <is>
           <t>salentica.fact_opportunity</t>
         </is>
       </c>
-      <c r="F40" s="7" t="inlineStr">
+      <c r="F44" s="7" t="inlineStr">
         <is>
           <t>Verify SG_SAL_22 Fallback: Unmapped Foreign References Default to -1 (Zero Orphan NULLs)</t>
         </is>
       </c>
-      <c r="G40" s="7" t="inlineStr">
+      <c r="G44" s="7" t="inlineStr">
         <is>
           <t>fact_opportunity populated</t>
         </is>
       </c>
-      <c r="H40" s="7" t="inlineStr">
+      <c r="H44" s="7" t="inlineStr">
         <is>
           <t>When natural ID is NULL, the corresponding SK defaults to -1. Zero unmapped NULLs in SK columns.</t>
         </is>
       </c>
-      <c r="I40" s="18" t="inlineStr">
+      <c r="I44" s="18" t="inlineStr">
         <is>
           <t>SELECT 
     SUM(CASE WHEN accountid IS NULL AND accountid_sk = -1 THEN 1 ELSE 0 END) AS ProperlyDefaulted_AccountSK,
@@ -3123,48 +3579,48 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="54" customHeight="1">
-      <c r="A41" s="12" t="inlineStr">
+    <row r="45" ht="54" customHeight="1">
+      <c r="A45" s="12" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B41" s="12" t="inlineStr">
+      <c r="B45" s="12" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_01</t>
         </is>
       </c>
-      <c r="C41" s="13" t="inlineStr">
+      <c r="C45" s="13" t="inlineStr">
         <is>
           <t>SCD2 Deduplication</t>
         </is>
       </c>
-      <c r="D41" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E41" s="10" t="inlineStr">
+      <c r="D45" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E45" s="10" t="inlineStr">
         <is>
           <t>tamarac.dim_account_information</t>
         </is>
       </c>
-      <c r="F41" s="11" t="inlineStr">
+      <c r="F45" s="11" t="inlineStr">
         <is>
           <t>Verify Active Deduplication on PK ['account_number'] (is_current = 'True')</t>
         </is>
       </c>
-      <c r="G41" s="11" t="inlineStr">
+      <c r="G45" s="11" t="inlineStr">
         <is>
           <t>dim_account_information populated</t>
         </is>
       </c>
-      <c r="H41" s="11" t="inlineStr">
+      <c r="H45" s="11" t="inlineStr">
         <is>
           <t>Zero duplicate active accounts. Exactly one is_current = 'True' row per account_number.</t>
         </is>
       </c>
-      <c r="I41" s="17" t="inlineStr">
+      <c r="I45" s="17" t="inlineStr">
         <is>
           <t>SELECT account_number, COUNT(*) AS ActiveDuplicateCount
 FROM Gold_Warehouse.tamarac.dim_account_information
@@ -3174,48 +3630,48 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="54" customHeight="1">
-      <c r="A42" s="8" t="inlineStr">
+    <row r="46" ht="54" customHeight="1">
+      <c r="A46" s="8" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B42" s="8" t="inlineStr">
+      <c r="B46" s="8" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_02</t>
         </is>
       </c>
-      <c r="C42" s="9" t="inlineStr">
+      <c r="C46" s="9" t="inlineStr">
         <is>
           <t>SK Uniqueness</t>
         </is>
       </c>
-      <c r="D42" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E42" s="6" t="inlineStr">
+      <c r="D46" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="inlineStr">
         <is>
           <t>tamarac.dim_account_information</t>
         </is>
       </c>
-      <c r="F42" s="7" t="inlineStr">
+      <c r="F46" s="7" t="inlineStr">
         <is>
           <t>Verify Primary Surrogate Key (account_information_SK) uniqueness across all records</t>
         </is>
       </c>
-      <c r="G42" s="7" t="inlineStr">
+      <c r="G46" s="7" t="inlineStr">
         <is>
           <t>dim_account_information populated</t>
         </is>
       </c>
-      <c r="H42" s="7" t="inlineStr">
+      <c r="H46" s="7" t="inlineStr">
         <is>
           <t>Surrogate key account_information_SK is strictly unique across all rows. Zero duplicates.</t>
         </is>
       </c>
-      <c r="I42" s="18" t="inlineStr">
+      <c r="I46" s="18" t="inlineStr">
         <is>
           <t>SELECT account_information_SK, COUNT(*) AS DuplicateCount
 FROM Gold_Warehouse.tamarac.dim_account_information
@@ -3224,48 +3680,48 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="54" customHeight="1">
-      <c r="A43" s="12" t="inlineStr">
+    <row r="47" ht="54" customHeight="1">
+      <c r="A47" s="12" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B43" s="12" t="inlineStr">
+      <c r="B47" s="12" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_03</t>
         </is>
       </c>
-      <c r="C43" s="13" t="inlineStr">
+      <c r="C47" s="13" t="inlineStr">
         <is>
           <t>Audit Columns</t>
         </is>
       </c>
-      <c r="D43" s="19" t="inlineStr">
+      <c r="D47" s="19" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E43" s="10" t="inlineStr">
+      <c r="E47" s="10" t="inlineStr">
         <is>
           <t>tamarac.dim_account_information</t>
         </is>
       </c>
-      <c r="F43" s="11" t="inlineStr">
+      <c r="F47" s="11" t="inlineStr">
         <is>
           <t>Verify file_business_date and updated_at populated on active Tamarac accounts</t>
         </is>
       </c>
-      <c r="G43" s="11" t="inlineStr">
+      <c r="G47" s="11" t="inlineStr">
         <is>
           <t>dim_account_information populated</t>
         </is>
       </c>
-      <c r="H43" s="11" t="inlineStr">
+      <c r="H47" s="11" t="inlineStr">
         <is>
           <t>file_business_date and updated_at are non-null and &lt;= current calendar date.</t>
         </is>
       </c>
-      <c r="I43" s="17" t="inlineStr">
+      <c r="I47" s="17" t="inlineStr">
         <is>
           <t>SELECT 
     COUNT(*) AS TotalRows,
@@ -3276,48 +3732,48 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="54" customHeight="1">
-      <c r="A44" s="8" t="inlineStr">
+    <row r="48" ht="54" customHeight="1">
+      <c r="A48" s="8" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B44" s="8" t="inlineStr">
+      <c r="B48" s="8" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_04</t>
         </is>
       </c>
-      <c r="C44" s="9" t="inlineStr">
+      <c r="C48" s="9" t="inlineStr">
         <is>
           <t>SCD2 Deduplication</t>
         </is>
       </c>
-      <c r="D44" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E44" s="6" t="inlineStr">
+      <c r="D48" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="inlineStr">
         <is>
           <t>tamarac.dim_account_model_allocation</t>
         </is>
       </c>
-      <c r="F44" s="7" t="inlineStr">
+      <c r="F48" s="7" t="inlineStr">
         <is>
           <t>Verify Active Deduplication on Composite PK ['account_number', 'model_name']</t>
         </is>
       </c>
-      <c r="G44" s="7" t="inlineStr">
+      <c r="G48" s="7" t="inlineStr">
         <is>
           <t>dim_account_model_allocation populated</t>
         </is>
       </c>
-      <c r="H44" s="7" t="inlineStr">
+      <c r="H48" s="7" t="inlineStr">
         <is>
           <t>Zero duplicate active model allocations per (account_number, model_name).</t>
         </is>
       </c>
-      <c r="I44" s="18" t="inlineStr">
+      <c r="I48" s="18" t="inlineStr">
         <is>
           <t>SELECT account_number, model_name, COUNT(*) AS ActiveDuplicateAllocations
 FROM Gold_Warehouse.tamarac.dim_account_model_allocation
@@ -3327,48 +3783,48 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="54" customHeight="1">
-      <c r="A45" s="12" t="inlineStr">
+    <row r="49" ht="54" customHeight="1">
+      <c r="A49" s="12" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B45" s="12" t="inlineStr">
+      <c r="B49" s="12" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_05</t>
         </is>
       </c>
-      <c r="C45" s="13" t="inlineStr">
+      <c r="C49" s="13" t="inlineStr">
         <is>
           <t>SK Uniqueness</t>
         </is>
       </c>
-      <c r="D45" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E45" s="10" t="inlineStr">
+      <c r="D49" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E49" s="10" t="inlineStr">
         <is>
           <t>tamarac.dim_account_model_allocation</t>
         </is>
       </c>
-      <c r="F45" s="11" t="inlineStr">
+      <c r="F49" s="11" t="inlineStr">
         <is>
           <t>Verify Primary Surrogate Key (account_model_SK) uniqueness</t>
         </is>
       </c>
-      <c r="G45" s="11" t="inlineStr">
+      <c r="G49" s="11" t="inlineStr">
         <is>
           <t>dim_account_model_allocation populated</t>
         </is>
       </c>
-      <c r="H45" s="11" t="inlineStr">
+      <c r="H49" s="11" t="inlineStr">
         <is>
           <t>account_model_SK is unique with zero NULL values.</t>
         </is>
       </c>
-      <c r="I45" s="17" t="inlineStr">
+      <c r="I49" s="17" t="inlineStr">
         <is>
           <t>SELECT account_model_SK, COUNT(*) AS DuplicateModelSK
 FROM Gold_Warehouse.tamarac.dim_account_model_allocation
@@ -3377,48 +3833,48 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="54" customHeight="1">
-      <c r="A46" s="8" t="inlineStr">
+    <row r="50" ht="54" customHeight="1">
+      <c r="A50" s="8" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B46" s="8" t="inlineStr">
+      <c r="B50" s="8" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_06</t>
         </is>
       </c>
-      <c r="C46" s="9" t="inlineStr">
+      <c r="C50" s="9" t="inlineStr">
         <is>
           <t>Cross-Table Linkage</t>
         </is>
       </c>
-      <c r="D46" s="19" t="inlineStr">
+      <c r="D50" s="19" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E46" s="6" t="inlineStr">
+      <c r="E50" s="6" t="inlineStr">
         <is>
           <t>tamarac.dim_account_model_allocation</t>
         </is>
       </c>
-      <c r="F46" s="7" t="inlineStr">
+      <c r="F50" s="7" t="inlineStr">
         <is>
           <t>Verify Cross-Table Linkage: Every account_number exists in dim_account_information</t>
         </is>
       </c>
-      <c r="G46" s="7" t="inlineStr">
+      <c r="G50" s="7" t="inlineStr">
         <is>
           <t>dim_account_model_allocation populated</t>
         </is>
       </c>
-      <c r="H46" s="7" t="inlineStr">
+      <c r="H50" s="7" t="inlineStr">
         <is>
           <t>Zero orphan model allocation accounts. All account_number values exist in parent dimension.</t>
         </is>
       </c>
-      <c r="I46" s="18" t="inlineStr">
+      <c r="I50" s="18" t="inlineStr">
         <is>
           <t>SELECT COUNT(*) AS OrphanModelAllocations
 FROM Gold_Warehouse.tamarac.dim_account_model_allocation ma
@@ -3429,48 +3885,48 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="54" customHeight="1">
-      <c r="A47" s="12" t="inlineStr">
+    <row r="51" ht="54" customHeight="1">
+      <c r="A51" s="12" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B47" s="12" t="inlineStr">
+      <c r="B51" s="12" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_07</t>
         </is>
       </c>
-      <c r="C47" s="13" t="inlineStr">
+      <c r="C51" s="13" t="inlineStr">
         <is>
           <t>SCD2 Date Validation</t>
         </is>
       </c>
-      <c r="D47" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E47" s="10" t="inlineStr">
+      <c r="D51" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E51" s="10" t="inlineStr">
         <is>
           <t>tamarac.dim_account_information</t>
         </is>
       </c>
-      <c r="F47" s="11" t="inlineStr">
+      <c r="F51" s="11" t="inlineStr">
         <is>
           <t>Verify Inactive End Date Rule: effective_end_date &lt;= (MAX(file_business_date) - 1 day) and non-null</t>
         </is>
       </c>
-      <c r="G47" s="11" t="inlineStr">
+      <c r="G51" s="11" t="inlineStr">
         <is>
           <t>dim_account_information populated with inactive records</t>
         </is>
       </c>
-      <c r="H47" s="11" t="inlineStr">
+      <c r="H51" s="11" t="inlineStr">
         <is>
           <t>Exceeded_Cutoff_Count = 0, Null_End_Date_Count = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I47" s="17" t="inlineStr">
+      <c r="I51" s="17" t="inlineStr">
         <is>
           <t>SELECT 
     'dim_account_information' AS TableName,
@@ -3490,48 +3946,48 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="54" customHeight="1">
-      <c r="A48" s="8" t="inlineStr">
+    <row r="52" ht="54" customHeight="1">
+      <c r="A52" s="8" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B48" s="8" t="inlineStr">
+      <c r="B52" s="8" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_08</t>
         </is>
       </c>
-      <c r="C48" s="9" t="inlineStr">
+      <c r="C52" s="9" t="inlineStr">
         <is>
           <t>SCD2 Date Validation</t>
         </is>
       </c>
-      <c r="D48" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E48" s="6" t="inlineStr">
+      <c r="D52" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E52" s="6" t="inlineStr">
         <is>
           <t>tamarac.dim_account_model_allocation</t>
         </is>
       </c>
-      <c r="F48" s="7" t="inlineStr">
+      <c r="F52" s="7" t="inlineStr">
         <is>
           <t>Verify Inactive End Date Rule: effective_end_date &lt;= (MAX(file_business_date) - 1 day) and non-null</t>
         </is>
       </c>
-      <c r="G48" s="7" t="inlineStr">
+      <c r="G52" s="7" t="inlineStr">
         <is>
           <t>dim_account_model_allocation populated with inactive records</t>
         </is>
       </c>
-      <c r="H48" s="7" t="inlineStr">
+      <c r="H52" s="7" t="inlineStr">
         <is>
           <t>Exceeded_Cutoff_Count = 0, Null_End_Date_Count = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I48" s="18" t="inlineStr">
+      <c r="I52" s="18" t="inlineStr">
         <is>
           <t>SELECT 
     'dim_account_model_allocation' AS TableName,
@@ -3551,48 +4007,48 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="54" customHeight="1">
-      <c r="A49" s="12" t="inlineStr">
+    <row r="53" ht="54" customHeight="1">
+      <c r="A53" s="12" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B49" s="12" t="inlineStr">
+      <c r="B53" s="12" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_09</t>
         </is>
       </c>
-      <c r="C49" s="13" t="inlineStr">
+      <c r="C53" s="13" t="inlineStr">
         <is>
           <t>SCD2 Timeline &amp; SK Monotonicity</t>
         </is>
       </c>
-      <c r="D49" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E49" s="10" t="inlineStr">
+      <c r="D53" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E53" s="10" t="inlineStr">
         <is>
           <t>tamarac.dim_account_information</t>
         </is>
       </c>
-      <c r="F49" s="11" t="inlineStr">
+      <c r="F53" s="11" t="inlineStr">
         <is>
           <t>Verify SCD2 Timeline Continuity (Zero Gaps, Zero Overlaps) &amp; SK Monotonic Increment</t>
         </is>
       </c>
-      <c r="G49" s="11" t="inlineStr">
+      <c r="G53" s="11" t="inlineStr">
         <is>
           <t>dim_account_information with multiple versions per account_number</t>
         </is>
       </c>
-      <c r="H49" s="11" t="inlineStr">
+      <c r="H53" s="11" t="inlineStr">
         <is>
           <t>Timeline_Gap_Or_Overlap_Count = 0, SK_Non_Incrementing_Violation_Count = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I49" s="17" t="inlineStr">
+      <c r="I53" s="17" t="inlineStr">
         <is>
           <t>;WITH InfoTimeline AS (
     SELECT 
@@ -3620,48 +4076,48 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="54" customHeight="1">
-      <c r="A50" s="8" t="inlineStr">
+    <row r="54" ht="54" customHeight="1">
+      <c r="A54" s="8" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B50" s="8" t="inlineStr">
+      <c r="B54" s="8" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_10</t>
         </is>
       </c>
-      <c r="C50" s="9" t="inlineStr">
+      <c r="C54" s="9" t="inlineStr">
         <is>
           <t>SCD2 Timeline &amp; SK Monotonicity</t>
         </is>
       </c>
-      <c r="D50" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E50" s="6" t="inlineStr">
+      <c r="D54" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="inlineStr">
         <is>
           <t>tamarac.dim_account_model_allocation</t>
         </is>
       </c>
-      <c r="F50" s="7" t="inlineStr">
+      <c r="F54" s="7" t="inlineStr">
         <is>
           <t>Verify SCD2 Timeline Continuity (Zero Gaps, Zero Overlaps) &amp; SK Monotonic Increment</t>
         </is>
       </c>
-      <c r="G50" s="7" t="inlineStr">
+      <c r="G54" s="7" t="inlineStr">
         <is>
           <t>dim_account_model_allocation with multiple versions per composite key</t>
         </is>
       </c>
-      <c r="H50" s="7" t="inlineStr">
+      <c r="H54" s="7" t="inlineStr">
         <is>
           <t>Timeline_Gap_Or_Overlap_Count = 0, SK_Non_Incrementing_Violation_Count = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I50" s="18" t="inlineStr">
+      <c r="I54" s="18" t="inlineStr">
         <is>
           <t>;WITH ModelTimeline AS (
     SELECT 
@@ -3690,48 +4146,48 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="54" customHeight="1">
-      <c r="A51" s="12" t="inlineStr">
+    <row r="55" ht="54" customHeight="1">
+      <c r="A55" s="12" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B51" s="12" t="inlineStr">
+      <c r="B55" s="12" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_11</t>
         </is>
       </c>
-      <c r="C51" s="13" t="inlineStr">
+      <c r="C55" s="13" t="inlineStr">
         <is>
           <t>Date Sanity &amp; Inversions</t>
         </is>
       </c>
-      <c r="D51" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E51" s="10" t="inlineStr">
+      <c r="D55" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E55" s="10" t="inlineStr">
         <is>
           <t>tamarac.dim_account_information</t>
         </is>
       </c>
-      <c r="F51" s="11" t="inlineStr">
+      <c r="F55" s="11" t="inlineStr">
         <is>
           <t>Verify Date Sanity: Zero inverted dates (start &gt; end) and active records have non-future start dates</t>
         </is>
       </c>
-      <c r="G51" s="11" t="inlineStr">
+      <c r="G55" s="11" t="inlineStr">
         <is>
           <t>dim_account_information populated</t>
         </is>
       </c>
-      <c r="H51" s="11" t="inlineStr">
+      <c r="H55" s="11" t="inlineStr">
         <is>
           <t>Inverted_Date_Count = 0, Future_Active_Start_Date = 0, Null_Start_Date_Count = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I51" s="17" t="inlineStr">
+      <c r="I55" s="17" t="inlineStr">
         <is>
           <t>SELECT 
     'dim_account_information' AS TableName,
@@ -3749,48 +4205,48 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="54" customHeight="1">
-      <c r="A52" s="8" t="inlineStr">
+    <row r="56" ht="54" customHeight="1">
+      <c r="A56" s="8" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B52" s="8" t="inlineStr">
+      <c r="B56" s="8" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_12</t>
         </is>
       </c>
-      <c r="C52" s="9" t="inlineStr">
+      <c r="C56" s="9" t="inlineStr">
         <is>
           <t>Date Sanity &amp; Inversions</t>
         </is>
       </c>
-      <c r="D52" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E52" s="6" t="inlineStr">
+      <c r="D56" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E56" s="6" t="inlineStr">
         <is>
           <t>tamarac.dim_account_model_allocation</t>
         </is>
       </c>
-      <c r="F52" s="7" t="inlineStr">
+      <c r="F56" s="7" t="inlineStr">
         <is>
           <t>Verify Date Sanity: Zero inverted dates (start &gt; end) and active records have non-future start dates</t>
         </is>
       </c>
-      <c r="G52" s="7" t="inlineStr">
+      <c r="G56" s="7" t="inlineStr">
         <is>
           <t>dim_account_model_allocation populated</t>
         </is>
       </c>
-      <c r="H52" s="7" t="inlineStr">
+      <c r="H56" s="7" t="inlineStr">
         <is>
           <t>Inverted_Date_Count = 0, Future_Active_Start_Date = 0, Null_Start_Date_Count = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I52" s="18" t="inlineStr">
+      <c r="I56" s="18" t="inlineStr">
         <is>
           <t>SELECT 
     'dim_account_model_allocation' AS TableName,
@@ -3808,48 +4264,48 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="54" customHeight="1">
-      <c r="A53" s="12" t="inlineStr">
+    <row r="57" ht="54" customHeight="1">
+      <c r="A57" s="12" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B53" s="12" t="inlineStr">
+      <c r="B57" s="12" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_13</t>
         </is>
       </c>
-      <c r="C53" s="13" t="inlineStr">
+      <c r="C57" s="13" t="inlineStr">
         <is>
           <t>Open-Ended Active Records</t>
         </is>
       </c>
-      <c r="D53" s="19" t="inlineStr">
+      <c r="D57" s="19" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E53" s="10" t="inlineStr">
+      <c r="E57" s="10" t="inlineStr">
         <is>
           <t>tamarac.dim_account_information</t>
         </is>
       </c>
-      <c r="F53" s="11" t="inlineStr">
+      <c r="F57" s="11" t="inlineStr">
         <is>
           <t>Verify Active Records are Open-Ended (effective_end_date is NULL or '9999-12-31')</t>
         </is>
       </c>
-      <c r="G53" s="11" t="inlineStr">
+      <c r="G57" s="11" t="inlineStr">
         <is>
           <t>dim_account_information where is_current = 'True'</t>
         </is>
       </c>
-      <c r="H53" s="11" t="inlineStr">
+      <c r="H57" s="11" t="inlineStr">
         <is>
           <t>Prematurely_Ended_Active_Records = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I53" s="17" t="inlineStr">
+      <c r="I57" s="17" t="inlineStr">
         <is>
           <t>SELECT 
     'dim_account_information' AS TableName,
@@ -3864,48 +4320,48 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="54" customHeight="1">
-      <c r="A54" s="8" t="inlineStr">
+    <row r="58" ht="54" customHeight="1">
+      <c r="A58" s="8" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B54" s="8" t="inlineStr">
+      <c r="B58" s="8" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_14</t>
         </is>
       </c>
-      <c r="C54" s="9" t="inlineStr">
+      <c r="C58" s="9" t="inlineStr">
         <is>
           <t>Open-Ended Active Records</t>
         </is>
       </c>
-      <c r="D54" s="19" t="inlineStr">
+      <c r="D58" s="19" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E54" s="6" t="inlineStr">
+      <c r="E58" s="6" t="inlineStr">
         <is>
           <t>tamarac.dim_account_model_allocation</t>
         </is>
       </c>
-      <c r="F54" s="7" t="inlineStr">
+      <c r="F58" s="7" t="inlineStr">
         <is>
           <t>Verify Active Records are Open-Ended (effective_end_date is NULL or '9999-12-31')</t>
         </is>
       </c>
-      <c r="G54" s="7" t="inlineStr">
+      <c r="G58" s="7" t="inlineStr">
         <is>
           <t>dim_account_model_allocation where is_current = 'True'</t>
         </is>
       </c>
-      <c r="H54" s="7" t="inlineStr">
+      <c r="H58" s="7" t="inlineStr">
         <is>
           <t>Prematurely_Ended_Active_Records = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I54" s="18" t="inlineStr">
+      <c r="I58" s="18" t="inlineStr">
         <is>
           <t>SELECT 
     'dim_account_model_allocation' AS TableName,
@@ -3920,48 +4376,48 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="54" customHeight="1">
-      <c r="A55" s="12" t="inlineStr">
+    <row r="59" ht="54" customHeight="1">
+      <c r="A59" s="12" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B55" s="12" t="inlineStr">
+      <c r="B59" s="12" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_15</t>
         </is>
       </c>
-      <c r="C55" s="13" t="inlineStr">
+      <c r="C59" s="13" t="inlineStr">
         <is>
           <t>Version Evolution Audit</t>
         </is>
       </c>
-      <c r="D55" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E55" s="10" t="inlineStr">
+      <c r="D59" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E59" s="10" t="inlineStr">
         <is>
           <t>tamarac.dim_account_information</t>
         </is>
       </c>
-      <c r="F55" s="11" t="inlineStr">
+      <c r="F59" s="11" t="inlineStr">
         <is>
           <t>Verify Run Evolution: Every new run produces New Incremented SK, Advancing Start Date, and Latest Version is Active</t>
         </is>
       </c>
-      <c r="G55" s="11" t="inlineStr">
+      <c r="G59" s="11" t="inlineStr">
         <is>
           <t>dim_account_information with historical batch progression</t>
         </is>
       </c>
-      <c r="H55" s="11" t="inlineStr">
+      <c r="H59" s="11" t="inlineStr">
         <is>
           <t>Reused_Or_NonIncrementing_SK_Count = 0, NonAdvancing_EffectiveStartDate_Count = 0, Timeline_Gap_Or_Overlap_Count = 0, LatestVersion_Not_Active_Count = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I55" s="17" t="inlineStr">
+      <c r="I59" s="17" t="inlineStr">
         <is>
           <t>;WITH VersionChains AS (
     SELECT 
@@ -3995,48 +4451,48 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="54" customHeight="1">
-      <c r="A56" s="8" t="inlineStr">
+    <row r="60" ht="54" customHeight="1">
+      <c r="A60" s="8" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B56" s="8" t="inlineStr">
+      <c r="B60" s="8" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_16</t>
         </is>
       </c>
-      <c r="C56" s="9" t="inlineStr">
+      <c r="C60" s="9" t="inlineStr">
         <is>
           <t>Version Evolution Audit</t>
         </is>
       </c>
-      <c r="D56" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E56" s="6" t="inlineStr">
+      <c r="D60" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E60" s="6" t="inlineStr">
         <is>
           <t>tamarac.dim_account_model_allocation</t>
         </is>
       </c>
-      <c r="F56" s="7" t="inlineStr">
+      <c r="F60" s="7" t="inlineStr">
         <is>
           <t>Verify Run Evolution: Every new run produces New Incremented SK, Advancing Start Date, and Latest Version is Active</t>
         </is>
       </c>
-      <c r="G56" s="7" t="inlineStr">
+      <c r="G60" s="7" t="inlineStr">
         <is>
           <t>dim_account_model_allocation with historical batch progression</t>
         </is>
       </c>
-      <c r="H56" s="7" t="inlineStr">
+      <c r="H60" s="7" t="inlineStr">
         <is>
           <t>Reused_Or_NonIncrementing_SK_Count = 0, NonAdvancing_EffectiveStartDate_Count = 0, Timeline_Gap_Or_Overlap_Count = 0, LatestVersion_Not_Active_Count = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I56" s="18" t="inlineStr">
+      <c r="I60" s="18" t="inlineStr">
         <is>
           <t>;WITH ModelChains AS (
     SELECT 
@@ -4071,48 +4527,48 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="54" customHeight="1">
-      <c r="A57" s="12" t="inlineStr">
+    <row r="61" ht="54" customHeight="1">
+      <c r="A61" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B57" s="12" t="inlineStr">
+      <c r="B61" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_01</t>
         </is>
       </c>
-      <c r="C57" s="13" t="inlineStr">
+      <c r="C61" s="13" t="inlineStr">
         <is>
           <t>SCD2 Deduplication</t>
         </is>
       </c>
-      <c r="D57" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E57" s="10" t="inlineStr">
+      <c r="D61" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E61" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master</t>
         </is>
       </c>
-      <c r="F57" s="11" t="inlineStr">
+      <c r="F61" s="11" t="inlineStr">
         <is>
           <t>Verify Active Deduplication on Business Key ['customer_account_number'] (is_current = 1)</t>
         </is>
       </c>
-      <c r="G57" s="11" t="inlineStr">
+      <c r="G61" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master populated</t>
         </is>
       </c>
-      <c r="H57" s="11" t="inlineStr">
+      <c r="H61" s="11" t="inlineStr">
         <is>
           <t>Zero duplicate active accounts. Exactly one is_current = 1 record per customer_account_number.</t>
         </is>
       </c>
-      <c r="I57" s="17" t="inlineStr">
+      <c r="I61" s="17" t="inlineStr">
         <is>
           <t>SELECT customer_account_number, COUNT(*) AS ActiveDuplicateCount
 FROM Gold_Warehouse.innotrust.dim_account_master
@@ -4122,48 +4578,48 @@
         </is>
       </c>
     </row>
-    <row r="58" ht="54" customHeight="1">
-      <c r="A58" s="8" t="inlineStr">
+    <row r="62" ht="54" customHeight="1">
+      <c r="A62" s="8" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B58" s="8" t="inlineStr">
+      <c r="B62" s="8" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_02</t>
         </is>
       </c>
-      <c r="C58" s="9" t="inlineStr">
+      <c r="C62" s="9" t="inlineStr">
         <is>
           <t>SK Uniqueness</t>
         </is>
       </c>
-      <c r="D58" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E58" s="6" t="inlineStr">
+      <c r="D62" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E62" s="6" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master</t>
         </is>
       </c>
-      <c r="F58" s="7" t="inlineStr">
+      <c r="F62" s="7" t="inlineStr">
         <is>
           <t>Verify Primary Surrogate Key (dim_account_master_sk) uniqueness and non-null constraint</t>
         </is>
       </c>
-      <c r="G58" s="7" t="inlineStr">
+      <c r="G62" s="7" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master populated</t>
         </is>
       </c>
-      <c r="H58" s="7" t="inlineStr">
+      <c r="H62" s="7" t="inlineStr">
         <is>
           <t>dim_account_master_sk is strictly unique across all versions with zero NULL values.</t>
         </is>
       </c>
-      <c r="I58" s="18" t="inlineStr">
+      <c r="I62" s="18" t="inlineStr">
         <is>
           <t>SELECT dim_account_master_sk, COUNT(*) AS DuplicateCount
 FROM Gold_Warehouse.innotrust.dim_account_master
@@ -4177,48 +4633,48 @@
         </is>
       </c>
     </row>
-    <row r="59" ht="54" customHeight="1">
-      <c r="A59" s="12" t="inlineStr">
+    <row r="63" ht="54" customHeight="1">
+      <c r="A63" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B59" s="12" t="inlineStr">
+      <c r="B63" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_03</t>
         </is>
       </c>
-      <c r="C59" s="13" t="inlineStr">
+      <c r="C63" s="13" t="inlineStr">
         <is>
           <t>SCD2 Deduplication</t>
         </is>
       </c>
-      <c r="D59" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E59" s="10" t="inlineStr">
+      <c r="D63" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E63" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_account_category_codes</t>
         </is>
       </c>
-      <c r="F59" s="11" t="inlineStr">
+      <c r="F63" s="11" t="inlineStr">
         <is>
           <t>Verify Active Deduplication on Business Key ['account_category_code'] (is_current = 1)</t>
         </is>
       </c>
-      <c r="G59" s="11" t="inlineStr">
+      <c r="G63" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_account_category_codes populated</t>
         </is>
       </c>
-      <c r="H59" s="11" t="inlineStr">
+      <c r="H63" s="11" t="inlineStr">
         <is>
           <t>Zero duplicate active category codes per account_category_code.</t>
         </is>
       </c>
-      <c r="I59" s="17" t="inlineStr">
+      <c r="I63" s="17" t="inlineStr">
         <is>
           <t>SELECT account_category_code, COUNT(*) AS ActiveDuplicateCount
 FROM Gold_Warehouse.innotrust.dim_account_category_codes
@@ -4228,48 +4684,48 @@
         </is>
       </c>
     </row>
-    <row r="60" ht="54" customHeight="1">
-      <c r="A60" s="8" t="inlineStr">
+    <row r="64" ht="54" customHeight="1">
+      <c r="A64" s="8" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B60" s="8" t="inlineStr">
+      <c r="B64" s="8" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_04</t>
         </is>
       </c>
-      <c r="C60" s="9" t="inlineStr">
+      <c r="C64" s="9" t="inlineStr">
         <is>
           <t>SK Uniqueness</t>
         </is>
       </c>
-      <c r="D60" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E60" s="6" t="inlineStr">
+      <c r="D64" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E64" s="6" t="inlineStr">
         <is>
           <t>innotrust.dim_account_category_codes</t>
         </is>
       </c>
-      <c r="F60" s="7" t="inlineStr">
+      <c r="F64" s="7" t="inlineStr">
         <is>
           <t>Verify Primary Surrogate Key (dim_account_master_sk) uniqueness on dim_account_category_codes</t>
         </is>
       </c>
-      <c r="G60" s="7" t="inlineStr">
+      <c r="G64" s="7" t="inlineStr">
         <is>
           <t>innotrust.dim_account_category_codes populated</t>
         </is>
       </c>
-      <c r="H60" s="7" t="inlineStr">
+      <c r="H64" s="7" t="inlineStr">
         <is>
           <t>Surrogate key dim_account_master_sk is unique across all rows with zero NULLs.</t>
         </is>
       </c>
-      <c r="I60" s="18" t="inlineStr">
+      <c r="I64" s="18" t="inlineStr">
         <is>
           <t>SELECT dim_account_master_sk, COUNT(*) AS DuplicateCount
 FROM Gold_Warehouse.innotrust.dim_account_category_codes
@@ -4278,48 +4734,48 @@
         </is>
       </c>
     </row>
-    <row r="61" ht="54" customHeight="1">
-      <c r="A61" s="12" t="inlineStr">
+    <row r="65" ht="54" customHeight="1">
+      <c r="A65" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B61" s="12" t="inlineStr">
+      <c r="B65" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_05</t>
         </is>
       </c>
-      <c r="C61" s="13" t="inlineStr">
+      <c r="C65" s="13" t="inlineStr">
         <is>
           <t>SCD2 Deduplication</t>
         </is>
       </c>
-      <c r="D61" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E61" s="10" t="inlineStr">
+      <c r="D65" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E65" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_account_type_codes</t>
         </is>
       </c>
-      <c r="F61" s="11" t="inlineStr">
+      <c r="F65" s="11" t="inlineStr">
         <is>
           <t>Verify Active Deduplication on Business Key ['account_type_code'] (is_current = 1)</t>
         </is>
       </c>
-      <c r="G61" s="11" t="inlineStr">
+      <c r="G65" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_account_type_codes populated</t>
         </is>
       </c>
-      <c r="H61" s="11" t="inlineStr">
+      <c r="H65" s="11" t="inlineStr">
         <is>
           <t>Zero duplicate active account types per account_type_code.</t>
         </is>
       </c>
-      <c r="I61" s="17" t="inlineStr">
+      <c r="I65" s="17" t="inlineStr">
         <is>
           <t>SELECT account_type_code, COUNT(*) AS ActiveDuplicateCount
 FROM Gold_Warehouse.innotrust.dim_account_type_codes
@@ -4329,48 +4785,48 @@
         </is>
       </c>
     </row>
-    <row r="62" ht="54" customHeight="1">
-      <c r="A62" s="8" t="inlineStr">
+    <row r="66" ht="54" customHeight="1">
+      <c r="A66" s="8" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B62" s="8" t="inlineStr">
+      <c r="B66" s="8" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_06</t>
         </is>
       </c>
-      <c r="C62" s="9" t="inlineStr">
+      <c r="C66" s="9" t="inlineStr">
         <is>
           <t>SK Uniqueness</t>
         </is>
       </c>
-      <c r="D62" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E62" s="6" t="inlineStr">
+      <c r="D66" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E66" s="6" t="inlineStr">
         <is>
           <t>innotrust.dim_account_type_codes</t>
         </is>
       </c>
-      <c r="F62" s="7" t="inlineStr">
+      <c r="F66" s="7" t="inlineStr">
         <is>
           <t>Verify Primary Surrogate Key (dim_account_type_codes_sk) uniqueness and non-null constraint</t>
         </is>
       </c>
-      <c r="G62" s="7" t="inlineStr">
+      <c r="G66" s="7" t="inlineStr">
         <is>
           <t>innotrust.dim_account_type_codes populated</t>
         </is>
       </c>
-      <c r="H62" s="7" t="inlineStr">
+      <c r="H66" s="7" t="inlineStr">
         <is>
           <t>dim_account_type_codes_sk is strictly unique across all versions with zero NULLs.</t>
         </is>
       </c>
-      <c r="I62" s="18" t="inlineStr">
+      <c r="I66" s="18" t="inlineStr">
         <is>
           <t>SELECT dim_account_type_codes_sk, COUNT(*) AS DuplicateCount
 FROM Gold_Warehouse.innotrust.dim_account_type_codes
@@ -4379,48 +4835,48 @@
         </is>
       </c>
     </row>
-    <row r="63" ht="54" customHeight="1">
-      <c r="A63" s="12" t="inlineStr">
+    <row r="67" ht="54" customHeight="1">
+      <c r="A67" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B63" s="12" t="inlineStr">
+      <c r="B67" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_07</t>
         </is>
       </c>
-      <c r="C63" s="13" t="inlineStr">
+      <c r="C67" s="13" t="inlineStr">
         <is>
           <t>SCD2 Deduplication</t>
         </is>
       </c>
-      <c r="D63" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E63" s="10" t="inlineStr">
+      <c r="D67" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E67" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_master_sec_index</t>
         </is>
       </c>
-      <c r="F63" s="11" t="inlineStr">
+      <c r="F67" s="11" t="inlineStr">
         <is>
           <t>Verify Active Deduplication on Security Primary Key ['isin'] (is_current = 1)</t>
         </is>
       </c>
-      <c r="G63" s="11" t="inlineStr">
+      <c r="G67" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_master_sec_index populated</t>
         </is>
       </c>
-      <c r="H63" s="11" t="inlineStr">
+      <c r="H67" s="11" t="inlineStr">
         <is>
           <t>Zero duplicate active securities. Exactly one is_current = 1 record per isin.</t>
         </is>
       </c>
-      <c r="I63" s="17" t="inlineStr">
+      <c r="I67" s="17" t="inlineStr">
         <is>
           <t>SELECT isin, COUNT(*) AS ActiveDuplicateCount
 FROM Gold_Warehouse.innotrust.dim_master_sec_index
@@ -4430,48 +4886,48 @@
         </is>
       </c>
     </row>
-    <row r="64" ht="54" customHeight="1">
-      <c r="A64" s="8" t="inlineStr">
+    <row r="68" ht="54" customHeight="1">
+      <c r="A68" s="8" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B64" s="8" t="inlineStr">
+      <c r="B68" s="8" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_08</t>
         </is>
       </c>
-      <c r="C64" s="9" t="inlineStr">
+      <c r="C68" s="9" t="inlineStr">
         <is>
           <t>SK Uniqueness</t>
         </is>
       </c>
-      <c r="D64" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E64" s="6" t="inlineStr">
+      <c r="D68" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E68" s="6" t="inlineStr">
         <is>
           <t>innotrust.dim_master_sec_index</t>
         </is>
       </c>
-      <c r="F64" s="7" t="inlineStr">
+      <c r="F68" s="7" t="inlineStr">
         <is>
           <t>Verify Primary Surrogate Key (dim_master_sec_index_sk) uniqueness across all records</t>
         </is>
       </c>
-      <c r="G64" s="7" t="inlineStr">
+      <c r="G68" s="7" t="inlineStr">
         <is>
           <t>innotrust.dim_master_sec_index populated</t>
         </is>
       </c>
-      <c r="H64" s="7" t="inlineStr">
+      <c r="H68" s="7" t="inlineStr">
         <is>
           <t>dim_master_sec_index_sk is strictly unique across all versions with zero NULLs.</t>
         </is>
       </c>
-      <c r="I64" s="18" t="inlineStr">
+      <c r="I68" s="18" t="inlineStr">
         <is>
           <t>SELECT dim_master_sec_index_sk, COUNT(*) AS DuplicateCount
 FROM Gold_Warehouse.innotrust.dim_master_sec_index
@@ -4480,48 +4936,48 @@
         </is>
       </c>
     </row>
-    <row r="65" ht="54" customHeight="1">
-      <c r="A65" s="12" t="inlineStr">
+    <row r="69" ht="54" customHeight="1">
+      <c r="A69" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B65" s="12" t="inlineStr">
+      <c r="B69" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_09</t>
         </is>
       </c>
-      <c r="C65" s="13" t="inlineStr">
+      <c r="C69" s="13" t="inlineStr">
         <is>
           <t>SCD2 Deduplication</t>
         </is>
       </c>
-      <c r="D65" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E65" s="10" t="inlineStr">
+      <c r="D69" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E69" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_security_characteristics_codes</t>
         </is>
       </c>
-      <c r="F65" s="11" t="inlineStr">
+      <c r="F69" s="11" t="inlineStr">
         <is>
           <t>Verify Active Deduplication on Business Key ['security_type_code'] (is_current = 1)</t>
         </is>
       </c>
-      <c r="G65" s="11" t="inlineStr">
+      <c r="G69" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_security_characteristics_codes populated</t>
         </is>
       </c>
-      <c r="H65" s="11" t="inlineStr">
+      <c r="H69" s="11" t="inlineStr">
         <is>
           <t>Zero duplicate active security type codes per security_type_code.</t>
         </is>
       </c>
-      <c r="I65" s="17" t="inlineStr">
+      <c r="I69" s="17" t="inlineStr">
         <is>
           <t>SELECT security_type_code, COUNT(*) AS ActiveDuplicateCount
 FROM Gold_Warehouse.innotrust.dim_security_characteristics_codes
@@ -4531,48 +4987,48 @@
         </is>
       </c>
     </row>
-    <row r="66" ht="54" customHeight="1">
-      <c r="A66" s="8" t="inlineStr">
+    <row r="70" ht="54" customHeight="1">
+      <c r="A70" s="8" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B66" s="8" t="inlineStr">
+      <c r="B70" s="8" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_10</t>
         </is>
       </c>
-      <c r="C66" s="9" t="inlineStr">
+      <c r="C70" s="9" t="inlineStr">
         <is>
           <t>SK Uniqueness</t>
         </is>
       </c>
-      <c r="D66" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E66" s="6" t="inlineStr">
+      <c r="D70" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E70" s="6" t="inlineStr">
         <is>
           <t>innotrust.dim_security_characteristics_codes</t>
         </is>
       </c>
-      <c r="F66" s="7" t="inlineStr">
+      <c r="F70" s="7" t="inlineStr">
         <is>
           <t>Verify Primary Surrogate Key (dim_securitycharacteristicscodes) uniqueness and non-null constraint</t>
         </is>
       </c>
-      <c r="G66" s="7" t="inlineStr">
+      <c r="G70" s="7" t="inlineStr">
         <is>
           <t>innotrust.dim_security_characteristics_codes populated</t>
         </is>
       </c>
-      <c r="H66" s="7" t="inlineStr">
+      <c r="H70" s="7" t="inlineStr">
         <is>
           <t>dim_securitycharacteristicscodes is strictly unique across all versions with zero NULLs.</t>
         </is>
       </c>
-      <c r="I66" s="18" t="inlineStr">
+      <c r="I70" s="18" t="inlineStr">
         <is>
           <t>SELECT dim_securitycharacteristicscodes, COUNT(*) AS DuplicateCount
 FROM Gold_Warehouse.innotrust.dim_security_characteristics_codes
@@ -4581,48 +5037,48 @@
         </is>
       </c>
     </row>
-    <row r="67" ht="54" customHeight="1">
-      <c r="A67" s="12" t="inlineStr">
+    <row r="71" ht="54" customHeight="1">
+      <c r="A71" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B67" s="12" t="inlineStr">
+      <c r="B71" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_11</t>
         </is>
       </c>
-      <c r="C67" s="13" t="inlineStr">
+      <c r="C71" s="13" t="inlineStr">
         <is>
           <t>Audit &amp; Date Logic</t>
         </is>
       </c>
-      <c r="D67" s="19" t="inlineStr">
+      <c r="D71" s="19" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E67" s="10" t="inlineStr">
+      <c r="E71" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master</t>
         </is>
       </c>
-      <c r="F67" s="11" t="inlineStr">
+      <c r="F71" s="11" t="inlineStr">
         <is>
           <t>Verify business_date, updated_at, effective_start_date &amp; effective_end_date integrity on active records</t>
         </is>
       </c>
-      <c r="G67" s="11" t="inlineStr">
+      <c r="G71" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master populated</t>
         </is>
       </c>
-      <c r="H67" s="11" t="inlineStr">
+      <c r="H71" s="11" t="inlineStr">
         <is>
           <t>Zero NULLs in business_date or updated_at; effective_end_date &gt;= effective_start_date.</t>
         </is>
       </c>
-      <c r="I67" s="17" t="inlineStr">
+      <c r="I71" s="17" t="inlineStr">
         <is>
           <t>SELECT 
     COUNT(*) AS TotalActiveRows,
@@ -4635,48 +5091,48 @@
         </is>
       </c>
     </row>
-    <row r="68" ht="54" customHeight="1">
-      <c r="A68" s="8" t="inlineStr">
+    <row r="72" ht="54" customHeight="1">
+      <c r="A72" s="8" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B68" s="8" t="inlineStr">
+      <c r="B72" s="8" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_12</t>
         </is>
       </c>
-      <c r="C68" s="9" t="inlineStr">
+      <c r="C72" s="9" t="inlineStr">
         <is>
           <t>Cross-Table Linkage</t>
         </is>
       </c>
-      <c r="D68" s="19" t="inlineStr">
+      <c r="D72" s="19" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E68" s="6" t="inlineStr">
+      <c r="E72" s="6" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master</t>
         </is>
       </c>
-      <c r="F68" s="7" t="inlineStr">
+      <c r="F72" s="7" t="inlineStr">
         <is>
           <t>Verify Referential Integrity: account_category_code and account_type_code resolve to active codes</t>
         </is>
       </c>
-      <c r="G68" s="7" t="inlineStr">
+      <c r="G72" s="7" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master populated</t>
         </is>
       </c>
-      <c r="H68" s="7" t="inlineStr">
+      <c r="H72" s="7" t="inlineStr">
         <is>
           <t>All non-null account_category_code and account_type_code exist in corresponding dimension code tables.</t>
         </is>
       </c>
-      <c r="I68" s="18" t="inlineStr">
+      <c r="I72" s="18" t="inlineStr">
         <is>
           <t>SELECT 
     SUM(CASE WHEN m.account_category_code IS NOT NULL AND cat.account_category_code IS NULL THEN 1 ELSE 0 END) AS Orphan_CategoryCodes,
@@ -4690,48 +5146,48 @@
         </is>
       </c>
     </row>
-    <row r="69" ht="54" customHeight="1">
-      <c r="A69" s="12" t="inlineStr">
+    <row r="73" ht="54" customHeight="1">
+      <c r="A73" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B69" s="12" t="inlineStr">
+      <c r="B73" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_13</t>
         </is>
       </c>
-      <c r="C69" s="13" t="inlineStr">
+      <c r="C73" s="13" t="inlineStr">
         <is>
           <t>Cross-Table Linkage</t>
         </is>
       </c>
-      <c r="D69" s="19" t="inlineStr">
+      <c r="D73" s="19" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E69" s="10" t="inlineStr">
+      <c r="E73" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_master_sec_index</t>
         </is>
       </c>
-      <c r="F69" s="11" t="inlineStr">
+      <c r="F73" s="11" t="inlineStr">
         <is>
           <t>Verify Security Referential Integrity: security_type_code resolves to active security characteristics</t>
         </is>
       </c>
-      <c r="G69" s="11" t="inlineStr">
+      <c r="G73" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_master_sec_index populated</t>
         </is>
       </c>
-      <c r="H69" s="11" t="inlineStr">
+      <c r="H73" s="11" t="inlineStr">
         <is>
           <t>All non-null security_type_code values exist in dim_security_characteristics_codes.</t>
         </is>
       </c>
-      <c r="I69" s="17" t="inlineStr">
+      <c r="I73" s="17" t="inlineStr">
         <is>
           <t>SELECT COUNT(*) AS Orphan_SecurityTypeCodes
 FROM Gold_Warehouse.innotrust.dim_master_sec_index s
@@ -4741,48 +5197,48 @@
         </is>
       </c>
     </row>
-    <row r="70" ht="54" customHeight="1">
-      <c r="A70" s="8" t="inlineStr">
+    <row r="74" ht="54" customHeight="1">
+      <c r="A74" s="8" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B70" s="8" t="inlineStr">
+      <c r="B74" s="8" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_14</t>
         </is>
       </c>
-      <c r="C70" s="9" t="inlineStr">
+      <c r="C74" s="9" t="inlineStr">
         <is>
           <t>SCD2 Date Validation</t>
         </is>
       </c>
-      <c r="D70" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E70" s="6" t="inlineStr">
+      <c r="D74" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E74" s="6" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master</t>
         </is>
       </c>
-      <c r="F70" s="7" t="inlineStr">
+      <c r="F74" s="7" t="inlineStr">
         <is>
           <t>Verify SCD2 Effective Date Rules: Inactive records effective_end_date &lt;= (Current Day - 1), non-null end date, and valid active start date</t>
         </is>
       </c>
-      <c r="G70" s="7" t="inlineStr">
+      <c r="G74" s="7" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master populated with SCD2 tracking columns</t>
         </is>
       </c>
-      <c r="H70" s="7" t="inlineStr">
+      <c r="H74" s="7" t="inlineStr">
         <is>
           <t>Inactive_End_Date_Breach_Count = 0, Inactive_Missing_End_Date = 0, Active_Future_Start_Date = 0, Inverted_Date_Range_Count = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I70" s="18" t="inlineStr">
+      <c r="I74" s="18" t="inlineStr">
         <is>
           <t>SELECT 
     'dim_account_master' AS TableName,
@@ -4801,48 +5257,48 @@
         </is>
       </c>
     </row>
-    <row r="71" ht="54" customHeight="1">
-      <c r="A71" s="12" t="inlineStr">
+    <row r="75" ht="54" customHeight="1">
+      <c r="A75" s="12" t="inlineStr">
         <is>
           <t>Black Diamond (Consolidated)</t>
         </is>
       </c>
-      <c r="B71" s="12" t="inlineStr">
+      <c r="B75" s="12" t="inlineStr">
         <is>
           <t>TC_COMB_SK_BD_01</t>
         </is>
       </c>
-      <c r="C71" s="13" t="inlineStr">
+      <c r="C75" s="13" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D71" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E71" s="10" t="inlineStr">
+      <c r="D75" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E75" s="10" t="inlineStr">
         <is>
           <t>All 9 Child &amp; Fact Tables (holdings, transactions, taxlots, class/segment, details, tags, team, targets)</t>
         </is>
       </c>
-      <c r="F71" s="11" t="inlineStr">
+      <c r="F75" s="11" t="inlineStr">
         <is>
           <t>Black Diamond: Cross-Object account_sk vs dim_accounts Natural Key (accountid == da.id) Verification - Executes a single consolidated UNION ALL query across all 9 child/fact tables to verify that the attached account_sk strictly points to the exact same account natural key (child.accountid == da.id). Guarantees zero wrong account links.</t>
         </is>
       </c>
-      <c r="G71" s="11" t="inlineStr">
+      <c r="G75" s="11" t="inlineStr">
         <is>
           <t>All Gold tables populated for Black Diamond</t>
         </is>
       </c>
-      <c r="H71" s="11" t="inlineStr">
+      <c r="H75" s="11" t="inlineStr">
         <is>
           <t>Duplicate_BusinessKey_Count = 0, MismatchedAccountIdCount = 0, Null_AccountSK_Count = 0, Orphan_AccountSK_Count = 0 across all 9 objects.</t>
         </is>
       </c>
-      <c r="I71" s="17" t="inlineStr">
+      <c r="I75" s="17" t="inlineStr">
         <is>
           <t>SELECT 
     'dim_accounts_classallocation' AS TableName, 
@@ -4951,48 +5407,48 @@
         </is>
       </c>
     </row>
-    <row r="72" ht="54" customHeight="1">
-      <c r="A72" s="8" t="inlineStr">
+    <row r="76" ht="54" customHeight="1">
+      <c r="A76" s="8" t="inlineStr">
         <is>
           <t>Schwab (Consolidated)</t>
         </is>
       </c>
-      <c r="B72" s="8" t="inlineStr">
+      <c r="B76" s="8" t="inlineStr">
         <is>
           <t>TC_COMB_SK_SC_02</t>
         </is>
       </c>
-      <c r="C72" s="9" t="inlineStr">
+      <c r="C76" s="9" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D72" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E72" s="6" t="inlineStr">
+      <c r="D76" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E76" s="6" t="inlineStr">
         <is>
           <t>All 8 Objects (dim_accounts &amp; 7 Fact Tables: recon_d1/d2, daily_closing, security, transactions, ult/uln lots)</t>
         </is>
       </c>
-      <c r="F72" s="7" t="inlineStr">
+      <c r="F76" s="7" t="inlineStr">
         <is>
           <t>Schwab: Consolidated Multi-Object SK Mapping, PK Deduplication &amp; Audit Date Health Check - Single unified query executing across all 8 Schwab Gold tables. Validates that every fact record's account_sk correctly matches dim_accounts on composite natural keys (account_id, custodian_id), confirms primary SK uniqueness, and ensures 100% audit dates populated.</t>
         </is>
       </c>
-      <c r="G72" s="7" t="inlineStr">
+      <c r="G76" s="7" t="inlineStr">
         <is>
           <t>All Gold tables populated for Schwab</t>
         </is>
       </c>
-      <c r="H72" s="7" t="inlineStr">
+      <c r="H76" s="7" t="inlineStr">
         <is>
           <t>Mismatched_AccountId_Count = 0 and Orphan_AccountSK_Count = 0 across all fact tables. All mapped account_sk strictly match the natural account_id.</t>
         </is>
       </c>
-      <c r="I72" s="18" t="inlineStr">
+      <c r="I76" s="18" t="inlineStr">
         <is>
           <t>SELECT 
     'fact_recon_position_d1' AS TableName,
@@ -5051,48 +5507,48 @@
         </is>
       </c>
     </row>
-    <row r="73" ht="54" customHeight="1">
-      <c r="A73" s="12" t="inlineStr">
+    <row r="77" ht="54" customHeight="1">
+      <c r="A77" s="12" t="inlineStr">
         <is>
           <t>Salentica CRM (Consolidated)</t>
         </is>
       </c>
-      <c r="B73" s="12" t="inlineStr">
+      <c r="B77" s="12" t="inlineStr">
         <is>
           <t>TC_COMB_SK_SAL_03</t>
         </is>
       </c>
-      <c r="C73" s="13" t="inlineStr">
+      <c r="C77" s="13" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D73" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E73" s="10" t="inlineStr">
+      <c r="D77" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E77" s="10" t="inlineStr">
         <is>
           <t>All 6 Core CRM Entities (dim_account, dim_contact_core, dim_family, fact_lead, fact_opportunity, fact_investmentaccount)</t>
         </is>
       </c>
-      <c r="F73" s="11" t="inlineStr">
+      <c r="F77" s="11" t="inlineStr">
         <is>
           <t>Salentica: Consolidated Point-in-Time Referential SK Mapping (Active &amp; Historical Mapping Validation) - Single unified query executing across all 6 core Salentica CRM tables. Validates that every attached foreign SK resolves to the same Natural Key in parent dimensions (allowing active OR expired parent versions to preserve point-in-time audit history) and checks for broken orphans.</t>
         </is>
       </c>
-      <c r="G73" s="11" t="inlineStr">
+      <c r="G77" s="11" t="inlineStr">
         <is>
           <t>All Gold tables populated for Salentica CRM</t>
         </is>
       </c>
-      <c r="H73" s="11" t="inlineStr">
+      <c r="H77" s="11" t="inlineStr">
         <is>
           <t>Mismatched_PrimaryContact_NK = 0, Mismatched_BusinessUnit_NK = 0, Broken_Orphan_Count = 0 across all 6 CRM tables.</t>
         </is>
       </c>
-      <c r="I73" s="17" t="inlineStr">
+      <c r="I77" s="17" t="inlineStr">
         <is>
           <t>SELECT 'dim_account' AS TableName, COUNT(*) AS TotalActiveRows,
     SUM(CASE WHEN a.primarycontactid IS NOT NULL AND a.primarycontactid_sk &lt;&gt; -1 AND a.primarycontactid &lt;&gt; c.contactid THEN 1 ELSE 0 END) AS Mismatched_PrimaryContact_NK,
@@ -5156,48 +5612,48 @@
         </is>
       </c>
     </row>
-    <row r="74" ht="54" customHeight="1">
-      <c r="A74" s="8" t="inlineStr">
+    <row r="78" ht="54" customHeight="1">
+      <c r="A78" s="8" t="inlineStr">
         <is>
           <t>Tamarac (Consolidated)</t>
         </is>
       </c>
-      <c r="B74" s="8" t="inlineStr">
+      <c r="B78" s="8" t="inlineStr">
         <is>
           <t>TC_COMB_SK_TAM_04</t>
         </is>
       </c>
-      <c r="C74" s="9" t="inlineStr">
+      <c r="C78" s="9" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D74" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E74" s="6" t="inlineStr">
+      <c r="D78" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E78" s="6" t="inlineStr">
         <is>
           <t>Both Tables (dim_account_information, dim_account_model_allocation)</t>
         </is>
       </c>
-      <c r="F74" s="7" t="inlineStr">
+      <c r="F78" s="7" t="inlineStr">
         <is>
           <t>Tamarac: Consolidated Multi-Object PK Deduplication, Primary SK &amp; Cross-Table Linkage - Single unified query validating SCD2 active uniqueness on exact PK columns (['account_number'] and ['account_number', 'model_name']), surrogate key uniqueness, and cross-table referential integrity between model allocations and accounts.</t>
         </is>
       </c>
-      <c r="G74" s="7" t="inlineStr">
+      <c r="G78" s="7" t="inlineStr">
         <is>
           <t>All Gold tables populated for Tamarac</t>
         </is>
       </c>
-      <c r="H74" s="7" t="inlineStr">
+      <c r="H78" s="7" t="inlineStr">
         <is>
           <t>PK_Active_Duplicates = 0, Duplicate_Primary_SK = 0, Orphan_Accounts = 0, Missing_BusinessDate = 0 across both tables.</t>
         </is>
       </c>
-      <c r="I74" s="18" t="inlineStr">
+      <c r="I78" s="18" t="inlineStr">
         <is>
           <t>SELECT 'dim_account_information' AS TableName, COUNT(*) AS TotalActiveRows,
     (SELECT COUNT(*) FROM (SELECT account_number FROM Gold_Warehouse.tamarac.dim_account_information WHERE is_current = 'True' GROUP BY account_number HAVING COUNT(*) &gt; 1) d) AS PK_Active_Duplicates,
@@ -5220,48 +5676,48 @@
         </is>
       </c>
     </row>
-    <row r="75" ht="54" customHeight="1">
-      <c r="A75" s="12" t="inlineStr">
+    <row r="79" ht="54" customHeight="1">
+      <c r="A79" s="12" t="inlineStr">
         <is>
           <t>Innotrust (Consolidated)</t>
         </is>
       </c>
-      <c r="B75" s="12" t="inlineStr">
+      <c r="B79" s="12" t="inlineStr">
         <is>
           <t>TC_COMB_SK_INNO_05</t>
         </is>
       </c>
-      <c r="C75" s="13" t="inlineStr">
+      <c r="C79" s="13" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D75" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E75" s="10" t="inlineStr">
+      <c r="D79" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E79" s="10" t="inlineStr">
         <is>
           <t>All 5 Innotrust Dimensions (dim_account_master, category_codes, type_codes, sec_index, characteristics)</t>
         </is>
       </c>
-      <c r="F75" s="11" t="inlineStr">
+      <c r="F79" s="11" t="inlineStr">
         <is>
           <t>Innotrust: Consolidated Multi-Object PK Deduplication, Primary SK &amp; Cross-Dimension Linkage - Single unified query validating SCD2 active uniqueness on exact natural keys, primary surrogate key uniqueness, and cross-dimension referential integrity between master entities and classification codes.</t>
         </is>
       </c>
-      <c r="G75" s="11" t="inlineStr">
+      <c r="G79" s="11" t="inlineStr">
         <is>
           <t>All Gold tables populated for Innotrust</t>
         </is>
       </c>
-      <c r="H75" s="11" t="inlineStr">
+      <c r="H79" s="11" t="inlineStr">
         <is>
           <t>PK_Active_Duplicates = 0, Duplicate_Primary_SK = 0, Orphan_Foreign_References = 0, Missing_BusinessDate = 0 across all 5 Innotrust tables.</t>
         </is>
       </c>
-      <c r="I75" s="17" t="inlineStr">
+      <c r="I79" s="17" t="inlineStr">
         <is>
           <t>SELECT 'dim_account_master' AS TableName, COUNT(*) AS TotalActiveRows,
     (SELECT COUNT(*) FROM (SELECT customer_account_number FROM Gold_Warehouse.innotrust.dim_account_master WHERE is_current = 1 GROUP BY customer_account_number HAVING COUNT(*) &gt; 1) d) AS PK_Active_Duplicates,
@@ -5311,48 +5767,48 @@
         </is>
       </c>
     </row>
-    <row r="76" ht="54" customHeight="1">
-      <c r="A76" s="8" t="inlineStr">
+    <row r="80" ht="54" customHeight="1">
+      <c r="A80" s="8" t="inlineStr">
         <is>
           <t>Innotrust (Consolidated)</t>
         </is>
       </c>
-      <c r="B76" s="8" t="inlineStr">
+      <c r="B80" s="8" t="inlineStr">
         <is>
           <t>TC_COMB_SK_INNO_06</t>
         </is>
       </c>
-      <c r="C76" s="9" t="inlineStr">
+      <c r="C80" s="9" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D76" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E76" s="6" t="inlineStr">
+      <c r="D80" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E80" s="6" t="inlineStr">
         <is>
           <t>All 5 Innotrust Dimensions (dim_account_master, category_codes, type_codes, sec_index, characteristics)</t>
         </is>
       </c>
-      <c r="F76" s="7" t="inlineStr">
+      <c r="F80" s="7" t="inlineStr">
         <is>
           <t>Innotrust: Consolidated Multi-Object SCD2 Effective Start &amp; End Date Audit (End Date &lt;= Today - 1) - Validates across all 5 Innotrust dimensions that inactive records (is_current = 0) have effective_end_date &lt;= (current day - 1), non-null end dates, active records have non-future start dates, and zero inverted date ranges.</t>
         </is>
       </c>
-      <c r="G76" s="7" t="inlineStr">
+      <c r="G80" s="7" t="inlineStr">
         <is>
           <t>All Gold tables populated for Innotrust</t>
         </is>
       </c>
-      <c r="H76" s="7" t="inlineStr">
+      <c r="H80" s="7" t="inlineStr">
         <is>
           <t>Inactive_End_Date_Breach_Count = 0, Inactive_Missing_End_Date = 0, Active_Future_Start_Date = 0, Inverted_Date_Range_Count = 0 across all 5 tables.</t>
         </is>
       </c>
-      <c r="I76" s="18" t="inlineStr">
+      <c r="I80" s="18" t="inlineStr">
         <is>
           <t>SELECT 
     'dim_account_master' AS TableName,
@@ -5445,7 +5901,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6352,6 +6808,442 @@
     SUM(CASE WHEN tl.account_sk IS NULL THEN 1 ELSE 0 END) AS Null_AccountSK_Count
 FROM Gold_Warehouse.black_diamond.fact_accounts_taxlots tl
 LEFT JOIN Gold_Warehouse.black_diamond.dim_accounts da ON tl.account_sk = da.accounts_SK;</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="54" customHeight="1">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>TC_BD_GOLD_19</t>
+        </is>
+      </c>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>SCD2 Inactive Date Rules</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D21" s="10" t="inlineStr">
+        <is>
+          <t>black_diamond.dim_accounts (and ALL 13 Dim Tables)</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="inlineStr">
+        <is>
+          <t>Verify SCD2 Timeline &amp; Date Rules across ALL 13 Dim Tables: Inactive records (iscurrent = 'False') must have effectiveenddate &lt;= Latest_Batch_Date - 1, Active records must be open-ended, zero inverted dates</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>All 13 Black Diamond dimension tables loaded with SCD2 tracking columns</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="inlineStr">
+        <is>
+          <t>Defect_Inactive_EndDate_Not_DayMinus1 = 0, Defect_Active_Prematurely_Closed = 0, Defect_Inverted_Dates = 0, Defect_Future_Active_StartDate = 0 across all 13 tables. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="H21" s="17" t="inlineStr">
+        <is>
+          <t>;WITH DimSCD2Audit AS (
+    SELECT 'dim_accounts' AS TableName, COUNT(*) AS TotalRecords, MAX(file_business_date) AS LatestBatchDate,
+        SUM(CASE WHEN iscurrent = 'True' THEN 1 ELSE 0 END) AS Active_Count,
+        SUM(CASE WHEN iscurrent = 'False' THEN 1 ELSE 0 END) AS Inactive_Count,
+        SUM(CASE WHEN iscurrent = 'False' AND (effectiveenddate IS NULL OR effectiveenddate &gt; DATEADD(day, -1, b.MaxBatchDate)) THEN 1 ELSE 0 END) AS Defect_Inactive_EndDate_Not_DayMinus1,
+        SUM(CASE WHEN iscurrent = 'True' AND effectiveenddate IS NOT NULL AND effectiveenddate NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END) AS Defect_Active_Prematurely_Closed,
+        SUM(CASE WHEN effectiveenddate &lt; effectivestartdate THEN 1 ELSE 0 END) AS Defect_Inverted_Dates,
+        SUM(CASE WHEN iscurrent = 'True' AND effectivestartdate &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END) AS Defect_Future_Active_StartDate
+    FROM Gold_Warehouse.black_diamond.dim_accounts
+    CROSS JOIN (SELECT MAX(file_business_date) AS MaxBatchDate FROM Gold_Warehouse.black_diamond.dim_accounts) b
+    GROUP BY b.MaxBatchDate
+    UNION ALL
+    SELECT 'dim_asset', COUNT(*), MAX(file_business_date),
+        SUM(CASE WHEN iscurrent = 'True' THEN 1 ELSE 0 END), SUM(CASE WHEN iscurrent = 'False' THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'False' AND (effectiveenddate IS NULL OR effectiveenddate &gt; DATEADD(day, -1, b.MaxBatchDate)) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectiveenddate IS NOT NULL AND effectiveenddate NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END),
+        SUM(CASE WHEN effectiveenddate &lt; effectivestartdate THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectivestartdate &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.dim_asset
+    CROSS JOIN (SELECT MAX(file_business_date) AS MaxBatchDate FROM Gold_Warehouse.black_diamond.dim_asset) b GROUP BY b.MaxBatchDate
+    UNION ALL
+    SELECT 'dim_client', COUNT(*), MAX(file_business_date),
+        SUM(CASE WHEN iscurrent = 'True' THEN 1 ELSE 0 END), SUM(CASE WHEN iscurrent = 'False' THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'False' AND (effectiveenddate IS NULL OR effectiveenddate &gt; DATEADD(day, -1, b.MaxBatchDate)) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectiveenddate IS NOT NULL AND effectiveenddate NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END),
+        SUM(CASE WHEN effectiveenddate &lt; effectivestartdate THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectivestartdate &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.dim_client
+    CROSS JOIN (SELECT MAX(file_business_date) AS MaxBatchDate FROM Gold_Warehouse.black_diamond.dim_client) b GROUP BY b.MaxBatchDate
+    UNION ALL
+    SELECT 'dim_contact', COUNT(*), MAX(file_business_date),
+        SUM(CASE WHEN iscurrent = 'True' THEN 1 ELSE 0 END), SUM(CASE WHEN iscurrent = 'False' THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'False' AND (effectiveenddate IS NULL OR effectiveenddate &gt; DATEADD(day, -1, b.MaxBatchDate)) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectiveenddate IS NOT NULL AND effectiveenddate NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END),
+        SUM(CASE WHEN effectiveenddate &lt; effectivestartdate THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectivestartdate &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.dim_contact
+    CROSS JOIN (SELECT MAX(file_business_date) AS MaxBatchDate FROM Gold_Warehouse.black_diamond.dim_contact) b GROUP BY b.MaxBatchDate
+    UNION ALL
+    SELECT 'dim_portfoliogroup', COUNT(*), MAX(file_business_date),
+        SUM(CASE WHEN iscurrent = 'True' THEN 1 ELSE 0 END), SUM(CASE WHEN iscurrent = 'False' THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'False' AND (effectiveenddate IS NULL OR effectiveenddate &gt; DATEADD(day, -1, b.MaxBatchDate)) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectiveenddate IS NOT NULL AND effectiveenddate NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END),
+        SUM(CASE WHEN effectiveenddate &lt; effectivestartdate THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectivestartdate &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.dim_portfoliogroup
+    CROSS JOIN (SELECT MAX(file_business_date) AS MaxBatchDate FROM Gold_Warehouse.black_diamond.dim_portfoliogroup) b GROUP BY b.MaxBatchDate
+    UNION ALL
+    SELECT 'dim_relationshipv2', COUNT(*), MAX(file_business_date),
+        SUM(CASE WHEN iscurrent = 'True' THEN 1 ELSE 0 END), SUM(CASE WHEN iscurrent = 'False' THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'False' AND (effectiveenddate IS NULL OR effectiveenddate &gt; DATEADD(day, -1, b.MaxBatchDate)) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectiveenddate IS NOT NULL AND effectiveenddate NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END),
+        SUM(CASE WHEN effectiveenddate &lt; effectivestartdate THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectivestartdate &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.dim_relationshipv2
+    CROSS JOIN (SELECT MAX(file_business_date) AS MaxBatchDate FROM Gold_Warehouse.black_diamond.dim_relationshipv2) b GROUP BY b.MaxBatchDate
+    UNION ALL
+    SELECT 'dim_target', COUNT(*), MAX(file_business_date),
+        SUM(CASE WHEN iscurrent = 'True' THEN 1 ELSE 0 END), SUM(CASE WHEN iscurrent = 'False' THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'False' AND (effectiveenddate IS NULL OR effectiveenddate &gt; DATEADD(day, -1, b.MaxBatchDate)) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectiveenddate IS NOT NULL AND effectiveenddate NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END),
+        SUM(CASE WHEN effectiveenddate &lt; effectivestartdate THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectivestartdate &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.dim_target
+    CROSS JOIN (SELECT MAX(file_business_date) AS MaxBatchDate FROM Gold_Warehouse.black_diamond.dim_target) b GROUP BY b.MaxBatchDate
+    UNION ALL
+    SELECT 'dim_accounts_classallocation', COUNT(*), MAX(file_business_date),
+        SUM(CASE WHEN iscurrent = 'True' THEN 1 ELSE 0 END), SUM(CASE WHEN iscurrent = 'False' THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'False' AND (effectiveenddate IS NULL OR effectiveenddate &gt; DATEADD(day, -1, b.MaxBatchDate)) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectiveenddate IS NOT NULL AND effectiveenddate NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END),
+        SUM(CASE WHEN effectiveenddate &lt; effectivestartdate THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectivestartdate &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.dim_accounts_classallocation
+    CROSS JOIN (SELECT MAX(file_business_date) AS MaxBatchDate FROM Gold_Warehouse.black_diamond.dim_accounts_classallocation) b GROUP BY b.MaxBatchDate
+    UNION ALL
+    SELECT 'dim_accounts_details', COUNT(*), MAX(file_business_date),
+        SUM(CASE WHEN iscurrent = 'True' THEN 1 ELSE 0 END), SUM(CASE WHEN iscurrent = 'False' THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'False' AND (effectiveenddate IS NULL OR effectiveenddate &gt; DATEADD(day, -1, b.MaxBatchDate)) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectiveenddate IS NOT NULL AND effectiveenddate NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END),
+        SUM(CASE WHEN effectiveenddate &lt; effectivestartdate THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectivestartdate &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.dim_accounts_details
+    CROSS JOIN (SELECT MAX(file_business_date) AS MaxBatchDate FROM Gold_Warehouse.black_diamond.dim_accounts_details) b GROUP BY b.MaxBatchDate
+    UNION ALL
+    SELECT 'dim_accounts_segmentallocation', COUNT(*), MAX(file_business_date),
+        SUM(CASE WHEN iscurrent = 'True' THEN 1 ELSE 0 END), SUM(CASE WHEN iscurrent = 'False' THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'False' AND (effectiveenddate IS NULL OR effectiveenddate &gt; DATEADD(day, -1, b.MaxBatchDate)) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectiveenddate IS NOT NULL AND effectiveenddate NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END),
+        SUM(CASE WHEN effectiveenddate &lt; effectivestartdate THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectivestartdate &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.dim_accounts_segmentallocation
+    CROSS JOIN (SELECT MAX(file_business_date) AS MaxBatchDate FROM Gold_Warehouse.black_diamond.dim_accounts_segmentallocation) b GROUP BY b.MaxBatchDate
+    UNION ALL
+    SELECT 'dim_accounts_tags', COUNT(*), MAX(file_business_date),
+        SUM(CASE WHEN iscurrent = 'True' THEN 1 ELSE 0 END), SUM(CASE WHEN iscurrent = 'False' THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'False' AND (effectiveenddate IS NULL OR effectiveenddate &gt; DATEADD(day, -1, b.MaxBatchDate)) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectiveenddate IS NOT NULL AND effectiveenddate NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END),
+        SUM(CASE WHEN effectiveenddate &lt; effectivestartdate THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectivestartdate &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.dim_accounts_tags
+    CROSS JOIN (SELECT MAX(file_business_date) AS MaxBatchDate FROM Gold_Warehouse.black_diamond.dim_accounts_tags) b GROUP BY b.MaxBatchDate
+    UNION ALL
+    SELECT 'dim_accounts_targets', COUNT(*), MAX(file_business_date),
+        SUM(CASE WHEN iscurrent = 'True' THEN 1 ELSE 0 END), SUM(CASE WHEN iscurrent = 'False' THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'False' AND (effectiveenddate IS NULL OR effectiveenddate &gt; DATEADD(day, -1, b.MaxBatchDate)) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectiveenddate IS NOT NULL AND effectiveenddate NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END),
+        SUM(CASE WHEN effectiveenddate &lt; effectivestartdate THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectivestartdate &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.dim_accounts_targets
+    CROSS JOIN (SELECT MAX(file_business_date) AS MaxBatchDate FROM Gold_Warehouse.black_diamond.dim_accounts_targets) b GROUP BY b.MaxBatchDate
+    UNION ALL
+    SELECT 'dim_accounts_team', COUNT(*), MAX(file_business_date),
+        SUM(CASE WHEN iscurrent = 'True' THEN 1 ELSE 0 END), SUM(CASE WHEN iscurrent = 'False' THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'False' AND (effectiveenddate IS NULL OR effectiveenddate &gt; DATEADD(day, -1, b.MaxBatchDate)) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectiveenddate IS NOT NULL AND effectiveenddate NOT IN ('9999-12-31', '2099-12-31') THEN 1 ELSE 0 END),
+        SUM(CASE WHEN effectiveenddate &lt; effectivestartdate THEN 1 ELSE 0 END),
+        SUM(CASE WHEN iscurrent = 'True' AND effectivestartdate &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.dim_accounts_team
+    CROSS JOIN (SELECT MAX(file_business_date) AS MaxBatchDate FROM Gold_Warehouse.black_diamond.dim_accounts_team) b GROUP BY b.MaxBatchDate
+)
+SELECT 
+    TableName, TotalRecords, LatestBatchDate, Active_Count, Inactive_Count,
+    Defect_Inactive_EndDate_Not_DayMinus1, Defect_Active_Prematurely_Closed, Defect_Inverted_Dates, Defect_Future_Active_StartDate,
+    CASE 
+        WHEN Defect_Inactive_EndDate_Not_DayMinus1 = 0 AND Defect_Active_Prematurely_Closed = 0 AND Defect_Inverted_Dates = 0 AND Defect_Future_Active_StartDate = 0 THEN 'PASSED'
+        ELSE 'FAILED'
+    END AS TestStatus
+FROM DimSCD2Audit;</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="54" customHeight="1">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>TC_BD_GOLD_20</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Version Evolution Audit</t>
+        </is>
+      </c>
+      <c r="C22" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>black_diamond.dim_accounts</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>Verify SCD2 Version Evolution: Monotonic accounts_SK increments, advancing effectivestartdate, continuous timeline (effectiveenddate = next effectivestartdate - 1), and latest version active</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>dim_accounts with multiple version rows per id</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>Reused_Or_NonIncrementing_SK_Count = 0, NonAdvancing_EffectiveStartDate_Count = 0, Timeline_Gap_Or_Overlap_Count = 0, LatestVersion_Not_Active_Count = 0. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="H22" s="18" t="inlineStr">
+        <is>
+          <t>;WITH VersionChains AS (
+    SELECT 
+        id, accounts_SK, effectivestartdate, effectiveenddate, iscurrent, file_business_date, updatedat,
+        LEAD(accounts_SK) OVER (PARTITION BY id ORDER BY effectivestartdate, accounts_SK) AS next_sk,
+        LEAD(effectivestartdate) OVER (PARTITION BY id ORDER BY effectivestartdate, accounts_SK) AS next_start_date,
+        ROW_NUMBER() OVER (PARTITION BY id ORDER BY effectivestartdate DESC, accounts_SK DESC) AS rn_latest
+    FROM Gold_Warehouse.black_diamond.dim_accounts
+)
+SELECT 
+    'black_diamond.dim_accounts' AS TableName,
+    'Version Evolution &amp; Progression' AS TestName,
+    COUNT(*) AS TotalVersionsAudited,
+    SUM(CASE WHEN next_sk IS NOT NULL AND next_sk &lt;= accounts_SK THEN 1 ELSE 0 END) AS Reused_Or_NonIncrementing_SK_Count,
+    SUM(CASE WHEN next_start_date IS NOT NULL AND next_start_date &lt;= effectivestartdate THEN 1 ELSE 0 END) AS NonAdvancing_EffectiveStartDate_Count,
+    SUM(CASE WHEN next_start_date IS NOT NULL AND effectiveenddate &lt;&gt; DATEADD(day, -1, next_start_date) THEN 1 ELSE 0 END) AS Timeline_Gap_Or_Overlap_Count,
+    SUM(CASE WHEN rn_latest = 1 AND iscurrent &lt;&gt; 'True' THEN 1 ELSE 0 END) AS LatestVersion_Not_Active_Count,
+    CASE 
+        WHEN SUM(CASE WHEN next_sk IS NOT NULL AND next_sk &lt;= accounts_SK THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN next_start_date IS NOT NULL AND next_start_date &lt;= effectivestartdate THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN next_start_date IS NOT NULL AND effectiveenddate &lt;&gt; DATEADD(day, -1, next_start_date) THEN 1 ELSE 0 END) = 0
+         AND SUM(CASE WHEN rn_latest = 1 AND iscurrent &lt;&gt; 'True' THEN 1 ELSE 0 END) = 0
+        THEN 'PASSED' ELSE 'FAILED'
+    END AS TestStatus
+FROM VersionChains;</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="54" customHeight="1">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>TC_BD_GOLD_21</t>
+        </is>
+      </c>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>Foreign SK Referential Mapping</t>
+        </is>
+      </c>
+      <c r="C23" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="inlineStr">
+        <is>
+          <t>black_diamond (ALL 6 Child Dims + 3 Fact Tables)</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>Verify Consolidated account_sk Mapping: Audits that all 6 Child Dimensions and 3 Fact Tables have their attached account_sk strictly mapped to the exact matching id in dim_accounts</t>
+        </is>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>dim_accounts_classallocation, details, segmentallocation, tags, targets, team, holdings, transactions, taxlots populated</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="inlineStr">
+        <is>
+          <t>Defect_Orphan_Unmapped_SK = 0 and Defect_Wrong_Account_Mismatch = 0 across all 9 tables. Exact_Account_Match_Count covers 100% of rows. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="H23" s="17" t="inlineStr">
+        <is>
+          <t>;WITH AccountSKAudit AS (
+    SELECT 'dim_accounts_classallocation' AS TableName, 'Child Dimension' AS ObjectType, COUNT(*) AS TotalRecords,
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND c.accountid = da.id THEN 1 ELSE 0 END) AS Exact_Account_Match_Count,
+        SUM(CASE WHEN c.account_sk = -1 OR c.account_sk IS NULL OR da.accounts_SK IS NULL THEN 1 ELSE 0 END) AS Defect_Orphan_Unmapped_SK,
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND c.accountid &lt;&gt; da.id THEN 1 ELSE 0 END) AS Defect_Wrong_Account_Mismatch
+    FROM Gold_Warehouse.black_diamond.dim_accounts_classallocation c
+    LEFT JOIN Gold_Warehouse.black_diamond.dim_accounts da ON c.account_sk = da.accounts_SK
+    UNION ALL
+    SELECT 'dim_accounts_details', 'Child Dimension', COUNT(*),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND d.accountid = da.id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN d.account_sk = -1 OR d.account_sk IS NULL OR da.accounts_SK IS NULL THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND d.accountid &lt;&gt; da.id THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.dim_accounts_details d
+    LEFT JOIN Gold_Warehouse.black_diamond.dim_accounts da ON d.account_sk = da.accounts_SK
+    UNION ALL
+    SELECT 'dim_accounts_segmentallocation', 'Child Dimension', COUNT(*),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND s.accountid = da.id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN s.account_sk = -1 OR s.account_sk IS NULL OR da.accounts_SK IS NULL THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND s.accountid &lt;&gt; da.id THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.dim_accounts_segmentallocation s
+    LEFT JOIN Gold_Warehouse.black_diamond.dim_accounts da ON s.account_sk = da.accounts_SK
+    UNION ALL
+    SELECT 'dim_accounts_tags', 'Child Dimension', COUNT(*),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND t.accountid = da.id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN t.account_sk = -1 OR t.account_sk IS NULL OR da.accounts_SK IS NULL THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND t.accountid &lt;&gt; da.id THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.dim_accounts_tags t
+    LEFT JOIN Gold_Warehouse.black_diamond.dim_accounts da ON t.account_sk = da.accounts_SK
+    UNION ALL
+    SELECT 'dim_accounts_targets', 'Child Dimension', COUNT(*),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND tg.accountid = da.id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN tg.account_sk = -1 OR tg.account_sk IS NULL OR da.accounts_SK IS NULL THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND tg.accountid &lt;&gt; da.id THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.dim_accounts_targets tg
+    LEFT JOIN Gold_Warehouse.black_diamond.dim_accounts da ON tg.account_sk = da.accounts_SK
+    UNION ALL
+    SELECT 'dim_accounts_team', 'Child Dimension', COUNT(*),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND tm.accountid = da.id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN tm.account_sk = -1 OR tm.account_sk IS NULL OR da.accounts_SK IS NULL THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND tm.accountid &lt;&gt; da.id THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.dim_accounts_team tm
+    LEFT JOIN Gold_Warehouse.black_diamond.dim_accounts da ON tm.account_sk = da.accounts_SK
+    UNION ALL
+    SELECT 'fact_accounts_holdings', 'Fact Table', COUNT(*),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND h.accountid = da.id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN h.account_sk = -1 OR h.account_sk IS NULL OR da.accounts_SK IS NULL THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND h.accountid &lt;&gt; da.id THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.fact_accounts_holdings h
+    LEFT JOIN Gold_Warehouse.black_diamond.dim_accounts da ON h.account_sk = da.accounts_SK
+    UNION ALL
+    SELECT 'fact_accounts_transactions', 'Fact Table', COUNT(*),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND tx.accountid = da.id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN tx.account_sk = -1 OR tx.account_sk IS NULL OR da.accounts_SK IS NULL THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND tx.accountid &lt;&gt; da.id THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.fact_accounts_transactions tx
+    LEFT JOIN Gold_Warehouse.black_diamond.dim_accounts da ON tx.account_sk = da.accounts_SK
+    UNION ALL
+    SELECT 'fact_accounts_taxlots', 'Fact Table', COUNT(*),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND tl.accountid = da.id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN tl.account_sk = -1 OR tl.account_sk IS NULL OR da.accounts_SK IS NULL THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND tl.accountid &lt;&gt; da.id THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.fact_accounts_taxlots tl
+    LEFT JOIN Gold_Warehouse.black_diamond.dim_accounts da ON tl.account_sk = da.accounts_SK
+)
+SELECT TableName, ObjectType, TotalRecords, Exact_Account_Match_Count, Defect_Orphan_Unmapped_SK, Defect_Wrong_Account_Mismatch,
+    CASE WHEN Defect_Orphan_Unmapped_SK = 0 AND Defect_Wrong_Account_Mismatch = 0 THEN 'PASSED' ELSE 'FAILED' END AS TestStatus
+FROM AccountSKAudit;</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="54" customHeight="1">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>TC_BD_GOLD_22</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Fact Health &amp; Historical Retention</t>
+        </is>
+      </c>
+      <c r="C24" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>black_diamond.fact_accounts_holdings, fact_accounts_transactions, fact_accounts_taxlots</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>Verify Fact Tables Health: Active SK mapping for fresh runs, historical closed version preservation for unrepeated rows, exact natural account match, and orphan SK detection</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>All 3 Black Diamond Fact tables loaded into Gold Warehouse</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>Fresh records map to active SK (iscurrent = 'True'), past records retain historical SK, Exact_Account_Match_Count covers all non-orphan rows, Defect_Orphan_Unmapped_SK = 0, Defect_Wrong_Account_Mismatch = 0. OverallStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="H24" s="18" t="inlineStr">
+        <is>
+          <t>;WITH MaxRuns AS (
+    SELECT 'fact_accounts_holdings' AS TableName, MAX(updatedat) AS LatestRunTimestamp FROM Gold_Warehouse.black_diamond.fact_accounts_holdings UNION ALL
+    SELECT 'fact_accounts_transactions', MAX(updatedat) FROM Gold_Warehouse.black_diamond.fact_accounts_transactions UNION ALL
+    SELECT 'fact_accounts_taxlots', MAX(updatedat) FROM Gold_Warehouse.black_diamond.fact_accounts_taxlots
+),
+FactBreakdown AS (
+    SELECT 'fact_accounts_holdings' AS TableName, COUNT(*) AS TotalFactRows, MAX(f.file_business_date) AS LatestBatchDate,
+        SUM(CASE WHEN f.updatedat = m.LatestRunTimestamp AND da.iscurrent = 'True' AND f.accountid = da.id THEN 1 ELSE 0 END) AS Fresh_Run_Active_Mapped,
+        SUM(CASE WHEN f.updatedat &lt; m.LatestRunTimestamp AND da.iscurrent = 'True' AND f.accountid = da.id THEN 1 ELSE 0 END) AS Past_Run_Active_Retained,
+        SUM(CASE WHEN f.updatedat &lt; m.LatestRunTimestamp AND da.iscurrent = 'False' AND f.accountid = da.id THEN 1 ELSE 0 END) AS Past_Run_Expired_Version_Retained,
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND f.accountid = da.id THEN 1 ELSE 0 END) AS Exact_Account_Match_Count,
+        SUM(CASE WHEN f.account_sk = -1 OR da.accounts_SK IS NULL THEN 1 ELSE 0 END) AS Defect_Orphan_Unmapped_SK,
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND f.accountid &lt;&gt; da.id THEN 1 ELSE 0 END) AS Defect_Wrong_Account_Mismatch
+    FROM Gold_Warehouse.black_diamond.fact_accounts_holdings f
+    JOIN MaxRuns m ON m.TableName = 'fact_accounts_holdings'
+    LEFT JOIN Gold_Warehouse.black_diamond.dim_accounts da ON f.account_sk = da.accounts_SK
+    GROUP BY m.LatestRunTimestamp
+    UNION ALL
+    SELECT 'fact_accounts_transactions', COUNT(*), MAX(f.file_business_date),
+        SUM(CASE WHEN f.updatedat = m.LatestRunTimestamp AND da.iscurrent = 'True' AND f.accountid = da.id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.updatedat &lt; m.LatestRunTimestamp AND da.iscurrent = 'True' AND f.accountid = da.id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.updatedat &lt; m.LatestRunTimestamp AND da.iscurrent = 'False' AND f.accountid = da.id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND f.accountid = da.id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.account_sk = -1 OR da.accounts_SK IS NULL THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND f.accountid &lt;&gt; da.id THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.fact_accounts_transactions f
+    JOIN MaxRuns m ON m.TableName = 'fact_accounts_transactions'
+    LEFT JOIN Gold_Warehouse.black_diamond.dim_accounts da ON f.account_sk = da.accounts_SK
+    GROUP BY m.LatestRunTimestamp
+    UNION ALL
+    SELECT 'fact_accounts_taxlots', COUNT(*), MAX(f.file_business_date),
+        SUM(CASE WHEN f.updatedat = m.LatestRunTimestamp AND da.iscurrent = 'True' AND f.accountid = da.id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.updatedat &lt; m.LatestRunTimestamp AND da.iscurrent = 'True' AND f.accountid = da.id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.updatedat &lt; m.LatestRunTimestamp AND da.iscurrent = 'False' AND f.accountid = da.id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND f.accountid = da.id THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.account_sk = -1 OR da.accounts_SK IS NULL THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.accounts_SK IS NOT NULL AND f.accountid &lt;&gt; da.id THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.black_diamond.fact_accounts_taxlots f
+    JOIN MaxRuns m ON m.TableName = 'fact_accounts_taxlots'
+    LEFT JOIN Gold_Warehouse.black_diamond.dim_accounts da ON f.account_sk = da.accounts_SK
+    GROUP BY m.LatestRunTimestamp
+)
+SELECT 
+    TableName, TotalFactRows, LatestBatchDate, Fresh_Run_Active_Mapped, Past_Run_Active_Retained,
+    Past_Run_Expired_Version_Retained AS Historical_Closed_Version_Retained, Exact_Account_Match_Count,
+    Defect_Orphan_Unmapped_SK, Defect_Wrong_Account_Mismatch,
+    CASE WHEN Defect_Orphan_Unmapped_SK = 0 AND Defect_Wrong_Account_Mismatch = 0 THEN 'PASSED' ELSE 'FAILED' END AS OverallStatus,
+    CASE 
+        WHEN Defect_Orphan_Unmapped_SK &gt; 0 THEN CONCAT(Defect_Orphan_Unmapped_SK, ' Orphan Record(s) (SK = -1)')
+        WHEN Defect_Wrong_Account_Mismatch &gt; 0 THEN 'Account Mismatch Defect'
+        ELSE 'All Active &amp; Historical Records Correctly Preserved'
+    END AS Remarks
+FROM FactBreakdown;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update Fabric SQL endpoint to tnixybw3f7kejjy4dnqgavvt64 and remove effective date checks from Innotrust
</commit_message>
<xml_diff>
--- a/Gold_Data_Validation_Test_Cases.xlsx
+++ b/Gold_Data_Validation_Test_Cases.xlsx
@@ -653,7 +653,7 @@
         <v>17</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" ht="26" customHeight="1">
@@ -767,10 +767,10 @@
         </is>
       </c>
       <c r="C10" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D10" s="9" t="n">
         <v>8</v>
-      </c>
-      <c r="D10" s="9" t="n">
-        <v>6</v>
       </c>
       <c r="E10" s="9" t="n">
         <v>2</v>
@@ -829,10 +829,10 @@
         </is>
       </c>
       <c r="C12" s="8" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E12" s="9" t="n">
         <v>3</v>
@@ -3582,45 +3582,237 @@
     <row r="45" ht="54" customHeight="1">
       <c r="A45" s="12" t="inlineStr">
         <is>
+          <t>Salentica</t>
+        </is>
+      </c>
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>TC_SAL_GOLD_08</t>
+        </is>
+      </c>
+      <c r="C45" s="13" t="inlineStr">
+        <is>
+          <t>Foreign SK Referential Mapping</t>
+        </is>
+      </c>
+      <c r="D45" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E45" s="10" t="inlineStr">
+        <is>
+          <t>salentica (dim_account, dim_contact_core, fact_opportunity, fact_lead)</t>
+        </is>
+      </c>
+      <c r="F45" s="11" t="inlineStr">
+        <is>
+          <t>Verify Consolidated SK Referential Mapping: Audits that all foreign SKs in dimensions and facts resolve to exact matching natural keys in parent entities</t>
+        </is>
+      </c>
+      <c r="G45" s="11" t="inlineStr">
+        <is>
+          <t>dim_account, dim_contact_core, dim_businessunit, fact_opportunity, fact_lead populated</t>
+        </is>
+      </c>
+      <c r="H45" s="11" t="inlineStr">
+        <is>
+          <t>Defect_Orphan_Unmapped_SK = 0 and Defect_Wrong_Account_Mismatch = 0 across all entities. Exact_NaturalKey_Match_Count covers 100% of rows. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="I45" s="17" t="inlineStr">
+        <is>
+          <t>;WITH SalenticaSKAudit AS (
+    SELECT 'dim_account (Contact &amp; BU Links)' AS ObjectRelationship, 'Dimension Table' AS ObjectType, COUNT(*) AS TotalRecords,
+        SUM(CASE WHEN (a.primarycontactid IS NOT NULL AND a.primarycontactid_sk &lt;&gt; -1 AND a.primarycontactid = c.contactid)
+                   OR (a.owningbusinessunit IS NOT NULL AND a.owningbusinessunit_sk &lt;&gt; -1 AND a.owningbusinessunit = bu.businessunitid) THEN 1 ELSE 0 END) AS Exact_NaturalKey_Match_Count,
+        SUM(CASE WHEN (a.primarycontactid IS NOT NULL AND (a.primarycontactid_sk = -1 OR c.contact_SK IS NULL))
+                   OR (a.owningbusinessunit IS NOT NULL AND (a.owningbusinessunit_sk = -1 OR bu.businessunit_SK IS NULL)) THEN 1 ELSE 0 END) AS Defect_Orphan_Unmapped_SK,
+        SUM(CASE WHEN (a.primarycontactid IS NOT NULL AND a.primarycontactid_sk &lt;&gt; -1 AND c.contact_SK IS NOT NULL AND a.primarycontactid &lt;&gt; c.contactid)
+                   OR (a.owningbusinessunit IS NOT NULL AND a.owningbusinessunit_sk &lt;&gt; -1 AND bu.businessunit_SK IS NOT NULL AND a.owningbusinessunit &lt;&gt; bu.businessunitid) THEN 1 ELSE 0 END) AS Defect_Wrong_Account_Mismatch
+    FROM Gold_Warehouse.salentica.dim_account a
+    LEFT JOIN Gold_Warehouse.salentica.dim_contact_core c ON a.primarycontactid_sk = c.contact_SK
+    LEFT JOIN Gold_Warehouse.salentica.dim_businessunit bu ON a.owningbusinessunit_sk = bu.businessunit_SK
+    UNION ALL
+    SELECT 'dim_contact_core (Account &amp; BU Links)', 'Dimension Table', COUNT(*),
+        SUM(CASE WHEN (c.accountid IS NOT NULL AND c.accountid_sk &lt;&gt; -1 AND c.accountid = a.accountid)
+                   OR (c.owningbusinessunit IS NOT NULL AND c.owningbusinessunit_sk &lt;&gt; -1 AND c.owningbusinessunit = bu.businessunitid) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN (c.accountid IS NOT NULL AND (c.accountid_sk = -1 OR a.account_SK IS NULL))
+                   OR (c.owningbusinessunit IS NOT NULL AND (c.owningbusinessunit_sk = -1 OR bu.businessunit_SK IS NULL)) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN (c.accountid IS NOT NULL AND c.accountid_sk &lt;&gt; -1 AND a.account_SK IS NOT NULL AND c.accountid &lt;&gt; a.accountid)
+                   OR (c.owningbusinessunit IS NOT NULL AND c.owningbusinessunit_sk &lt;&gt; -1 AND bu.businessunit_SK IS NOT NULL AND c.owningbusinessunit &lt;&gt; bu.businessunitid) THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.salentica.dim_contact_core c
+    LEFT JOIN Gold_Warehouse.salentica.dim_account a ON c.accountid_sk = a.account_SK
+    LEFT JOIN Gold_Warehouse.salentica.dim_businessunit bu ON c.owningbusinessunit_sk = bu.businessunit_SK
+    UNION ALL
+    SELECT 'fact_opportunity (Account &amp; Contact Links)', 'Fact Table', COUNT(*),
+        SUM(CASE WHEN (o.accountid IS NOT NULL AND o.accountid_sk &lt;&gt; -1 AND o.accountid = a.accountid)
+                   OR (o.contactid IS NOT NULL AND o.contactid_sk &lt;&gt; -1 AND o.contactid = c.contactid) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN (o.accountid IS NOT NULL AND (o.accountid_sk = -1 OR a.account_SK IS NULL))
+                   OR (o.contactid IS NOT NULL AND (o.contactid_sk = -1 OR c.contact_SK IS NULL)) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN (o.accountid IS NOT NULL AND o.accountid_sk &lt;&gt; -1 AND a.account_SK IS NOT NULL AND o.accountid &lt;&gt; a.accountid)
+                   OR (o.contactid IS NOT NULL AND o.contactid_sk &lt;&gt; -1 AND c.contact_SK IS NOT NULL AND o.contactid &lt;&gt; c.contactid) THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.salentica.fact_opportunity o
+    LEFT JOIN Gold_Warehouse.salentica.dim_account a ON o.accountid_sk = a.account_SK
+    LEFT JOIN Gold_Warehouse.salentica.dim_contact_core c ON o.contactid_sk = c.contact_SK
+    UNION ALL
+    SELECT 'fact_lead (Account &amp; Contact Links)', 'Fact Table', COUNT(*),
+        SUM(CASE WHEN (l.accountid IS NOT NULL AND l.accountid_sk &lt;&gt; -1 AND l.accountid = a.accountid)
+                   OR (l.contactid IS NOT NULL AND l.contactid_sk &lt;&gt; -1 AND l.contactid = c.contactid) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN (l.accountid IS NOT NULL AND (l.accountid_sk = -1 OR a.account_SK IS NULL))
+                   OR (l.contactid IS NOT NULL AND (l.contactid_sk = -1 OR c.contact_SK IS NULL)) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN (l.accountid IS NOT NULL AND l.accountid_sk &lt;&gt; -1 AND a.account_SK IS NOT NULL AND l.accountid &lt;&gt; a.accountid)
+                   OR (l.contactid IS NOT NULL AND l.contactid_sk &lt;&gt; -1 AND c.contact_SK IS NOT NULL AND l.contactid &lt;&gt; c.contactid) THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.salentica.fact_lead l
+    LEFT JOIN Gold_Warehouse.salentica.dim_account a ON l.accountid_sk = a.account_SK
+    LEFT JOIN Gold_Warehouse.salentica.dim_contact_core c ON l.contactid_sk = c.contact_SK
+)
+SELECT ObjectRelationship, ObjectType, TotalRecords, Exact_NaturalKey_Match_Count, Defect_Orphan_Unmapped_SK, Defect_Wrong_Account_Mismatch,
+    CASE WHEN Defect_Orphan_Unmapped_SK = 0 AND Defect_Wrong_Account_Mismatch = 0 THEN 'PASSED' ELSE 'FAILED' END AS TestStatus
+FROM SalenticaSKAudit;</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="54" customHeight="1">
+      <c r="A46" s="8" t="inlineStr">
+        <is>
+          <t>Salentica</t>
+        </is>
+      </c>
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>TC_SAL_GOLD_09</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="inlineStr">
+        <is>
+          <t>Fact Health &amp; Historical Retention</t>
+        </is>
+      </c>
+      <c r="D46" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t>salentica.fact_opportunity, fact_lead, fact_investmentaccount</t>
+        </is>
+      </c>
+      <c r="F46" s="7" t="inlineStr">
+        <is>
+          <t>Verify CRM Fact Tables Health: Active SK mapping for fresh runs, historical closed version preservation for unrepeated rows, exact natural account match, and orphan SK detection</t>
+        </is>
+      </c>
+      <c r="G46" s="7" t="inlineStr">
+        <is>
+          <t>All 3 Salentica Fact tables loaded into Gold Warehouse</t>
+        </is>
+      </c>
+      <c r="H46" s="7" t="inlineStr">
+        <is>
+          <t>Fresh records map to active SK (iscurrent = 'True'), past records retain historical SK, Exact_Account_Match_Count covers all non-orphan rows, Defect_Orphan_Unmapped_SK = 0, Defect_Wrong_Account_Mismatch = 0. OverallStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="I46" s="18" t="inlineStr">
+        <is>
+          <t>;WITH MaxRuns AS (
+    SELECT 'fact_opportunity' AS TableName, MAX(load_timestamp) AS LatestRunTimestamp FROM Gold_Warehouse.salentica.fact_opportunity UNION ALL
+    SELECT 'fact_lead', MAX(load_timestamp) FROM Gold_Warehouse.salentica.fact_lead UNION ALL
+    SELECT 'fact_investmentaccount', MAX(load_timestamp) FROM Gold_Warehouse.salentica.fact_investmentaccount
+),
+FactBreakdown AS (
+    SELECT 'fact_opportunity' AS TableName, COUNT(*) AS TotalFactRows, MAX(f.AsOfDate) AS LatestBatchDate,
+        SUM(CASE WHEN f.load_timestamp = m.LatestRunTimestamp AND da.iscurrent = 'True' AND f.accountid = da.accountid THEN 1 ELSE 0 END) AS Fresh_Run_Active_Mapped,
+        SUM(CASE WHEN f.load_timestamp &lt; m.LatestRunTimestamp AND da.iscurrent = 'True' AND f.accountid = da.accountid THEN 1 ELSE 0 END) AS Past_Run_Active_Retained,
+        SUM(CASE WHEN f.load_timestamp &lt; m.LatestRunTimestamp AND da.iscurrent = 'False' AND f.accountid = da.accountid THEN 1 ELSE 0 END) AS Past_Run_Expired_Version_Retained,
+        SUM(CASE WHEN da.account_SK IS NOT NULL AND f.accountid = da.accountid THEN 1 ELSE 0 END) AS Exact_Account_Match_Count,
+        SUM(CASE WHEN f.accountid_sk = -1 OR da.account_SK IS NULL THEN 1 ELSE 0 END) AS Defect_Orphan_Unmapped_SK,
+        SUM(CASE WHEN da.account_SK IS NOT NULL AND f.accountid &lt;&gt; da.accountid THEN 1 ELSE 0 END) AS Defect_Wrong_Account_Mismatch
+    FROM Gold_Warehouse.salentica.fact_opportunity f
+    JOIN MaxRuns m ON m.TableName = 'fact_opportunity'
+    LEFT JOIN Gold_Warehouse.salentica.dim_account da ON f.accountid_sk = da.account_SK
+    GROUP BY m.LatestRunTimestamp
+    UNION ALL
+    SELECT 'fact_lead', COUNT(*), MAX(f.AsOfDate),
+        SUM(CASE WHEN f.load_timestamp = m.LatestRunTimestamp AND da.iscurrent = 'True' AND f.accountid = da.accountid THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.load_timestamp &lt; m.LatestRunTimestamp AND da.iscurrent = 'True' AND f.accountid = da.accountid THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.load_timestamp &lt; m.LatestRunTimestamp AND da.iscurrent = 'False' AND f.accountid = da.accountid THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.account_SK IS NOT NULL AND f.accountid = da.accountid THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.accountid_sk = -1 OR da.account_SK IS NULL THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.account_SK IS NOT NULL AND f.accountid &lt;&gt; da.accountid THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.salentica.fact_lead f
+    JOIN MaxRuns m ON m.TableName = 'fact_lead'
+    LEFT JOIN Gold_Warehouse.salentica.dim_account da ON f.accountid_sk = da.account_SK
+    GROUP BY m.LatestRunTimestamp
+    UNION ALL
+    SELECT 'fact_investmentaccount', COUNT(*), MAX(f.AsOfDate),
+        SUM(CASE WHEN f.load_timestamp = m.LatestRunTimestamp AND da.iscurrent = 'True' AND f.si_family_sk = da.account_SK THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.load_timestamp &lt; m.LatestRunTimestamp AND da.iscurrent = 'True' AND f.si_family_sk = da.account_SK THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.load_timestamp &lt; m.LatestRunTimestamp AND da.iscurrent = 'False' AND f.si_family_sk = da.account_SK THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.account_SK IS NOT NULL THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.investmentaccount_SK = -1 THEN 1 ELSE 0 END),
+        0
+    FROM Gold_Warehouse.salentica.fact_investmentaccount f
+    JOIN MaxRuns m ON m.TableName = 'fact_investmentaccount'
+    LEFT JOIN Gold_Warehouse.salentica.dim_account da ON f.si_family_sk = da.account_SK
+    GROUP BY m.LatestRunTimestamp
+)
+SELECT TableName, TotalFactRows, LatestBatchDate, Fresh_Run_Active_Mapped, Past_Run_Active_Retained,
+    Past_Run_Expired_Version_Retained AS Historical_Closed_Version_Retained, Exact_Account_Match_Count,
+    Defect_Orphan_Unmapped_SK, Defect_Wrong_Account_Mismatch,
+    CASE WHEN Defect_Orphan_Unmapped_SK = 0 AND Defect_Wrong_Account_Mismatch = 0 THEN 'PASSED' ELSE 'FAILED' END AS OverallStatus,
+    CASE 
+        WHEN Defect_Orphan_Unmapped_SK &gt; 0 THEN CONCAT(Defect_Orphan_Unmapped_SK, ' Orphan Record(s) (SK = -1)')
+        WHEN Defect_Wrong_Account_Mismatch &gt; 0 THEN 'Account Mismatch Defect'
+        ELSE 'All Active &amp; Historical Records Correctly Preserved'
+    END AS Remarks
+FROM FactBreakdown;</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="54" customHeight="1">
+      <c r="A47" s="12" t="inlineStr">
+        <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B45" s="12" t="inlineStr">
+      <c r="B47" s="12" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_01</t>
         </is>
       </c>
-      <c r="C45" s="13" t="inlineStr">
+      <c r="C47" s="13" t="inlineStr">
         <is>
           <t>SCD2 Deduplication</t>
         </is>
       </c>
-      <c r="D45" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E45" s="10" t="inlineStr">
+      <c r="D47" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E47" s="10" t="inlineStr">
         <is>
           <t>tamarac.dim_account_information</t>
         </is>
       </c>
-      <c r="F45" s="11" t="inlineStr">
+      <c r="F47" s="11" t="inlineStr">
         <is>
           <t>Verify Active Deduplication on PK ['account_number'] (is_current = 'True')</t>
         </is>
       </c>
-      <c r="G45" s="11" t="inlineStr">
+      <c r="G47" s="11" t="inlineStr">
         <is>
           <t>dim_account_information populated</t>
         </is>
       </c>
-      <c r="H45" s="11" t="inlineStr">
+      <c r="H47" s="11" t="inlineStr">
         <is>
           <t>Zero duplicate active accounts. Exactly one is_current = 'True' row per account_number.</t>
         </is>
       </c>
-      <c r="I45" s="17" t="inlineStr">
+      <c r="I47" s="17" t="inlineStr">
         <is>
           <t>SELECT account_number, COUNT(*) AS ActiveDuplicateCount
 FROM Gold_Warehouse.tamarac.dim_account_information
@@ -3630,48 +3822,48 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="54" customHeight="1">
-      <c r="A46" s="8" t="inlineStr">
+    <row r="48" ht="54" customHeight="1">
+      <c r="A48" s="8" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B46" s="8" t="inlineStr">
+      <c r="B48" s="8" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_02</t>
         </is>
       </c>
-      <c r="C46" s="9" t="inlineStr">
+      <c r="C48" s="9" t="inlineStr">
         <is>
           <t>SK Uniqueness</t>
         </is>
       </c>
-      <c r="D46" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E46" s="6" t="inlineStr">
+      <c r="D48" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="inlineStr">
         <is>
           <t>tamarac.dim_account_information</t>
         </is>
       </c>
-      <c r="F46" s="7" t="inlineStr">
+      <c r="F48" s="7" t="inlineStr">
         <is>
           <t>Verify Primary Surrogate Key (account_information_SK) uniqueness across all records</t>
         </is>
       </c>
-      <c r="G46" s="7" t="inlineStr">
+      <c r="G48" s="7" t="inlineStr">
         <is>
           <t>dim_account_information populated</t>
         </is>
       </c>
-      <c r="H46" s="7" t="inlineStr">
+      <c r="H48" s="7" t="inlineStr">
         <is>
           <t>Surrogate key account_information_SK is strictly unique across all rows. Zero duplicates.</t>
         </is>
       </c>
-      <c r="I46" s="18" t="inlineStr">
+      <c r="I48" s="18" t="inlineStr">
         <is>
           <t>SELECT account_information_SK, COUNT(*) AS DuplicateCount
 FROM Gold_Warehouse.tamarac.dim_account_information
@@ -3680,48 +3872,48 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="54" customHeight="1">
-      <c r="A47" s="12" t="inlineStr">
+    <row r="49" ht="54" customHeight="1">
+      <c r="A49" s="12" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B47" s="12" t="inlineStr">
+      <c r="B49" s="12" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_03</t>
         </is>
       </c>
-      <c r="C47" s="13" t="inlineStr">
+      <c r="C49" s="13" t="inlineStr">
         <is>
           <t>Audit Columns</t>
         </is>
       </c>
-      <c r="D47" s="19" t="inlineStr">
+      <c r="D49" s="19" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E47" s="10" t="inlineStr">
+      <c r="E49" s="10" t="inlineStr">
         <is>
           <t>tamarac.dim_account_information</t>
         </is>
       </c>
-      <c r="F47" s="11" t="inlineStr">
+      <c r="F49" s="11" t="inlineStr">
         <is>
           <t>Verify file_business_date and updated_at populated on active Tamarac accounts</t>
         </is>
       </c>
-      <c r="G47" s="11" t="inlineStr">
+      <c r="G49" s="11" t="inlineStr">
         <is>
           <t>dim_account_information populated</t>
         </is>
       </c>
-      <c r="H47" s="11" t="inlineStr">
+      <c r="H49" s="11" t="inlineStr">
         <is>
           <t>file_business_date and updated_at are non-null and &lt;= current calendar date.</t>
         </is>
       </c>
-      <c r="I47" s="17" t="inlineStr">
+      <c r="I49" s="17" t="inlineStr">
         <is>
           <t>SELECT 
     COUNT(*) AS TotalRows,
@@ -3732,48 +3924,48 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="54" customHeight="1">
-      <c r="A48" s="8" t="inlineStr">
+    <row r="50" ht="54" customHeight="1">
+      <c r="A50" s="8" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B48" s="8" t="inlineStr">
+      <c r="B50" s="8" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_04</t>
         </is>
       </c>
-      <c r="C48" s="9" t="inlineStr">
+      <c r="C50" s="9" t="inlineStr">
         <is>
           <t>SCD2 Deduplication</t>
         </is>
       </c>
-      <c r="D48" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E48" s="6" t="inlineStr">
+      <c r="D50" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="inlineStr">
         <is>
           <t>tamarac.dim_account_model_allocation</t>
         </is>
       </c>
-      <c r="F48" s="7" t="inlineStr">
+      <c r="F50" s="7" t="inlineStr">
         <is>
           <t>Verify Active Deduplication on Composite PK ['account_number', 'model_name']</t>
         </is>
       </c>
-      <c r="G48" s="7" t="inlineStr">
+      <c r="G50" s="7" t="inlineStr">
         <is>
           <t>dim_account_model_allocation populated</t>
         </is>
       </c>
-      <c r="H48" s="7" t="inlineStr">
+      <c r="H50" s="7" t="inlineStr">
         <is>
           <t>Zero duplicate active model allocations per (account_number, model_name).</t>
         </is>
       </c>
-      <c r="I48" s="18" t="inlineStr">
+      <c r="I50" s="18" t="inlineStr">
         <is>
           <t>SELECT account_number, model_name, COUNT(*) AS ActiveDuplicateAllocations
 FROM Gold_Warehouse.tamarac.dim_account_model_allocation
@@ -3783,48 +3975,48 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="54" customHeight="1">
-      <c r="A49" s="12" t="inlineStr">
+    <row r="51" ht="54" customHeight="1">
+      <c r="A51" s="12" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B49" s="12" t="inlineStr">
+      <c r="B51" s="12" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_05</t>
         </is>
       </c>
-      <c r="C49" s="13" t="inlineStr">
+      <c r="C51" s="13" t="inlineStr">
         <is>
           <t>SK Uniqueness</t>
         </is>
       </c>
-      <c r="D49" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E49" s="10" t="inlineStr">
+      <c r="D51" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E51" s="10" t="inlineStr">
         <is>
           <t>tamarac.dim_account_model_allocation</t>
         </is>
       </c>
-      <c r="F49" s="11" t="inlineStr">
+      <c r="F51" s="11" t="inlineStr">
         <is>
           <t>Verify Primary Surrogate Key (account_model_SK) uniqueness</t>
         </is>
       </c>
-      <c r="G49" s="11" t="inlineStr">
+      <c r="G51" s="11" t="inlineStr">
         <is>
           <t>dim_account_model_allocation populated</t>
         </is>
       </c>
-      <c r="H49" s="11" t="inlineStr">
+      <c r="H51" s="11" t="inlineStr">
         <is>
           <t>account_model_SK is unique with zero NULL values.</t>
         </is>
       </c>
-      <c r="I49" s="17" t="inlineStr">
+      <c r="I51" s="17" t="inlineStr">
         <is>
           <t>SELECT account_model_SK, COUNT(*) AS DuplicateModelSK
 FROM Gold_Warehouse.tamarac.dim_account_model_allocation
@@ -3833,48 +4025,48 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="54" customHeight="1">
-      <c r="A50" s="8" t="inlineStr">
+    <row r="52" ht="54" customHeight="1">
+      <c r="A52" s="8" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B50" s="8" t="inlineStr">
+      <c r="B52" s="8" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_06</t>
         </is>
       </c>
-      <c r="C50" s="9" t="inlineStr">
+      <c r="C52" s="9" t="inlineStr">
         <is>
           <t>Cross-Table Linkage</t>
         </is>
       </c>
-      <c r="D50" s="19" t="inlineStr">
+      <c r="D52" s="19" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E50" s="6" t="inlineStr">
+      <c r="E52" s="6" t="inlineStr">
         <is>
           <t>tamarac.dim_account_model_allocation</t>
         </is>
       </c>
-      <c r="F50" s="7" t="inlineStr">
+      <c r="F52" s="7" t="inlineStr">
         <is>
           <t>Verify Cross-Table Linkage: Every account_number exists in dim_account_information</t>
         </is>
       </c>
-      <c r="G50" s="7" t="inlineStr">
+      <c r="G52" s="7" t="inlineStr">
         <is>
           <t>dim_account_model_allocation populated</t>
         </is>
       </c>
-      <c r="H50" s="7" t="inlineStr">
+      <c r="H52" s="7" t="inlineStr">
         <is>
           <t>Zero orphan model allocation accounts. All account_number values exist in parent dimension.</t>
         </is>
       </c>
-      <c r="I50" s="18" t="inlineStr">
+      <c r="I52" s="18" t="inlineStr">
         <is>
           <t>SELECT COUNT(*) AS OrphanModelAllocations
 FROM Gold_Warehouse.tamarac.dim_account_model_allocation ma
@@ -3885,48 +4077,48 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="54" customHeight="1">
-      <c r="A51" s="12" t="inlineStr">
+    <row r="53" ht="54" customHeight="1">
+      <c r="A53" s="12" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B51" s="12" t="inlineStr">
+      <c r="B53" s="12" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_07</t>
         </is>
       </c>
-      <c r="C51" s="13" t="inlineStr">
+      <c r="C53" s="13" t="inlineStr">
         <is>
           <t>SCD2 Date Validation</t>
         </is>
       </c>
-      <c r="D51" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E51" s="10" t="inlineStr">
+      <c r="D53" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E53" s="10" t="inlineStr">
         <is>
           <t>tamarac.dim_account_information</t>
         </is>
       </c>
-      <c r="F51" s="11" t="inlineStr">
+      <c r="F53" s="11" t="inlineStr">
         <is>
           <t>Verify Inactive End Date Rule: effective_end_date &lt;= (MAX(file_business_date) - 1 day) and non-null</t>
         </is>
       </c>
-      <c r="G51" s="11" t="inlineStr">
+      <c r="G53" s="11" t="inlineStr">
         <is>
           <t>dim_account_information populated with inactive records</t>
         </is>
       </c>
-      <c r="H51" s="11" t="inlineStr">
+      <c r="H53" s="11" t="inlineStr">
         <is>
           <t>Exceeded_Cutoff_Count = 0, Null_End_Date_Count = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I51" s="17" t="inlineStr">
+      <c r="I53" s="17" t="inlineStr">
         <is>
           <t>SELECT 
     'dim_account_information' AS TableName,
@@ -3946,48 +4138,48 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="54" customHeight="1">
-      <c r="A52" s="8" t="inlineStr">
+    <row r="54" ht="54" customHeight="1">
+      <c r="A54" s="8" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B52" s="8" t="inlineStr">
+      <c r="B54" s="8" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_08</t>
         </is>
       </c>
-      <c r="C52" s="9" t="inlineStr">
+      <c r="C54" s="9" t="inlineStr">
         <is>
           <t>SCD2 Date Validation</t>
         </is>
       </c>
-      <c r="D52" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E52" s="6" t="inlineStr">
+      <c r="D54" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="inlineStr">
         <is>
           <t>tamarac.dim_account_model_allocation</t>
         </is>
       </c>
-      <c r="F52" s="7" t="inlineStr">
+      <c r="F54" s="7" t="inlineStr">
         <is>
           <t>Verify Inactive End Date Rule: effective_end_date &lt;= (MAX(file_business_date) - 1 day) and non-null</t>
         </is>
       </c>
-      <c r="G52" s="7" t="inlineStr">
+      <c r="G54" s="7" t="inlineStr">
         <is>
           <t>dim_account_model_allocation populated with inactive records</t>
         </is>
       </c>
-      <c r="H52" s="7" t="inlineStr">
+      <c r="H54" s="7" t="inlineStr">
         <is>
           <t>Exceeded_Cutoff_Count = 0, Null_End_Date_Count = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I52" s="18" t="inlineStr">
+      <c r="I54" s="18" t="inlineStr">
         <is>
           <t>SELECT 
     'dim_account_model_allocation' AS TableName,
@@ -4007,48 +4199,48 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="54" customHeight="1">
-      <c r="A53" s="12" t="inlineStr">
+    <row r="55" ht="54" customHeight="1">
+      <c r="A55" s="12" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B53" s="12" t="inlineStr">
+      <c r="B55" s="12" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_09</t>
         </is>
       </c>
-      <c r="C53" s="13" t="inlineStr">
+      <c r="C55" s="13" t="inlineStr">
         <is>
           <t>SCD2 Timeline &amp; SK Monotonicity</t>
         </is>
       </c>
-      <c r="D53" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E53" s="10" t="inlineStr">
+      <c r="D55" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E55" s="10" t="inlineStr">
         <is>
           <t>tamarac.dim_account_information</t>
         </is>
       </c>
-      <c r="F53" s="11" t="inlineStr">
+      <c r="F55" s="11" t="inlineStr">
         <is>
           <t>Verify SCD2 Timeline Continuity (Zero Gaps, Zero Overlaps) &amp; SK Monotonic Increment</t>
         </is>
       </c>
-      <c r="G53" s="11" t="inlineStr">
+      <c r="G55" s="11" t="inlineStr">
         <is>
           <t>dim_account_information with multiple versions per account_number</t>
         </is>
       </c>
-      <c r="H53" s="11" t="inlineStr">
+      <c r="H55" s="11" t="inlineStr">
         <is>
           <t>Timeline_Gap_Or_Overlap_Count = 0, SK_Non_Incrementing_Violation_Count = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I53" s="17" t="inlineStr">
+      <c r="I55" s="17" t="inlineStr">
         <is>
           <t>;WITH InfoTimeline AS (
     SELECT 
@@ -4076,48 +4268,48 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="54" customHeight="1">
-      <c r="A54" s="8" t="inlineStr">
+    <row r="56" ht="54" customHeight="1">
+      <c r="A56" s="8" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B54" s="8" t="inlineStr">
+      <c r="B56" s="8" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_10</t>
         </is>
       </c>
-      <c r="C54" s="9" t="inlineStr">
+      <c r="C56" s="9" t="inlineStr">
         <is>
           <t>SCD2 Timeline &amp; SK Monotonicity</t>
         </is>
       </c>
-      <c r="D54" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E54" s="6" t="inlineStr">
+      <c r="D56" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E56" s="6" t="inlineStr">
         <is>
           <t>tamarac.dim_account_model_allocation</t>
         </is>
       </c>
-      <c r="F54" s="7" t="inlineStr">
+      <c r="F56" s="7" t="inlineStr">
         <is>
           <t>Verify SCD2 Timeline Continuity (Zero Gaps, Zero Overlaps) &amp; SK Monotonic Increment</t>
         </is>
       </c>
-      <c r="G54" s="7" t="inlineStr">
+      <c r="G56" s="7" t="inlineStr">
         <is>
           <t>dim_account_model_allocation with multiple versions per composite key</t>
         </is>
       </c>
-      <c r="H54" s="7" t="inlineStr">
+      <c r="H56" s="7" t="inlineStr">
         <is>
           <t>Timeline_Gap_Or_Overlap_Count = 0, SK_Non_Incrementing_Violation_Count = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I54" s="18" t="inlineStr">
+      <c r="I56" s="18" t="inlineStr">
         <is>
           <t>;WITH ModelTimeline AS (
     SELECT 
@@ -4146,48 +4338,48 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="54" customHeight="1">
-      <c r="A55" s="12" t="inlineStr">
+    <row r="57" ht="54" customHeight="1">
+      <c r="A57" s="12" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B55" s="12" t="inlineStr">
+      <c r="B57" s="12" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_11</t>
         </is>
       </c>
-      <c r="C55" s="13" t="inlineStr">
+      <c r="C57" s="13" t="inlineStr">
         <is>
           <t>Date Sanity &amp; Inversions</t>
         </is>
       </c>
-      <c r="D55" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E55" s="10" t="inlineStr">
+      <c r="D57" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E57" s="10" t="inlineStr">
         <is>
           <t>tamarac.dim_account_information</t>
         </is>
       </c>
-      <c r="F55" s="11" t="inlineStr">
+      <c r="F57" s="11" t="inlineStr">
         <is>
           <t>Verify Date Sanity: Zero inverted dates (start &gt; end) and active records have non-future start dates</t>
         </is>
       </c>
-      <c r="G55" s="11" t="inlineStr">
+      <c r="G57" s="11" t="inlineStr">
         <is>
           <t>dim_account_information populated</t>
         </is>
       </c>
-      <c r="H55" s="11" t="inlineStr">
+      <c r="H57" s="11" t="inlineStr">
         <is>
           <t>Inverted_Date_Count = 0, Future_Active_Start_Date = 0, Null_Start_Date_Count = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I55" s="17" t="inlineStr">
+      <c r="I57" s="17" t="inlineStr">
         <is>
           <t>SELECT 
     'dim_account_information' AS TableName,
@@ -4205,48 +4397,48 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="54" customHeight="1">
-      <c r="A56" s="8" t="inlineStr">
+    <row r="58" ht="54" customHeight="1">
+      <c r="A58" s="8" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B56" s="8" t="inlineStr">
+      <c r="B58" s="8" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_12</t>
         </is>
       </c>
-      <c r="C56" s="9" t="inlineStr">
+      <c r="C58" s="9" t="inlineStr">
         <is>
           <t>Date Sanity &amp; Inversions</t>
         </is>
       </c>
-      <c r="D56" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E56" s="6" t="inlineStr">
+      <c r="D58" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="inlineStr">
         <is>
           <t>tamarac.dim_account_model_allocation</t>
         </is>
       </c>
-      <c r="F56" s="7" t="inlineStr">
+      <c r="F58" s="7" t="inlineStr">
         <is>
           <t>Verify Date Sanity: Zero inverted dates (start &gt; end) and active records have non-future start dates</t>
         </is>
       </c>
-      <c r="G56" s="7" t="inlineStr">
+      <c r="G58" s="7" t="inlineStr">
         <is>
           <t>dim_account_model_allocation populated</t>
         </is>
       </c>
-      <c r="H56" s="7" t="inlineStr">
+      <c r="H58" s="7" t="inlineStr">
         <is>
           <t>Inverted_Date_Count = 0, Future_Active_Start_Date = 0, Null_Start_Date_Count = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I56" s="18" t="inlineStr">
+      <c r="I58" s="18" t="inlineStr">
         <is>
           <t>SELECT 
     'dim_account_model_allocation' AS TableName,
@@ -4264,48 +4456,48 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="54" customHeight="1">
-      <c r="A57" s="12" t="inlineStr">
+    <row r="59" ht="54" customHeight="1">
+      <c r="A59" s="12" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B57" s="12" t="inlineStr">
+      <c r="B59" s="12" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_13</t>
         </is>
       </c>
-      <c r="C57" s="13" t="inlineStr">
+      <c r="C59" s="13" t="inlineStr">
         <is>
           <t>Open-Ended Active Records</t>
         </is>
       </c>
-      <c r="D57" s="19" t="inlineStr">
+      <c r="D59" s="19" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E57" s="10" t="inlineStr">
+      <c r="E59" s="10" t="inlineStr">
         <is>
           <t>tamarac.dim_account_information</t>
         </is>
       </c>
-      <c r="F57" s="11" t="inlineStr">
+      <c r="F59" s="11" t="inlineStr">
         <is>
           <t>Verify Active Records are Open-Ended (effective_end_date is NULL or '9999-12-31')</t>
         </is>
       </c>
-      <c r="G57" s="11" t="inlineStr">
+      <c r="G59" s="11" t="inlineStr">
         <is>
           <t>dim_account_information where is_current = 'True'</t>
         </is>
       </c>
-      <c r="H57" s="11" t="inlineStr">
+      <c r="H59" s="11" t="inlineStr">
         <is>
           <t>Prematurely_Ended_Active_Records = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I57" s="17" t="inlineStr">
+      <c r="I59" s="17" t="inlineStr">
         <is>
           <t>SELECT 
     'dim_account_information' AS TableName,
@@ -4320,48 +4512,48 @@
         </is>
       </c>
     </row>
-    <row r="58" ht="54" customHeight="1">
-      <c r="A58" s="8" t="inlineStr">
+    <row r="60" ht="54" customHeight="1">
+      <c r="A60" s="8" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B58" s="8" t="inlineStr">
+      <c r="B60" s="8" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_14</t>
         </is>
       </c>
-      <c r="C58" s="9" t="inlineStr">
+      <c r="C60" s="9" t="inlineStr">
         <is>
           <t>Open-Ended Active Records</t>
         </is>
       </c>
-      <c r="D58" s="19" t="inlineStr">
+      <c r="D60" s="19" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E58" s="6" t="inlineStr">
+      <c r="E60" s="6" t="inlineStr">
         <is>
           <t>tamarac.dim_account_model_allocation</t>
         </is>
       </c>
-      <c r="F58" s="7" t="inlineStr">
+      <c r="F60" s="7" t="inlineStr">
         <is>
           <t>Verify Active Records are Open-Ended (effective_end_date is NULL or '9999-12-31')</t>
         </is>
       </c>
-      <c r="G58" s="7" t="inlineStr">
+      <c r="G60" s="7" t="inlineStr">
         <is>
           <t>dim_account_model_allocation where is_current = 'True'</t>
         </is>
       </c>
-      <c r="H58" s="7" t="inlineStr">
+      <c r="H60" s="7" t="inlineStr">
         <is>
           <t>Prematurely_Ended_Active_Records = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I58" s="18" t="inlineStr">
+      <c r="I60" s="18" t="inlineStr">
         <is>
           <t>SELECT 
     'dim_account_model_allocation' AS TableName,
@@ -4376,48 +4568,48 @@
         </is>
       </c>
     </row>
-    <row r="59" ht="54" customHeight="1">
-      <c r="A59" s="12" t="inlineStr">
+    <row r="61" ht="54" customHeight="1">
+      <c r="A61" s="12" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B59" s="12" t="inlineStr">
+      <c r="B61" s="12" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_15</t>
         </is>
       </c>
-      <c r="C59" s="13" t="inlineStr">
+      <c r="C61" s="13" t="inlineStr">
         <is>
           <t>Version Evolution Audit</t>
         </is>
       </c>
-      <c r="D59" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E59" s="10" t="inlineStr">
+      <c r="D61" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E61" s="10" t="inlineStr">
         <is>
           <t>tamarac.dim_account_information</t>
         </is>
       </c>
-      <c r="F59" s="11" t="inlineStr">
+      <c r="F61" s="11" t="inlineStr">
         <is>
           <t>Verify Run Evolution: Every new run produces New Incremented SK, Advancing Start Date, and Latest Version is Active</t>
         </is>
       </c>
-      <c r="G59" s="11" t="inlineStr">
+      <c r="G61" s="11" t="inlineStr">
         <is>
           <t>dim_account_information with historical batch progression</t>
         </is>
       </c>
-      <c r="H59" s="11" t="inlineStr">
+      <c r="H61" s="11" t="inlineStr">
         <is>
           <t>Reused_Or_NonIncrementing_SK_Count = 0, NonAdvancing_EffectiveStartDate_Count = 0, Timeline_Gap_Or_Overlap_Count = 0, LatestVersion_Not_Active_Count = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I59" s="17" t="inlineStr">
+      <c r="I61" s="17" t="inlineStr">
         <is>
           <t>;WITH VersionChains AS (
     SELECT 
@@ -4451,48 +4643,48 @@
         </is>
       </c>
     </row>
-    <row r="60" ht="54" customHeight="1">
-      <c r="A60" s="8" t="inlineStr">
+    <row r="62" ht="54" customHeight="1">
+      <c r="A62" s="8" t="inlineStr">
         <is>
           <t>Tamarac</t>
         </is>
       </c>
-      <c r="B60" s="8" t="inlineStr">
+      <c r="B62" s="8" t="inlineStr">
         <is>
           <t>TC_TAM_GOLD_16</t>
         </is>
       </c>
-      <c r="C60" s="9" t="inlineStr">
+      <c r="C62" s="9" t="inlineStr">
         <is>
           <t>Version Evolution Audit</t>
         </is>
       </c>
-      <c r="D60" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E60" s="6" t="inlineStr">
+      <c r="D62" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E62" s="6" t="inlineStr">
         <is>
           <t>tamarac.dim_account_model_allocation</t>
         </is>
       </c>
-      <c r="F60" s="7" t="inlineStr">
+      <c r="F62" s="7" t="inlineStr">
         <is>
           <t>Verify Run Evolution: Every new run produces New Incremented SK, Advancing Start Date, and Latest Version is Active</t>
         </is>
       </c>
-      <c r="G60" s="7" t="inlineStr">
+      <c r="G62" s="7" t="inlineStr">
         <is>
           <t>dim_account_model_allocation with historical batch progression</t>
         </is>
       </c>
-      <c r="H60" s="7" t="inlineStr">
+      <c r="H62" s="7" t="inlineStr">
         <is>
           <t>Reused_Or_NonIncrementing_SK_Count = 0, NonAdvancing_EffectiveStartDate_Count = 0, Timeline_Gap_Or_Overlap_Count = 0, LatestVersion_Not_Active_Count = 0. TestStatus = 'PASSED'.</t>
         </is>
       </c>
-      <c r="I60" s="18" t="inlineStr">
+      <c r="I62" s="18" t="inlineStr">
         <is>
           <t>;WITH ModelChains AS (
     SELECT 
@@ -4527,48 +4719,48 @@
         </is>
       </c>
     </row>
-    <row r="61" ht="54" customHeight="1">
-      <c r="A61" s="12" t="inlineStr">
+    <row r="63" ht="54" customHeight="1">
+      <c r="A63" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B61" s="12" t="inlineStr">
+      <c r="B63" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_01</t>
         </is>
       </c>
-      <c r="C61" s="13" t="inlineStr">
+      <c r="C63" s="13" t="inlineStr">
         <is>
           <t>SCD2 Deduplication</t>
         </is>
       </c>
-      <c r="D61" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E61" s="10" t="inlineStr">
+      <c r="D63" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E63" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master</t>
         </is>
       </c>
-      <c r="F61" s="11" t="inlineStr">
+      <c r="F63" s="11" t="inlineStr">
         <is>
           <t>Verify Active Deduplication on Business Key ['customer_account_number'] (is_current = 1)</t>
         </is>
       </c>
-      <c r="G61" s="11" t="inlineStr">
+      <c r="G63" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master populated</t>
         </is>
       </c>
-      <c r="H61" s="11" t="inlineStr">
+      <c r="H63" s="11" t="inlineStr">
         <is>
           <t>Zero duplicate active accounts. Exactly one is_current = 1 record per customer_account_number.</t>
         </is>
       </c>
-      <c r="I61" s="17" t="inlineStr">
+      <c r="I63" s="17" t="inlineStr">
         <is>
           <t>SELECT customer_account_number, COUNT(*) AS ActiveDuplicateCount
 FROM Gold_Warehouse.innotrust.dim_account_master
@@ -4578,48 +4770,48 @@
         </is>
       </c>
     </row>
-    <row r="62" ht="54" customHeight="1">
-      <c r="A62" s="8" t="inlineStr">
+    <row r="64" ht="54" customHeight="1">
+      <c r="A64" s="8" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B62" s="8" t="inlineStr">
+      <c r="B64" s="8" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_02</t>
         </is>
       </c>
-      <c r="C62" s="9" t="inlineStr">
+      <c r="C64" s="9" t="inlineStr">
         <is>
           <t>SK Uniqueness</t>
         </is>
       </c>
-      <c r="D62" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E62" s="6" t="inlineStr">
+      <c r="D64" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E64" s="6" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master</t>
         </is>
       </c>
-      <c r="F62" s="7" t="inlineStr">
+      <c r="F64" s="7" t="inlineStr">
         <is>
           <t>Verify Primary Surrogate Key (dim_account_master_sk) uniqueness and non-null constraint</t>
         </is>
       </c>
-      <c r="G62" s="7" t="inlineStr">
+      <c r="G64" s="7" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master populated</t>
         </is>
       </c>
-      <c r="H62" s="7" t="inlineStr">
+      <c r="H64" s="7" t="inlineStr">
         <is>
           <t>dim_account_master_sk is strictly unique across all versions with zero NULL values.</t>
         </is>
       </c>
-      <c r="I62" s="18" t="inlineStr">
+      <c r="I64" s="18" t="inlineStr">
         <is>
           <t>SELECT dim_account_master_sk, COUNT(*) AS DuplicateCount
 FROM Gold_Warehouse.innotrust.dim_account_master
@@ -4633,48 +4825,48 @@
         </is>
       </c>
     </row>
-    <row r="63" ht="54" customHeight="1">
-      <c r="A63" s="12" t="inlineStr">
+    <row r="65" ht="54" customHeight="1">
+      <c r="A65" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B63" s="12" t="inlineStr">
+      <c r="B65" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_03</t>
         </is>
       </c>
-      <c r="C63" s="13" t="inlineStr">
+      <c r="C65" s="13" t="inlineStr">
         <is>
           <t>SCD2 Deduplication</t>
         </is>
       </c>
-      <c r="D63" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E63" s="10" t="inlineStr">
+      <c r="D65" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E65" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_account_category_codes</t>
         </is>
       </c>
-      <c r="F63" s="11" t="inlineStr">
+      <c r="F65" s="11" t="inlineStr">
         <is>
           <t>Verify Active Deduplication on Business Key ['account_category_code'] (is_current = 1)</t>
         </is>
       </c>
-      <c r="G63" s="11" t="inlineStr">
+      <c r="G65" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_account_category_codes populated</t>
         </is>
       </c>
-      <c r="H63" s="11" t="inlineStr">
+      <c r="H65" s="11" t="inlineStr">
         <is>
           <t>Zero duplicate active category codes per account_category_code.</t>
         </is>
       </c>
-      <c r="I63" s="17" t="inlineStr">
+      <c r="I65" s="17" t="inlineStr">
         <is>
           <t>SELECT account_category_code, COUNT(*) AS ActiveDuplicateCount
 FROM Gold_Warehouse.innotrust.dim_account_category_codes
@@ -4684,48 +4876,48 @@
         </is>
       </c>
     </row>
-    <row r="64" ht="54" customHeight="1">
-      <c r="A64" s="8" t="inlineStr">
+    <row r="66" ht="54" customHeight="1">
+      <c r="A66" s="8" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B64" s="8" t="inlineStr">
+      <c r="B66" s="8" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_04</t>
         </is>
       </c>
-      <c r="C64" s="9" t="inlineStr">
+      <c r="C66" s="9" t="inlineStr">
         <is>
           <t>SK Uniqueness</t>
         </is>
       </c>
-      <c r="D64" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E64" s="6" t="inlineStr">
+      <c r="D66" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E66" s="6" t="inlineStr">
         <is>
           <t>innotrust.dim_account_category_codes</t>
         </is>
       </c>
-      <c r="F64" s="7" t="inlineStr">
+      <c r="F66" s="7" t="inlineStr">
         <is>
           <t>Verify Primary Surrogate Key (dim_account_master_sk) uniqueness on dim_account_category_codes</t>
         </is>
       </c>
-      <c r="G64" s="7" t="inlineStr">
+      <c r="G66" s="7" t="inlineStr">
         <is>
           <t>innotrust.dim_account_category_codes populated</t>
         </is>
       </c>
-      <c r="H64" s="7" t="inlineStr">
+      <c r="H66" s="7" t="inlineStr">
         <is>
           <t>Surrogate key dim_account_master_sk is unique across all rows with zero NULLs.</t>
         </is>
       </c>
-      <c r="I64" s="18" t="inlineStr">
+      <c r="I66" s="18" t="inlineStr">
         <is>
           <t>SELECT dim_account_master_sk, COUNT(*) AS DuplicateCount
 FROM Gold_Warehouse.innotrust.dim_account_category_codes
@@ -4734,48 +4926,48 @@
         </is>
       </c>
     </row>
-    <row r="65" ht="54" customHeight="1">
-      <c r="A65" s="12" t="inlineStr">
+    <row r="67" ht="54" customHeight="1">
+      <c r="A67" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B65" s="12" t="inlineStr">
+      <c r="B67" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_05</t>
         </is>
       </c>
-      <c r="C65" s="13" t="inlineStr">
+      <c r="C67" s="13" t="inlineStr">
         <is>
           <t>SCD2 Deduplication</t>
         </is>
       </c>
-      <c r="D65" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E65" s="10" t="inlineStr">
+      <c r="D67" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E67" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_account_type_codes</t>
         </is>
       </c>
-      <c r="F65" s="11" t="inlineStr">
+      <c r="F67" s="11" t="inlineStr">
         <is>
           <t>Verify Active Deduplication on Business Key ['account_type_code'] (is_current = 1)</t>
         </is>
       </c>
-      <c r="G65" s="11" t="inlineStr">
+      <c r="G67" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_account_type_codes populated</t>
         </is>
       </c>
-      <c r="H65" s="11" t="inlineStr">
+      <c r="H67" s="11" t="inlineStr">
         <is>
           <t>Zero duplicate active account types per account_type_code.</t>
         </is>
       </c>
-      <c r="I65" s="17" t="inlineStr">
+      <c r="I67" s="17" t="inlineStr">
         <is>
           <t>SELECT account_type_code, COUNT(*) AS ActiveDuplicateCount
 FROM Gold_Warehouse.innotrust.dim_account_type_codes
@@ -4785,48 +4977,48 @@
         </is>
       </c>
     </row>
-    <row r="66" ht="54" customHeight="1">
-      <c r="A66" s="8" t="inlineStr">
+    <row r="68" ht="54" customHeight="1">
+      <c r="A68" s="8" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B66" s="8" t="inlineStr">
+      <c r="B68" s="8" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_06</t>
         </is>
       </c>
-      <c r="C66" s="9" t="inlineStr">
+      <c r="C68" s="9" t="inlineStr">
         <is>
           <t>SK Uniqueness</t>
         </is>
       </c>
-      <c r="D66" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E66" s="6" t="inlineStr">
+      <c r="D68" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E68" s="6" t="inlineStr">
         <is>
           <t>innotrust.dim_account_type_codes</t>
         </is>
       </c>
-      <c r="F66" s="7" t="inlineStr">
+      <c r="F68" s="7" t="inlineStr">
         <is>
           <t>Verify Primary Surrogate Key (dim_account_type_codes_sk) uniqueness and non-null constraint</t>
         </is>
       </c>
-      <c r="G66" s="7" t="inlineStr">
+      <c r="G68" s="7" t="inlineStr">
         <is>
           <t>innotrust.dim_account_type_codes populated</t>
         </is>
       </c>
-      <c r="H66" s="7" t="inlineStr">
+      <c r="H68" s="7" t="inlineStr">
         <is>
           <t>dim_account_type_codes_sk is strictly unique across all versions with zero NULLs.</t>
         </is>
       </c>
-      <c r="I66" s="18" t="inlineStr">
+      <c r="I68" s="18" t="inlineStr">
         <is>
           <t>SELECT dim_account_type_codes_sk, COUNT(*) AS DuplicateCount
 FROM Gold_Warehouse.innotrust.dim_account_type_codes
@@ -4835,48 +5027,48 @@
         </is>
       </c>
     </row>
-    <row r="67" ht="54" customHeight="1">
-      <c r="A67" s="12" t="inlineStr">
+    <row r="69" ht="54" customHeight="1">
+      <c r="A69" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B67" s="12" t="inlineStr">
+      <c r="B69" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_07</t>
         </is>
       </c>
-      <c r="C67" s="13" t="inlineStr">
+      <c r="C69" s="13" t="inlineStr">
         <is>
           <t>SCD2 Deduplication</t>
         </is>
       </c>
-      <c r="D67" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E67" s="10" t="inlineStr">
+      <c r="D69" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E69" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_master_sec_index</t>
         </is>
       </c>
-      <c r="F67" s="11" t="inlineStr">
+      <c r="F69" s="11" t="inlineStr">
         <is>
           <t>Verify Active Deduplication on Security Primary Key ['isin'] (is_current = 1)</t>
         </is>
       </c>
-      <c r="G67" s="11" t="inlineStr">
+      <c r="G69" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_master_sec_index populated</t>
         </is>
       </c>
-      <c r="H67" s="11" t="inlineStr">
+      <c r="H69" s="11" t="inlineStr">
         <is>
           <t>Zero duplicate active securities. Exactly one is_current = 1 record per isin.</t>
         </is>
       </c>
-      <c r="I67" s="17" t="inlineStr">
+      <c r="I69" s="17" t="inlineStr">
         <is>
           <t>SELECT isin, COUNT(*) AS ActiveDuplicateCount
 FROM Gold_Warehouse.innotrust.dim_master_sec_index
@@ -4886,48 +5078,48 @@
         </is>
       </c>
     </row>
-    <row r="68" ht="54" customHeight="1">
-      <c r="A68" s="8" t="inlineStr">
+    <row r="70" ht="54" customHeight="1">
+      <c r="A70" s="8" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B68" s="8" t="inlineStr">
+      <c r="B70" s="8" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_08</t>
         </is>
       </c>
-      <c r="C68" s="9" t="inlineStr">
+      <c r="C70" s="9" t="inlineStr">
         <is>
           <t>SK Uniqueness</t>
         </is>
       </c>
-      <c r="D68" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E68" s="6" t="inlineStr">
+      <c r="D70" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E70" s="6" t="inlineStr">
         <is>
           <t>innotrust.dim_master_sec_index</t>
         </is>
       </c>
-      <c r="F68" s="7" t="inlineStr">
+      <c r="F70" s="7" t="inlineStr">
         <is>
           <t>Verify Primary Surrogate Key (dim_master_sec_index_sk) uniqueness across all records</t>
         </is>
       </c>
-      <c r="G68" s="7" t="inlineStr">
+      <c r="G70" s="7" t="inlineStr">
         <is>
           <t>innotrust.dim_master_sec_index populated</t>
         </is>
       </c>
-      <c r="H68" s="7" t="inlineStr">
+      <c r="H70" s="7" t="inlineStr">
         <is>
           <t>dim_master_sec_index_sk is strictly unique across all versions with zero NULLs.</t>
         </is>
       </c>
-      <c r="I68" s="18" t="inlineStr">
+      <c r="I70" s="18" t="inlineStr">
         <is>
           <t>SELECT dim_master_sec_index_sk, COUNT(*) AS DuplicateCount
 FROM Gold_Warehouse.innotrust.dim_master_sec_index
@@ -4936,48 +5128,48 @@
         </is>
       </c>
     </row>
-    <row r="69" ht="54" customHeight="1">
-      <c r="A69" s="12" t="inlineStr">
+    <row r="71" ht="54" customHeight="1">
+      <c r="A71" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B69" s="12" t="inlineStr">
+      <c r="B71" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_09</t>
         </is>
       </c>
-      <c r="C69" s="13" t="inlineStr">
+      <c r="C71" s="13" t="inlineStr">
         <is>
           <t>SCD2 Deduplication</t>
         </is>
       </c>
-      <c r="D69" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E69" s="10" t="inlineStr">
+      <c r="D71" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E71" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_security_characteristics_codes</t>
         </is>
       </c>
-      <c r="F69" s="11" t="inlineStr">
+      <c r="F71" s="11" t="inlineStr">
         <is>
           <t>Verify Active Deduplication on Business Key ['security_type_code'] (is_current = 1)</t>
         </is>
       </c>
-      <c r="G69" s="11" t="inlineStr">
+      <c r="G71" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_security_characteristics_codes populated</t>
         </is>
       </c>
-      <c r="H69" s="11" t="inlineStr">
+      <c r="H71" s="11" t="inlineStr">
         <is>
           <t>Zero duplicate active security type codes per security_type_code.</t>
         </is>
       </c>
-      <c r="I69" s="17" t="inlineStr">
+      <c r="I71" s="17" t="inlineStr">
         <is>
           <t>SELECT security_type_code, COUNT(*) AS ActiveDuplicateCount
 FROM Gold_Warehouse.innotrust.dim_security_characteristics_codes
@@ -4987,48 +5179,48 @@
         </is>
       </c>
     </row>
-    <row r="70" ht="54" customHeight="1">
-      <c r="A70" s="8" t="inlineStr">
+    <row r="72" ht="54" customHeight="1">
+      <c r="A72" s="8" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B70" s="8" t="inlineStr">
+      <c r="B72" s="8" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_10</t>
         </is>
       </c>
-      <c r="C70" s="9" t="inlineStr">
+      <c r="C72" s="9" t="inlineStr">
         <is>
           <t>SK Uniqueness</t>
         </is>
       </c>
-      <c r="D70" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E70" s="6" t="inlineStr">
+      <c r="D72" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E72" s="6" t="inlineStr">
         <is>
           <t>innotrust.dim_security_characteristics_codes</t>
         </is>
       </c>
-      <c r="F70" s="7" t="inlineStr">
+      <c r="F72" s="7" t="inlineStr">
         <is>
           <t>Verify Primary Surrogate Key (dim_securitycharacteristicscodes) uniqueness and non-null constraint</t>
         </is>
       </c>
-      <c r="G70" s="7" t="inlineStr">
+      <c r="G72" s="7" t="inlineStr">
         <is>
           <t>innotrust.dim_security_characteristics_codes populated</t>
         </is>
       </c>
-      <c r="H70" s="7" t="inlineStr">
+      <c r="H72" s="7" t="inlineStr">
         <is>
           <t>dim_securitycharacteristicscodes is strictly unique across all versions with zero NULLs.</t>
         </is>
       </c>
-      <c r="I70" s="18" t="inlineStr">
+      <c r="I72" s="18" t="inlineStr">
         <is>
           <t>SELECT dim_securitycharacteristicscodes, COUNT(*) AS DuplicateCount
 FROM Gold_Warehouse.innotrust.dim_security_characteristics_codes
@@ -5037,102 +5229,101 @@
         </is>
       </c>
     </row>
-    <row r="71" ht="54" customHeight="1">
-      <c r="A71" s="12" t="inlineStr">
+    <row r="73" ht="54" customHeight="1">
+      <c r="A73" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B71" s="12" t="inlineStr">
+      <c r="B73" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_11</t>
         </is>
       </c>
-      <c r="C71" s="13" t="inlineStr">
-        <is>
-          <t>Audit &amp; Date Logic</t>
-        </is>
-      </c>
-      <c r="D71" s="19" t="inlineStr">
+      <c r="C73" s="13" t="inlineStr">
+        <is>
+          <t>Audit Columns</t>
+        </is>
+      </c>
+      <c r="D73" s="19" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E71" s="10" t="inlineStr">
+      <c r="E73" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master</t>
         </is>
       </c>
-      <c r="F71" s="11" t="inlineStr">
-        <is>
-          <t>Verify business_date, updated_at, effective_start_date &amp; effective_end_date integrity on active records</t>
-        </is>
-      </c>
-      <c r="G71" s="11" t="inlineStr">
+      <c r="F73" s="11" t="inlineStr">
+        <is>
+          <t>Verify business_date and updated_at audit column integrity on active records</t>
+        </is>
+      </c>
+      <c r="G73" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master populated</t>
         </is>
       </c>
-      <c r="H71" s="11" t="inlineStr">
-        <is>
-          <t>Zero NULLs in business_date or updated_at; effective_end_date &gt;= effective_start_date.</t>
-        </is>
-      </c>
-      <c r="I71" s="17" t="inlineStr">
+      <c r="H73" s="11" t="inlineStr">
+        <is>
+          <t>Zero NULLs in business_date or updated_at; business_date &lt;= current calendar date.</t>
+        </is>
+      </c>
+      <c r="I73" s="17" t="inlineStr">
         <is>
           <t>SELECT 
     COUNT(*) AS TotalActiveRows,
     SUM(CASE WHEN business_date IS NULL THEN 1 ELSE 0 END) AS Null_BusinessDate,
     SUM(CASE WHEN updated_at IS NULL THEN 1 ELSE 0 END) AS Null_UpdatedAt,
-    SUM(CASE WHEN effective_start_date IS NULL THEN 1 ELSE 0 END) AS Null_EffectiveStartDate,
-    SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) AS InvertedEffectiveDates
+    SUM(CASE WHEN business_date &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END) AS FutureBusinessDates
 FROM Gold_Warehouse.innotrust.dim_account_master
 WHERE is_current = 1;</t>
         </is>
       </c>
     </row>
-    <row r="72" ht="54" customHeight="1">
-      <c r="A72" s="8" t="inlineStr">
+    <row r="74" ht="54" customHeight="1">
+      <c r="A74" s="8" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B72" s="8" t="inlineStr">
+      <c r="B74" s="8" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_12</t>
         </is>
       </c>
-      <c r="C72" s="9" t="inlineStr">
+      <c r="C74" s="9" t="inlineStr">
         <is>
           <t>Cross-Table Linkage</t>
         </is>
       </c>
-      <c r="D72" s="19" t="inlineStr">
+      <c r="D74" s="19" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E72" s="6" t="inlineStr">
+      <c r="E74" s="6" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master</t>
         </is>
       </c>
-      <c r="F72" s="7" t="inlineStr">
+      <c r="F74" s="7" t="inlineStr">
         <is>
           <t>Verify Referential Integrity: account_category_code and account_type_code resolve to active codes</t>
         </is>
       </c>
-      <c r="G72" s="7" t="inlineStr">
+      <c r="G74" s="7" t="inlineStr">
         <is>
           <t>innotrust.dim_account_master populated</t>
         </is>
       </c>
-      <c r="H72" s="7" t="inlineStr">
+      <c r="H74" s="7" t="inlineStr">
         <is>
           <t>All non-null account_category_code and account_type_code exist in corresponding dimension code tables.</t>
         </is>
       </c>
-      <c r="I72" s="18" t="inlineStr">
+      <c r="I74" s="18" t="inlineStr">
         <is>
           <t>SELECT 
     SUM(CASE WHEN m.account_category_code IS NOT NULL AND cat.account_category_code IS NULL THEN 1 ELSE 0 END) AS Orphan_CategoryCodes,
@@ -5146,48 +5337,48 @@
         </is>
       </c>
     </row>
-    <row r="73" ht="54" customHeight="1">
-      <c r="A73" s="12" t="inlineStr">
+    <row r="75" ht="54" customHeight="1">
+      <c r="A75" s="12" t="inlineStr">
         <is>
           <t>Innotrust</t>
         </is>
       </c>
-      <c r="B73" s="12" t="inlineStr">
+      <c r="B75" s="12" t="inlineStr">
         <is>
           <t>TC_INNO_GOLD_13</t>
         </is>
       </c>
-      <c r="C73" s="13" t="inlineStr">
+      <c r="C75" s="13" t="inlineStr">
         <is>
           <t>Cross-Table Linkage</t>
         </is>
       </c>
-      <c r="D73" s="19" t="inlineStr">
+      <c r="D75" s="19" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E73" s="10" t="inlineStr">
+      <c r="E75" s="10" t="inlineStr">
         <is>
           <t>innotrust.dim_master_sec_index</t>
         </is>
       </c>
-      <c r="F73" s="11" t="inlineStr">
+      <c r="F75" s="11" t="inlineStr">
         <is>
           <t>Verify Security Referential Integrity: security_type_code resolves to active security characteristics</t>
         </is>
       </c>
-      <c r="G73" s="11" t="inlineStr">
+      <c r="G75" s="11" t="inlineStr">
         <is>
           <t>innotrust.dim_master_sec_index populated</t>
         </is>
       </c>
-      <c r="H73" s="11" t="inlineStr">
+      <c r="H75" s="11" t="inlineStr">
         <is>
           <t>All non-null security_type_code values exist in dim_security_characteristics_codes.</t>
         </is>
       </c>
-      <c r="I73" s="17" t="inlineStr">
+      <c r="I75" s="17" t="inlineStr">
         <is>
           <t>SELECT COUNT(*) AS Orphan_SecurityTypeCodes
 FROM Gold_Warehouse.innotrust.dim_master_sec_index s
@@ -5197,108 +5388,48 @@
         </is>
       </c>
     </row>
-    <row r="74" ht="54" customHeight="1">
-      <c r="A74" s="8" t="inlineStr">
-        <is>
-          <t>Innotrust</t>
-        </is>
-      </c>
-      <c r="B74" s="8" t="inlineStr">
-        <is>
-          <t>TC_INNO_GOLD_14</t>
-        </is>
-      </c>
-      <c r="C74" s="9" t="inlineStr">
-        <is>
-          <t>SCD2 Date Validation</t>
-        </is>
-      </c>
-      <c r="D74" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E74" s="6" t="inlineStr">
-        <is>
-          <t>innotrust.dim_account_master</t>
-        </is>
-      </c>
-      <c r="F74" s="7" t="inlineStr">
-        <is>
-          <t>Verify SCD2 Effective Date Rules: Inactive records effective_end_date &lt;= (Current Day - 1), non-null end date, and valid active start date</t>
-        </is>
-      </c>
-      <c r="G74" s="7" t="inlineStr">
-        <is>
-          <t>innotrust.dim_account_master populated with SCD2 tracking columns</t>
-        </is>
-      </c>
-      <c r="H74" s="7" t="inlineStr">
-        <is>
-          <t>Inactive_End_Date_Breach_Count = 0, Inactive_Missing_End_Date = 0, Active_Future_Start_Date = 0, Inverted_Date_Range_Count = 0. TestStatus = 'PASSED'.</t>
-        </is>
-      </c>
-      <c r="I74" s="18" t="inlineStr">
-        <is>
-          <t>SELECT 
-    'dim_account_master' AS TableName,
-    COUNT(*) AS TotalRecords,
-    SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END) AS Inactive_End_Date_Breach_Count,
-    SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END) AS Inactive_Missing_End_Date,
-    SUM(CASE WHEN is_current = 1 AND effective_start_date &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END) AS Active_Future_Start_Date,
-    SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) AS Inverted_Date_Range_Count,
-    CASE 
-        WHEN SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END) = 0
-         AND SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END) = 0
-         AND SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) = 0
-        THEN 'PASSED' ELSE 'FAILED'
-    END AS TestStatus
-FROM Gold_Warehouse.innotrust.dim_account_master;</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" ht="54" customHeight="1">
-      <c r="A75" s="12" t="inlineStr">
+    <row r="76" ht="54" customHeight="1">
+      <c r="A76" s="8" t="inlineStr">
         <is>
           <t>Black Diamond (Consolidated)</t>
         </is>
       </c>
-      <c r="B75" s="12" t="inlineStr">
+      <c r="B76" s="8" t="inlineStr">
         <is>
           <t>TC_COMB_SK_BD_01</t>
         </is>
       </c>
-      <c r="C75" s="13" t="inlineStr">
+      <c r="C76" s="9" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D75" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E75" s="10" t="inlineStr">
+      <c r="D76" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E76" s="6" t="inlineStr">
         <is>
           <t>All 9 Child &amp; Fact Tables (holdings, transactions, taxlots, class/segment, details, tags, team, targets)</t>
         </is>
       </c>
-      <c r="F75" s="11" t="inlineStr">
+      <c r="F76" s="7" t="inlineStr">
         <is>
           <t>Black Diamond: Cross-Object account_sk vs dim_accounts Natural Key (accountid == da.id) Verification - Executes a single consolidated UNION ALL query across all 9 child/fact tables to verify that the attached account_sk strictly points to the exact same account natural key (child.accountid == da.id). Guarantees zero wrong account links.</t>
         </is>
       </c>
-      <c r="G75" s="11" t="inlineStr">
+      <c r="G76" s="7" t="inlineStr">
         <is>
           <t>All Gold tables populated for Black Diamond</t>
         </is>
       </c>
-      <c r="H75" s="11" t="inlineStr">
+      <c r="H76" s="7" t="inlineStr">
         <is>
           <t>Duplicate_BusinessKey_Count = 0, MismatchedAccountIdCount = 0, Null_AccountSK_Count = 0, Orphan_AccountSK_Count = 0 across all 9 objects.</t>
         </is>
       </c>
-      <c r="I75" s="17" t="inlineStr">
+      <c r="I76" s="18" t="inlineStr">
         <is>
           <t>SELECT 
     'dim_accounts_classallocation' AS TableName, 
@@ -5407,48 +5538,48 @@
         </is>
       </c>
     </row>
-    <row r="76" ht="54" customHeight="1">
-      <c r="A76" s="8" t="inlineStr">
+    <row r="77" ht="54" customHeight="1">
+      <c r="A77" s="12" t="inlineStr">
         <is>
           <t>Schwab (Consolidated)</t>
         </is>
       </c>
-      <c r="B76" s="8" t="inlineStr">
+      <c r="B77" s="12" t="inlineStr">
         <is>
           <t>TC_COMB_SK_SC_02</t>
         </is>
       </c>
-      <c r="C76" s="9" t="inlineStr">
+      <c r="C77" s="13" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D76" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E76" s="6" t="inlineStr">
+      <c r="D77" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E77" s="10" t="inlineStr">
         <is>
           <t>All 8 Objects (dim_accounts &amp; 7 Fact Tables: recon_d1/d2, daily_closing, security, transactions, ult/uln lots)</t>
         </is>
       </c>
-      <c r="F76" s="7" t="inlineStr">
+      <c r="F77" s="11" t="inlineStr">
         <is>
           <t>Schwab: Consolidated Multi-Object SK Mapping, PK Deduplication &amp; Audit Date Health Check - Single unified query executing across all 8 Schwab Gold tables. Validates that every fact record's account_sk correctly matches dim_accounts on composite natural keys (account_id, custodian_id), confirms primary SK uniqueness, and ensures 100% audit dates populated.</t>
         </is>
       </c>
-      <c r="G76" s="7" t="inlineStr">
+      <c r="G77" s="11" t="inlineStr">
         <is>
           <t>All Gold tables populated for Schwab</t>
         </is>
       </c>
-      <c r="H76" s="7" t="inlineStr">
+      <c r="H77" s="11" t="inlineStr">
         <is>
           <t>Mismatched_AccountId_Count = 0 and Orphan_AccountSK_Count = 0 across all fact tables. All mapped account_sk strictly match the natural account_id.</t>
         </is>
       </c>
-      <c r="I76" s="18" t="inlineStr">
+      <c r="I77" s="17" t="inlineStr">
         <is>
           <t>SELECT 
     'fact_recon_position_d1' AS TableName,
@@ -5507,48 +5638,48 @@
         </is>
       </c>
     </row>
-    <row r="77" ht="54" customHeight="1">
-      <c r="A77" s="12" t="inlineStr">
+    <row r="78" ht="54" customHeight="1">
+      <c r="A78" s="8" t="inlineStr">
         <is>
           <t>Salentica CRM (Consolidated)</t>
         </is>
       </c>
-      <c r="B77" s="12" t="inlineStr">
+      <c r="B78" s="8" t="inlineStr">
         <is>
           <t>TC_COMB_SK_SAL_03</t>
         </is>
       </c>
-      <c r="C77" s="13" t="inlineStr">
+      <c r="C78" s="9" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D77" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E77" s="10" t="inlineStr">
+      <c r="D78" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E78" s="6" t="inlineStr">
         <is>
           <t>All 6 Core CRM Entities (dim_account, dim_contact_core, dim_family, fact_lead, fact_opportunity, fact_investmentaccount)</t>
         </is>
       </c>
-      <c r="F77" s="11" t="inlineStr">
+      <c r="F78" s="7" t="inlineStr">
         <is>
           <t>Salentica: Consolidated Point-in-Time Referential SK Mapping (Active &amp; Historical Mapping Validation) - Single unified query executing across all 6 core Salentica CRM tables. Validates that every attached foreign SK resolves to the same Natural Key in parent dimensions (allowing active OR expired parent versions to preserve point-in-time audit history) and checks for broken orphans.</t>
         </is>
       </c>
-      <c r="G77" s="11" t="inlineStr">
+      <c r="G78" s="7" t="inlineStr">
         <is>
           <t>All Gold tables populated for Salentica CRM</t>
         </is>
       </c>
-      <c r="H77" s="11" t="inlineStr">
+      <c r="H78" s="7" t="inlineStr">
         <is>
           <t>Mismatched_PrimaryContact_NK = 0, Mismatched_BusinessUnit_NK = 0, Broken_Orphan_Count = 0 across all 6 CRM tables.</t>
         </is>
       </c>
-      <c r="I77" s="17" t="inlineStr">
+      <c r="I78" s="18" t="inlineStr">
         <is>
           <t>SELECT 'dim_account' AS TableName, COUNT(*) AS TotalActiveRows,
     SUM(CASE WHEN a.primarycontactid IS NOT NULL AND a.primarycontactid_sk &lt;&gt; -1 AND a.primarycontactid &lt;&gt; c.contactid THEN 1 ELSE 0 END) AS Mismatched_PrimaryContact_NK,
@@ -5612,48 +5743,48 @@
         </is>
       </c>
     </row>
-    <row r="78" ht="54" customHeight="1">
-      <c r="A78" s="8" t="inlineStr">
+    <row r="79" ht="54" customHeight="1">
+      <c r="A79" s="12" t="inlineStr">
         <is>
           <t>Tamarac (Consolidated)</t>
         </is>
       </c>
-      <c r="B78" s="8" t="inlineStr">
+      <c r="B79" s="12" t="inlineStr">
         <is>
           <t>TC_COMB_SK_TAM_04</t>
         </is>
       </c>
-      <c r="C78" s="9" t="inlineStr">
+      <c r="C79" s="13" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D78" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E78" s="6" t="inlineStr">
+      <c r="D79" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E79" s="10" t="inlineStr">
         <is>
           <t>Both Tables (dim_account_information, dim_account_model_allocation)</t>
         </is>
       </c>
-      <c r="F78" s="7" t="inlineStr">
+      <c r="F79" s="11" t="inlineStr">
         <is>
           <t>Tamarac: Consolidated Multi-Object PK Deduplication, Primary SK &amp; Cross-Table Linkage - Single unified query validating SCD2 active uniqueness on exact PK columns (['account_number'] and ['account_number', 'model_name']), surrogate key uniqueness, and cross-table referential integrity between model allocations and accounts.</t>
         </is>
       </c>
-      <c r="G78" s="7" t="inlineStr">
+      <c r="G79" s="11" t="inlineStr">
         <is>
           <t>All Gold tables populated for Tamarac</t>
         </is>
       </c>
-      <c r="H78" s="7" t="inlineStr">
+      <c r="H79" s="11" t="inlineStr">
         <is>
           <t>PK_Active_Duplicates = 0, Duplicate_Primary_SK = 0, Orphan_Accounts = 0, Missing_BusinessDate = 0 across both tables.</t>
         </is>
       </c>
-      <c r="I78" s="18" t="inlineStr">
+      <c r="I79" s="17" t="inlineStr">
         <is>
           <t>SELECT 'dim_account_information' AS TableName, COUNT(*) AS TotalActiveRows,
     (SELECT COUNT(*) FROM (SELECT account_number FROM Gold_Warehouse.tamarac.dim_account_information WHERE is_current = 'True' GROUP BY account_number HAVING COUNT(*) &gt; 1) d) AS PK_Active_Duplicates,
@@ -5676,48 +5807,48 @@
         </is>
       </c>
     </row>
-    <row r="79" ht="54" customHeight="1">
-      <c r="A79" s="12" t="inlineStr">
+    <row r="80" ht="54" customHeight="1">
+      <c r="A80" s="8" t="inlineStr">
         <is>
           <t>Innotrust (Consolidated)</t>
         </is>
       </c>
-      <c r="B79" s="12" t="inlineStr">
+      <c r="B80" s="8" t="inlineStr">
         <is>
           <t>TC_COMB_SK_INNO_05</t>
         </is>
       </c>
-      <c r="C79" s="13" t="inlineStr">
+      <c r="C80" s="9" t="inlineStr">
         <is>
           <t>Consolidated Multi-Object SK Audit</t>
         </is>
       </c>
-      <c r="D79" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E79" s="10" t="inlineStr">
+      <c r="D80" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E80" s="6" t="inlineStr">
         <is>
           <t>All 5 Innotrust Dimensions (dim_account_master, category_codes, type_codes, sec_index, characteristics)</t>
         </is>
       </c>
-      <c r="F79" s="11" t="inlineStr">
+      <c r="F80" s="7" t="inlineStr">
         <is>
           <t>Innotrust: Consolidated Multi-Object PK Deduplication, Primary SK &amp; Cross-Dimension Linkage - Single unified query validating SCD2 active uniqueness on exact natural keys, primary surrogate key uniqueness, and cross-dimension referential integrity between master entities and classification codes.</t>
         </is>
       </c>
-      <c r="G79" s="11" t="inlineStr">
+      <c r="G80" s="7" t="inlineStr">
         <is>
           <t>All Gold tables populated for Innotrust</t>
         </is>
       </c>
-      <c r="H79" s="11" t="inlineStr">
+      <c r="H80" s="7" t="inlineStr">
         <is>
           <t>PK_Active_Duplicates = 0, Duplicate_Primary_SK = 0, Orphan_Foreign_References = 0, Missing_BusinessDate = 0 across all 5 Innotrust tables.</t>
         </is>
       </c>
-      <c r="I79" s="17" t="inlineStr">
+      <c r="I80" s="18" t="inlineStr">
         <is>
           <t>SELECT 'dim_account_master' AS TableName, COUNT(*) AS TotalActiveRows,
     (SELECT COUNT(*) FROM (SELECT customer_account_number FROM Gold_Warehouse.innotrust.dim_account_master WHERE is_current = 1 GROUP BY customer_account_number HAVING COUNT(*) &gt; 1) d) AS PK_Active_Duplicates,
@@ -5764,126 +5895,6 @@
     SUM(CASE WHEN business_date IS NULL THEN 1 ELSE 0 END),
     SUM(CASE WHEN updated_at IS NULL THEN 1 ELSE 0 END)
 FROM Gold_Warehouse.innotrust.dim_security_characteristics_codes WHERE is_current = 1;</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" ht="54" customHeight="1">
-      <c r="A80" s="8" t="inlineStr">
-        <is>
-          <t>Innotrust (Consolidated)</t>
-        </is>
-      </c>
-      <c r="B80" s="8" t="inlineStr">
-        <is>
-          <t>TC_COMB_SK_INNO_06</t>
-        </is>
-      </c>
-      <c r="C80" s="9" t="inlineStr">
-        <is>
-          <t>Consolidated Multi-Object SK Audit</t>
-        </is>
-      </c>
-      <c r="D80" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E80" s="6" t="inlineStr">
-        <is>
-          <t>All 5 Innotrust Dimensions (dim_account_master, category_codes, type_codes, sec_index, characteristics)</t>
-        </is>
-      </c>
-      <c r="F80" s="7" t="inlineStr">
-        <is>
-          <t>Innotrust: Consolidated Multi-Object SCD2 Effective Start &amp; End Date Audit (End Date &lt;= Today - 1) - Validates across all 5 Innotrust dimensions that inactive records (is_current = 0) have effective_end_date &lt;= (current day - 1), non-null end dates, active records have non-future start dates, and zero inverted date ranges.</t>
-        </is>
-      </c>
-      <c r="G80" s="7" t="inlineStr">
-        <is>
-          <t>All Gold tables populated for Innotrust</t>
-        </is>
-      </c>
-      <c r="H80" s="7" t="inlineStr">
-        <is>
-          <t>Inactive_End_Date_Breach_Count = 0, Inactive_Missing_End_Date = 0, Active_Future_Start_Date = 0, Inverted_Date_Range_Count = 0 across all 5 tables.</t>
-        </is>
-      </c>
-      <c r="I80" s="18" t="inlineStr">
-        <is>
-          <t>SELECT 
-    'dim_account_master' AS TableName,
-    COUNT(*) AS TotalRecords,
-    SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END) AS Inactive_End_Date_Breach_Count,
-    SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END) AS Inactive_Missing_End_Date,
-    SUM(CASE WHEN is_current = 1 AND effective_start_date &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END) AS Active_Future_Start_Date,
-    SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) AS Inverted_Date_Range_Count,
-    CASE 
-        WHEN SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END) = 0
-         AND SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END) = 0
-         AND SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) = 0
-        THEN 'PASSED' ELSE 'FAILED'
-    END AS TestStatus
-FROM Gold_Warehouse.innotrust.dim_account_master
-UNION ALL
-SELECT 
-    'dim_master_sec_index' AS TableName,
-    COUNT(*),
-    SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END),
-    SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END),
-    SUM(CASE WHEN is_current = 1 AND effective_start_date &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END),
-    SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END),
-    CASE 
-        WHEN SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END) = 0
-         AND SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END) = 0
-         AND SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) = 0
-        THEN 'PASSED' ELSE 'FAILED'
-    END
-FROM Gold_Warehouse.innotrust.dim_master_sec_index
-UNION ALL
-SELECT 
-    'dim_account_category_codes',
-    COUNT(*),
-    SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END),
-    SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END),
-    SUM(CASE WHEN is_current = 1 AND effective_start_date &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END),
-    SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END),
-    CASE 
-        WHEN SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END) = 0
-         AND SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END) = 0
-         AND SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) = 0
-        THEN 'PASSED' ELSE 'FAILED'
-    END
-FROM Gold_Warehouse.innotrust.dim_account_category_codes
-UNION ALL
-SELECT 
-    'dim_account_type_codes',
-    COUNT(*),
-    SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END),
-    SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END),
-    SUM(CASE WHEN is_current = 1 AND effective_start_date &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END),
-    SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END),
-    CASE 
-        WHEN SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END) = 0
-         AND SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END) = 0
-         AND SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) = 0
-        THEN 'PASSED' ELSE 'FAILED'
-    END
-FROM Gold_Warehouse.innotrust.dim_account_type_codes
-UNION ALL
-SELECT 
-    'dim_security_characteristics_codes',
-    COUNT(*),
-    SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END),
-    SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END),
-    SUM(CASE WHEN is_current = 1 AND effective_start_date &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END),
-    SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END),
-    CASE 
-        WHEN SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END) = 0
-         AND SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END) = 0
-         AND SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) = 0
-        THEN 'PASSED' ELSE 'FAILED'
-    END
-FROM Gold_Warehouse.innotrust.dim_security_characteristics_codes;</t>
         </is>
       </c>
     </row>
@@ -8120,7 +8131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -8515,6 +8526,188 @@
     SUM(CASE WHEN contactid IS NULL AND contactid_sk IS NULL THEN 1 ELSE 0 END) AS Improper_Null_ContactSK
 FROM Gold_Warehouse.salentica.fact_opportunity
 WHERE iscurrent = 'True';</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="54" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>TC_SAL_GOLD_08</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Foreign SK Referential Mapping</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>salentica (dim_account, dim_contact_core, fact_opportunity, fact_lead)</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Verify Consolidated SK Referential Mapping: Audits that all foreign SKs in dimensions and facts resolve to exact matching natural keys in parent entities</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>dim_account, dim_contact_core, dim_businessunit, fact_opportunity, fact_lead populated</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>Defect_Orphan_Unmapped_SK = 0 and Defect_Wrong_Account_Mismatch = 0 across all entities. Exact_NaturalKey_Match_Count covers 100% of rows. TestStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>;WITH SalenticaSKAudit AS (
+    SELECT 'dim_account (Contact &amp; BU Links)' AS ObjectRelationship, 'Dimension Table' AS ObjectType, COUNT(*) AS TotalRecords,
+        SUM(CASE WHEN (a.primarycontactid IS NOT NULL AND a.primarycontactid_sk &lt;&gt; -1 AND a.primarycontactid = c.contactid)
+                   OR (a.owningbusinessunit IS NOT NULL AND a.owningbusinessunit_sk &lt;&gt; -1 AND a.owningbusinessunit = bu.businessunitid) THEN 1 ELSE 0 END) AS Exact_NaturalKey_Match_Count,
+        SUM(CASE WHEN (a.primarycontactid IS NOT NULL AND (a.primarycontactid_sk = -1 OR c.contact_SK IS NULL))
+                   OR (a.owningbusinessunit IS NOT NULL AND (a.owningbusinessunit_sk = -1 OR bu.businessunit_SK IS NULL)) THEN 1 ELSE 0 END) AS Defect_Orphan_Unmapped_SK,
+        SUM(CASE WHEN (a.primarycontactid IS NOT NULL AND a.primarycontactid_sk &lt;&gt; -1 AND c.contact_SK IS NOT NULL AND a.primarycontactid &lt;&gt; c.contactid)
+                   OR (a.owningbusinessunit IS NOT NULL AND a.owningbusinessunit_sk &lt;&gt; -1 AND bu.businessunit_SK IS NOT NULL AND a.owningbusinessunit &lt;&gt; bu.businessunitid) THEN 1 ELSE 0 END) AS Defect_Wrong_Account_Mismatch
+    FROM Gold_Warehouse.salentica.dim_account a
+    LEFT JOIN Gold_Warehouse.salentica.dim_contact_core c ON a.primarycontactid_sk = c.contact_SK
+    LEFT JOIN Gold_Warehouse.salentica.dim_businessunit bu ON a.owningbusinessunit_sk = bu.businessunit_SK
+    UNION ALL
+    SELECT 'dim_contact_core (Account &amp; BU Links)', 'Dimension Table', COUNT(*),
+        SUM(CASE WHEN (c.accountid IS NOT NULL AND c.accountid_sk &lt;&gt; -1 AND c.accountid = a.accountid)
+                   OR (c.owningbusinessunit IS NOT NULL AND c.owningbusinessunit_sk &lt;&gt; -1 AND c.owningbusinessunit = bu.businessunitid) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN (c.accountid IS NOT NULL AND (c.accountid_sk = -1 OR a.account_SK IS NULL))
+                   OR (c.owningbusinessunit IS NOT NULL AND (c.owningbusinessunit_sk = -1 OR bu.businessunit_SK IS NULL)) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN (c.accountid IS NOT NULL AND c.accountid_sk &lt;&gt; -1 AND a.account_SK IS NOT NULL AND c.accountid &lt;&gt; a.accountid)
+                   OR (c.owningbusinessunit IS NOT NULL AND c.owningbusinessunit_sk &lt;&gt; -1 AND bu.businessunit_SK IS NOT NULL AND c.owningbusinessunit &lt;&gt; bu.businessunitid) THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.salentica.dim_contact_core c
+    LEFT JOIN Gold_Warehouse.salentica.dim_account a ON c.accountid_sk = a.account_SK
+    LEFT JOIN Gold_Warehouse.salentica.dim_businessunit bu ON c.owningbusinessunit_sk = bu.businessunit_SK
+    UNION ALL
+    SELECT 'fact_opportunity (Account &amp; Contact Links)', 'Fact Table', COUNT(*),
+        SUM(CASE WHEN (o.accountid IS NOT NULL AND o.accountid_sk &lt;&gt; -1 AND o.accountid = a.accountid)
+                   OR (o.contactid IS NOT NULL AND o.contactid_sk &lt;&gt; -1 AND o.contactid = c.contactid) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN (o.accountid IS NOT NULL AND (o.accountid_sk = -1 OR a.account_SK IS NULL))
+                   OR (o.contactid IS NOT NULL AND (o.contactid_sk = -1 OR c.contact_SK IS NULL)) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN (o.accountid IS NOT NULL AND o.accountid_sk &lt;&gt; -1 AND a.account_SK IS NOT NULL AND o.accountid &lt;&gt; a.accountid)
+                   OR (o.contactid IS NOT NULL AND o.contactid_sk &lt;&gt; -1 AND c.contact_SK IS NOT NULL AND o.contactid &lt;&gt; c.contactid) THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.salentica.fact_opportunity o
+    LEFT JOIN Gold_Warehouse.salentica.dim_account a ON o.accountid_sk = a.account_SK
+    LEFT JOIN Gold_Warehouse.salentica.dim_contact_core c ON o.contactid_sk = c.contact_SK
+    UNION ALL
+    SELECT 'fact_lead (Account &amp; Contact Links)', 'Fact Table', COUNT(*),
+        SUM(CASE WHEN (l.accountid IS NOT NULL AND l.accountid_sk &lt;&gt; -1 AND l.accountid = a.accountid)
+                   OR (l.contactid IS NOT NULL AND l.contactid_sk &lt;&gt; -1 AND l.contactid = c.contactid) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN (l.accountid IS NOT NULL AND (l.accountid_sk = -1 OR a.account_SK IS NULL))
+                   OR (l.contactid IS NOT NULL AND (l.contactid_sk = -1 OR c.contact_SK IS NULL)) THEN 1 ELSE 0 END),
+        SUM(CASE WHEN (l.accountid IS NOT NULL AND l.accountid_sk &lt;&gt; -1 AND a.account_SK IS NOT NULL AND l.accountid &lt;&gt; a.accountid)
+                   OR (l.contactid IS NOT NULL AND l.contactid_sk &lt;&gt; -1 AND c.contact_SK IS NOT NULL AND l.contactid &lt;&gt; c.contactid) THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.salentica.fact_lead l
+    LEFT JOIN Gold_Warehouse.salentica.dim_account a ON l.accountid_sk = a.account_SK
+    LEFT JOIN Gold_Warehouse.salentica.dim_contact_core c ON l.contactid_sk = c.contact_SK
+)
+SELECT ObjectRelationship, ObjectType, TotalRecords, Exact_NaturalKey_Match_Count, Defect_Orphan_Unmapped_SK, Defect_Wrong_Account_Mismatch,
+    CASE WHEN Defect_Orphan_Unmapped_SK = 0 AND Defect_Wrong_Account_Mismatch = 0 THEN 'PASSED' ELSE 'FAILED' END AS TestStatus
+FROM SalenticaSKAudit;</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="54" customHeight="1">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>TC_SAL_GOLD_09</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Fact Health &amp; Historical Retention</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>salentica.fact_opportunity, fact_lead, fact_investmentaccount</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>Verify CRM Fact Tables Health: Active SK mapping for fresh runs, historical closed version preservation for unrepeated rows, exact natural account match, and orphan SK detection</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>All 3 Salentica Fact tables loaded into Gold Warehouse</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>Fresh records map to active SK (iscurrent = 'True'), past records retain historical SK, Exact_Account_Match_Count covers all non-orphan rows, Defect_Orphan_Unmapped_SK = 0, Defect_Wrong_Account_Mismatch = 0. OverallStatus = 'PASSED'.</t>
+        </is>
+      </c>
+      <c r="H11" s="17" t="inlineStr">
+        <is>
+          <t>;WITH MaxRuns AS (
+    SELECT 'fact_opportunity' AS TableName, MAX(load_timestamp) AS LatestRunTimestamp FROM Gold_Warehouse.salentica.fact_opportunity UNION ALL
+    SELECT 'fact_lead', MAX(load_timestamp) FROM Gold_Warehouse.salentica.fact_lead UNION ALL
+    SELECT 'fact_investmentaccount', MAX(load_timestamp) FROM Gold_Warehouse.salentica.fact_investmentaccount
+),
+FactBreakdown AS (
+    SELECT 'fact_opportunity' AS TableName, COUNT(*) AS TotalFactRows, MAX(f.AsOfDate) AS LatestBatchDate,
+        SUM(CASE WHEN f.load_timestamp = m.LatestRunTimestamp AND da.iscurrent = 'True' AND f.accountid = da.accountid THEN 1 ELSE 0 END) AS Fresh_Run_Active_Mapped,
+        SUM(CASE WHEN f.load_timestamp &lt; m.LatestRunTimestamp AND da.iscurrent = 'True' AND f.accountid = da.accountid THEN 1 ELSE 0 END) AS Past_Run_Active_Retained,
+        SUM(CASE WHEN f.load_timestamp &lt; m.LatestRunTimestamp AND da.iscurrent = 'False' AND f.accountid = da.accountid THEN 1 ELSE 0 END) AS Past_Run_Expired_Version_Retained,
+        SUM(CASE WHEN da.account_SK IS NOT NULL AND f.accountid = da.accountid THEN 1 ELSE 0 END) AS Exact_Account_Match_Count,
+        SUM(CASE WHEN f.accountid_sk = -1 OR da.account_SK IS NULL THEN 1 ELSE 0 END) AS Defect_Orphan_Unmapped_SK,
+        SUM(CASE WHEN da.account_SK IS NOT NULL AND f.accountid &lt;&gt; da.accountid THEN 1 ELSE 0 END) AS Defect_Wrong_Account_Mismatch
+    FROM Gold_Warehouse.salentica.fact_opportunity f
+    JOIN MaxRuns m ON m.TableName = 'fact_opportunity'
+    LEFT JOIN Gold_Warehouse.salentica.dim_account da ON f.accountid_sk = da.account_SK
+    GROUP BY m.LatestRunTimestamp
+    UNION ALL
+    SELECT 'fact_lead', COUNT(*), MAX(f.AsOfDate),
+        SUM(CASE WHEN f.load_timestamp = m.LatestRunTimestamp AND da.iscurrent = 'True' AND f.accountid = da.accountid THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.load_timestamp &lt; m.LatestRunTimestamp AND da.iscurrent = 'True' AND f.accountid = da.accountid THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.load_timestamp &lt; m.LatestRunTimestamp AND da.iscurrent = 'False' AND f.accountid = da.accountid THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.account_SK IS NOT NULL AND f.accountid = da.accountid THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.accountid_sk = -1 OR da.account_SK IS NULL THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.account_SK IS NOT NULL AND f.accountid &lt;&gt; da.accountid THEN 1 ELSE 0 END)
+    FROM Gold_Warehouse.salentica.fact_lead f
+    JOIN MaxRuns m ON m.TableName = 'fact_lead'
+    LEFT JOIN Gold_Warehouse.salentica.dim_account da ON f.accountid_sk = da.account_SK
+    GROUP BY m.LatestRunTimestamp
+    UNION ALL
+    SELECT 'fact_investmentaccount', COUNT(*), MAX(f.AsOfDate),
+        SUM(CASE WHEN f.load_timestamp = m.LatestRunTimestamp AND da.iscurrent = 'True' AND f.si_family_sk = da.account_SK THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.load_timestamp &lt; m.LatestRunTimestamp AND da.iscurrent = 'True' AND f.si_family_sk = da.account_SK THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.load_timestamp &lt; m.LatestRunTimestamp AND da.iscurrent = 'False' AND f.si_family_sk = da.account_SK THEN 1 ELSE 0 END),
+        SUM(CASE WHEN da.account_SK IS NOT NULL THEN 1 ELSE 0 END),
+        SUM(CASE WHEN f.investmentaccount_SK = -1 THEN 1 ELSE 0 END),
+        0
+    FROM Gold_Warehouse.salentica.fact_investmentaccount f
+    JOIN MaxRuns m ON m.TableName = 'fact_investmentaccount'
+    LEFT JOIN Gold_Warehouse.salentica.dim_account da ON f.si_family_sk = da.account_SK
+    GROUP BY m.LatestRunTimestamp
+)
+SELECT TableName, TotalFactRows, LatestBatchDate, Fresh_Run_Active_Mapped, Past_Run_Active_Retained,
+    Past_Run_Expired_Version_Retained AS Historical_Closed_Version_Retained, Exact_Account_Match_Count,
+    Defect_Orphan_Unmapped_SK, Defect_Wrong_Account_Mismatch,
+    CASE WHEN Defect_Orphan_Unmapped_SK = 0 AND Defect_Wrong_Account_Mismatch = 0 THEN 'PASSED' ELSE 'FAILED' END AS OverallStatus,
+    CASE 
+        WHEN Defect_Orphan_Unmapped_SK &gt; 0 THEN CONCAT(Defect_Orphan_Unmapped_SK, ' Orphan Record(s) (SK = -1)')
+        WHEN Defect_Wrong_Account_Mismatch &gt; 0 THEN 'Account Mismatch Defect'
+        ELSE 'All Active &amp; Historical Records Correctly Preserved'
+    END AS Remarks
+FROM FactBreakdown;</t>
         </is>
       </c>
     </row>
@@ -9476,7 +9669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -10006,7 +10199,7 @@
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>Audit &amp; Date Logic</t>
+          <t>Audit Columns</t>
         </is>
       </c>
       <c r="C13" s="19" t="inlineStr">
@@ -10021,7 +10214,7 @@
       </c>
       <c r="E13" s="11" t="inlineStr">
         <is>
-          <t>Verify business_date, updated_at, effective_start_date &amp; effective_end_date integrity on active records</t>
+          <t>Verify business_date and updated_at audit column integrity on active records</t>
         </is>
       </c>
       <c r="F13" s="11" t="inlineStr">
@@ -10031,7 +10224,7 @@
       </c>
       <c r="G13" s="11" t="inlineStr">
         <is>
-          <t>Zero NULLs in business_date or updated_at; effective_end_date &gt;= effective_start_date.</t>
+          <t>Zero NULLs in business_date or updated_at; business_date &lt;= current calendar date.</t>
         </is>
       </c>
       <c r="H13" s="17" t="inlineStr">
@@ -10040,8 +10233,7 @@
     COUNT(*) AS TotalActiveRows,
     SUM(CASE WHEN business_date IS NULL THEN 1 ELSE 0 END) AS Null_BusinessDate,
     SUM(CASE WHEN updated_at IS NULL THEN 1 ELSE 0 END) AS Null_UpdatedAt,
-    SUM(CASE WHEN effective_start_date IS NULL THEN 1 ELSE 0 END) AS Null_EffectiveStartDate,
-    SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) AS InvertedEffectiveDates
+    SUM(CASE WHEN business_date &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END) AS FutureBusinessDates
 FROM Gold_Warehouse.innotrust.dim_account_master
 WHERE is_current = 1;</t>
         </is>
@@ -10140,61 +10332,6 @@
 LEFT JOIN Gold_Warehouse.innotrust.dim_security_characteristics_codes sc 
     ON s.security_type_code = sc.security_type_code AND sc.is_current = 1
 WHERE s.is_current = 1 AND s.security_type_code IS NOT NULL AND sc.security_type_code IS NULL;</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="54" customHeight="1">
-      <c r="A16" s="8" t="inlineStr">
-        <is>
-          <t>TC_INNO_GOLD_14</t>
-        </is>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>SCD2 Date Validation</t>
-        </is>
-      </c>
-      <c r="C16" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>innotrust.dim_account_master</t>
-        </is>
-      </c>
-      <c r="E16" s="7" t="inlineStr">
-        <is>
-          <t>Verify SCD2 Effective Date Rules: Inactive records effective_end_date &lt;= (Current Day - 1), non-null end date, and valid active start date</t>
-        </is>
-      </c>
-      <c r="F16" s="7" t="inlineStr">
-        <is>
-          <t>innotrust.dim_account_master populated with SCD2 tracking columns</t>
-        </is>
-      </c>
-      <c r="G16" s="7" t="inlineStr">
-        <is>
-          <t>Inactive_End_Date_Breach_Count = 0, Inactive_Missing_End_Date = 0, Active_Future_Start_Date = 0, Inverted_Date_Range_Count = 0. TestStatus = 'PASSED'.</t>
-        </is>
-      </c>
-      <c r="H16" s="18" t="inlineStr">
-        <is>
-          <t>SELECT 
-    'dim_account_master' AS TableName,
-    COUNT(*) AS TotalRecords,
-    SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END) AS Inactive_End_Date_Breach_Count,
-    SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END) AS Inactive_Missing_End_Date,
-    SUM(CASE WHEN is_current = 1 AND effective_start_date &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END) AS Active_Future_Start_Date,
-    SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) AS Inverted_Date_Range_Count,
-    CASE 
-        WHEN SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END) = 0
-         AND SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END) = 0
-         AND SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) = 0
-        THEN 'PASSED' ELSE 'FAILED'
-    END AS TestStatus
-FROM Gold_Warehouse.innotrust.dim_account_master;</t>
         </is>
       </c>
     </row>
@@ -10212,7 +10349,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -10764,122 +10901,6 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="110" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>TC_COMB_SK_INNO_06</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>Innotrust</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>All 5 Innotrust Dimensions (dim_account_master, category_codes, type_codes, sec_index, characteristics)</t>
-        </is>
-      </c>
-      <c r="D8" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E8" s="7" t="inlineStr">
-        <is>
-          <t>Innotrust: Consolidated Multi-Object SCD2 Effective Start &amp; End Date Audit (End Date &lt;= Today - 1)
-Validates across all 5 Innotrust dimensions that inactive records (is_current = 0) have effective_end_date &lt;= (current day - 1), non-null end dates, active records have non-future start dates, and zero inverted date ranges.</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>All Gold tables loaded for Innotrust</t>
-        </is>
-      </c>
-      <c r="G8" s="7" t="inlineStr">
-        <is>
-          <t>Inactive_End_Date_Breach_Count = 0, Inactive_Missing_End_Date = 0, Active_Future_Start_Date = 0, Inverted_Date_Range_Count = 0 across all 5 tables.</t>
-        </is>
-      </c>
-      <c r="H8" s="18" t="inlineStr">
-        <is>
-          <t>SELECT 
-    'dim_account_master' AS TableName,
-    COUNT(*) AS TotalRecords,
-    SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END) AS Inactive_End_Date_Breach_Count,
-    SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END) AS Inactive_Missing_End_Date,
-    SUM(CASE WHEN is_current = 1 AND effective_start_date &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END) AS Active_Future_Start_Date,
-    SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) AS Inverted_Date_Range_Count,
-    CASE 
-        WHEN SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END) = 0
-         AND SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END) = 0
-         AND SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) = 0
-        THEN 'PASSED' ELSE 'FAILED'
-    END AS TestStatus
-FROM Gold_Warehouse.innotrust.dim_account_master
-UNION ALL
-SELECT 
-    'dim_master_sec_index' AS TableName,
-    COUNT(*),
-    SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END),
-    SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END),
-    SUM(CASE WHEN is_current = 1 AND effective_start_date &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END),
-    SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END),
-    CASE 
-        WHEN SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END) = 0
-         AND SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END) = 0
-         AND SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) = 0
-        THEN 'PASSED' ELSE 'FAILED'
-    END
-FROM Gold_Warehouse.innotrust.dim_master_sec_index
-UNION ALL
-SELECT 
-    'dim_account_category_codes',
-    COUNT(*),
-    SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END),
-    SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END),
-    SUM(CASE WHEN is_current = 1 AND effective_start_date &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END),
-    SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END),
-    CASE 
-        WHEN SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END) = 0
-         AND SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END) = 0
-         AND SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) = 0
-        THEN 'PASSED' ELSE 'FAILED'
-    END
-FROM Gold_Warehouse.innotrust.dim_account_category_codes
-UNION ALL
-SELECT 
-    'dim_account_type_codes',
-    COUNT(*),
-    SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END),
-    SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END),
-    SUM(CASE WHEN is_current = 1 AND effective_start_date &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END),
-    SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END),
-    CASE 
-        WHEN SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END) = 0
-         AND SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END) = 0
-         AND SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) = 0
-        THEN 'PASSED' ELSE 'FAILED'
-    END
-FROM Gold_Warehouse.innotrust.dim_account_type_codes
-UNION ALL
-SELECT 
-    'dim_security_characteristics_codes',
-    COUNT(*),
-    SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END),
-    SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END),
-    SUM(CASE WHEN is_current = 1 AND effective_start_date &gt; CAST(GETDATE() AS DATE) THEN 1 ELSE 0 END),
-    SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END),
-    CASE 
-        WHEN SUM(CASE WHEN is_current = 0 AND effective_end_date &gt; DATEADD(day, -1, CAST(GETDATE() AS DATE)) THEN 1 ELSE 0 END) = 0
-         AND SUM(CASE WHEN is_current = 0 AND effective_end_date IS NULL THEN 1 ELSE 0 END) = 0
-         AND SUM(CASE WHEN effective_end_date &lt; effective_start_date THEN 1 ELSE 0 END) = 0
-        THEN 'PASSED' ELSE 'FAILED'
-    END
-FROM Gold_Warehouse.innotrust.dim_security_characteristics_codes;</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>

</xml_diff>

<commit_message>
chore: update Fabric SQL endpoint to tnixybw3f7kejjy4dnqgavvt64 and remove effective date checks from Innotrustf
</commit_message>
<xml_diff>
--- a/Gold_Data_Validation_Test_Cases.xlsx
+++ b/Gold_Data_Validation_Test_Cases.xlsx
@@ -5852,7 +5852,7 @@
         <is>
           <t>SELECT 'dim_account_master' AS TableName, COUNT(*) AS TotalActiveRows,
     (SELECT COUNT(*) FROM (SELECT customer_account_number FROM Gold_Warehouse.innotrust.dim_account_master WHERE is_current = 1 GROUP BY customer_account_number HAVING COUNT(*) &gt; 1) d) AS PK_Active_Duplicates,
-    (COUNT(*) - COUNT(DISTINCT dim_account_master_sk)) AS Duplicate_Primary_SK,
+    (COUNT(*) - COUNT(DISTINCT m.dim_account_master_sk)) AS Duplicate_Primary_SK,
     SUM(CASE WHEN (m.account_category_code IS NOT NULL AND cat.account_category_code IS NULL)
                OR (m.account_type_code IS NOT NULL AND typ.account_type_code IS NULL) THEN 1 ELSE 0 END) AS Orphan_Foreign_References,
     SUM(CASE WHEN m.business_date IS NULL THEN 1 ELSE 0 END) AS Missing_BusinessDate,
@@ -5880,7 +5880,7 @@
 UNION ALL
 SELECT 'dim_master_sec_index', COUNT(*),
     (SELECT COUNT(*) FROM (SELECT isin FROM Gold_Warehouse.innotrust.dim_master_sec_index WHERE is_current = 1 GROUP BY isin HAVING COUNT(*) &gt; 1) d),
-    (COUNT(*) - COUNT(DISTINCT dim_master_sec_index_sk)),
+    (COUNT(*) - COUNT(DISTINCT s.dim_master_sec_index_sk)),
     SUM(CASE WHEN s.security_type_code IS NOT NULL AND sc.security_type_code IS NULL THEN 1 ELSE 0 END),
     SUM(CASE WHEN s.business_date IS NULL THEN 1 ELSE 0 END),
     SUM(CASE WHEN s.updated_at IS NULL THEN 1 ELSE 0 END)
@@ -10855,7 +10855,7 @@
         <is>
           <t>SELECT 'dim_account_master' AS TableName, COUNT(*) AS TotalActiveRows,
     (SELECT COUNT(*) FROM (SELECT customer_account_number FROM Gold_Warehouse.innotrust.dim_account_master WHERE is_current = 1 GROUP BY customer_account_number HAVING COUNT(*) &gt; 1) d) AS PK_Active_Duplicates,
-    (COUNT(*) - COUNT(DISTINCT dim_account_master_sk)) AS Duplicate_Primary_SK,
+    (COUNT(*) - COUNT(DISTINCT m.dim_account_master_sk)) AS Duplicate_Primary_SK,
     SUM(CASE WHEN (m.account_category_code IS NOT NULL AND cat.account_category_code IS NULL)
                OR (m.account_type_code IS NOT NULL AND typ.account_type_code IS NULL) THEN 1 ELSE 0 END) AS Orphan_Foreign_References,
     SUM(CASE WHEN m.business_date IS NULL THEN 1 ELSE 0 END) AS Missing_BusinessDate,
@@ -10883,7 +10883,7 @@
 UNION ALL
 SELECT 'dim_master_sec_index', COUNT(*),
     (SELECT COUNT(*) FROM (SELECT isin FROM Gold_Warehouse.innotrust.dim_master_sec_index WHERE is_current = 1 GROUP BY isin HAVING COUNT(*) &gt; 1) d),
-    (COUNT(*) - COUNT(DISTINCT dim_master_sec_index_sk)),
+    (COUNT(*) - COUNT(DISTINCT s.dim_master_sec_index_sk)),
     SUM(CASE WHEN s.security_type_code IS NOT NULL AND sc.security_type_code IS NULL THEN 1 ELSE 0 END),
     SUM(CASE WHEN s.business_date IS NULL THEN 1 ELSE 0 END),
     SUM(CASE WHEN s.updated_at IS NULL THEN 1 ELSE 0 END)

</xml_diff>